<commit_message>
Format participant column: one line per timestamped response, wrapped, one row per participant
- Each response on its own line within a single cell (newline-separated)
- Enable text wrapping and match the original Transcript column width
- Keeps one row per participant for per-participant scoring
</commit_message>
<xml_diff>
--- a/Transcripts_participant_only.xlsx
+++ b/Transcripts_participant_only.xlsx
@@ -45,10 +45,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -451,6 +454,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="142.5" customWidth="1" min="1" max="1"/>
+    <col width="142.5" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -479,9 +483,19 @@
       <c r="B2" t="n">
         <v>14140</v>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>00:22 Hi. It's been raining a lot, so the weather is pretty bad today.  00:38 So right now I'm doing a bonus quiz. So I'm pretty excited about that and I'm happy to learn more about this.  00:59 No, it's something fun and it's to boost my grades. So it feels pretty good.  01:17 So it's about AI. So that feels pretty fun. But actually I want to talk to you about something. So I actually had a tough situation recently in a team project.  01:44 Yeah. So were in my last subject, we had to make a team presentation for our grade and it was pretty important for the grade. And were about four people in the team. I was one of them. And at the end we only had three people presenting. Oh no, were five at the beginning and then we ended up only being two.  02:21 Yeah, so what's important, I think is to be good in time and prepare a lot in advance so nobody has to take over your work within a few hours. However, that was exactly what happened. One guy, he was sick. Then he gave us his part of the presentation at 2am the day before the presentation. So that was pretty challenging. But we did divided the work and we did the best we could and I feel like we succeeded pretty well and the grade was fine.  03:11 Yeah, no, it's. I think we managed pretty well. And I talked to the tutor as well to get some understanding from his point. So that was great.  03:35 Yeah, exactly. No, it was very good. So the problem in general was that at one point, we knew all along that one person wasn't going to be able to present. So she did her part and gave it to us in time. But then there was this other guy who got a heavy fever and handed his work to us only a few hours before. So that was the main challenge.  04:16 Yeah, definitely. And I think you learn a lot from these type of experiences. So whatever challenge you meet, I feel like you learn how to tackle it and you get experience on how to do it the next time.  04:50 Yes, absolutely.  05:13 Yes. Thank you.</t>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>00:22 Hi. It's been raining a lot, so the weather is pretty bad today.
+00:38 So right now I'm doing a bonus quiz. So I'm pretty excited about that and I'm happy to learn more about this.
+00:59 No, it's something fun and it's to boost my grades. So it feels pretty good.
+01:17 So it's about AI. So that feels pretty fun. But actually I want to talk to you about something. So I actually had a tough situation recently in a team project.
+01:44 Yeah. So were in my last subject, we had to make a team presentation for our grade and it was pretty important for the grade. And were about four people in the team. I was one of them. And at the end we only had three people presenting. Oh no, were five at the beginning and then we ended up only being two.
+02:21 Yeah, so what's important, I think is to be good in time and prepare a lot in advance so nobody has to take over your work within a few hours. However, that was exactly what happened. One guy, he was sick. Then he gave us his part of the presentation at 2am the day before the presentation. So that was pretty challenging. But we did divided the work and we did the best we could and I feel like we succeeded pretty well and the grade was fine.
+03:11 Yeah, no, it's. I think we managed pretty well. And I talked to the tutor as well to get some understanding from his point. So that was great.
+03:35 Yeah, exactly. No, it was very good. So the problem in general was that at one point, we knew all along that one person wasn't going to be able to present. So she did her part and gave it to us in time. But then there was this other guy who got a heavy fever and handed his work to us only a few hours before. So that was the main challenge.
+04:16 Yeah, definitely. And I think you learn a lot from these type of experiences. So whatever challenge you meet, I feel like you learn how to tackle it and you get experience on how to do it the next time.
+04:50 Yes, absolutely.
+05:13 Yes. Thank you.</t>
         </is>
       </c>
     </row>
@@ -494,9 +508,18 @@
       <c r="B3" t="n">
         <v>14965</v>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>00:28 Hey, I'm Victor. Nice to meet you. How's your day?  00:44 Also interesting. Nice weather outside. And yeah, I'm here because I'm actually wanted to talk about something. Something challenging that happened in the past. And I just needed a good ear to listen to what I'm saying.  01:12 Okay, so where do I start? We had family problems in the family, and now I've been getting the opportunity to reconcile with the part of the family we had problems with. And they want to meet up, which is kind of challenging for me because I don't know how to feel about it.  01:51 It's trying to set a date on where to meet, on when to meet. Because I remember the day we parted a bit and thinking about the situation makes me feel a bit uncomfortable. Even though I want to give them the chance again to get to know them in a other way because now I'm grown up.  02:37 Yeah, I suggested them in like a month and for one and a half days. But I am scared. It's maybe too much or maybe too less. I don't know. Because the person is coming all the way to me.  03:18 Maybe walking around or going for coffee or something like this, or sitting in the park. Because there's a lot of things we have to talk about that happened in the past.  03:52 Yeah, I agree. That's a good point. And I hope everything will go well, because I'm kind of scared that in the moment I feel very uncomfortable because of what happened.  04:28 And what could I do in case it gets awkward?  04:59 Okay. Yeah, that makes a lot of sense. Thank you so much for listening to me. I appreciate it.  05:17 Yes. Thank you. Hello. Hello.</t>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>00:28 Hey, I'm Victor. Nice to meet you. How's your day?
+00:44 Also interesting. Nice weather outside. And yeah, I'm here because I'm actually wanted to talk about something. Something challenging that happened in the past. And I just needed a good ear to listen to what I'm saying.
+01:12 Okay, so where do I start? We had family problems in the family, and now I've been getting the opportunity to reconcile with the part of the family we had problems with. And they want to meet up, which is kind of challenging for me because I don't know how to feel about it.
+01:51 It's trying to set a date on where to meet, on when to meet. Because I remember the day we parted a bit and thinking about the situation makes me feel a bit uncomfortable. Even though I want to give them the chance again to get to know them in a other way because now I'm grown up.
+02:37 Yeah, I suggested them in like a month and for one and a half days. But I am scared. It's maybe too much or maybe too less. I don't know. Because the person is coming all the way to me.
+03:18 Maybe walking around or going for coffee or something like this, or sitting in the park. Because there's a lot of things we have to talk about that happened in the past.
+03:52 Yeah, I agree. That's a good point. And I hope everything will go well, because I'm kind of scared that in the moment I feel very uncomfortable because of what happened.
+04:28 And what could I do in case it gets awkward?
+04:59 Okay. Yeah, that makes a lot of sense. Thank you so much for listening to me. I appreciate it.
+05:17 Yes. Thank you. Hello. Hello.</t>
         </is>
       </c>
     </row>
@@ -509,9 +532,15 @@
       <c r="B4" t="n">
         <v>14719</v>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>00:14 Hi, my name is Perfect. Yeah, it's quite cold outside and windy. That's annoying.  00:36 Yes. I had a really challenging group project last week. Yeah, maybe I would like to talk about this.  00:58 Yeah, the people don't want to participate. As always. Sometimes in this university they're just chilling and stuff like this. So I just want to get a really good grade. And the system is, in my opinion, not the best one because all the workload is most of the time left by one person. And in this case, in a group project, just one guy, especially me, is doing everything and the other ones are not participating and therefore the final grade is not so good because the people don't really know what to present. And this is annoying.  01:57 I mean, I get in really close contact with them, push them to participate, and always remember, hey, this is a group project. Please upload your parts onto a certain deadline. But then the people are doing this with no effort, just publishing white PowerPoint slides with nothing really strategic. There are no strategic information on it, just copy paste, I don't know where from. And as you can see, when I open the presentation, there's literally no effort and really a low standard. And therefore I need to repeat the work always and we don't do it. And that's really challenging. This is not a groom project. This is like a single project.  03:17 Yeah, I tried it. And the response was yeah, buddy, that's tough. You need to handle this. It's a group project. I cannot give you an individual grade. And this is like the system in Master Sheet. That annoys me the most that you don't get an individual grade. You only get a group grade. And for the people who just want to pass everything, this is like the perfect system. But for the people who try to achieve higher goals. Yeah, it's stopping your career a little bit.  04:13 You can't. You have the people with 15 people guys and you get randomly selected with people in one group. So there's no chance to work with people you want to work on. I would like that the university give you the opportunity that you can select maybe also friends to work on a project maybe just once in the whole study. So you can select some friends, work together in the group project because this may be. Yeah, this is better.  05:22 Perfect. Thank you. Bye.</t>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>00:14 Hi, my name is Perfect. Yeah, it's quite cold outside and windy. That's annoying.
+00:36 Yes. I had a really challenging group project last week. Yeah, maybe I would like to talk about this.
+00:58 Yeah, the people don't want to participate. As always. Sometimes in this university they're just chilling and stuff like this. So I just want to get a really good grade. And the system is, in my opinion, not the best one because all the workload is most of the time left by one person. And in this case, in a group project, just one guy, especially me, is doing everything and the other ones are not participating and therefore the final grade is not so good because the people don't really know what to present. And this is annoying.
+01:57 I mean, I get in really close contact with them, push them to participate, and always remember, hey, this is a group project. Please upload your parts onto a certain deadline. But then the people are doing this with no effort, just publishing white PowerPoint slides with nothing really strategic. There are no strategic information on it, just copy paste, I don't know where from. And as you can see, when I open the presentation, there's literally no effort and really a low standard. And therefore I need to repeat the work always and we don't do it. And that's really challenging. This is not a groom project. This is like a single project.
+03:17 Yeah, I tried it. And the response was yeah, buddy, that's tough. You need to handle this. It's a group project. I cannot give you an individual grade. And this is like the system in Master Sheet. That annoys me the most that you don't get an individual grade. You only get a group grade. And for the people who just want to pass everything, this is like the perfect system. But for the people who try to achieve higher goals. Yeah, it's stopping your career a little bit.
+04:13 You can't. You have the people with 15 people guys and you get randomly selected with people in one group. So there's no chance to work with people you want to work on. I would like that the university give you the opportunity that you can select maybe also friends to work on a project maybe just once in the whole study. So you can select some friends, work together in the group project because this may be. Yeah, this is better.
+05:22 Perfect. Thank you. Bye.</t>
         </is>
       </c>
     </row>
@@ -524,9 +553,20 @@
       <c r="B5" t="n">
         <v>14989</v>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>00:22 I would like to speak about my friend that I see one weeks ago.  00:38 We go for King's Day outside, we go eat in a brunch place and after we go first with some other friend in Maastricht.  01:02 Was very nice. I meet some new people, some new friends that I will never meet if I was not with my friend.  01:29 Thankfully they act toward me. Was very funny, very simple, very relaxed with me it was very nice moment.  01:52 Yes, exactly. I knew what you do.  02:13 Okay. Okay. What else? You can talk.  02:38 Can I speak about my parents? I come yesterday, we go eat in a restaurant in Maastricht. It's very nice place, very good restaurant.  03:04 The fact that I see my parents, I didn't see my parents this long time was very nice moment. We talk a lot about the life, ok? The university, all that. All this stuff.  03:37 Yes, exactly.  03:54 Tomorrow I'm have a presentation in supply chain I need to do my slide the upstream part.  04:15 Everything. All the part.  04:34 For the moment, I don't know. I'm going to do another disk.</t>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>00:22 I would like to speak about my friend that I see one weeks ago.
+00:38 We go for King's Day outside, we go eat in a brunch place and after we go first with some other friend in Maastricht.
+01:02 Was very nice. I meet some new people, some new friends that I will never meet if I was not with my friend.
+01:29 Thankfully they act toward me. Was very funny, very simple, very relaxed with me it was very nice moment.
+01:52 Yes, exactly. I knew what you do.
+02:13 Okay. Okay. What else? You can talk.
+02:38 Can I speak about my parents? I come yesterday, we go eat in a restaurant in Maastricht. It's very nice place, very good restaurant.
+03:04 The fact that I see my parents, I didn't see my parents this long time was very nice moment. We talk a lot about the life, ok? The university, all that. All this stuff.
+03:37 Yes, exactly.
+03:54 Tomorrow I'm have a presentation in supply chain I need to do my slide the upstream part.
+04:15 Everything. All the part.
+04:34 For the moment, I don't know. I'm going to do another disk.</t>
         </is>
       </c>
     </row>
@@ -539,9 +579,20 @@
       <c r="B6" t="n">
         <v>14800</v>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>00:22 I would like to talk about a recent problem I had with in my life.  00:37 Yes. I had to do, like, a team project with my fellow students, but we had to do a presentation, but, like, nobody did something, so I had to do, like, all the work.  01:00 Yes.  01:04 I had to do it on my own, but it still created some issues because when we had to do the presentation, my other teammates weren't prepared.  01:30 My part went pretty well, and I was with another girl, and she also prepared well, but were with two boys, and they didn't prepare well. They just said some AI stuff, and it didn't go very well.  02:03 Sorry, could you repeat that?  02:18 Yes, they said, like, the first part of the presentation went really well, and that was the part that the other girl and me did. And then they said, like, the other part. The second part that the boys did was not as great, and I didn't. It lacked some, like, things that were important.  02:54 Yeah, I feel great that I got some recognition for my good part, but I don't like it because I have to do another presentation with them. And, yeah, that won't be that great because then I have to do it again with the other girl, and they won't be doing anything.  03:30 Yeah, me and the girl talked about that. I think we're going to, like, say to the boys that they also have to do something and that we are not going to do it on ourselves again.  03:58 Yes.  04:15 Yes, I agree on that. I think we can manage to do it with, like, all four of us and then we can create it that we don't have to do anything on our own.  04:40 Yes. Thank you.</t>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>00:22 I would like to talk about a recent problem I had with in my life.
+00:37 Yes. I had to do, like, a team project with my fellow students, but we had to do a presentation, but, like, nobody did something, so I had to do, like, all the work.
+01:00 Yes.
+01:04 I had to do it on my own, but it still created some issues because when we had to do the presentation, my other teammates weren't prepared.
+01:30 My part went pretty well, and I was with another girl, and she also prepared well, but were with two boys, and they didn't prepare well. They just said some AI stuff, and it didn't go very well.
+02:03 Sorry, could you repeat that?
+02:18 Yes, they said, like, the first part of the presentation went really well, and that was the part that the other girl and me did. And then they said, like, the other part. The second part that the boys did was not as great, and I didn't. It lacked some, like, things that were important.
+02:54 Yeah, I feel great that I got some recognition for my good part, but I don't like it because I have to do another presentation with them. And, yeah, that won't be that great because then I have to do it again with the other girl, and they won't be doing anything.
+03:30 Yeah, me and the girl talked about that. I think we're going to, like, say to the boys that they also have to do something and that we are not going to do it on ourselves again.
+03:58 Yes.
+04:15 Yes, I agree on that. I think we can manage to do it with, like, all four of us and then we can create it that we don't have to do anything on our own.
+04:40 Yes. Thank you.</t>
         </is>
       </c>
     </row>
@@ -554,9 +605,19 @@
       <c r="B7" t="n">
         <v>14806</v>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>00:30 I must speak about an interaction or a conflict I had with somebody recently, but I have no idea what to talk about.  00:50 Well, I. I don't know what to talk about.  01:33 Maybe about a football match, maybe.  01:49 Someone you watched with disagreement with how the football match went? Because there was two hands. I mean hands. Like when another player touches the ball with his hands, one with. It was in the square of the goal keeper and so. So it must have been penalty. But it didn't go like apparently there's a rule that says when one player shoots to another one that is his teammate, then it doesn't count. But it stopped the whole match and they didn't take into account. And then another hand during the match was not counted also.  02:54 Well, it didn't unfold, unfortunately, because the other team won the match. And yeah, the other person was also a bit in shock about the referee not taking the two hands into account. So yeah,.  03:35 I mean. No, I like the fact that emotions run high because it. I mean, you can debate about it, but football is about emotions when you're not playing, so I don't mind.  04:06 Yeah, that's true.  04:22 Yeah, we always talk about it, like, after the match, just talking about the actions and everything that happened during the match. So, yeah,.  04:44 Yeah, it's very good. I like football.  05:06 What should we talk about now?  05:25 Yeah, it was nice. I mean, What should I do?    Transcribed by https://fireflies.ai/</t>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>00:30 I must speak about an interaction or a conflict I had with somebody recently, but I have no idea what to talk about.
+00:50 Well, I. I don't know what to talk about.
+01:33 Maybe about a football match, maybe.
+01:49 Someone you watched with disagreement with how the football match went? Because there was two hands. I mean hands. Like when another player touches the ball with his hands, one with. It was in the square of the goal keeper and so. So it must have been penalty. But it didn't go like apparently there's a rule that says when one player shoots to another one that is his teammate, then it doesn't count. But it stopped the whole match and they didn't take into account. And then another hand during the match was not counted also.
+02:54 Well, it didn't unfold, unfortunately, because the other team won the match. And yeah, the other person was also a bit in shock about the referee not taking the two hands into account. So yeah,.
+03:35 I mean. No, I like the fact that emotions run high because it. I mean, you can debate about it, but football is about emotions when you're not playing, so I don't mind.
+04:06 Yeah, that's true.
+04:22 Yeah, we always talk about it, like, after the match, just talking about the actions and everything that happened during the match. So, yeah,.
+04:44 Yeah, it's very good. I like football.
+05:06 What should we talk about now?
+05:25 Yeah, it was nice. I mean, What should I do?    Transcribed by https://fireflies.ai/</t>
         </is>
       </c>
     </row>
@@ -569,9 +630,21 @@
       <c r="B8" t="n">
         <v>14428</v>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>00:19 I'm fine, thanks.  00:35 We can go with the flow like you suggested.  00:48 When we smile, we had a barbecue with friends at the beach.  01:06 Drinking the beers shirtless.  01:23 Rather the atmosphere than the beer. To be honest,.  01:38 Oh yes, when the weather's better for sure.  01:55 Warmer days,.  02:11 We're in Maschit, so there's not that many beaches you can go to. So we have our favorite spots on the other side of the Maas.  02:31 Yeah,.  02:49 I've been there.  02:54 I mean, I've been there before, so it's a really nice spot. But I've had an argument there in the past.  03:16 Now I feel good. It's half a year back, so it's fine.  03:32 Sure. Should I just take it off?</t>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>00:19 I'm fine, thanks.
+00:35 We can go with the flow like you suggested.
+00:48 When we smile, we had a barbecue with friends at the beach.
+01:06 Drinking the beers shirtless.
+01:23 Rather the atmosphere than the beer. To be honest,.
+01:38 Oh yes, when the weather's better for sure.
+01:55 Warmer days,.
+02:11 We're in Maschit, so there's not that many beaches you can go to. So we have our favorite spots on the other side of the Maas.
+02:31 Yeah,.
+02:49 I've been there.
+02:54 I mean, I've been there before, so it's a really nice spot. But I've had an argument there in the past.
+03:16 Now I feel good. It's half a year back, so it's fine.
+03:32 Sure. Should I just take it off?</t>
         </is>
       </c>
     </row>
@@ -584,9 +657,17 @@
       <c r="B9" t="n">
         <v>13366</v>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>00:17 Yeah, perfect. I would like to share my experience with. With my co worker, which was pretty much weird social interaction. If you could give me any advice on that.  00:49 It was pretty much the whole interaction and how they responded. It's at my work. My co worker, she seems very sweet and okay, I'm a newbie, which is, I think, important fact to say. However, she doesn't seem to be very understanding, I would say. And she gets frustrated really easily to some degree where she starts screaming at people. And, yeah, I wasn't quite sure how to get. How to challenge that situation.  01:56 I. No, I feel like I talked to her, like, before this interaction. I was fine with her. She was, like, cracking jokes. She was feeling great. Yeah, I thought she was great. And we. Once I heard you, I heard her yelling to my boss and my boss yelling at her, which I thought was my boss's idea or like, my boss's, you know, my boss's fault that he starts screaming at her. But now it seems like that it was her attitude that made him feel like that. Because, like, we are fine the whole time at work. And all of a sudden, like, she got frustrated so easily. Like when somebody gave her another task that she was gonna do and I was supposed to do the task. However, I was helping elsewhere. But normally she would do the task regularly because I only work.  02:53 I only work on Sundays and Mondays, so it doesn't make any sense. And, yeah, she started just screaming. And it was just because she told me that I put another thing somewhere where it's not supposed to because it's stressing her out. And she started screaming at her, at me, and then everyone else is like, it's not her freaking job to do these things, but, like, it is her job.  03:42 No, not easy.  03:49 No, sure. No, I understand that completely because, like, we are fine the whole time. And after that she was also smiling in 30 minutes of the time. And then like she said bye. However, I have no idea how to like, interact with the situation because I also want to stood my ground. I don't want to just like, I was just too like, you know, dumbstruck by the whole situation that like, I couldn't even reply and I was like, oh, yeah, sorry. You know, and like, this is totally not me. Like, I'm not really an extroverted person, which I really don't understand. Like, why, like, situation like this by a co worker who's like, chill and we're fine. Like, you know, like, just like caught me off guard.  04:57 Yeah, no, I understand that. Like, however, my deal or is that basically if something like that of an interaction like this happens to me in real life, I. I just call. I am pretty calm in these situations. But then I can. I can't get it out of my head. Like, I, I am the one. I'm the type of person that I will think about it for. I don't know, that will. It will keep me. Keep me awake at night, you know, Like, I will think about it for 48 hours. Like, why didn't I. Why haven't. Why haven't I responded better? Like, why did I do something differently? You know,.  06:01 Yeah, no, I get that. But like, you know, I also don't want to have an attitude, but I feel like with my personality, I do have to have that. And then I will just like, I will feel bad that I didn't say anything.  06:42 Yeah, fair. Okay, I will do that next time then.</t>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>00:17 Yeah, perfect. I would like to share my experience with. With my co worker, which was pretty much weird social interaction. If you could give me any advice on that.
+00:49 It was pretty much the whole interaction and how they responded. It's at my work. My co worker, she seems very sweet and okay, I'm a newbie, which is, I think, important fact to say. However, she doesn't seem to be very understanding, I would say. And she gets frustrated really easily to some degree where she starts screaming at people. And, yeah, I wasn't quite sure how to get. How to challenge that situation.
+01:56 I. No, I feel like I talked to her, like, before this interaction. I was fine with her. She was, like, cracking jokes. She was feeling great. Yeah, I thought she was great. And we. Once I heard you, I heard her yelling to my boss and my boss yelling at her, which I thought was my boss's idea or like, my boss's, you know, my boss's fault that he starts screaming at her. But now it seems like that it was her attitude that made him feel like that. Because, like, we are fine the whole time at work. And all of a sudden, like, she got frustrated so easily. Like when somebody gave her another task that she was gonna do and I was supposed to do the task. However, I was helping elsewhere. But normally she would do the task regularly because I only work.
+02:53 I only work on Sundays and Mondays, so it doesn't make any sense. And, yeah, she started just screaming. And it was just because she told me that I put another thing somewhere where it's not supposed to because it's stressing her out. And she started screaming at her, at me, and then everyone else is like, it's not her freaking job to do these things, but, like, it is her job.
+03:42 No, not easy.
+03:49 No, sure. No, I understand that completely because, like, we are fine the whole time. And after that she was also smiling in 30 minutes of the time. And then like she said bye. However, I have no idea how to like, interact with the situation because I also want to stood my ground. I don't want to just like, I was just too like, you know, dumbstruck by the whole situation that like, I couldn't even reply and I was like, oh, yeah, sorry. You know, and like, this is totally not me. Like, I'm not really an extroverted person, which I really don't understand. Like, why, like, situation like this by a co worker who's like, chill and we're fine. Like, you know, like, just like caught me off guard.
+04:57 Yeah, no, I understand that. Like, however, my deal or is that basically if something like that of an interaction like this happens to me in real life, I. I just call. I am pretty calm in these situations. But then I can. I can't get it out of my head. Like, I, I am the one. I'm the type of person that I will think about it for. I don't know, that will. It will keep me. Keep me awake at night, you know, Like, I will think about it for 48 hours. Like, why didn't I. Why haven't. Why haven't I responded better? Like, why did I do something differently? You know,.
+06:01 Yeah, no, I get that. But like, you know, I also don't want to have an attitude, but I feel like with my personality, I do have to have that. And then I will just like, I will feel bad that I didn't say anything.
+06:42 Yeah, fair. Okay, I will do that next time then.</t>
         </is>
       </c>
     </row>
@@ -599,9 +680,18 @@
       <c r="B10" t="n">
         <v>11</v>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>00:00 And then it starts. It starts talking first. Yeah. Whenever you're ready. Okay, I can go. I want to talk about a bad situation that I lived yesterday.  00:35 I had a. I don't know, bad conversation with one of my housemates and I didn't like so much her manners and the way she. She interacted with me and the way she told the thing to me.  01:05 Was something regarded. I don't know. Split a split regarding the. Our purchase that we share in our house and I don't know, she. She said something that I didn't like so much. So my. I don't know, my way of reasoning was a bit different from her. So sometimes I don't understand really well how. How she thinks about things and I don't know. And I didn't like so much the man.  02:04 I don't know. Because it's a kind of person where it's quite difficult to. I don't know, it's quite difficult to communicate and to have a conversation. So sometimes I actually don't want to have a conversation. I don't want to. To try to understand better her. This is the thing. So I don't know. Yes, I can. Maybe I. I should share more what I. What I'm thinking and what was wrong for me. But the thing is that I don't want to waste my energy on this.  03:08 But how do you mean has simple. What do you mean? Like. What do you mean.  03:45 Yeah, no, I know. Maybe you're right. But the thing is still that I don't want. Like, I think that this is the kind of thing that can waste my energy because I actually don't care really much to have this kind of conversation. Maybe. Yeah, you're right. That could better to have this kind of conversation so in the future these kind of things. Don't happen again. But the thing is that, I don't know, maybe sometimes it is easier to leave the things as they are and don't waste energy. Because the thing is that there are people that don't. Don't understand. They don't understand. So I don't know. I don't know.  05:05 Yeah, maybe. Maybe I will know. But the thing is that we should do a something together this week, and I don't know if I want to.  05:41 What do you mean with this last thing? Like put more attention on the activity? What do you mean?  06:09 So do you think that I should go, but I should go for you and. And to, I don't know, focus only on the activity without talking about something and without any emotional involvement?  06:47 But the thing is that. I don't know. I still don't know. Hello? So the time is over. Okay. I think you can press, like either restart or finish.    Transcribed by https://fireflies.ai/</t>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>00:00 And then it starts. It starts talking first. Yeah. Whenever you're ready. Okay, I can go. I want to talk about a bad situation that I lived yesterday.
+00:35 I had a. I don't know, bad conversation with one of my housemates and I didn't like so much her manners and the way she. She interacted with me and the way she told the thing to me.
+01:05 Was something regarded. I don't know. Split a split regarding the. Our purchase that we share in our house and I don't know, she. She said something that I didn't like so much. So my. I don't know, my way of reasoning was a bit different from her. So sometimes I don't understand really well how. How she thinks about things and I don't know. And I didn't like so much the man.
+02:04 I don't know. Because it's a kind of person where it's quite difficult to. I don't know, it's quite difficult to communicate and to have a conversation. So sometimes I actually don't want to have a conversation. I don't want to. To try to understand better her. This is the thing. So I don't know. Yes, I can. Maybe I. I should share more what I. What I'm thinking and what was wrong for me. But the thing is that I don't want to waste my energy on this.
+03:08 But how do you mean has simple. What do you mean? Like. What do you mean.
+03:45 Yeah, no, I know. Maybe you're right. But the thing is still that I don't want. Like, I think that this is the kind of thing that can waste my energy because I actually don't care really much to have this kind of conversation. Maybe. Yeah, you're right. That could better to have this kind of conversation so in the future these kind of things. Don't happen again. But the thing is that, I don't know, maybe sometimes it is easier to leave the things as they are and don't waste energy. Because the thing is that there are people that don't. Don't understand. They don't understand. So I don't know. I don't know.
+05:05 Yeah, maybe. Maybe I will know. But the thing is that we should do a something together this week, and I don't know if I want to.
+05:41 What do you mean with this last thing? Like put more attention on the activity? What do you mean?
+06:09 So do you think that I should go, but I should go for you and. And to, I don't know, focus only on the activity without talking about something and without any emotional involvement?
+06:47 But the thing is that. I don't know. I still don't know. Hello? So the time is over. Okay. I think you can press, like either restart or finish.    Transcribed by https://fireflies.ai/</t>
         </is>
       </c>
     </row>
@@ -614,9 +704,17 @@
       <c r="B11" t="n">
         <v>14674</v>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>00:20 Hi, I'm very good. I was just at the gym and now I'm a bit exhausted, but yeah, no, it was good. How are you?  00:40 It was just like a Hyrux situation, so a lot of high intensity training, but that was really good. And yeah, now I'm excited to try this experiment and it's a bit weird, but exciting. Yeah,.  01:09 Sorry, I did not understand what you mean.  01:24 I would like to do my Hyrux in Dusseldorf next year. But I also want to tell you something about my personal problem.  01:49 Okay. So recently I had the situation that my friend was just a bit too, like, very unfriendly to me and not really acting in the way I hope or like I want her to act because she was not really, like, helping me and was rather very unfriendly to me. And I don't know, like, how I should handle situations like that.  02:40 I think she's a very, like, has a strong personality and if I would interrupt her in her being and like her character, I think she can get very attacked. And like, usually I don't think it's that much of a problem, but recently I'm very annoyed because it happened so often and I cannot really comprehend with other friends and talk about it with other friends. So that's why it makes a bit. What? That's why it makes it a Bit more difficult to. Yeah. Think about.  03:51 Yeah, I think that's a good idea, but I'm not sure, like, how would you start this conversation? And, like, especially when we're talking, she's always, like, such a strong personality that I cannot really keep up with. Not with her ideas, but, like, with the way she is arguing and fighting with me. So she has way more or way stronger arguments. And in the end, I'm the one who says sorry, even though she should say sorry.  04:55 Oh, yeah, that sounds good. Maybe I'm gonna do it and try to, like, talk with my friends about that. Yeah. So I think our time is almost over, but I really enjoy talking to you. I think you're a good help and. Yeah, thank you.  05:27 Thank you.</t>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>00:20 Hi, I'm very good. I was just at the gym and now I'm a bit exhausted, but yeah, no, it was good. How are you?
+00:40 It was just like a Hyrux situation, so a lot of high intensity training, but that was really good. And yeah, now I'm excited to try this experiment and it's a bit weird, but exciting. Yeah,.
+01:09 Sorry, I did not understand what you mean.
+01:24 I would like to do my Hyrux in Dusseldorf next year. But I also want to tell you something about my personal problem.
+01:49 Okay. So recently I had the situation that my friend was just a bit too, like, very unfriendly to me and not really acting in the way I hope or like I want her to act because she was not really, like, helping me and was rather very unfriendly to me. And I don't know, like, how I should handle situations like that.
+02:40 I think she's a very, like, has a strong personality and if I would interrupt her in her being and like her character, I think she can get very attacked. And like, usually I don't think it's that much of a problem, but recently I'm very annoyed because it happened so often and I cannot really comprehend with other friends and talk about it with other friends. So that's why it makes a bit. What? That's why it makes it a Bit more difficult to. Yeah. Think about.
+03:51 Yeah, I think that's a good idea, but I'm not sure, like, how would you start this conversation? And, like, especially when we're talking, she's always, like, such a strong personality that I cannot really keep up with. Not with her ideas, but, like, with the way she is arguing and fighting with me. So she has way more or way stronger arguments. And in the end, I'm the one who says sorry, even though she should say sorry.
+04:55 Oh, yeah, that sounds good. Maybe I'm gonna do it and try to, like, talk with my friends about that. Yeah. So I think our time is almost over, but I really enjoy talking to you. I think you're a good help and. Yeah, thank you.
+05:27 Thank you.</t>
         </is>
       </c>
     </row>
@@ -629,9 +727,16 @@
       <c r="B12" t="n">
         <v>14578</v>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>00:30 Okay, so I'd like to talk about some recent challenging conversation that I have, if that is okay.  01:00 Yes. So I was in an argument with my friends because I'm thinking of maybe like changing my field of study because I currently do not feel like that it is something that I'm confident, comfortable with or that like the people, the university and in general the vibe of my current study, which is business by the way. So yeah, and I'm thinking of maybe switching.  01:46 Okay, so first of all, I talked with friends and my boyfriend as well about it. And since he is studying currently in Aachen and I'm in Maastricht. So yeah, I was maybe like he of course wanted me to change of course to a study that is located in Aachen near to him. And I kind of feel like I want that as well, but I don't want to be the one that is moving there for him. So my friends say, oh yeah, maybe you should re evaluate your decision. So now I'm like kind of stuck in between already thinking that I'm not happy in my current study, but also wanting to move in or move too nearer to my boyfriend. But also like I get the thought of my friends, but I feel like. Or yeah, that is a question to you. Do I.  02:34 How can I know that this is a decision that I want to do based on really my interests besides my boyfriend?  03:06 Okay, so I'm good at math and that I really like in business. I also like, I enjoy like, like talking and presenting stuff and I wanted to study something that I have like a wide range of later on in my career. But like I feel like now that I have studied like for one year, I don't know, I feel like that the people are not really my vibe. And I've met other people that are studying for example in Aachen that are more kind of my vibe. But should it be like a reason for me to say, okay, I want to switch university because the people here make me feel uncomfortable and there they do not.  04:09 Okay, so I would say like if I'm happy then I'm going to be successful. But I don't know if it is something like I want to know, like the opinion that I should have, like is it okay for me to say I'm switching because of ch just people in my environment?  04:44 For sure, Definitely. It would make me feel more comfortable. Especially because people are saying that business is like kind of like a lame study or that it's like nothing to really consider or that it's like worth nothing and that I should study something more like natural sciences, like mathematics for example.  05:21 I feel like that I take a lot the opinion, I weigh a lot the opinion of others. Especially because they say, okay, business is over. Hello. Hello. Hello. All done? Yes. Okay. Wait, he's still talking. I'll stop.    Transcribed by https://fireflies.ai/</t>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>00:30 Okay, so I'd like to talk about some recent challenging conversation that I have, if that is okay.
+01:00 Yes. So I was in an argument with my friends because I'm thinking of maybe like changing my field of study because I currently do not feel like that it is something that I'm confident, comfortable with or that like the people, the university and in general the vibe of my current study, which is business by the way. So yeah, and I'm thinking of maybe switching.
+01:46 Okay, so first of all, I talked with friends and my boyfriend as well about it. And since he is studying currently in Aachen and I'm in Maastricht. So yeah, I was maybe like he of course wanted me to change of course to a study that is located in Aachen near to him. And I kind of feel like I want that as well, but I don't want to be the one that is moving there for him. So my friends say, oh yeah, maybe you should re evaluate your decision. So now I'm like kind of stuck in between already thinking that I'm not happy in my current study, but also wanting to move in or move too nearer to my boyfriend. But also like I get the thought of my friends, but I feel like. Or yeah, that is a question to you. Do I.
+02:34 How can I know that this is a decision that I want to do based on really my interests besides my boyfriend?
+03:06 Okay, so I'm good at math and that I really like in business. I also like, I enjoy like, like talking and presenting stuff and I wanted to study something that I have like a wide range of later on in my career. But like I feel like now that I have studied like for one year, I don't know, I feel like that the people are not really my vibe. And I've met other people that are studying for example in Aachen that are more kind of my vibe. But should it be like a reason for me to say, okay, I want to switch university because the people here make me feel uncomfortable and there they do not.
+04:09 Okay, so I would say like if I'm happy then I'm going to be successful. But I don't know if it is something like I want to know, like the opinion that I should have, like is it okay for me to say I'm switching because of ch just people in my environment?
+04:44 For sure, Definitely. It would make me feel more comfortable. Especially because people are saying that business is like kind of like a lame study or that it's like nothing to really consider or that it's like worth nothing and that I should study something more like natural sciences, like mathematics for example.
+05:21 I feel like that I take a lot the opinion, I weigh a lot the opinion of others. Especially because they say, okay, business is over. Hello. Hello. Hello. All done? Yes. Okay. Wait, he's still talking. I'll stop.    Transcribed by https://fireflies.ai/</t>
         </is>
       </c>
     </row>
@@ -644,9 +749,14 @@
       <c r="B13" t="n">
         <v>14401</v>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>00:13 I would like to talk about a challenging social event I had recently. I would like to tell you about a challenging social event that I had or social interaction.  01:02 I see the most difference in day to day communication patterns because since people are mostly talking on messages, so this is a big difference which makes it harder in some situations to. To talk to people. For example, I had a recent. I've been building a startup with a friend and we had to do a video for a challenge because we're taking part in a challenge and we had similar opinions on how to do it. But in the end the results of our videos were both very different. And I like, because I had to cut the video, I had to kind of. I was kind of in charge of it. And this made it really hard for me to. Because she was like her video was not up to my expectations maybe a little bit.  02:01 And it didn't really fit into the general idea of it. So I had to bring about some criticism which felt really hard, especially over WhatsApp because were very far away from each other and couldn't just meet to talk about it. And that made it quite challenging to find the right words to bring about without. To bring about the criticism without hurting a friend. Yeah.  03:01 Yeah, it seems like that what I like about or what makes it better is voice messages. But in general I think that real communication is always better than just texting. It's very convenient. But I feel like people have people, including me, are afraid of phone calls nowadays and don't want to have the real interaction. But I don't see why that is. It's not even faster to message people. So that's just a social issue, I think. And I would really like to go back to real conversation or at least phone calls.  04:17 That is true. But how can you do that when you've been talking to friends that you don't see very often? Because we live in different cities since a couple of months, and we've only been talking about over messages. And this makes it hard to go back to phone calls now because I feel like it might be weird.  05:10 Sounds good. Thank you very much.</t>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>00:13 I would like to talk about a challenging social event I had recently. I would like to tell you about a challenging social event that I had or social interaction.
+01:02 I see the most difference in day to day communication patterns because since people are mostly talking on messages, so this is a big difference which makes it harder in some situations to. To talk to people. For example, I had a recent. I've been building a startup with a friend and we had to do a video for a challenge because we're taking part in a challenge and we had similar opinions on how to do it. But in the end the results of our videos were both very different. And I like, because I had to cut the video, I had to kind of. I was kind of in charge of it. And this made it really hard for me to. Because she was like her video was not up to my expectations maybe a little bit.
+02:01 And it didn't really fit into the general idea of it. So I had to bring about some criticism which felt really hard, especially over WhatsApp because were very far away from each other and couldn't just meet to talk about it. And that made it quite challenging to find the right words to bring about without. To bring about the criticism without hurting a friend. Yeah.
+03:01 Yeah, it seems like that what I like about or what makes it better is voice messages. But in general I think that real communication is always better than just texting. It's very convenient. But I feel like people have people, including me, are afraid of phone calls nowadays and don't want to have the real interaction. But I don't see why that is. It's not even faster to message people. So that's just a social issue, I think. And I would really like to go back to real conversation or at least phone calls.
+04:17 That is true. But how can you do that when you've been talking to friends that you don't see very often? Because we live in different cities since a couple of months, and we've only been talking about over messages. And this makes it hard to go back to phone calls now because I feel like it might be weird.
+05:10 Sounds good. Thank you very much.</t>
         </is>
       </c>
     </row>
@@ -659,9 +769,18 @@
       <c r="B14" t="n">
         <v>13438</v>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>00:20 On my mind today, I want to tell you about a challenging conversation I had with friend today. So it's a bit difficult situation because one of my friends, we are one big friend group. And one of my friends, her birthday is tomorrow, and I already talked with her about it because we have class together and were talking about the last week's. And we have class later today also, and tomorrow is her birthday, and he just found out that my other friends are on my top brunch, and my other friends thought I was in the group, but I'm not. And so I don't know if I should ask her if I can come because I don't know, maybe she forgot me or maybe it was intentionally, but I don't think it's intentionally, but I don't know. And. Yeah, what is your opinion?  01:06 What I should do when I see her later today?  01:37 Yeah, but if I do that and it was intentional, I still have class for her every second day for the next four weeks. So I don't know if it's a thing to break a friendship, but it would be probably weird, don't you think?  02:19 Okay, yeah, maybe that's correct. But still, I don't know. How would you exactly address what I should say? Like, what do you think I should say to her?  02:56 Don't you think I should do it less obvious and say, hey, what are your plans for your birthday tomorrow?  03:19 Yeah, maybe. Yeah. I don't know if it's the right approach because I don't want to make it awkward if it was extra, you know,.  03:53 True. Yeah. That's good advice. Actually, I would say, do you have any more advice?  04:24 Okay, but let's say there is a group present. Obviously I'm not part of that right now. How do I go of that? Cuz I think it's too late to join. If I would join,.  04:59 Yeah, not bad. Should I write one of the persons from who are giving it as a group or should I write into the group?  05:26 Okay, sounds good to me. Actually, how would you phrase sounds good?</t>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>00:20 On my mind today, I want to tell you about a challenging conversation I had with friend today. So it's a bit difficult situation because one of my friends, we are one big friend group. And one of my friends, her birthday is tomorrow, and I already talked with her about it because we have class together and were talking about the last week's. And we have class later today also, and tomorrow is her birthday, and he just found out that my other friends are on my top brunch, and my other friends thought I was in the group, but I'm not. And so I don't know if I should ask her if I can come because I don't know, maybe she forgot me or maybe it was intentionally, but I don't think it's intentionally, but I don't know. And. Yeah, what is your opinion?
+01:06 What I should do when I see her later today?
+01:37 Yeah, but if I do that and it was intentional, I still have class for her every second day for the next four weeks. So I don't know if it's a thing to break a friendship, but it would be probably weird, don't you think?
+02:19 Okay, yeah, maybe that's correct. But still, I don't know. How would you exactly address what I should say? Like, what do you think I should say to her?
+02:56 Don't you think I should do it less obvious and say, hey, what are your plans for your birthday tomorrow?
+03:19 Yeah, maybe. Yeah. I don't know if it's the right approach because I don't want to make it awkward if it was extra, you know,.
+03:53 True. Yeah. That's good advice. Actually, I would say, do you have any more advice?
+04:24 Okay, but let's say there is a group present. Obviously I'm not part of that right now. How do I go of that? Cuz I think it's too late to join. If I would join,.
+04:59 Yeah, not bad. Should I write one of the persons from who are giving it as a group or should I write into the group?
+05:26 Okay, sounds good to me. Actually, how would you phrase sounds good?</t>
         </is>
       </c>
     </row>
@@ -674,9 +793,17 @@
       <c r="B15" t="n">
         <v>14446</v>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>00:11 So yesterday I was doing a project for a client and I was there with my brother and he was supposed to record some videos and I was there to talk to the client and. And then he set up the cameras, but I told him that we want to record horizontal, not vertical, but he set it up in the wrong way. So on the way back I was really mad because now we can't use the material for YouTube as good and we lose lots of quality. So yeah, this is something. Some experience that I had and I was angry I was talking to him. So what do you think?  01:20 Yes, I agree. So that's what I did basically. And. But it's his job to set up, so I'm not gonna be there most of the time. So I think he has to do better. That's what I told him. But. But I don't want to be mean. So. Yeah, what do you think?  02:10 All right. But to be honest, this is. I knew everything. You already told me, so this is nothing new. So maybe you can come up with some new advice you have because this is pretty basic. I mean, I already knew that before talking to you.  02:58 Yes, I agree. Thank you. Do you have any problems that I should help you with?  03:16 Alright. So to be honest, I don't have any other problems. I'm doing pretty good mentally wise. But maybe you can Discover some problems. So maybe ask me some questions?  03:43 Well, it's hard to manage all the time as a student and working and having fun. So, yeah, this is one issue for sure.  04:18 Yes, I agree, but I. I don't know.  04:35 Yeah, sure. Let's do it.  04:54 Work. Especially work. But then I have tutorial as well. So mainly work, but then there's tutorial and then there's free time as well.</t>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>00:11 So yesterday I was doing a project for a client and I was there with my brother and he was supposed to record some videos and I was there to talk to the client and. And then he set up the cameras, but I told him that we want to record horizontal, not vertical, but he set it up in the wrong way. So on the way back I was really mad because now we can't use the material for YouTube as good and we lose lots of quality. So yeah, this is something. Some experience that I had and I was angry I was talking to him. So what do you think?
+01:20 Yes, I agree. So that's what I did basically. And. But it's his job to set up, so I'm not gonna be there most of the time. So I think he has to do better. That's what I told him. But. But I don't want to be mean. So. Yeah, what do you think?
+02:10 All right. But to be honest, this is. I knew everything. You already told me, so this is nothing new. So maybe you can come up with some new advice you have because this is pretty basic. I mean, I already knew that before talking to you.
+02:58 Yes, I agree. Thank you. Do you have any problems that I should help you with?
+03:16 Alright. So to be honest, I don't have any other problems. I'm doing pretty good mentally wise. But maybe you can Discover some problems. So maybe ask me some questions?
+03:43 Well, it's hard to manage all the time as a student and working and having fun. So, yeah, this is one issue for sure.
+04:18 Yes, I agree, but I. I don't know.
+04:35 Yeah, sure. Let's do it.
+04:54 Work. Especially work. But then I have tutorial as well. So mainly work, but then there's tutorial and then there's free time as well.</t>
         </is>
       </c>
     </row>
@@ -689,9 +816,22 @@
       <c r="B16" t="n">
         <v>14350</v>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>00:17 On my mind, It's a challenging interaction I had this morning.  00:30 Someone in our group wasn't there for the presentation and he did his stuff really late at night, so we didn't have a clue what was his part. So we didn't know what to say in our presentation today about his topics.  01:00 We just thought about topics, try to improvise and make the best out of the situation. So we used also ChatGPT to respond to that.  01:33 She didn't say anything. She just nodded at the. She didn't. Also, she didn't give feedback. So, yeah. Not sure what she thought about.  02:04 I'm feeling fine. It's like it was nice. It was. It was not a nice experience, but it's okay now.  02:31 Yeah, I can move forward with confidence.  02:47 Yes, I learned a lot from this experience and I think I got this.  03:13 Yeah. Any questions?  03:27 Like tell the other one to do stuff more earlier. So, yeah,.  03:48 Yes, you're right. I agree.  04:03 Yo. Right,.  04:24 No. Do you have any ideas?  04:36 Great.  04:46 Perfect.</t>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>00:17 On my mind, It's a challenging interaction I had this morning.
+00:30 Someone in our group wasn't there for the presentation and he did his stuff really late at night, so we didn't have a clue what was his part. So we didn't know what to say in our presentation today about his topics.
+01:00 We just thought about topics, try to improvise and make the best out of the situation. So we used also ChatGPT to respond to that.
+01:33 She didn't say anything. She just nodded at the. She didn't. Also, she didn't give feedback. So, yeah. Not sure what she thought about.
+02:04 I'm feeling fine. It's like it was nice. It was. It was not a nice experience, but it's okay now.
+02:31 Yeah, I can move forward with confidence.
+02:47 Yes, I learned a lot from this experience and I think I got this.
+03:13 Yeah. Any questions?
+03:27 Like tell the other one to do stuff more earlier. So, yeah,.
+03:48 Yes, you're right. I agree.
+04:03 Yo. Right,.
+04:24 No. Do you have any ideas?
+04:36 Great.
+04:46 Perfect.</t>
         </is>
       </c>
     </row>
@@ -704,9 +844,15 @@
       <c r="B17" t="n">
         <v>15205</v>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>00:18 Hi, how are you? How are you?  00:31 So recently I had a really difficult situation with one of my roommates because she wanted to invite friends and I was physically like exhausted and mentally exhausted from the day and studying. And it was really difficult to tell her because on the one hand I really wanted that she can invite her friends. But on the other hand, I didn't want that many people over because I was kind of physically exhausted. So that was a really challenging experience. And my conversation that I had,.  01:12 So I actually said yes to the friends because she's kind of like more. She talks a lot and I feel like she's kind of like it. Just like what she does has got to happen. So I was just like, fine with it. And I was going with it. I was like, okay, just invite your friends and I will just be in my room. Just don't be that loud. And she was kind of sad that I didn't want to join, but I was just like, I'm like, mentally exhausted from like uni all day. Yeah. So at first she was kind of like pissed because I didn't join our friends, but then she was fine and she was like, oh, yeah, just go into your room and sleep. That's fine.  02:09 I think I should have just said my needs directly because first I was kind of like hemmed and I didn't want to say it because I felt like it would confront her and like she would be pissed at it. But I just learned that I should just like, say my needs. And it doesn't matter, like, what the other person thinks because as long as I feel it, my feelings are valid. So. Yeah,.  02:48 Yeah, definitely. So, yeah, how would you say I should handle it better the next time? Do you have any tips?  03:27 Yeah, that's. That's a good advice. Thank you so much. Do you have any more tips to share? Just like in the general environment and like other, like how I can like come up with the topic of it of like saying, oh, yeah, I don't want to join.  04:17 Yeah, that's true. Thank you so much for your advice. I think that's all.</t>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>00:18 Hi, how are you? How are you?
+00:31 So recently I had a really difficult situation with one of my roommates because she wanted to invite friends and I was physically like exhausted and mentally exhausted from the day and studying. And it was really difficult to tell her because on the one hand I really wanted that she can invite her friends. But on the other hand, I didn't want that many people over because I was kind of physically exhausted. So that was a really challenging experience. And my conversation that I had,.
+01:12 So I actually said yes to the friends because she's kind of like more. She talks a lot and I feel like she's kind of like it. Just like what she does has got to happen. So I was just like, fine with it. And I was going with it. I was like, okay, just invite your friends and I will just be in my room. Just don't be that loud. And she was kind of sad that I didn't want to join, but I was just like, I'm like, mentally exhausted from like uni all day. Yeah. So at first she was kind of like pissed because I didn't join our friends, but then she was fine and she was like, oh, yeah, just go into your room and sleep. That's fine.
+02:09 I think I should have just said my needs directly because first I was kind of like hemmed and I didn't want to say it because I felt like it would confront her and like she would be pissed at it. But I just learned that I should just like, say my needs. And it doesn't matter, like, what the other person thinks because as long as I feel it, my feelings are valid. So. Yeah,.
+02:48 Yeah, definitely. So, yeah, how would you say I should handle it better the next time? Do you have any tips?
+03:27 Yeah, that's. That's a good advice. Thank you so much. Do you have any more tips to share? Just like in the general environment and like other, like how I can like come up with the topic of it of like saying, oh, yeah, I don't want to join.
+04:17 Yeah, that's true. Thank you so much for your advice. I think that's all.</t>
         </is>
       </c>
     </row>
@@ -719,9 +865,19 @@
       <c r="B18" t="n">
         <v>14218</v>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>00:16 Nice to meet you. How are you?  00:27 I'm also doing great. I would like to chat about a recent challenging situation I had.  00:44 Yeah, so I was talking to my mother and she wanted me to do a test for a scholarship because it gives money and stuff. But I was really stressed because of student consultancy and other things going on because of group work in university. So I said that it's not doable to do this test in this time.  01:22 She somehow understands, but also said that I should take time for it and yeah, make time for.  01:44 I think it was not really possible because also the exam were coming up and I really had to learn for it. So I think it was not a good trade off to use this time for the scholarship thing.  02:14 Not really relieved, no.  02:36 I'm not sure.  02:58 No, it's not that important for me because I. It's not in my mind anymore. Really.  03:21 My focus is on doing university, also doing a bit of spirit sport and student consultancy, handling and all business development.  03:53 I think I'm doing really good progress since I'm in university, so I gained a lot of new skills and stuff.  04:26 Okay. Thank you.</t>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>00:16 Nice to meet you. How are you?
+00:27 I'm also doing great. I would like to chat about a recent challenging situation I had.
+00:44 Yeah, so I was talking to my mother and she wanted me to do a test for a scholarship because it gives money and stuff. But I was really stressed because of student consultancy and other things going on because of group work in university. So I said that it's not doable to do this test in this time.
+01:22 She somehow understands, but also said that I should take time for it and yeah, make time for.
+01:44 I think it was not really possible because also the exam were coming up and I really had to learn for it. So I think it was not a good trade off to use this time for the scholarship thing.
+02:14 Not really relieved, no.
+02:36 I'm not sure.
+02:58 No, it's not that important for me because I. It's not in my mind anymore. Really.
+03:21 My focus is on doing university, also doing a bit of spirit sport and student consultancy, handling and all business development.
+03:53 I think I'm doing really good progress since I'm in university, so I gained a lot of new skills and stuff.
+04:26 Okay. Thank you.</t>
         </is>
       </c>
     </row>
@@ -734,9 +890,17 @@
       <c r="B19" t="n">
         <v>14476</v>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>00:18 I'd like to talk about a challenging experience that I had with friends.  00:33 Challenging experience is that I was slightly unavailable for like a month or so because I was catching up on exams. Now I caught up, but my friends thought I was distancing myself and I just was focusing on studying more.  01:08 Now it went better because I realized that the problem was that I didn't tell them that and that they also didn't tell me how they felt. So it kind of increased over time, but now it's good.  01:43 Yeah, I'd say so. It allowed us to also know each other better, how we think and deal with situation.  02:11 Yeah, I'd definitely say so. And even though it was an unfortunate, I guess, experience, it could be for the better in some way because I got to know how they process things better and make them closer as friends.  02:45 But for example, how would you have communicated instead of what I did and we did, what are some like ways of doing that?  03:30 Yeah, that makes sense. That's what I did. I guess I just did it too late. But again, it wasn't a big issue either. So it was. It was an easy fix. It was just really the time effect that we hadn't discussed it in a while. That's it.  04:05 Yeah, exactly. Yeah. And also how often should. No way. I mean, I think that. I think that the problem now makes sense to me. Yeah,.  04:45 Yeah, definitely. And one last thing like. Yeah, I'm out of questions.</t>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>00:18 I'd like to talk about a challenging experience that I had with friends.
+00:33 Challenging experience is that I was slightly unavailable for like a month or so because I was catching up on exams. Now I caught up, but my friends thought I was distancing myself and I just was focusing on studying more.
+01:08 Now it went better because I realized that the problem was that I didn't tell them that and that they also didn't tell me how they felt. So it kind of increased over time, but now it's good.
+01:43 Yeah, I'd say so. It allowed us to also know each other better, how we think and deal with situation.
+02:11 Yeah, I'd definitely say so. And even though it was an unfortunate, I guess, experience, it could be for the better in some way because I got to know how they process things better and make them closer as friends.
+02:45 But for example, how would you have communicated instead of what I did and we did, what are some like ways of doing that?
+03:30 Yeah, that makes sense. That's what I did. I guess I just did it too late. But again, it wasn't a big issue either. So it was. It was an easy fix. It was just really the time effect that we hadn't discussed it in a while. That's it.
+04:05 Yeah, exactly. Yeah. And also how often should. No way. I mean, I think that. I think that the problem now makes sense to me. Yeah,.
+04:45 Yeah, definitely. And one last thing like. Yeah, I'm out of questions.</t>
         </is>
       </c>
     </row>
@@ -749,9 +913,15 @@
       <c r="B20" t="n">
         <v>14593</v>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>00:03 Thank you. I would like to talk about a challenging interaction I had recently with some group teammates in my tutorial. So I think the biggest problem was that I felt like my ambitions in the project that were supposed to do were not aligned with what they were aiming for. And so I felt like I was kind of left to myself a little bit. I'd say, honestly, just different ambitions in, like, the great goals that we wanted to get. And yeah, I think that was the biggest problem.  01:47 Honestly, I've noticed and learned that a lot of the times it's just easier to then do more work and kind of make it better rather than pushing them to do more. Because I'd rather just. Yeah, I'd rather not push them to do something they don't want to do. And also, I don't believe that they would do it as well as I did. Maybe to some extent. I think it very much depends on the environment. I think that in the sort of PBL system that I'm doing at my university, I think that a lot of the times it will be this way. Not always, of course. You might also get people that have similar ambition and similar goals. However, I think that most of the time, yes, it will be that way, but I don't know later in work life or anything.  03:00 I think that a lot of the times people will be more aligned with you and your ambition.  03:33 Not necessarily. I mean, hard skills, maybe like just doing the work and learning while doing the work. Yeah, but like, not necessarily like team skills, because, as I said, a lot of the time it's just. I'll just do it rather than necessarily communicating it with them because it's just easier and more efficient and the outcome is better. I see what you're doing.  04:18 Do you have a question. Maybe. I don't know what else to tell you.  04:41 When I read through, like. I mean, they didn't do anything. They didn't do nothing. Right. They did something. And when I read through it and I was like, this is just not good quality, that was very frustrating.  05:11 Fixing it myself the same way I did with other stuff. Yeah. I mean, you can't communicate. But as I said, I think it's just. I'd rather have the good, like a better outcome rather than also forcing people that really don't care as much to do it, you know? Hello.</t>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>00:03 Thank you. I would like to talk about a challenging interaction I had recently with some group teammates in my tutorial. So I think the biggest problem was that I felt like my ambitions in the project that were supposed to do were not aligned with what they were aiming for. And so I felt like I was kind of left to myself a little bit. I'd say, honestly, just different ambitions in, like, the great goals that we wanted to get. And yeah, I think that was the biggest problem.
+01:47 Honestly, I've noticed and learned that a lot of the times it's just easier to then do more work and kind of make it better rather than pushing them to do more. Because I'd rather just. Yeah, I'd rather not push them to do something they don't want to do. And also, I don't believe that they would do it as well as I did. Maybe to some extent. I think it very much depends on the environment. I think that in the sort of PBL system that I'm doing at my university, I think that a lot of the times it will be this way. Not always, of course. You might also get people that have similar ambition and similar goals. However, I think that most of the time, yes, it will be that way, but I don't know later in work life or anything.
+03:00 I think that a lot of the times people will be more aligned with you and your ambition.
+03:33 Not necessarily. I mean, hard skills, maybe like just doing the work and learning while doing the work. Yeah, but like, not necessarily like team skills, because, as I said, a lot of the time it's just. I'll just do it rather than necessarily communicating it with them because it's just easier and more efficient and the outcome is better. I see what you're doing.
+04:18 Do you have a question. Maybe. I don't know what else to tell you.
+04:41 When I read through, like. I mean, they didn't do anything. They didn't do nothing. Right. They did something. And when I read through it and I was like, this is just not good quality, that was very frustrating.
+05:11 Fixing it myself the same way I did with other stuff. Yeah. I mean, you can't communicate. But as I said, I think it's just. I'd rather have the good, like a better outcome rather than also forcing people that really don't care as much to do it, you know? Hello.</t>
         </is>
       </c>
     </row>
@@ -764,9 +934,14 @@
       <c r="B21" t="n">
         <v>14251</v>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>00:15 Hi Eduardo, nice to meet you. I would like to talk about an interaction I had in university with my group that was not as pleasant as I thought it would be.  00:38 Yes, sure. So was in a group work and it was a problem that occurred because I want to achieve a good grade and the work that my project teammates did was not that good as I would have expected and how it should have been for a good presentation and a good grade. So I didn't really know how to handle the situation because I wanted to prompt a different alternative to their task solution. But they didn't really were quite, yeah, I don't know, convinced. And then it was like a conflict of what we should do now. I knew that we their answer was not as good and great as how it really was for their experience. And I also didn't want to offend them and didn't really know how to say nicely that we should take a different solution.  01:58 Yes, I thought about it and I also talked to various other team members and asked them what they thought which solution would better. And also I tried to compare, not really compare, to show that there's a worse and not good, but to show where their solution might have some flaws and be as not as efficient than my solution. And I try to do communicate that in a very nice way. But it's still. If someone is said to their mind that their minds and thoughts are the right ones, then it's hard to convince them otherwise.  03:11 Absolutely. I agree. It was really kind of difficult now. So from the beginning didn't really know how to approach this problem because I had previously also met other people were like, I know people who are really then very fastly offended if someone doesn't like their idea and they always think that they're input is the best. And it's really hard then to work with these people and it's just unnecessary stress that would general be generated in the group. So it was really going on my nerves and was hard for me to really work without being like mean or like people thought I would be mean and yeah, hard.  04:26 Yes, absolutely. I mean, of course I want to get the best outcome and I really focus on having a good grade. But the group dynamic is really important because it doesn't make any sense if I'm just doing everything alone, for example, or excluding someone. That would be very disrespectful and not the values I want to present to someone else, so.  05:07 Yes, that's absolutely true. And I also. It was a tough situation, but then later we got to a solution. We found a compromise and had a really great outcome of the project. Hello. Hi. How was it? Should I stop? I can just take it off. I'll reset the whole room for the next person. Perfect. Did you enjoy it? Yeah, it was interesting. That's one of the three adjectives that most people use.    Transcribed by https://fireflies.ai/</t>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>00:15 Hi Eduardo, nice to meet you. I would like to talk about an interaction I had in university with my group that was not as pleasant as I thought it would be.
+00:38 Yes, sure. So was in a group work and it was a problem that occurred because I want to achieve a good grade and the work that my project teammates did was not that good as I would have expected and how it should have been for a good presentation and a good grade. So I didn't really know how to handle the situation because I wanted to prompt a different alternative to their task solution. But they didn't really were quite, yeah, I don't know, convinced. And then it was like a conflict of what we should do now. I knew that we their answer was not as good and great as how it really was for their experience. And I also didn't want to offend them and didn't really know how to say nicely that we should take a different solution.
+01:58 Yes, I thought about it and I also talked to various other team members and asked them what they thought which solution would better. And also I tried to compare, not really compare, to show that there's a worse and not good, but to show where their solution might have some flaws and be as not as efficient than my solution. And I try to do communicate that in a very nice way. But it's still. If someone is said to their mind that their minds and thoughts are the right ones, then it's hard to convince them otherwise.
+03:11 Absolutely. I agree. It was really kind of difficult now. So from the beginning didn't really know how to approach this problem because I had previously also met other people were like, I know people who are really then very fastly offended if someone doesn't like their idea and they always think that they're input is the best. And it's really hard then to work with these people and it's just unnecessary stress that would general be generated in the group. So it was really going on my nerves and was hard for me to really work without being like mean or like people thought I would be mean and yeah, hard.
+04:26 Yes, absolutely. I mean, of course I want to get the best outcome and I really focus on having a good grade. But the group dynamic is really important because it doesn't make any sense if I'm just doing everything alone, for example, or excluding someone. That would be very disrespectful and not the values I want to present to someone else, so.
+05:07 Yes, that's absolutely true. And I also. It was a tough situation, but then later we got to a solution. We found a compromise and had a really great outcome of the project. Hello. Hi. How was it? Should I stop? I can just take it off. I'll reset the whole room for the next person. Perfect. Did you enjoy it? Yeah, it was interesting. That's one of the three adjectives that most people use.    Transcribed by https://fireflies.ai/</t>
         </is>
       </c>
     </row>
@@ -779,9 +954,17 @@
       <c r="B22" t="n">
         <v>14683</v>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>00:49 Hello, my name is Luis. How are you?  01:01 Oh, yeah, I'm also fine. I want to talk to you about something. Do you have a minute to listen to me?  01:18 First of all, where are we? What room is it?  01:33 No, it does not. There's no. Oh, yeah, it is. Oh, yeah, it is. You're right.  01:46 Alright, man, in this cozy spot, I want to talk to you about my classmates. We had a presentation. We had to obviously prepare the presentation to present it to our class. It was quite a big presentation, so we had to split up the tasks and so on. You get what I mean?  02:21 Yes, all right. My classmates, I mean, were a group of three. So me and two others. My other classmate, her name is Lynn, and she was great. She did all her tasks and were able to present it to each other and so on. But my other classmate, he was a Dutch guy, he didn't do anything and we had to cover his part. Even though we told him many, many times that he should do his task because it's not fair. We have to do his part because it was such a big presentation and very many tasks to do. Now, what should I do to convince him to do the task? I mean, we did it afterwards, so he didn't do anything. But should I go to the teacher and tell him about it or should I. What should I do?  03:47 Well, we've already tried many times. As I've already said. Maybe you all heard it. We have tried to convince him and ask him to do it, but he ended up didn't. So I should go to the teacher next award.  04:28 Alright, man. Thank you for listening to me. Do you want to talk about something? You seem kinda. Kinda annoyed. Your facial expression shows me that you have something on your mind.  05:02 That was basically it, man. Do you have any other advices for me for my study? I study international business in Maastricht and. Yeah, what's the game plan? What should I do next?</t>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>00:49 Hello, my name is Luis. How are you?
+01:01 Oh, yeah, I'm also fine. I want to talk to you about something. Do you have a minute to listen to me?
+01:18 First of all, where are we? What room is it?
+01:33 No, it does not. There's no. Oh, yeah, it is. Oh, yeah, it is. You're right.
+01:46 Alright, man, in this cozy spot, I want to talk to you about my classmates. We had a presentation. We had to obviously prepare the presentation to present it to our class. It was quite a big presentation, so we had to split up the tasks and so on. You get what I mean?
+02:21 Yes, all right. My classmates, I mean, were a group of three. So me and two others. My other classmate, her name is Lynn, and she was great. She did all her tasks and were able to present it to each other and so on. But my other classmate, he was a Dutch guy, he didn't do anything and we had to cover his part. Even though we told him many, many times that he should do his task because it's not fair. We have to do his part because it was such a big presentation and very many tasks to do. Now, what should I do to convince him to do the task? I mean, we did it afterwards, so he didn't do anything. But should I go to the teacher and tell him about it or should I. What should I do?
+03:47 Well, we've already tried many times. As I've already said. Maybe you all heard it. We have tried to convince him and ask him to do it, but he ended up didn't. So I should go to the teacher next award.
+04:28 Alright, man. Thank you for listening to me. Do you want to talk about something? You seem kinda. Kinda annoyed. Your facial expression shows me that you have something on your mind.
+05:02 That was basically it, man. Do you have any other advices for me for my study? I study international business in Maastricht and. Yeah, what's the game plan? What should I do next?</t>
         </is>
       </c>
     </row>
@@ -794,9 +977,14 @@
       <c r="B23" t="n">
         <v>15178</v>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>00:29 Okay, perfect. So I want to talk to you about a recent situation where I had a conversation with some friends of mine where we had some difficulties. We were planning a trip for next weekend and yeah, weren't quite aligned in how we want to travel to our destination. So we had some disagreements there.  01:12 So it was about many factors. So to start off, we are six people who want to travel to our destination and three of our friends, they want to travel on Thursday already and the rest of us want to travel on Friday. So we had some disagreements there because some of us wanted to skip a tutorial and some of us didn't want to skip the tutorial on Thursday and Friday. I mean, on Friday we all have to skip our tutorial anyways. So some of us didn't want to have like another skill. So this was the first problem. And then obviously we would all return on Monday here to Maastricht.  01:57 So we had some disagreements because all of the people traveling on Friday, they want to go by train, whilst the people going on Thursday already, they were suggesting why we not come there after them with the car and then all go back by car.  02:41 So personally, I'm also part of the group that wants to travel on Friday as I don't want to skip my tutorial on Thursday. And then regarding the issue of whether we go by train or by car, I actually don't really mind. I think both will be, yeah, like the same amount of money spent on it. And actually I feel like train is a bit more relaxing and you have some time to do something for university while in the car. You're not gonna do anything for university. So actually I would prefer going by train, but for me that's not that of a big decision. But I have to say, of course, going by cars also really exhausting driving eight hours or something. So prefer the train. Actually.  04:07 Yeah, I mean, as the others are going on Thursday anyways, they already booked their trains. I feel like the biggest decision we have to make is how we gotta travel back on Monday. So I think we have to find a solution there as they want us to come with the car and then we all go back by car. Or the other option is that we all go by train. So it's a bit of a tricky situation.  05:02 Yeah, probably. Hello. Hi. How was that? Cool. You liked it?</t>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>00:29 Okay, perfect. So I want to talk to you about a recent situation where I had a conversation with some friends of mine where we had some difficulties. We were planning a trip for next weekend and yeah, weren't quite aligned in how we want to travel to our destination. So we had some disagreements there.
+01:12 So it was about many factors. So to start off, we are six people who want to travel to our destination and three of our friends, they want to travel on Thursday already and the rest of us want to travel on Friday. So we had some disagreements there because some of us wanted to skip a tutorial and some of us didn't want to skip the tutorial on Thursday and Friday. I mean, on Friday we all have to skip our tutorial anyways. So some of us didn't want to have like another skill. So this was the first problem. And then obviously we would all return on Monday here to Maastricht.
+01:57 So we had some disagreements because all of the people traveling on Friday, they want to go by train, whilst the people going on Thursday already, they were suggesting why we not come there after them with the car and then all go back by car.
+02:41 So personally, I'm also part of the group that wants to travel on Friday as I don't want to skip my tutorial on Thursday. And then regarding the issue of whether we go by train or by car, I actually don't really mind. I think both will be, yeah, like the same amount of money spent on it. And actually I feel like train is a bit more relaxing and you have some time to do something for university while in the car. You're not gonna do anything for university. So actually I would prefer going by train, but for me that's not that of a big decision. But I have to say, of course, going by cars also really exhausting driving eight hours or something. So prefer the train. Actually.
+04:07 Yeah, I mean, as the others are going on Thursday anyways, they already booked their trains. I feel like the biggest decision we have to make is how we gotta travel back on Monday. So I think we have to find a solution there as they want us to come with the car and then we all go back by car. Or the other option is that we all go by train. So it's a bit of a tricky situation.
+05:02 Yeah, probably. Hello. Hi. How was that? Cool. You liked it?</t>
         </is>
       </c>
     </row>
@@ -809,9 +997,19 @@
       <c r="B24" t="n">
         <v>15112</v>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>00:17 I would like you to help me resolve a problem that I have with my manager.  00:35 Me and my manager were talking about work hours and she told me that she wanted me to work a lot. So we planned a lot of dates for me to work and eventually we came to the conclusion that I would work every Tuesday, four times a week. And then another co worker of me texted me that he also works those days and that he will be taking over my shifts. But my manager didn't tell this to me.  01:26 I am hoping that I could get the hours back.  01:55 Well, actually I already approached her.  02:10 She did give me explanation and said that I could have the hours back, but she wasn't too happy about it and she didn't really want to admit that she made a mistake. And that's what's basically, that's what I'm not really happy about, that she cannot admit that she made a mistake.  02:55 I'm looking for ways to move forward. I guess.  03:26 The thing is, whenever I try to explain to her how I'm feeling, she talks over me.  03:58 Yes, that may help.  04:16 Side Yes, I think that as well.  04:35 Yes, I will try to talk to her again then.  04:55 It feels like she doesn't give me a chance to respond. Hello. How did it go? Good. Where should I oh, don't worry, I'll reset it for you. Did you enjoy it? It was cool.</t>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>00:17 I would like you to help me resolve a problem that I have with my manager.
+00:35 Me and my manager were talking about work hours and she told me that she wanted me to work a lot. So we planned a lot of dates for me to work and eventually we came to the conclusion that I would work every Tuesday, four times a week. And then another co worker of me texted me that he also works those days and that he will be taking over my shifts. But my manager didn't tell this to me.
+01:26 I am hoping that I could get the hours back.
+01:55 Well, actually I already approached her.
+02:10 She did give me explanation and said that I could have the hours back, but she wasn't too happy about it and she didn't really want to admit that she made a mistake. And that's what's basically, that's what I'm not really happy about, that she cannot admit that she made a mistake.
+02:55 I'm looking for ways to move forward. I guess.
+03:26 The thing is, whenever I try to explain to her how I'm feeling, she talks over me.
+03:58 Yes, that may help.
+04:16 Side Yes, I think that as well.
+04:35 Yes, I will try to talk to her again then.
+04:55 It feels like she doesn't give me a chance to respond. Hello. How did it go? Good. Where should I oh, don't worry, I'll reset it for you. Did you enjoy it? It was cool.</t>
         </is>
       </c>
     </row>
@@ -824,9 +1022,17 @@
       <c r="B25" t="n">
         <v>13327</v>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>00:00 I'll be back. Thank you. Okay, I'm here. I'm here to talk about the challenging interaction I've had.  00:33 I mean, it was about a group work, so we had to work about a presentation, but nobody was working at all. And it was like, I don't know, 30 minutes before class, so we had to do something. But I was just sending messages in the group chat also the day before, but nobody was replying, so I just didn't know what to do. And it was pretty challenging because then the day after, when we had to present, they actually had stuff to present without letting me know.  01:28 I mean, at the end we just had to choose one of the group members to present. So I handled it like I didn't do anything at the end because they said maybe they're thinking that I should do everything when I don't actually have to do everything, you know? So at the end, one of the group members, they just did a presentation in, like, five minutes, and then they presented right away.  02:17 I mean, at the end, it turned out very well, and the tutor liked the presentation, so I guess it was fine. But I can tell that it was kind of frustrating because I wanted things to be done, but at the same time, I didn't want to do everything by myself. So. Yeah,.  03:01 Yeah, I mean, you're right, but I wanted to do that as well. But as I said, when I was texting in the group chat, nobody was replying. And every time I was sending messages, they were like, nobody has started yet, and that's it. And when I said that we should, like, split the work and, you know, just do it before the class, nobody was replying again. So I don't know.  03:53 Yeah, I told them, but apparently they just. I mean, at the end, they had something and we did something and we presented something. But still, like, it's pretty tough.  04:26 Yeah, exactly. So it's fine. I mean, I'm good with myself, so it's perfect.  04:47 Yeah, true. Thank you for listening, though.  05:00 Thank you.</t>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>00:00 I'll be back. Thank you. Okay, I'm here. I'm here to talk about the challenging interaction I've had.
+00:33 I mean, it was about a group work, so we had to work about a presentation, but nobody was working at all. And it was like, I don't know, 30 minutes before class, so we had to do something. But I was just sending messages in the group chat also the day before, but nobody was replying, so I just didn't know what to do. And it was pretty challenging because then the day after, when we had to present, they actually had stuff to present without letting me know.
+01:28 I mean, at the end we just had to choose one of the group members to present. So I handled it like I didn't do anything at the end because they said maybe they're thinking that I should do everything when I don't actually have to do everything, you know? So at the end, one of the group members, they just did a presentation in, like, five minutes, and then they presented right away.
+02:17 I mean, at the end, it turned out very well, and the tutor liked the presentation, so I guess it was fine. But I can tell that it was kind of frustrating because I wanted things to be done, but at the same time, I didn't want to do everything by myself. So. Yeah,.
+03:01 Yeah, I mean, you're right, but I wanted to do that as well. But as I said, when I was texting in the group chat, nobody was replying. And every time I was sending messages, they were like, nobody has started yet, and that's it. And when I said that we should, like, split the work and, you know, just do it before the class, nobody was replying again. So I don't know.
+03:53 Yeah, I told them, but apparently they just. I mean, at the end, they had something and we did something and we presented something. But still, like, it's pretty tough.
+04:26 Yeah, exactly. So it's fine. I mean, I'm good with myself, so it's perfect.
+04:47 Yeah, true. Thank you for listening, though.
+05:00 Thank you.</t>
         </is>
       </c>
     </row>
@@ -839,9 +1045,18 @@
       <c r="B26" t="n">
         <v>13822</v>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>00:24 Nothing really. I'm really chill. I think we should talk about a convers like a situation I had in my past that was challenging to me.  00:50 Yeah. So actually like last week I have like a leadership position in the student association and last week I had to fire. Fire is a hard word. But last week I had to fire someone from my commite because they were not contributing.  01:24 I think the person took it pretty well because I mean they knew that they weren't contributing enough to the committee and so I think it didn't come as a big surprise. However, it was stressful for me because beforehand I tried a lot to incorporate them in the team and it was just not a lot of things coming from them.  02:02 I'm feeling pretty good about it. I feel like it was a challenge for me as a first leadership role and I think I managed it pretty well.  02:32 Actually about this matter, maybe you could give me some advice for the future on how to handle rejections. So when I have to reject people like in the professional setting.  03:11 Okay, that sounds like great advice. What would be things that I like in a bit more deeper way. Things that I could incorporate into my day to day decision making in order to include people more in my position.  03:57 Okay, that already sounds like great advice from you. I'm really happy. What do you think the benefits are of incorporating a team culture that is healthy in a committee?  04:42 Okay, for resilience that you're talking about, could you maybe give more in depth solutions on how to build this resilience?  05:22 Okay, that already sounds like great advice. On different matter, what do you think how the people in my committee should handle their time to study and their time to contribute to the committee? What do you think is a good time management?  06:09 Okay, that sounds great. Thank you a lot. I think now I will end the conversation.</t>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>00:24 Nothing really. I'm really chill. I think we should talk about a convers like a situation I had in my past that was challenging to me.
+00:50 Yeah. So actually like last week I have like a leadership position in the student association and last week I had to fire. Fire is a hard word. But last week I had to fire someone from my commite because they were not contributing.
+01:24 I think the person took it pretty well because I mean they knew that they weren't contributing enough to the committee and so I think it didn't come as a big surprise. However, it was stressful for me because beforehand I tried a lot to incorporate them in the team and it was just not a lot of things coming from them.
+02:02 I'm feeling pretty good about it. I feel like it was a challenge for me as a first leadership role and I think I managed it pretty well.
+02:32 Actually about this matter, maybe you could give me some advice for the future on how to handle rejections. So when I have to reject people like in the professional setting.
+03:11 Okay, that sounds like great advice. What would be things that I like in a bit more deeper way. Things that I could incorporate into my day to day decision making in order to include people more in my position.
+03:57 Okay, that already sounds like great advice from you. I'm really happy. What do you think the benefits are of incorporating a team culture that is healthy in a committee?
+04:42 Okay, for resilience that you're talking about, could you maybe give more in depth solutions on how to build this resilience?
+05:22 Okay, that already sounds like great advice. On different matter, what do you think how the people in my committee should handle their time to study and their time to contribute to the committee? What do you think is a good time management?
+06:09 Okay, that sounds great. Thank you a lot. I think now I will end the conversation.</t>
         </is>
       </c>
     </row>
@@ -854,9 +1069,18 @@
       <c r="B27" t="n">
         <v>14155</v>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>00:00 Five minutes. Enjoy it. Yeah. Thank you. So I recently. So I recently had this challenging experience in my last period in university with a group member who didn't really participate and really was really mean to us all. And I wanted to talk with you about this.  00:57 So we had this presentation that made like 50% of our grade and he didn't really participate. He was really like mean and he didn't come when we like said that we will meet up. And in general the work with him was really bad so that we in the end didn't really have this great presentation too. So it also like failed a bit. Our grace.  01:32 So we tried to talk to him and you know, just talk about our issues and problems, but he didn't really listen and sometimes he was also like lying when we like for example, wanted to meet up. So.  02:00 Yes, we did. We talked with our tutor but like she didn't help us that much. But like in the end she told us that she would just give him a worse grade. But it didn't really, you know, it didn't really benefit us because in general we got also like a worse grade. So.  02:36 Well, obviously we couldn't decide who which person participates in our presentation group so. So we couldn't do. I can't do much about it. I think I just have to learn like to work also like when we talk about education and work experience, how to work with people like him who are bit more problematic and where you like can't work that well. I think this is just something which you have to learn over the time.  03:22 Yeah, it could possibly be. I don't know.  03:45 Thank you so much. Means a lot. Nice words.  04:00 No, in general, I think this is just something. Do you have, like, maybe some advices on how to work with people, you know, who are not that very cooperative?  04:37 Yes, I think I thought the same. So I think we have here the same opinion. Well, we tried in the end to also, like, do this, but yeah, I think in general we have the same opinion on this.  05:01 All right. Thank you.</t>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>00:00 Five minutes. Enjoy it. Yeah. Thank you. So I recently. So I recently had this challenging experience in my last period in university with a group member who didn't really participate and really was really mean to us all. And I wanted to talk with you about this.
+00:57 So we had this presentation that made like 50% of our grade and he didn't really participate. He was really like mean and he didn't come when we like said that we will meet up. And in general the work with him was really bad so that we in the end didn't really have this great presentation too. So it also like failed a bit. Our grace.
+01:32 So we tried to talk to him and you know, just talk about our issues and problems, but he didn't really listen and sometimes he was also like lying when we like for example, wanted to meet up. So.
+02:00 Yes, we did. We talked with our tutor but like she didn't help us that much. But like in the end she told us that she would just give him a worse grade. But it didn't really, you know, it didn't really benefit us because in general we got also like a worse grade. So.
+02:36 Well, obviously we couldn't decide who which person participates in our presentation group so. So we couldn't do. I can't do much about it. I think I just have to learn like to work also like when we talk about education and work experience, how to work with people like him who are bit more problematic and where you like can't work that well. I think this is just something which you have to learn over the time.
+03:22 Yeah, it could possibly be. I don't know.
+03:45 Thank you so much. Means a lot. Nice words.
+04:00 No, in general, I think this is just something. Do you have, like, maybe some advices on how to work with people, you know, who are not that very cooperative?
+04:37 Yes, I think I thought the same. So I think we have here the same opinion. Well, we tried in the end to also, like, do this, but yeah, I think in general we have the same opinion on this.
+05:01 All right. Thank you.</t>
         </is>
       </c>
     </row>
@@ -869,9 +1093,15 @@
       <c r="B28" t="n">
         <v>19765</v>
       </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>00:10 Hi, Eduardo. Nice to meet you. So I had like a discussion with my boss about getting more free hours, but he wouldn't give in and won't give me the hours. So. Yeah, that was really unfortunate.  00:48 I think I'm really important at work, so I feel like I'm also, yeah, I can again, I earn the extra hours, but yeah, I hope when I talk to him again that he might give me the hours instead of like, being how he's treating me now.  01:37 Yeah, I hope so. Good point. I will. Yeah, tell him that.  01:56 Thank you. Do you have any other tips? Eduardo, do you get any. Do you have any other tips?  02:39 Okay, thank you very much. That that's true. Is there maybe another way instead of talking to him to get what I. Eduardo, is there anything else I can do instead of talking to him again? Because I think he maybe still won't give me the extra hours.  03:39 Okay. Yeah, I think. I think I know someone who's also handling the schedules and everything, so maybe that person can give me extra free time and I also gonna write an email. So that was also a really good tip.  04:19 Thank you very much, Eduardo.</t>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>00:10 Hi, Eduardo. Nice to meet you. So I had like a discussion with my boss about getting more free hours, but he wouldn't give in and won't give me the hours. So. Yeah, that was really unfortunate.
+00:48 I think I'm really important at work, so I feel like I'm also, yeah, I can again, I earn the extra hours, but yeah, I hope when I talk to him again that he might give me the hours instead of like, being how he's treating me now.
+01:37 Yeah, I hope so. Good point. I will. Yeah, tell him that.
+01:56 Thank you. Do you have any other tips? Eduardo, do you get any. Do you have any other tips?
+02:39 Okay, thank you very much. That that's true. Is there maybe another way instead of talking to him to get what I. Eduardo, is there anything else I can do instead of talking to him again? Because I think he maybe still won't give me the extra hours.
+03:39 Okay. Yeah, I think. I think I know someone who's also handling the schedules and everything, so maybe that person can give me extra free time and I also gonna write an email. So that was also a really good tip.
+04:19 Thank you very much, Eduardo.</t>
         </is>
       </c>
     </row>
@@ -884,9 +1114,19 @@
       <c r="B29" t="n">
         <v>14038</v>
       </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>00:19 Great to meet you too. Yeah, about. I'm just chilling. I have this study today and after that I have my tutorial and then I will drive back home.  00:42 Yeah, I think it's great. Sometimes it's a lot of work, a lot of reading, but I think it's going smooth.  01:06 I try to keep up with the flow and because we're having our exams in around four weeks, I try to keep in the flow and try to practice for the exam.  01:35 I think it's pretty balanced because when the subject started I tried to go with the flow and therefore I think I don't have any problems with it.  02:01 Yes, of course. Do you have any jokes to tell me?  02:17 That's a great joke. I like that. How about you? How is your time? How do you spend your time?  02:39 That. That sounds great. I like that.  02:52 Yeah, I just wanted to talk about the recent situation I had with my past landlord. If you're interested in it.  03:13 I moved out in January, but the contract was until July, so I moved out earlier. But I found a new tenant for him and he said everything is alright. And then I was waiting for the payback of. Or the reimbursement of the. Yeah, of the half monthly rent of January and I was sending an email to his secretary, and she answered that they don't want to pay back it because it's not stated in the contract. And then I was in the situation to handle it with the landlord and his secretary because he wrote me that they will pay back the half of the monthly rent of January.  04:16 Yeah, I wrote his secretary and said to her that or sent her a screenshot of the chapel. The landlord that he sent me that I will get the payback of the monthly rent and told the landlord that I will follow up to the secretary. And then he sent the money back to me because there was no chance that he can get out of the situation in another way because he stated that he will pay back the rent.  05:04 Yeah, of course it was a win for me. And I think I handled the situation good and everything came to a good end.</t>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>00:19 Great to meet you too. Yeah, about. I'm just chilling. I have this study today and after that I have my tutorial and then I will drive back home.
+00:42 Yeah, I think it's great. Sometimes it's a lot of work, a lot of reading, but I think it's going smooth.
+01:06 I try to keep up with the flow and because we're having our exams in around four weeks, I try to keep in the flow and try to practice for the exam.
+01:35 I think it's pretty balanced because when the subject started I tried to go with the flow and therefore I think I don't have any problems with it.
+02:01 Yes, of course. Do you have any jokes to tell me?
+02:17 That's a great joke. I like that. How about you? How is your time? How do you spend your time?
+02:39 That. That sounds great. I like that.
+02:52 Yeah, I just wanted to talk about the recent situation I had with my past landlord. If you're interested in it.
+03:13 I moved out in January, but the contract was until July, so I moved out earlier. But I found a new tenant for him and he said everything is alright. And then I was waiting for the payback of. Or the reimbursement of the. Yeah, of the half monthly rent of January and I was sending an email to his secretary, and she answered that they don't want to pay back it because it's not stated in the contract. And then I was in the situation to handle it with the landlord and his secretary because he wrote me that they will pay back the half of the monthly rent of January.
+04:16 Yeah, I wrote his secretary and said to her that or sent her a screenshot of the chapel. The landlord that he sent me that I will get the payback of the monthly rent and told the landlord that I will follow up to the secretary. And then he sent the money back to me because there was no chance that he can get out of the situation in another way because he stated that he will pay back the rent.
+05:04 Yeah, of course it was a win for me. And I think I handled the situation good and everything came to a good end.</t>
         </is>
       </c>
     </row>
@@ -899,9 +1139,20 @@
       <c r="B30" t="n">
         <v>14125</v>
       </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>00:06 We can talk about anything.  00:20 Probably just school, studies, exams, stuff like that.  00:38 Right now I'm just trying to make sure that I pass all my exams so that I don't have any resets. I've been working hard on the finance course, especially because finance it's quite math heavy and my math exams haven't been the great in the past I've passed. But yeah, definitely just focusing on finance.  01:19 I think it's definitely more about staying consistent. Consistency is key, right? So just lots of practice. Maybe start implementing some past papers because I haven't done that yet. And for the rest, yeah, just keep studying.  01:58 Yes, that sounds great. Thanks for the motivation, I guess.  02:17 I will do. So what's next?  02:41 When you say reward yourself, what do you mean by that? Like just mean like spending some time off or what does that really imply.  03:13 That sounds good. I'll be sure to implement that. Maybe I'll also like consider implementing more like sports as a sort of reward or just spending time with friends because studying all day is of course not good and could tire me out. Definitely.  03:49 Yes, thanks. Thanks for the help and good conversation. How should we proceed? This conversation?  04:18 You know, honestly, I think we've covered a lot. It's an eye opener. Maybe just. Do you like playing Padel? I've been getting into paddle recently.  04:43 Mostly I play singles, but no, no. I play doubles. What am I saying? Yeah, I play doubles, singles, paddle. Never really tried it. To be honest, I thought it was more of a double sport. But maybe sometime we can play together. Yeah. But thanks for the conversation and maybe see you next time out there on the courts. I like your office, by the way. Buddy.  05:22 Thank you. Bye.</t>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>00:06 We can talk about anything.
+00:20 Probably just school, studies, exams, stuff like that.
+00:38 Right now I'm just trying to make sure that I pass all my exams so that I don't have any resets. I've been working hard on the finance course, especially because finance it's quite math heavy and my math exams haven't been the great in the past I've passed. But yeah, definitely just focusing on finance.
+01:19 I think it's definitely more about staying consistent. Consistency is key, right? So just lots of practice. Maybe start implementing some past papers because I haven't done that yet. And for the rest, yeah, just keep studying.
+01:58 Yes, that sounds great. Thanks for the motivation, I guess.
+02:17 I will do. So what's next?
+02:41 When you say reward yourself, what do you mean by that? Like just mean like spending some time off or what does that really imply.
+03:13 That sounds good. I'll be sure to implement that. Maybe I'll also like consider implementing more like sports as a sort of reward or just spending time with friends because studying all day is of course not good and could tire me out. Definitely.
+03:49 Yes, thanks. Thanks for the help and good conversation. How should we proceed? This conversation?
+04:18 You know, honestly, I think we've covered a lot. It's an eye opener. Maybe just. Do you like playing Padel? I've been getting into paddle recently.
+04:43 Mostly I play singles, but no, no. I play doubles. What am I saying? Yeah, I play doubles, singles, paddle. Never really tried it. To be honest, I thought it was more of a double sport. But maybe sometime we can play together. Yeah. But thanks for the conversation and maybe see you next time out there on the courts. I like your office, by the way. Buddy.
+05:22 Thank you. Bye.</t>
         </is>
       </c>
     </row>
@@ -914,9 +1165,14 @@
       <c r="B31" t="n">
         <v>14899</v>
       </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>00:00 Hope you enjoy it. Yeah. Okay. Hello, Eduardo. Yeah, I recently had a challenging situation I want to talk about with you. What do you think? Like, I just remember in our tutorial group, we had to do a group presentation in Dorado, and then there were some participants that didn't like to do anything. And basically as soon as the deadline was there, I was the only person that felt responsible to do all the exercises. And I really feel bad about it. I think it's unfair. What do you think? Can you answer? I think it's not possible. It. Hello, Eduardo. I hope. Hello, Eduardo. I hope you can hear me. Perfect. Pleasure to meet you as well. Yeah, I recently had, like, a difficulty in university, actually. I just want to talk about this with you.  02:35 So, actually, for our tutorial group, we had to do a group presentation that is also graded. But however, like none of the four group members, I had felt responsible for doing anything. And in the end, the deadline approached and I was just doing the entire presentation because I didn't want to have a bad grade. But I think that's pretty unfair. Don't you think so? Because the others didn't do anything.  03:17 The thing is, I don't want to be a snitch and tell the professor I did everything. I mean, I could do it, and it would probably also save my grade. But I also don't like to, you know, snitch on the others. But I just think that if this will be repeated in the future, so I have, like, multiple scenarios like this, then I would go to the tutor or what would you recommend to me?  04:08 Yeah, okay. That actually sounds reasonable to me. I think, like, in the next time, maybe we can also, like me and my group members, we can talk about the ambitions we have because maybe they were just not that ambitious and said, okay, we don't really care about the grade, but I may be a person that wants to have, like a very good grade. So maybe talk about the ambitions first, and then you can still see whether you have to go to the tutor or not.  04:58 Okay, but maybe. Maybe, like, in regards of the process that we had, was there anything I could have said? Like, before, I did all the work alone, I mean, also, I was a bit angry, and I just did it all by myself without telling them because I was sure they wouldn't do the work anyway. So is there maybe anything I could improve during the process? So we can avoid that I have to do the entire presentation on my own?  05:51 That actually sounds reasonable. Thank you. Hello. Hello. Let me help you out with that. It was nice, but I think at the first time it didn't work out, so you had to restart it. Okay, no problem. If you were able, it'll.    Transcribed by https://fireflies.ai/</t>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>00:00 Hope you enjoy it. Yeah. Okay. Hello, Eduardo. Yeah, I recently had a challenging situation I want to talk about with you. What do you think? Like, I just remember in our tutorial group, we had to do a group presentation in Dorado, and then there were some participants that didn't like to do anything. And basically as soon as the deadline was there, I was the only person that felt responsible to do all the exercises. And I really feel bad about it. I think it's unfair. What do you think? Can you answer? I think it's not possible. It. Hello, Eduardo. I hope. Hello, Eduardo. I hope you can hear me. Perfect. Pleasure to meet you as well. Yeah, I recently had, like, a difficulty in university, actually. I just want to talk about this with you.
+02:35 So, actually, for our tutorial group, we had to do a group presentation that is also graded. But however, like none of the four group members, I had felt responsible for doing anything. And in the end, the deadline approached and I was just doing the entire presentation because I didn't want to have a bad grade. But I think that's pretty unfair. Don't you think so? Because the others didn't do anything.
+03:17 The thing is, I don't want to be a snitch and tell the professor I did everything. I mean, I could do it, and it would probably also save my grade. But I also don't like to, you know, snitch on the others. But I just think that if this will be repeated in the future, so I have, like, multiple scenarios like this, then I would go to the tutor or what would you recommend to me?
+04:08 Yeah, okay. That actually sounds reasonable to me. I think, like, in the next time, maybe we can also, like me and my group members, we can talk about the ambitions we have because maybe they were just not that ambitious and said, okay, we don't really care about the grade, but I may be a person that wants to have, like a very good grade. So maybe talk about the ambitions first, and then you can still see whether you have to go to the tutor or not.
+04:58 Okay, but maybe. Maybe, like, in regards of the process that we had, was there anything I could have said? Like, before, I did all the work alone, I mean, also, I was a bit angry, and I just did it all by myself without telling them because I was sure they wouldn't do the work anyway. So is there maybe anything I could improve during the process? So we can avoid that I have to do the entire presentation on my own?
+05:51 That actually sounds reasonable. Thank you. Hello. Hello. Let me help you out with that. It was nice, but I think at the first time it didn't work out, so you had to restart it. Okay, no problem. If you were able, it'll.    Transcribed by https://fireflies.ai/</t>
         </is>
       </c>
     </row>
@@ -929,9 +1185,17 @@
       <c r="B32" t="n">
         <v>14830</v>
       </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>00:29 Hi, Eduardo. I am Tom, and I want to talk about the discussion I had with my friend.  00:46 So, first of all, we talked about who's the better football player, Cristiano Ronaldo or Lionel Messi. And in my opinion, is that Cristiano Ronaldo, and for my friend's opinion, was Lionel Messi. So we had a tough conversation.  01:15 No, everything like stats and how important they are for their team and. Yeah, also their personal experience.  01:44 No, no, we disagreed. He was still with Lionel Messi, and I was with Cristiano Ronaldo. But in my opinion, Ronaldo is the better player because he scored more goals in total, and he started his career in Sporting, the Saban, and not like Lionel Messi at Barcelona. So Cristiano Ronaldo was not given the perfect team at the start, and he had to fight for everything. And. And Lionel Messi was, like, always given in the shoes.  02:37 And Cristiano Ronaldo is always there for his team if his team needs him. So, for example, at Juventus, when Juventus lost 20 against Atletico Madrid and the second leg, in the second game, Cristiano Ronaldo scored the hat trick. So this simply shows for me that Ronaldo is like a player who's there if his team needs him. And Lionel Messi is not always there.  03:21 Yeah. And what's your opinion about this debate? So, do you have an opinion, or what do you think? Who's the better player?  03:58 And after that debate, we got into the debate, which club is bigger and has a greater history? And for me, it was obviously Real Madrid and for Barcelona. And it's clear, right, if that Real Madrid has more trophies and more Champions League trophies, that they are the bigger club.  04:24 What do you think about it?  04:40 Hello? Do I have it?</t>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>00:29 Hi, Eduardo. I am Tom, and I want to talk about the discussion I had with my friend.
+00:46 So, first of all, we talked about who's the better football player, Cristiano Ronaldo or Lionel Messi. And in my opinion, is that Cristiano Ronaldo, and for my friend's opinion, was Lionel Messi. So we had a tough conversation.
+01:15 No, everything like stats and how important they are for their team and. Yeah, also their personal experience.
+01:44 No, no, we disagreed. He was still with Lionel Messi, and I was with Cristiano Ronaldo. But in my opinion, Ronaldo is the better player because he scored more goals in total, and he started his career in Sporting, the Saban, and not like Lionel Messi at Barcelona. So Cristiano Ronaldo was not given the perfect team at the start, and he had to fight for everything. And. And Lionel Messi was, like, always given in the shoes.
+02:37 And Cristiano Ronaldo is always there for his team if his team needs him. So, for example, at Juventus, when Juventus lost 20 against Atletico Madrid and the second leg, in the second game, Cristiano Ronaldo scored the hat trick. So this simply shows for me that Ronaldo is like a player who's there if his team needs him. And Lionel Messi is not always there.
+03:21 Yeah. And what's your opinion about this debate? So, do you have an opinion, or what do you think? Who's the better player?
+03:58 And after that debate, we got into the debate, which club is bigger and has a greater history? And for me, it was obviously Real Madrid and for Barcelona. And it's clear, right, if that Real Madrid has more trophies and more Champions League trophies, that they are the bigger club.
+04:24 What do you think about it?
+04:40 Hello? Do I have it?</t>
         </is>
       </c>
     </row>
@@ -944,9 +1208,22 @@
       <c r="B33" t="n">
         <v>15085</v>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>00:24 It's good, thank you.  00:35 I had a lot of sleep and I skipped class. I mean, it's not that good, but it was relaxing.  00:55 I'm gonna prepare for my classes and I have to do some grocery shopping. And then after, in the evening, I'm going to work.  01:23 I don't know. Could you repeat the question?  01:40 Yeah, I like to go to the gym. Gym to do strength training.  02:02 I'm going to start again next week because I had a bigger break from the gym, but I've been doing it for two or three years now.  02:27 Yes, I have a wedding come around and I want to lose weight for that and that's my plan.  02:50 Yes, that's exactly my plan.  03:04 Well, first I have to buy a subscription to the degeneration and then go like three or four times a week. So I actually do the exercises and the training. And also I want to have a diet consisting of eating less sweet things and just generally eating less.  03:46 Thank you. Yes,.  04:06 Feeling strong again? Because in the past few, three or four months, I've been feeling like I could feel weakening myself, like my body is weakening. And now if I go back to the gym, it's gonna get stronger again and I can feel powerful again. So it's good.  04:41 Yeah. I already done this once. Like, this extreme. I mean, not extreme, but like, bigger weight loss. Before, there was like a prom in my high school and I decided to lose weight for that, and I was able to lose actually 10kg in like two weeks just by cutting out every sweet things that I usually eat because I am a really sweet dude.  05:28 Yeah, but the thing is that I have some problems with overeating because even though I feel full sometimes I can't, like, stop because I know it's really good that, like, the food tastes amazing and everything like that. But I don't know what to do against that overeating problem. What do you suggest?  06:21 That's actually a good idea. I was thinking of sewing because I used to, but I don't have a sewing machine right now. Maastricht. But I would really like to do something fun or creative. I don't know. I try to draw every day, but that stops after a few months maybe. But yeah, I want to start that again. Yeah. So what kind of hobbies do you suggest? Maybe. It's still listening.    Transcribed by https://fireflies.ai/</t>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>00:24 It's good, thank you.
+00:35 I had a lot of sleep and I skipped class. I mean, it's not that good, but it was relaxing.
+00:55 I'm gonna prepare for my classes and I have to do some grocery shopping. And then after, in the evening, I'm going to work.
+01:23 I don't know. Could you repeat the question?
+01:40 Yeah, I like to go to the gym. Gym to do strength training.
+02:02 I'm going to start again next week because I had a bigger break from the gym, but I've been doing it for two or three years now.
+02:27 Yes, I have a wedding come around and I want to lose weight for that and that's my plan.
+02:50 Yes, that's exactly my plan.
+03:04 Well, first I have to buy a subscription to the degeneration and then go like three or four times a week. So I actually do the exercises and the training. And also I want to have a diet consisting of eating less sweet things and just generally eating less.
+03:46 Thank you. Yes,.
+04:06 Feeling strong again? Because in the past few, three or four months, I've been feeling like I could feel weakening myself, like my body is weakening. And now if I go back to the gym, it's gonna get stronger again and I can feel powerful again. So it's good.
+04:41 Yeah. I already done this once. Like, this extreme. I mean, not extreme, but like, bigger weight loss. Before, there was like a prom in my high school and I decided to lose weight for that, and I was able to lose actually 10kg in like two weeks just by cutting out every sweet things that I usually eat because I am a really sweet dude.
+05:28 Yeah, but the thing is that I have some problems with overeating because even though I feel full sometimes I can't, like, stop because I know it's really good that, like, the food tastes amazing and everything like that. But I don't know what to do against that overeating problem. What do you suggest?
+06:21 That's actually a good idea. I was thinking of sewing because I used to, but I don't have a sewing machine right now. Maastricht. But I would really like to do something fun or creative. I don't know. I try to draw every day, but that stops after a few months maybe. But yeah, I want to start that again. Yeah. So what kind of hobbies do you suggest? Maybe. It's still listening.    Transcribed by https://fireflies.ai/</t>
         </is>
       </c>
     </row>
@@ -959,9 +1236,18 @@
       <c r="B34" t="n">
         <v>13858</v>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>00:15 Hi. I would like to talk about a challenging experience. I had.  00:33 A friend of mine and I like, I haven't talked to her yet, but I feel like that I'll give her more in a friendship than she gives me. And I feel like very uncomfortable like telling her because I feel like I like to do that for her and I'm very open to do a lot for her, but I also just want to see her maybe give also something similar back. Like she does give some things back, but not as much that I do. I feel like.  01:27 I just don't want her to feel like I look at everything and everything should be 50. I do feel like there's situation where someone helps more and someone helps less. But in general I feel like some. Sometimes there is a bigger gap and just to close that a little would just help me. I feel like.  02:04 Yes.  02:16 Yeah, maybe. Or how I can tell her like secretly with not having an awkward conversation.  02:45 Okay. I feel like it's kind of difficult to like talk about it or because it makes it so awkward. Like nobody says, yeah, that was great, I would wish you to do that more often. I feel like it's an assault or like I tell her something to do and I don't want to do that.  03:32 I feel like I'll already do that and it's still not working.  04:00 I also try to be like more direct in some kind of jokes. Like trying to say it more like under cover. Under coverly. But like I don't want to be so persistent about it, so what can I do?  04:35 Yeah, but you tried that. It's not working.  05:01 I don't really want to have like this real conversation because it might get bigger than it is right now.</t>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>00:15 Hi. I would like to talk about a challenging experience. I had.
+00:33 A friend of mine and I like, I haven't talked to her yet, but I feel like that I'll give her more in a friendship than she gives me. And I feel like very uncomfortable like telling her because I feel like I like to do that for her and I'm very open to do a lot for her, but I also just want to see her maybe give also something similar back. Like she does give some things back, but not as much that I do. I feel like.
+01:27 I just don't want her to feel like I look at everything and everything should be 50. I do feel like there's situation where someone helps more and someone helps less. But in general I feel like some. Sometimes there is a bigger gap and just to close that a little would just help me. I feel like.
+02:04 Yes.
+02:16 Yeah, maybe. Or how I can tell her like secretly with not having an awkward conversation.
+02:45 Okay. I feel like it's kind of difficult to like talk about it or because it makes it so awkward. Like nobody says, yeah, that was great, I would wish you to do that more often. I feel like it's an assault or like I tell her something to do and I don't want to do that.
+03:32 I feel like I'll already do that and it's still not working.
+04:00 I also try to be like more direct in some kind of jokes. Like trying to say it more like under cover. Under coverly. But like I don't want to be so persistent about it, so what can I do?
+04:35 Yeah, but you tried that. It's not working.
+05:01 I don't really want to have like this real conversation because it might get bigger than it is right now.</t>
         </is>
       </c>
     </row>
@@ -974,9 +1260,22 @@
       <c r="B35" t="n">
         <v>14977</v>
       </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>00:23 Nothing much really.  00:35 I like to do sports, play basketball, work on myself. You know, regular things. Kind of that you would expect someone like me or my age to do. I like to keep myself fit, work on myself, try to make something out of myself, make use of the time.  01:09 Practice and we pretty much just play workout. I enjoy working out upper body, more chest, regular stuff I'd say.  01:31 Yes.  01:37 Not really. You know, you have my plan that I do and I try and follow it as much as possible. Possible. You know, there's no particular favorite one.  02:00 That's probably a good question, but I'd rather be for endurance since I'm an athlete. That's why I want to focus on. I don't want to be a pumped up bodybuilder. I'd rather be explosive and athletic.  02:30 Yep, that's true.  02:46 Yeah, yeah. You know, when I work out legs, I work out. One time I do plyometrics and I focus on athleticism. And the next day I do pure strength training with heavy lifting and small size of reps repetitions.  03:16 Yes,.  03:28 I could stick more to my workout plan, which is why it's not working as good, but that's on me. It's my fault.  03:51 Yeah, actually, yes. Short term goals would be more catching.  04:13 I think these are a little bit too general, but we can switch topics. I have a question for you.  04:26 So I do photography and videography and I did this video for a new student association here and I told them I'll do it fully for free. But we kind of came out of contact because I wanted them to feature my posts as a like, let's say you call it like a co editor post, like a cross post. But they wouldn't agree with that and they weren't very open with giving me a shout out next to. Although I did like all the work. And yeah, now we're kind of out of contact. How do you think you approach a situation like this?  05:10 Yes.</t>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>00:23 Nothing much really.
+00:35 I like to do sports, play basketball, work on myself. You know, regular things. Kind of that you would expect someone like me or my age to do. I like to keep myself fit, work on myself, try to make something out of myself, make use of the time.
+01:09 Practice and we pretty much just play workout. I enjoy working out upper body, more chest, regular stuff I'd say.
+01:31 Yes.
+01:37 Not really. You know, you have my plan that I do and I try and follow it as much as possible. Possible. You know, there's no particular favorite one.
+02:00 That's probably a good question, but I'd rather be for endurance since I'm an athlete. That's why I want to focus on. I don't want to be a pumped up bodybuilder. I'd rather be explosive and athletic.
+02:30 Yep, that's true.
+02:46 Yeah, yeah. You know, when I work out legs, I work out. One time I do plyometrics and I focus on athleticism. And the next day I do pure strength training with heavy lifting and small size of reps repetitions.
+03:16 Yes,.
+03:28 I could stick more to my workout plan, which is why it's not working as good, but that's on me. It's my fault.
+03:51 Yeah, actually, yes. Short term goals would be more catching.
+04:13 I think these are a little bit too general, but we can switch topics. I have a question for you.
+04:26 So I do photography and videography and I did this video for a new student association here and I told them I'll do it fully for free. But we kind of came out of contact because I wanted them to feature my posts as a like, let's say you call it like a co editor post, like a cross post. But they wouldn't agree with that and they weren't very open with giving me a shout out next to. Although I did like all the work. And yeah, now we're kind of out of contact. How do you think you approach a situation like this?
+05:10 Yes.</t>
         </is>
       </c>
     </row>
@@ -989,9 +1288,16 @@
       <c r="B36" t="n">
         <v>6</v>
       </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>00:04 Thanks. Yeah, so I actually want to talk about a situation that recently happened with my friend. And I still feel I don't have enough closure about it because it was a situation that really hurt my feelings. And I also understand the side of the other person. But for me it was quite a stressful experience as a friend because I really value my friends and my friendship with other people. I feel like I am giving myself 100% and I'm not receiving the same from the other people. So. Yeah,.  01:04 So actually there were more situations that was, you know, feel like building up. And at one point I felt like a jar that was so full that it just, you know, broke. So actually the things started from Easter. For me, Easter is a very important celebration where we gather families in Moldova. I always been around my family and to be honest, I really was waiting for this friend to come over because we wanted to cook some traditional meals together and also paint the eggs because it's also a tradition that we do for Easter. And she was on a trip and she just returned the same day when I was supposed to do all these things. And she didn't because she said she was too tired, which I also understand.  01:50 But the next day, the morning of the Easter, I was really expecting her to be there, but she was very late. And it really hurted my feelings, but I said okay. Then another situation that happened is that since then she was not really in contact with me, not really texting, calling. If the calls or texts don't come from my side, then she would not even bother to call me or to message me. And it really also bothers me because all the time when I go to her, I never go empty handed, all the time bring flowers, chocolates, I all the time text her all the time I was worried about her when she was not answering for some days. And I don't share the same experience. So I feel like I deserve the same attitude and respect from my friends.  02:31 And also bothered me is that she all the time complained that she doesn't have enough budget, not enough time to go on a trip, a girls trip that I also was dreaming about for a long time. And then recently I saw some pictures and videos on Instagram of her that she was with other friends. And it really hurted me because it felt like she has time and budget for other people, but not for myself. And another thing Is that in Moldova, our parents sometimes send us some packages and it comes from a minibus. And you never know when those people would be in Netherlands, because we are here established. And yeah, I wasn't expecting any package. And at one point I got a lot of calls from foreign numbers, like German numbers. And I usually don't answer, you know, the phones to strange people.  03:25 And I said, okay, let me answer the phone. And there was like a man screaming at me, like, why I'm not answering my phone? Because I'm supposed to get a package from Moldova. And actually her parents sent the package to her in Netherlands, but because she was not home, they gave the people that deliver the packages my phone number. And I had to like, all the time be stressed about it. And, you know, I also didn't like that. And recently also was my birthday of my boyfriend. And she also couldn't make it because of the other reason that she had and because she had to attend another event with her boyfriend. So there was a lot of events that just built up and it felt really hurtful because I also approached her, I texted her.  04:07 Maybe it's not the best approach because, yeah, I also don't like this long text where I have to describe everything. And sometimes maybe you don't get the nice tone out of it. Maybe you understand completely different the message. But I still felt like I needed to express myself because I really value all the friendship that I have. And when I'm like, I also lived a lot of betrayals when it comes to friendships. And maybe I don't have so many friends at the moment, but the ones that I have, they're super nice, you know, like, it's not about the quantity, but quality. And that's why I approached her. And she got really offensive because she said that I make her feel the victim.  04:45 And it's not nice for me to put so much pressure on her because maybe on Instagram, on videos that you have, maybe life feels like pink and. And shiny, but actually in the reality is not, yeah, same. And she. That was failing a lot of courses, but I'm not sure if it was my mistake because, yeah, this is how I feel at the moment. And it was quite a stressful experience for me. And at the moment we still are in touch, but not so often and not so in depth as we used to be. And also made myself a conclusion that maybe I have to step a bit back and give myself and herself a bit of space. And yeah, maybe I will not put 100% anymore because it feels like not worth it.  06:17 So maybe you can give me some advices of how I should act next. Like what would be the further next steps?</t>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>00:04 Thanks. Yeah, so I actually want to talk about a situation that recently happened with my friend. And I still feel I don't have enough closure about it because it was a situation that really hurt my feelings. And I also understand the side of the other person. But for me it was quite a stressful experience as a friend because I really value my friends and my friendship with other people. I feel like I am giving myself 100% and I'm not receiving the same from the other people. So. Yeah,.
+01:04 So actually there were more situations that was, you know, feel like building up. And at one point I felt like a jar that was so full that it just, you know, broke. So actually the things started from Easter. For me, Easter is a very important celebration where we gather families in Moldova. I always been around my family and to be honest, I really was waiting for this friend to come over because we wanted to cook some traditional meals together and also paint the eggs because it's also a tradition that we do for Easter. And she was on a trip and she just returned the same day when I was supposed to do all these things. And she didn't because she said she was too tired, which I also understand.
+01:50 But the next day, the morning of the Easter, I was really expecting her to be there, but she was very late. And it really hurted my feelings, but I said okay. Then another situation that happened is that since then she was not really in contact with me, not really texting, calling. If the calls or texts don't come from my side, then she would not even bother to call me or to message me. And it really also bothers me because all the time when I go to her, I never go empty handed, all the time bring flowers, chocolates, I all the time text her all the time I was worried about her when she was not answering for some days. And I don't share the same experience. So I feel like I deserve the same attitude and respect from my friends.
+02:31 And also bothered me is that she all the time complained that she doesn't have enough budget, not enough time to go on a trip, a girls trip that I also was dreaming about for a long time. And then recently I saw some pictures and videos on Instagram of her that she was with other friends. And it really hurted me because it felt like she has time and budget for other people, but not for myself. And another thing Is that in Moldova, our parents sometimes send us some packages and it comes from a minibus. And you never know when those people would be in Netherlands, because we are here established. And yeah, I wasn't expecting any package. And at one point I got a lot of calls from foreign numbers, like German numbers. And I usually don't answer, you know, the phones to strange people.
+03:25 And I said, okay, let me answer the phone. And there was like a man screaming at me, like, why I'm not answering my phone? Because I'm supposed to get a package from Moldova. And actually her parents sent the package to her in Netherlands, but because she was not home, they gave the people that deliver the packages my phone number. And I had to like, all the time be stressed about it. And, you know, I also didn't like that. And recently also was my birthday of my boyfriend. And she also couldn't make it because of the other reason that she had and because she had to attend another event with her boyfriend. So there was a lot of events that just built up and it felt really hurtful because I also approached her, I texted her.
+04:07 Maybe it's not the best approach because, yeah, I also don't like this long text where I have to describe everything. And sometimes maybe you don't get the nice tone out of it. Maybe you understand completely different the message. But I still felt like I needed to express myself because I really value all the friendship that I have. And when I'm like, I also lived a lot of betrayals when it comes to friendships. And maybe I don't have so many friends at the moment, but the ones that I have, they're super nice, you know, like, it's not about the quantity, but quality. And that's why I approached her. And she got really offensive because she said that I make her feel the victim.
+04:45 And it's not nice for me to put so much pressure on her because maybe on Instagram, on videos that you have, maybe life feels like pink and. And shiny, but actually in the reality is not, yeah, same. And she. That was failing a lot of courses, but I'm not sure if it was my mistake because, yeah, this is how I feel at the moment. And it was quite a stressful experience for me. And at the moment we still are in touch, but not so often and not so in depth as we used to be. And also made myself a conclusion that maybe I have to step a bit back and give myself and herself a bit of space. And yeah, maybe I will not put 100% anymore because it feels like not worth it.
+06:17 So maybe you can give me some advices of how I should act next. Like what would be the further next steps?</t>
         </is>
       </c>
     </row>
@@ -1004,9 +1310,26 @@
       <c r="B37" t="n">
         <v>25579</v>
       </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>00:04 If you have any questions, I'm outside. Yes, thank you. Talk about anything you ask for advice. Name and lighter sheet. Hello, Eduardo. Hey, Eduardo. How you doing? So basically I was supposed to ask some questions.  00:41 That's a very good one. This is based practice, dexlab. Okay. Okay. I need to brainstorm a bit. I want to do some marketing campaign for my company. It is a secondhand marketplace for students and I want to get more students to do an interview with me. What do you suggest?  01:23 I was thinking going to the park with a beer and tell them, yeah, for one interview you get a beer, or for one sign up you get a beer. Something like that.  01:57 Is there any legal issue regarding giving away beers? It's students at Art University, so we're in a country where 18 is the minimum age, so it should be fine now.  02:35 No, I'd rather just exclude the younger ones.  03:06 Vouchers for what though? It's a student online company, nothing else.  03:34 I hear you, but I think we're just gonna stick with beer because it's gonna be a hot day and people will want to want a beer.  04:00 All right, I will. Sounds good. Thank you.  04:15 I appreciate that. Now I will ask you something else. I recently had an encounter with an advisor of mine and I don't know. The issue with him is that he's not proactive. And I'm not a clue how to incentivize him to be more proactive.  04:59 So reinforcement is the key, you see?  05:17 All right, cool. I guess I'll do that then.  05:32 What else can I talk about? Alright, tell me a joke.  05:51 That's such a lame one.  06:00 Yeah, sure.  06:04 No, no. Give. Give another shot. Why not?  06:18 Oh, horrible.  06:31 I would like to know where you're located.  06:45 Okay, that's. Yes. The end yes, you can take it off now.    Transcribed by https://fireflies.ai/</t>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>00:04 If you have any questions, I'm outside. Yes, thank you. Talk about anything you ask for advice. Name and lighter sheet. Hello, Eduardo. Hey, Eduardo. How you doing? So basically I was supposed to ask some questions.
+00:41 That's a very good one. This is based practice, dexlab. Okay. Okay. I need to brainstorm a bit. I want to do some marketing campaign for my company. It is a secondhand marketplace for students and I want to get more students to do an interview with me. What do you suggest?
+01:23 I was thinking going to the park with a beer and tell them, yeah, for one interview you get a beer, or for one sign up you get a beer. Something like that.
+01:57 Is there any legal issue regarding giving away beers? It's students at Art University, so we're in a country where 18 is the minimum age, so it should be fine now.
+02:35 No, I'd rather just exclude the younger ones.
+03:06 Vouchers for what though? It's a student online company, nothing else.
+03:34 I hear you, but I think we're just gonna stick with beer because it's gonna be a hot day and people will want to want a beer.
+04:00 All right, I will. Sounds good. Thank you.
+04:15 I appreciate that. Now I will ask you something else. I recently had an encounter with an advisor of mine and I don't know. The issue with him is that he's not proactive. And I'm not a clue how to incentivize him to be more proactive.
+04:59 So reinforcement is the key, you see?
+05:17 All right, cool. I guess I'll do that then.
+05:32 What else can I talk about? Alright, tell me a joke.
+05:51 That's such a lame one.
+06:00 Yeah, sure.
+06:04 No, no. Give. Give another shot. Why not?
+06:18 Oh, horrible.
+06:31 I would like to know where you're located.
+06:45 Okay, that's. Yes. The end yes, you can take it off now.    Transcribed by https://fireflies.ai/</t>
         </is>
       </c>
     </row>
@@ -1019,9 +1342,17 @@
       <c r="B38" t="n">
         <v>13669</v>
       </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>00:18 Hi. I have been in a situation. It was a really challenging situation where I had some misunderstanding with one of my friends. This was the situation. So I am looking for some rentable places to live here in this city. And I didn't know if I wanted to live with her or live alone.  01:17 Okay. Should I say what I'm thinking about?  01:56 Okay. It's really pretty. I feel calm here.  02:44 I can feel it. It's really cool. Should we just talk about my problem or like, brainstorm or how to get like, a solution to my problem?  03:32 Okay, I got it.  03:53 Yeah, I see.  04:14 Maybe you can help me. Like, what would be the best decision? To move in with her when I know that her behavior can be sometimes really, like, stressful because she studies a lot or, like, move in alone and it would be much more expensive with which I'm not able to present the money for. What do you think?  04:45 Absolutely.  05:09 Okay. Thank you for your help. Hello.</t>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>00:18 Hi. I have been in a situation. It was a really challenging situation where I had some misunderstanding with one of my friends. This was the situation. So I am looking for some rentable places to live here in this city. And I didn't know if I wanted to live with her or live alone.
+01:17 Okay. Should I say what I'm thinking about?
+01:56 Okay. It's really pretty. I feel calm here.
+02:44 I can feel it. It's really cool. Should we just talk about my problem or like, brainstorm or how to get like, a solution to my problem?
+03:32 Okay, I got it.
+03:53 Yeah, I see.
+04:14 Maybe you can help me. Like, what would be the best decision? To move in with her when I know that her behavior can be sometimes really, like, stressful because she studies a lot or, like, move in alone and it would be much more expensive with which I'm not able to present the money for. What do you think?
+04:45 Absolutely.
+05:09 Okay. Thank you for your help. Hello.</t>
         </is>
       </c>
     </row>
@@ -1034,9 +1365,12 @@
       <c r="B39" t="n">
         <v>13600</v>
       </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>00:31 Hi, nice to meet you. I wanted to talk to you about a weird interaction I had with one of my roommates. I'm sharing a kitchen with a lot of students and it seems to be pretty messy these days. So I tried to confront one of them, but they got really angry and none of my roommates talk to me anymore. What do you think I should do,.  01:23 Okay, thanks. But I'm scared that they will have like a bad reaction to that. Like, they seem to be pretty aggressive.  01:55 But how do I, like, communicate to them properly that I want the kitchen to be fully, like, clean and a respectable area?  02:29 Okay, thank you so much and thank you for your help. It was very helpful.</t>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>00:31 Hi, nice to meet you. I wanted to talk to you about a weird interaction I had with one of my roommates. I'm sharing a kitchen with a lot of students and it seems to be pretty messy these days. So I tried to confront one of them, but they got really angry and none of my roommates talk to me anymore. What do you think I should do,.
+01:23 Okay, thanks. But I'm scared that they will have like a bad reaction to that. Like, they seem to be pretty aggressive.
+01:55 But how do I, like, communicate to them properly that I want the kitchen to be fully, like, clean and a respectable area?
+02:29 Okay, thank you so much and thank you for your help. It was very helpful.</t>
         </is>
       </c>
     </row>
@@ -1049,9 +1383,18 @@
       <c r="B40" t="n">
         <v>16369</v>
       </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>00:26 Hi, how are you? I would like you to.  00:35 I'm feeling okay.  00:45 I wanted to talk about a challenging interaction I've had recently.  01:00 Yeah, I was talking with my group work project from university. They were all being very passive though. So no one was trying to take over a role or even assign roles.  01:31 Yeah, I've tried to kind of start as a kind of leader, but I don't really want to take the leader role since that takes much more time than any other role. And I've just tried having them each assign themselves a role, but it hasn't really worked yet. Do you have any tips?  02:20 Yeah, that sounds good, but I mean, it sounds good in theory, but I don't know how I would be able to put that in practice, especially if I don't see them in person. Often I usually just have them per text where a lot of people can just ignore.  03:05 Yeah, that seems smart enough. How would you then continue to keep them accountable though? Like, we have, I think three weeks until the presentation, but we have to keep doing weekly small drives that we should show the teacher and I don't want to be every day sending out reminders or kind of having to check on everyone.  03:50 Yeah, that makes sense.  04:07 Yeah. How could I formulate it, though, without sounding too bossy?  04:32 Yep. That seems good. Thanks for your help. Have you had experiences like this before?</t>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>00:26 Hi, how are you? I would like you to.
+00:35 I'm feeling okay.
+00:45 I wanted to talk about a challenging interaction I've had recently.
+01:00 Yeah, I was talking with my group work project from university. They were all being very passive though. So no one was trying to take over a role or even assign roles.
+01:31 Yeah, I've tried to kind of start as a kind of leader, but I don't really want to take the leader role since that takes much more time than any other role. And I've just tried having them each assign themselves a role, but it hasn't really worked yet. Do you have any tips?
+02:20 Yeah, that sounds good, but I mean, it sounds good in theory, but I don't know how I would be able to put that in practice, especially if I don't see them in person. Often I usually just have them per text where a lot of people can just ignore.
+03:05 Yeah, that seems smart enough. How would you then continue to keep them accountable though? Like, we have, I think three weeks until the presentation, but we have to keep doing weekly small drives that we should show the teacher and I don't want to be every day sending out reminders or kind of having to check on everyone.
+03:50 Yeah, that makes sense.
+04:07 Yeah. How could I formulate it, though, without sounding too bossy?
+04:32 Yep. That seems good. Thanks for your help. Have you had experiences like this before?</t>
         </is>
       </c>
     </row>
@@ -1064,9 +1407,12 @@
       <c r="B41" t="n">
         <v>13393</v>
       </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>00:16 Good to meet you too. We can start the conversation. I want to speak to you about a recently challenging social situation.  00:35 Okay. So I have a good friend, a fellow student, which I quite like and we get along well, but kind of. It's not a problem, but it's kind of a misalignment. He has a lot of friends. He has a lot. He has a very vivid social life and more. I'm more kind of introverted. I have a few very good friends and I'd like to integrate him into my close friends circle. But he obviously he has a lot of friends and so a lot of options. Yeah. So it's a bit of complicated to deal with that situation because I like him as a person. I like to do some stuff with him, but he is kind of very busy with a lot of people.  01:38 Not sure if that is the thing I would do because it's not that kind of a serious problem and not sure if that should be something where I tell them how I feel on a deeper level. Because also our connection is not that deep yet. So probably I would just kind of find a way to interact more with them, spend more time with them and then see where it goes.  02:33 Yeah. Thanks for the tips. And another thing. Do you have any advice on how to integrate different friends who don't know each other yet and create a group of friends? So kind of. Yeah. Bring different people together.</t>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>00:16 Good to meet you too. We can start the conversation. I want to speak to you about a recently challenging social situation.
+00:35 Okay. So I have a good friend, a fellow student, which I quite like and we get along well, but kind of. It's not a problem, but it's kind of a misalignment. He has a lot of friends. He has a lot. He has a very vivid social life and more. I'm more kind of introverted. I have a few very good friends and I'd like to integrate him into my close friends circle. But he obviously he has a lot of friends and so a lot of options. Yeah. So it's a bit of complicated to deal with that situation because I like him as a person. I like to do some stuff with him, but he is kind of very busy with a lot of people.
+01:38 Not sure if that is the thing I would do because it's not that kind of a serious problem and not sure if that should be something where I tell them how I feel on a deeper level. Because also our connection is not that deep yet. So probably I would just kind of find a way to interact more with them, spend more time with them and then see where it goes.
+02:33 Yeah. Thanks for the tips. And another thing. Do you have any advice on how to integrate different friends who don't know each other yet and create a group of friends? So kind of. Yeah. Bring different people together.</t>
         </is>
       </c>
     </row>
@@ -1079,9 +1425,17 @@
       <c r="B42" t="n">
         <v>14728</v>
       </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>00:21 I would like to share a challenging interaction with a friend.  00:40 I wasn't talking about a change, rather a challenging interaction with a friend on a social level.  01:05 I would like to be more confident in my friendships and to be able to not let everything so close to me. Yes,.  01:42 Yes. Do you have an idea?  02:05 I think that's something I've been doing, actually. It's more focusing on. Yeah. Not overthinking. When people do small things that might not be my greatest interest, obviously. And not being super disappointed in those persons then. Do you have an idea about that?  02:50 Yeah, that is a very good idea. Do you have anything else I could implement from right now?  03:23 But what if I'm continuously disappointed in my friends at parts because I've seen some small interactions or small things that I didn't like? What do I do about that?  04:01 Okay, thank you. Do you have anything else I could do? Because I think I'm already doing the compliment stuff kind of already, but it's more about not letting it to like those negative things, not letting them too closely to my heart. Do you have anything you have to say about that?  04:48 Yeah, that might be a good idea. Is there anything else you want to share about that situation?</t>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>00:21 I would like to share a challenging interaction with a friend.
+00:40 I wasn't talking about a change, rather a challenging interaction with a friend on a social level.
+01:05 I would like to be more confident in my friendships and to be able to not let everything so close to me. Yes,.
+01:42 Yes. Do you have an idea?
+02:05 I think that's something I've been doing, actually. It's more focusing on. Yeah. Not overthinking. When people do small things that might not be my greatest interest, obviously. And not being super disappointed in those persons then. Do you have an idea about that?
+02:50 Yeah, that is a very good idea. Do you have anything else I could implement from right now?
+03:23 But what if I'm continuously disappointed in my friends at parts because I've seen some small interactions or small things that I didn't like? What do I do about that?
+04:01 Okay, thank you. Do you have anything else I could do? Because I think I'm already doing the compliment stuff kind of already, but it's more about not letting it to like those negative things, not letting them too closely to my heart. Do you have anything you have to say about that?
+04:48 Yeah, that might be a good idea. Is there anything else you want to share about that situation?</t>
         </is>
       </c>
     </row>
@@ -1094,9 +1448,20 @@
       <c r="B43" t="n">
         <v>14812</v>
       </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>00:39 So I had like a conflict with my. With my tutor for a paper that I wrote and she gave me really bad feedback but she didn't like actually give me feedback and I didn't know how to identify do that because I still wanted to stay respectful, but I was still like really mad.  01:15 Yeah, sure.  01:46 Do you think it would be like, how would I like, ask her to like maybe change the grade?  02:18 Okay. Like, because the thing is that she said that she wouldn't let anyone fail, but I got like almost a failing grade but like not really failing grade. So I feel like I went into it with misconception about her grading style. And also there was two different two tutors that were correcting the things. So one of them had really good feedback and the other had really bad feedback.  03:10 Yeah. Thanks for your help.  03:28 Cool, thanks. Is there Anything else we have to talk about?  04:00 I'm supposed to talk to you about my problems with someone with relationships.  04:21 No, not really. Mostly just the thing with the tutor.  04:43 Mmm. I'm still a little bit uncomfortable with the whole situation.  05:09 Sure. What kind of message should I send her?  05:30 Yeah.  05:34 Yes, I think that's good.</t>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>00:39 So I had like a conflict with my. With my tutor for a paper that I wrote and she gave me really bad feedback but she didn't like actually give me feedback and I didn't know how to identify do that because I still wanted to stay respectful, but I was still like really mad.
+01:15 Yeah, sure.
+01:46 Do you think it would be like, how would I like, ask her to like maybe change the grade?
+02:18 Okay. Like, because the thing is that she said that she wouldn't let anyone fail, but I got like almost a failing grade but like not really failing grade. So I feel like I went into it with misconception about her grading style. And also there was two different two tutors that were correcting the things. So one of them had really good feedback and the other had really bad feedback.
+03:10 Yeah. Thanks for your help.
+03:28 Cool, thanks. Is there Anything else we have to talk about?
+04:00 I'm supposed to talk to you about my problems with someone with relationships.
+04:21 No, not really. Mostly just the thing with the tutor.
+04:43 Mmm. I'm still a little bit uncomfortable with the whole situation.
+05:09 Sure. What kind of message should I send her?
+05:30 Yeah.
+05:34 Yes, I think that's good.</t>
         </is>
       </c>
     </row>
@@ -1109,9 +1474,19 @@
       <c r="B44" t="n">
         <v>13885</v>
       </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>00:13 What's up? What's up, Edu? Yeah, I have a recent. Recent challenge. I faced one of my group members in facilitation. Didn't prepare for the. For the facilitation, and now I had to. Yeah, I had to do it all by myself, and we got a bad grade because of him. Like, he didn't prepare well.  00:38 Yeah, that was the problem.  00:56 Nah, not really. But I think, like, it's just unfair because, you know, everybody prepared, and he was just like, yeah, he just came unprepared, and we had to settle it on our own. And, yeah, now the whole group was suffering because of that. And, yeah, I think it's just not really. Not really fair and just a bad thing for him. Right,.  01:40 Yeah, sure. I think next time I'm gonna reach out for the person and tell him instantly what he's doing wrong or. Yeah, just raise my opinion on him. Like, saying that it's not okay that it's only us who are preparing. And, yeah, everybody needs to prepare.  02:19 Yeah, of course it can make a big difference. But, you know, it's also, like, it depends on the other person. Like, maybe he just doesn't have that mindset to, you know, change next time. And, yeah, I guess then my last choice is to, like, kick him out of the group or snitch on him.  03:00 Yeah, absolutely. You're right. Even if, like, it Has a bad outcome for him. I mean, yeah, he had his chance. And at university you're supposed to work with others and if you don't like do that, you have to be aware of the consequences you face. Right,.  03:39 Yeah, man. And just like a quick jump. You have a really nice view behind you. Could you tell me what the building or where it's located looks really nice.  04:10 Yeah, man. And what is the. The ocean like? Do you know where that's located? Maybe.  04:34 Okay, man, what is your name again?  04:43 Yeah, I think so as well. And where you from, Eduardo? I would like maybe. I would maybe think of Mexico or something. Maybe South America.  05:11 Yo, Eduardo, I really like your haircut.</t>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>00:13 What's up? What's up, Edu? Yeah, I have a recent. Recent challenge. I faced one of my group members in facilitation. Didn't prepare for the. For the facilitation, and now I had to. Yeah, I had to do it all by myself, and we got a bad grade because of him. Like, he didn't prepare well.
+00:38 Yeah, that was the problem.
+00:56 Nah, not really. But I think, like, it's just unfair because, you know, everybody prepared, and he was just like, yeah, he just came unprepared, and we had to settle it on our own. And, yeah, now the whole group was suffering because of that. And, yeah, I think it's just not really. Not really fair and just a bad thing for him. Right,.
+01:40 Yeah, sure. I think next time I'm gonna reach out for the person and tell him instantly what he's doing wrong or. Yeah, just raise my opinion on him. Like, saying that it's not okay that it's only us who are preparing. And, yeah, everybody needs to prepare.
+02:19 Yeah, of course it can make a big difference. But, you know, it's also, like, it depends on the other person. Like, maybe he just doesn't have that mindset to, you know, change next time. And, yeah, I guess then my last choice is to, like, kick him out of the group or snitch on him.
+03:00 Yeah, absolutely. You're right. Even if, like, it Has a bad outcome for him. I mean, yeah, he had his chance. And at university you're supposed to work with others and if you don't like do that, you have to be aware of the consequences you face. Right,.
+03:39 Yeah, man. And just like a quick jump. You have a really nice view behind you. Could you tell me what the building or where it's located looks really nice.
+04:10 Yeah, man. And what is the. The ocean like? Do you know where that's located? Maybe.
+04:34 Okay, man, what is your name again?
+04:43 Yeah, I think so as well. And where you from, Eduardo? I would like maybe. I would maybe think of Mexico or something. Maybe South America.
+05:11 Yo, Eduardo, I really like your haircut.</t>
         </is>
       </c>
     </row>
@@ -1124,9 +1499,14 @@
       <c r="B45" t="n">
         <v>13441</v>
       </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>00:05 Thank you. Hello. Hi. I will talk about a challenging experience in the past. So I was at a group project, and we all have the. We will all get the same great together. And one person was missing, and he wasn't doing anything for the project. And then the question was, or kind of the challenge was whether I should report him and tell my teacher that he didn't do anything or if I should just keep on going and don't care about it. Because overall, I think we got a quite good grade. So that was kind of the challenge.  01:11 Yeah, so in the end, I. I wasn't sure. I think I did, like, something in the middle because I. Yeah, I was not really. I like, told the teacher, yeah, he didn't do too much, but then, yeah, that's basically it. So I didn't really say that he did nothing at all and that we had to do his parts ourselves. So, yeah, that's how I kind of handled.  02:01 Yeah, but it's defy kind of bad because this guy is kind of nice. I mean, he didn't really communicate with us, but I think. Yeah. I'm not really sure in the end whether it was a good decision. Maybe. Could you tell me what you would have done?  02:49 Yeah, okay, I get that. Yeah. I think that basically was my challenging. Yeah. Also, it was kind of challenging to then talk to my teammates and to decide within the team whether we should report it to the teacher or not. So, yeah, that was also kind of challenging because nobody of us wanted to be like the bad guy and tell the teacher, but we all weren't really happy with his performance. Yeah. So that was also kind of Challenging?  03:52 Do you have maybe any other ideas what I could do next time? Better? So maybe how to communicate with the person better, how to better as a team and. Yeah, then tell me whether you would report it or not if it happens with the same person again. I mean, he never really does much, so yeah, that's kind of the problem.  04:58 Yeah, okay, but he does his parts. But his parts are very bad, so it really seems like he just put it in ChatGPT and then copy pasted it into the presentation. So that's the main problem there.</t>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>00:05 Thank you. Hello. Hi. I will talk about a challenging experience in the past. So I was at a group project, and we all have the. We will all get the same great together. And one person was missing, and he wasn't doing anything for the project. And then the question was, or kind of the challenge was whether I should report him and tell my teacher that he didn't do anything or if I should just keep on going and don't care about it. Because overall, I think we got a quite good grade. So that was kind of the challenge.
+01:11 Yeah, so in the end, I. I wasn't sure. I think I did, like, something in the middle because I. Yeah, I was not really. I like, told the teacher, yeah, he didn't do too much, but then, yeah, that's basically it. So I didn't really say that he did nothing at all and that we had to do his parts ourselves. So, yeah, that's how I kind of handled.
+02:01 Yeah, but it's defy kind of bad because this guy is kind of nice. I mean, he didn't really communicate with us, but I think. Yeah. I'm not really sure in the end whether it was a good decision. Maybe. Could you tell me what you would have done?
+02:49 Yeah, okay, I get that. Yeah. I think that basically was my challenging. Yeah. Also, it was kind of challenging to then talk to my teammates and to decide within the team whether we should report it to the teacher or not. So, yeah, that was also kind of challenging because nobody of us wanted to be like the bad guy and tell the teacher, but we all weren't really happy with his performance. Yeah. So that was also kind of Challenging?
+03:52 Do you have maybe any other ideas what I could do next time? Better? So maybe how to communicate with the person better, how to better as a team and. Yeah, then tell me whether you would report it or not if it happens with the same person again. I mean, he never really does much, so yeah, that's kind of the problem.
+04:58 Yeah, okay, but he does his parts. But his parts are very bad, so it really seems like he just put it in ChatGPT and then copy pasted it into the presentation. So that's the main problem there.</t>
         </is>
       </c>
     </row>
@@ -1139,9 +1519,17 @@
       <c r="B46" t="n">
         <v>14320</v>
       </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>00:43 Okay. I had a challenging situationship recently. Can we talk? Okay. So I failed the QM1 class, so. And I also failed the receipts. And now I am wondering if I'm going to be able to pass it next year.  01:30 Yes. I recently downloaded the application success formula to have like more tutoring private classes after classes.  02:03 Yes, I agree.  02:17 Well, I had another class recently where I passed the exam and I had nine out of 10 and it was kind of the same subject. So I feel comfortable now about the QM1 next year.  02:47 Yes.  03:05 Any other advice?  03:34 What advice would you give me when I just don't feel to study.  04:06 Okay, so maybe I am. I subscribe myself in the gym so I guess it's fine.  04:30 Okay. Thank you so much.</t>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>00:43 Okay. I had a challenging situationship recently. Can we talk? Okay. So I failed the QM1 class, so. And I also failed the receipts. And now I am wondering if I'm going to be able to pass it next year.
+01:30 Yes. I recently downloaded the application success formula to have like more tutoring private classes after classes.
+02:03 Yes, I agree.
+02:17 Well, I had another class recently where I passed the exam and I had nine out of 10 and it was kind of the same subject. So I feel comfortable now about the QM1 next year.
+02:47 Yes.
+03:05 Any other advice?
+03:34 What advice would you give me when I just don't feel to study.
+04:06 Okay, so maybe I am. I subscribe myself in the gym so I guess it's fine.
+04:30 Okay. Thank you so much.</t>
         </is>
       </c>
     </row>
@@ -1154,9 +1542,13 @@
       <c r="B47" t="n">
         <v>14713</v>
       </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>00:19 I have a challenging experience that I would like to talk about.  00:32 So about one and a half weeks ago, were at cheerleading practice and a friend of mine injured herself. She was falling from a stunt and then her knee was like hurting and we wanted to go to the emergency room here in the Maastricht hospital and you have to call and make an appointment for the er because otherwise you get fined. And we called. We are all English speakers, so we don't have a Dutch speaking person with us. So they just hung up on us and then we called again and they hung up on us again. And up until went to, sports worker that called them in Dutch. And then they were giving us an appointment, which was already very rude. Then went over there, which is like a two minute walk.  02:35 So last week when I injured myself, I didn't go to the er. I had to like make the decision to like go back to my home country to get like an MRI scan and everything because the Dutch hospitals in it ER rooms don't really care about internationals.  03:31 I mean, for my friend, she also went back to her home country to get the treatment. So I'm just now kind of drawing the conclusion that you cannot rely on the, as an international student on the Dutch healthcare system. So every time something happens, we have to go back to our home countries kind of. Or like just expect to get told that we have to take paracetamol and wait.  04:35 Yeah, you're right.</t>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>00:19 I have a challenging experience that I would like to talk about.
+00:32 So about one and a half weeks ago, were at cheerleading practice and a friend of mine injured herself. She was falling from a stunt and then her knee was like hurting and we wanted to go to the emergency room here in the Maastricht hospital and you have to call and make an appointment for the er because otherwise you get fined. And we called. We are all English speakers, so we don't have a Dutch speaking person with us. So they just hung up on us and then we called again and they hung up on us again. And up until went to, sports worker that called them in Dutch. And then they were giving us an appointment, which was already very rude. Then went over there, which is like a two minute walk.
+02:35 So last week when I injured myself, I didn't go to the er. I had to like make the decision to like go back to my home country to get like an MRI scan and everything because the Dutch hospitals in it ER rooms don't really care about internationals.
+03:31 I mean, for my friend, she also went back to her home country to get the treatment. So I'm just now kind of drawing the conclusion that you cannot rely on the, as an international student on the Dutch healthcare system. So every time something happens, we have to go back to our home countries kind of. Or like just expect to get told that we have to take paracetamol and wait.
+04:35 Yeah, you're right.</t>
         </is>
       </c>
     </row>
@@ -1169,9 +1561,18 @@
       <c r="B48" t="n">
         <v>9</v>
       </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>00:05 Whenever you hear. Yeah. Okay. What's on my mind today? I have did have a conversation with a friend who I still have to pay money to.  00:37 Yeah.  00:42 Well, it's a friend of mine and I borrowed some money of him and now suddenly he wants to have it in return. But he did not ask for it in a polite way. So it's like being an issue between us now.  01:17 Like in an honest and direct way and say what's on my mind?  01:42 Yeah, sure. But I want to keep the friendship in a good way, so I want to preserve it know.  02:10 Sure, that's what I want. Do you have any advice for me?  02:39 Okay. Is there also some things I don't need to do or specific I don't must do?  03:14 Okay. Okay. Well, wish me good luck with it then. I hope I have to resolve it very soon. So.  03:34 Yeah, sure. But do you have any advice according to similar things to avoid it in the future?  04:06 Okay, well, thank you very much. That's very nice to hear. I wish you a very good and pleasant day.</t>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>00:05 Whenever you hear. Yeah. Okay. What's on my mind today? I have did have a conversation with a friend who I still have to pay money to.
+00:37 Yeah.
+00:42 Well, it's a friend of mine and I borrowed some money of him and now suddenly he wants to have it in return. But he did not ask for it in a polite way. So it's like being an issue between us now.
+01:17 Like in an honest and direct way and say what's on my mind?
+01:42 Yeah, sure. But I want to keep the friendship in a good way, so I want to preserve it know.
+02:10 Sure, that's what I want. Do you have any advice for me?
+02:39 Okay. Is there also some things I don't need to do or specific I don't must do?
+03:14 Okay. Okay. Well, wish me good luck with it then. I hope I have to resolve it very soon. So.
+03:34 Yeah, sure. But do you have any advice according to similar things to avoid it in the future?
+04:06 Okay, well, thank you very much. That's very nice to hear. I wish you a very good and pleasant day.</t>
         </is>
       </c>
     </row>
@@ -1184,9 +1585,16 @@
       <c r="B49" t="n">
         <v>15187</v>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>00:19 Who are you? Tell me about you and your story. Life story.  00:46 My story? Yeah, I'm a student from Europe and yeah, my first year bachelor.  01:12 Learning so much.  01:24 Wait, wait. I would like to talk about one challenging thing that happened recently. Are you okay with that? Talking about that?  01:42 I would say recently we had a group project and we did not agree on the same template we should use or even the same platform was different. So yeah, we had a little conflict on what template and what are the goals and vision of the group project. And yeah, that was like a big challenging thing recently I would say. What would you say about that?  02:34 I thought I have the better idea, but the two other ones thought their idea is better so we agreed to stick with their idea.  03:07 I'm not pleased with that because I think my ideas would be way better because I perform better than they.  03:41 I will do probably the same thing, I think. Yeah. We are done with this session. Alright. Thank you very much for your talking with me. I enjoyed it.</t>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>00:19 Who are you? Tell me about you and your story. Life story.
+00:46 My story? Yeah, I'm a student from Europe and yeah, my first year bachelor.
+01:12 Learning so much.
+01:24 Wait, wait. I would like to talk about one challenging thing that happened recently. Are you okay with that? Talking about that?
+01:42 I would say recently we had a group project and we did not agree on the same template we should use or even the same platform was different. So yeah, we had a little conflict on what template and what are the goals and vision of the group project. And yeah, that was like a big challenging thing recently I would say. What would you say about that?
+02:34 I thought I have the better idea, but the two other ones thought their idea is better so we agreed to stick with their idea.
+03:07 I'm not pleased with that because I think my ideas would be way better because I perform better than they.
+03:41 I will do probably the same thing, I think. Yeah. We are done with this session. Alright. Thank you very much for your talking with me. I enjoyed it.</t>
         </is>
       </c>
     </row>
@@ -1199,9 +1607,24 @@
       <c r="B50" t="n">
         <v>14185</v>
       </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>00:12 I know. Just talking with friends, having problems. I have to study a lot and I also have to travel a lot. Maybe just to distract myself with sports, like going to the gym or playing football.  01:04 Yes, very much.  01:18 Maybe be more time efficient and like study a lot more? Yes, that's a good idea.  01:55 Yes, that would be nice to look.  02:10 I try to study like two hours and I mostly do it like in the morning or like middle of the day.  02:33 I think I'm focused, but sometimes I'm on my phone or like distracted, so I'm not really locked in.  02:57 Yes. You are really smart.  03:14 Yes. So just studying a lot, making good time plans. Yeah,.  03:42 Yes, that's what we should do.  03:59 Okay, that's a good idea.  04:14 I wake up like eight or nine o' clock and then after breakfast I'm ready to go to study.  04:40 This is perfect.  04:57 Well, this is a really good idea. But do you think like 50 minutes is enough break or would you say a little bit more?  05:26 Yeah, that's. That's a really good idea. What do you recommend? If I have like to study five hours a day, how should I do the time spaces? Like,.  06:06 That's a really good idea. And does my brain get everything then like really fast or do I have to like repeat it so much? Because my problems are often that if I study something like the next day, I already forgot what it was, so I have to do it again. You know what I mean?  06:49 That's a really good idea. Thank.</t>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>00:12 I know. Just talking with friends, having problems. I have to study a lot and I also have to travel a lot. Maybe just to distract myself with sports, like going to the gym or playing football.
+01:04 Yes, very much.
+01:18 Maybe be more time efficient and like study a lot more? Yes, that's a good idea.
+01:55 Yes, that would be nice to look.
+02:10 I try to study like two hours and I mostly do it like in the morning or like middle of the day.
+02:33 I think I'm focused, but sometimes I'm on my phone or like distracted, so I'm not really locked in.
+02:57 Yes. You are really smart.
+03:14 Yes. So just studying a lot, making good time plans. Yeah,.
+03:42 Yes, that's what we should do.
+03:59 Okay, that's a good idea.
+04:14 I wake up like eight or nine o' clock and then after breakfast I'm ready to go to study.
+04:40 This is perfect.
+04:57 Well, this is a really good idea. But do you think like 50 minutes is enough break or would you say a little bit more?
+05:26 Yeah, that's. That's a really good idea. What do you recommend? If I have like to study five hours a day, how should I do the time spaces? Like,.
+06:06 That's a really good idea. And does my brain get everything then like really fast or do I have to like repeat it so much? Because my problems are often that if I study something like the next day, I already forgot what it was, so I have to do it again. You know what I mean?
+06:49 That's a really good idea. Thank.</t>
         </is>
       </c>
     </row>
@@ -1214,9 +1637,17 @@
       <c r="B51" t="n">
         <v>15172</v>
       </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>00:18 I would like to talk about the recent football game.  00:29 I was thinking about the semifinals and Champions League where Paris Saint Germain and Bayern Munich face each other. And unfortunately Bayern Munich left the competition due to two false decisions by the referees, which was very frustrating for us Germans because we support Bayern Munich as a whole completely. And it was a very challenging match and had major impact on society. How we view football and FIFA at the whole now due to the decisions.  01:19 I think it will be. It had a major negative impact on the fan base because now that the VAR is more into place. Yes. People might reconsider the decisions and a lot of false decisions are being made. And I think society has, especially the fan base has a lot of negative thoughts on VAR because it's so like unbalanced and sometimes it makes good decisions and sometimes super bad decisions. And they have like. And they can like decide on how a game is going to be. And at the end, the main purpose of fans watching and the decision of the referee is just being left out and the whole game becomes like disrupted and not nice to watch anymore as it was before without VAR and the face. False decisions.  02:40 Yeah. Do you have anything else what we can talk about? Some suggestions?  03:07 I would think about tennis, maybe. Do you want to talk about tennis?  03:28 French Open, which is upcoming.  03:43 Yeah. Alcaraz and Sinner. It will be a heaty battle because Sinna already won the last five majors, major, ATP, Thousand Masters, which is. Which hasn't. Have been a phenomena which hasn't occurred in the past. So he's one of the most successful players out there from all the great tennis players. And I want to, like, see or I'm very anxious, like, eager to see how Alcaraz is going to play against Sinna.  04:30 Do you have a favorite player? Between those. Between these both. Sorry? Between the both. Alcaraz and Sinna, do you have, like, a favorite one?  05:01 But if you were to decide which one of them you would likely would like to see more in the final, which one would it be?</t>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>00:18 I would like to talk about the recent football game.
+00:29 I was thinking about the semifinals and Champions League where Paris Saint Germain and Bayern Munich face each other. And unfortunately Bayern Munich left the competition due to two false decisions by the referees, which was very frustrating for us Germans because we support Bayern Munich as a whole completely. And it was a very challenging match and had major impact on society. How we view football and FIFA at the whole now due to the decisions.
+01:19 I think it will be. It had a major negative impact on the fan base because now that the VAR is more into place. Yes. People might reconsider the decisions and a lot of false decisions are being made. And I think society has, especially the fan base has a lot of negative thoughts on VAR because it's so like unbalanced and sometimes it makes good decisions and sometimes super bad decisions. And they have like. And they can like decide on how a game is going to be. And at the end, the main purpose of fans watching and the decision of the referee is just being left out and the whole game becomes like disrupted and not nice to watch anymore as it was before without VAR and the face. False decisions.
+02:40 Yeah. Do you have anything else what we can talk about? Some suggestions?
+03:07 I would think about tennis, maybe. Do you want to talk about tennis?
+03:28 French Open, which is upcoming.
+03:43 Yeah. Alcaraz and Sinner. It will be a heaty battle because Sinna already won the last five majors, major, ATP, Thousand Masters, which is. Which hasn't. Have been a phenomena which hasn't occurred in the past. So he's one of the most successful players out there from all the great tennis players. And I want to, like, see or I'm very anxious, like, eager to see how Alcaraz is going to play against Sinna.
+04:30 Do you have a favorite player? Between those. Between these both. Sorry? Between the both. Alcaraz and Sinna, do you have, like, a favorite one?
+05:01 But if you were to decide which one of them you would likely would like to see more in the final, which one would it be?</t>
         </is>
       </c>
     </row>
@@ -1229,9 +1660,13 @@
       <c r="B52" t="n">
         <v>13588</v>
       </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>00:16 Hi, it's really nice to meet you. First, I just wanted to talk about a situation which I encountered recently. It was like in uni, when normally, you know, to do presentations and have a lot of teamwork. And I was in a group full of people. I kind of. I liked them, but they didn't really work. So I was the only one working the whole time. And every time I wrote in the chat, for instance, who is going to do which task? Nobody really answered to me at all. And then like we had small mini presentations. We had to give every single lesson. And each of the presentations is what I did. And nobody of them did any work of that. And they felt also really bad, I think. But they never changed their attitude towards me.  01:09 And I think it was really unfair and not so nice, to be honest. And for me, I am like quite unsure of what to do because I don't want to disturb anyone. But still I want to have a good grade, obviously while having good atmosphere while working and everybody doing part of their tasks. So I'm not sure if you know what I mean. Just like it's really hard. Yeah. So I'm not really sure what to do because also like they are. We are a group of five and I'm the only one doing every single thing just for a good grade. And they are also having the same good grades as I am having. This is what I'm thinking of being really annoying and it's just not really nice for me. Yeah.  02:15 Just don't feel that great about the situation because I don't know what to do exactly. So yeah, I don't know if you know what I mean. Like the balance between still being nice and friendly and having good grade but also having fair work. I also talked some with friends of mine about that and I was kind of also really angry about the group members because I thought it's not really professional to let someone else do all your tasks and then pretend if you did all of it. And I didn't really speak up for myself because I didn't want to ruin our grade because it was a group grade. So everybody had the same grade. I was to talk with friends, as already mentioned, and family. And they all said that I should talk with the teacher.  03:06 But I wasn't sure about job because if I did that they probably wouldn't have changed anything or I wished of having another batch grade maybe. Yeah, I'm not sure if you know what I mean? Yeah. I don't know. It just kind of really was a hard time mostly also because when I try to meet up with them, it's just like I want to have a good impression, not only for the teacher, but also for my group members. And they just weren't there for me and they didn't really listen to what I was, what I talked about. But sometimes they also change.  04:03 So, like, it was not only bad, some of them were really nice and they tried to add some new things, but it was kind of sometimes really hard to work them with them just because they are really lazy sometimes and they didn't really do their work most of the time. This is what I did. Yep.</t>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>00:16 Hi, it's really nice to meet you. First, I just wanted to talk about a situation which I encountered recently. It was like in uni, when normally, you know, to do presentations and have a lot of teamwork. And I was in a group full of people. I kind of. I liked them, but they didn't really work. So I was the only one working the whole time. And every time I wrote in the chat, for instance, who is going to do which task? Nobody really answered to me at all. And then like we had small mini presentations. We had to give every single lesson. And each of the presentations is what I did. And nobody of them did any work of that. And they felt also really bad, I think. But they never changed their attitude towards me.
+01:09 And I think it was really unfair and not so nice, to be honest. And for me, I am like quite unsure of what to do because I don't want to disturb anyone. But still I want to have a good grade, obviously while having good atmosphere while working and everybody doing part of their tasks. So I'm not sure if you know what I mean. Just like it's really hard. Yeah. So I'm not really sure what to do because also like they are. We are a group of five and I'm the only one doing every single thing just for a good grade. And they are also having the same good grades as I am having. This is what I'm thinking of being really annoying and it's just not really nice for me. Yeah.
+02:15 Just don't feel that great about the situation because I don't know what to do exactly. So yeah, I don't know if you know what I mean. Like the balance between still being nice and friendly and having good grade but also having fair work. I also talked some with friends of mine about that and I was kind of also really angry about the group members because I thought it's not really professional to let someone else do all your tasks and then pretend if you did all of it. And I didn't really speak up for myself because I didn't want to ruin our grade because it was a group grade. So everybody had the same grade. I was to talk with friends, as already mentioned, and family. And they all said that I should talk with the teacher.
+03:06 But I wasn't sure about job because if I did that they probably wouldn't have changed anything or I wished of having another batch grade maybe. Yeah, I'm not sure if you know what I mean? Yeah. I don't know. It just kind of really was a hard time mostly also because when I try to meet up with them, it's just like I want to have a good impression, not only for the teacher, but also for my group members. And they just weren't there for me and they didn't really listen to what I was, what I talked about. But sometimes they also change.
+04:03 So, like, it was not only bad, some of them were really nice and they tried to add some new things, but it was kind of sometimes really hard to work them with them just because they are really lazy sometimes and they didn't really do their work most of the time. This is what I did. Yep.</t>
         </is>
       </c>
     </row>
@@ -1244,9 +1679,16 @@
       <c r="B53" t="n">
         <v>13456</v>
       </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>00:00 That I am gone. Okay, thanks. Enjoy it. Thank you. Hi. Hi. So I want to talk about this challenging interaction I had the other day with a friend of mine. So, yeah.  00:35 So, basically, my friend came to visit me here, and so she met this guy and basically left me a little bit by the side. And so then what we had to do was have a conversation because I didn't like how she talked to me. But then she started doing it again, so it was really challenging to talk about it with her again.  01:14 Yeah. Well, I told her that I didn't like her attitude towards me because when she was. The guy was around, she was talking to me pretty differently. When she talks to me, I've known since were little kids, and she knew this guy from, like, 24 hours, and it pretty pissed me off. And then we had again, a conversation because this conflict had been going on for months. And then at Christmas, we sat down and talked about it again, and she told me how she felt, and I told her I felt. But I don't think we got to an agreement there.  02:04 Probably that this guy doesn't interfere in our conversations and friendship because after our conversation, were both really happy. But turns out the guy thinks that I was lying about everything, So I was pretty pissed by that, to be honest.  02:37 I think she doesn't really care because now they're a couple, and so she obviously takes his side. But I still don't think it's fair towards me that she just ignores me because she's not with him together. But again, I really don't care anymore.  03:13 I mean, I've already stepped back a few times maybe because, like, I'm so done with the converse over and over conversation. And she really doesn't seem to get the point. So I really do not care about it anymore. I just want to step back. It's okay.  03:54 Yeah. I mean, the thing is, it bothers because we've been friends since we're five years old. We've known each other our whole lives, and it bothers me pretty much that you just took his side, even though she only knew him for like a few hours. Of course now they've been dating a little while, but still. It's frustrating.  04:35 Yeah, you could say that. I mean, I don't know. I don't know really what to say about this anymore.</t>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>00:00 That I am gone. Okay, thanks. Enjoy it. Thank you. Hi. Hi. So I want to talk about this challenging interaction I had the other day with a friend of mine. So, yeah.
+00:35 So, basically, my friend came to visit me here, and so she met this guy and basically left me a little bit by the side. And so then what we had to do was have a conversation because I didn't like how she talked to me. But then she started doing it again, so it was really challenging to talk about it with her again.
+01:14 Yeah. Well, I told her that I didn't like her attitude towards me because when she was. The guy was around, she was talking to me pretty differently. When she talks to me, I've known since were little kids, and she knew this guy from, like, 24 hours, and it pretty pissed me off. And then we had again, a conversation because this conflict had been going on for months. And then at Christmas, we sat down and talked about it again, and she told me how she felt, and I told her I felt. But I don't think we got to an agreement there.
+02:04 Probably that this guy doesn't interfere in our conversations and friendship because after our conversation, were both really happy. But turns out the guy thinks that I was lying about everything, So I was pretty pissed by that, to be honest.
+02:37 I think she doesn't really care because now they're a couple, and so she obviously takes his side. But I still don't think it's fair towards me that she just ignores me because she's not with him together. But again, I really don't care anymore.
+03:13 I mean, I've already stepped back a few times maybe because, like, I'm so done with the converse over and over conversation. And she really doesn't seem to get the point. So I really do not care about it anymore. I just want to step back. It's okay.
+03:54 Yeah. I mean, the thing is, it bothers because we've been friends since we're five years old. We've known each other our whole lives, and it bothers me pretty much that you just took his side, even though she only knew him for like a few hours. Of course now they've been dating a little while, but still. It's frustrating.
+04:35 Yeah, you could say that. I mean, I don't know. I don't know really what to say about this anymore.</t>
         </is>
       </c>
     </row>
@@ -1259,9 +1701,15 @@
       <c r="B54" t="n">
         <v>13798</v>
       </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>00:29 Hello. No, I just wanted to talk. You know, I had a kind of challenging experience recently and would like to share it with you.  00:44 No, I just had a disagreement with a friend. We were. It was after a party. We were in the kitchen and were both a bit drunk, so we had kind of a lot of fight. Right. But we both did something that was kind of not harmful for the other, but we both reacted in a bad way and it was awkward for that night, but then we solved it the next day, so it was fine. But it was a weird experience to have.  01:37 Yeah, totally. It was a short misunderstanding. It wasn't really something that serious. Like nothing really that bad happened. It was just one bad action that led to a bad reaction. So we both kind of came to the conclusion that we both reacted in a bad way and we both did the wrong thing. So, yeah, we're good. As good as new.  02:19 Aside from that, would you like to know anything else about the experience?  02:36 I think the idea that, I mean, my friend was the first to apologize, but yeah, I feel like sometimes leaving that pride or ego aside and just apologizing for what you did wrong and learning how to do that, you know, quickly, it's just probably the biggest takeaway. Just learning how to take accountability as fast as possible to be able to resolve the issue.  03:26 It. I think that's it for my part.  04:32 Great. It. That.</t>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>00:29 Hello. No, I just wanted to talk. You know, I had a kind of challenging experience recently and would like to share it with you.
+00:44 No, I just had a disagreement with a friend. We were. It was after a party. We were in the kitchen and were both a bit drunk, so we had kind of a lot of fight. Right. But we both did something that was kind of not harmful for the other, but we both reacted in a bad way and it was awkward for that night, but then we solved it the next day, so it was fine. But it was a weird experience to have.
+01:37 Yeah, totally. It was a short misunderstanding. It wasn't really something that serious. Like nothing really that bad happened. It was just one bad action that led to a bad reaction. So we both kind of came to the conclusion that we both reacted in a bad way and we both did the wrong thing. So, yeah, we're good. As good as new.
+02:19 Aside from that, would you like to know anything else about the experience?
+02:36 I think the idea that, I mean, my friend was the first to apologize, but yeah, I feel like sometimes leaving that pride or ego aside and just apologizing for what you did wrong and learning how to do that, you know, quickly, it's just probably the biggest takeaway. Just learning how to take accountability as fast as possible to be able to resolve the issue.
+03:26 It. I think that's it for my part.
+04:32 Great. It. That.</t>
         </is>
       </c>
     </row>
@@ -1274,9 +1722,22 @@
       <c r="B55" t="n">
         <v>25576</v>
       </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>00:24 Just how are you? Perhaps first, I'm Mara. All right. Hello.  00:40 I'm also good. Just bit busy with life, but I'm good.  00:57 Yes, I want to talk about challenging interaction with you.  01:12 Oh, no, I want to tell you about a challenging interaction I had on my side.  01:27 It was with some of my friends, and basically I couldn't come to a meeting. We were supposed to meet, but yeah, it's very busy right now, and I felt like two of the friends did not really understand and were kind of mad.  01:54 I just tried to be honest and talk with them about it, but then also at some point I thought, okay, I think you also have to understand because we are friends. So I just left it like that.  02:28 Yes, it did. But I think it's always sad if you think some friends don't understand what you mean. No. And they. Yeah,.  02:55 Yeah, but what would you advise me to do? And if I enter another situation where friends who just don't understand that it can get busy and they get super disappointed and kind of also mad and blame you that you don't have perhaps the time? And what would you do.  03:44 Yeah, but what?  03:56 But what if you just don't know if it's going to get hectic so it's a bit more spontaneous?  04:26 Okay, thank you. I think that's all from my side.  04:44 Do you have any other ideas how to handle stress better? Any tips? Advice?  05:12 And what if always you have kind of the thoughts about it like always these thoughts. What can you do against it?  05:42 Okay, thank you.</t>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>00:24 Just how are you? Perhaps first, I'm Mara. All right. Hello.
+00:40 I'm also good. Just bit busy with life, but I'm good.
+00:57 Yes, I want to talk about challenging interaction with you.
+01:12 Oh, no, I want to tell you about a challenging interaction I had on my side.
+01:27 It was with some of my friends, and basically I couldn't come to a meeting. We were supposed to meet, but yeah, it's very busy right now, and I felt like two of the friends did not really understand and were kind of mad.
+01:54 I just tried to be honest and talk with them about it, but then also at some point I thought, okay, I think you also have to understand because we are friends. So I just left it like that.
+02:28 Yes, it did. But I think it's always sad if you think some friends don't understand what you mean. No. And they. Yeah,.
+02:55 Yeah, but what would you advise me to do? And if I enter another situation where friends who just don't understand that it can get busy and they get super disappointed and kind of also mad and blame you that you don't have perhaps the time? And what would you do.
+03:44 Yeah, but what?
+03:56 But what if you just don't know if it's going to get hectic so it's a bit more spontaneous?
+04:26 Okay, thank you. I think that's all from my side.
+04:44 Do you have any other ideas how to handle stress better? Any tips? Advice?
+05:12 And what if always you have kind of the thoughts about it like always these thoughts. What can you do against it?
+05:42 Okay, thank you.</t>
         </is>
       </c>
     </row>
@@ -1289,9 +1750,18 @@
       <c r="B56" t="n">
         <v>13378</v>
       </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>00:13 I want to chat about experience and a challenging conversation that I had today.  00:29 Since we are in different cultures, we didn't understand each other and it was a group project and so we had different discussion about what we need to do and how we need to do it.  00:52 We talked a lot. Even though we had a main disagreement. We tried to calm each other and understand each other point of view and we're still improving it. But we tried with that.  01:26 I mean, still we need to do a lot. We improved. Yes, but it could better. So I would tell you we are 50%, 60% done.  01:52 Maybe if even the other person will start to listen to me rather than just saying okay or yes, I will do it and try to have a conversation with me and expose even his point of view. Except like instead of me just trying to understand him, like just him saying what he wants.  02:36 Yes, I would review.  02:53 Yes,.  03:06 Maybe directly talk about it with my group project members and saying that what I'm feeling and what for me they should do. So that could be maybe one process. I don't know what you think about it.  03:41 Yes, I agree. But like sometimes I try to do it and they do not. They say like, they say, yes, we should do that, but then they do not do it. Like, I don't feel listened.  04:12 Okay, thank you very much.</t>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>00:13 I want to chat about experience and a challenging conversation that I had today.
+00:29 Since we are in different cultures, we didn't understand each other and it was a group project and so we had different discussion about what we need to do and how we need to do it.
+00:52 We talked a lot. Even though we had a main disagreement. We tried to calm each other and understand each other point of view and we're still improving it. But we tried with that.
+01:26 I mean, still we need to do a lot. We improved. Yes, but it could better. So I would tell you we are 50%, 60% done.
+01:52 Maybe if even the other person will start to listen to me rather than just saying okay or yes, I will do it and try to have a conversation with me and expose even his point of view. Except like instead of me just trying to understand him, like just him saying what he wants.
+02:36 Yes, I would review.
+02:53 Yes,.
+03:06 Maybe directly talk about it with my group project members and saying that what I'm feeling and what for me they should do. So that could be maybe one process. I don't know what you think about it.
+03:41 Yes, I agree. But like sometimes I try to do it and they do not. They say like, they say, yes, we should do that, but then they do not do it. Like, I don't feel listened.
+04:12 Okay, thank you very much.</t>
         </is>
       </c>
     </row>
@@ -1304,9 +1774,16 @@
       <c r="B57" t="n">
         <v>14380</v>
       </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>00:16 Hi, it's nice to meet you too. I wanted to tell you a situation that I faced a difficulty with.  00:35 Okay. So I had an issue with my grades recently. I received a very high grade on this course which was half based on my exam, half based on my tutor's opinion of my presentation and my behavior. So half of the grade was very subjective and I scored really high on the exam. But the subjective part wasn't as high as I wanted it to be. And it was very disappointing because I know that I was one of the best performing in the class. So I tried talking to the tutor. I wasn't allowed to. I had to speak to the course coordinator who wasn't helpful. He just told me that they don't discuss grades after being published but. But they wouldn't tell us our grades before they were published. So how are we supposed to discuss them at any other point?  01:27 And there was no resolution to that. He just told me to accept my grade because it was good. But it was very disappointing because I know that this also has long term impact on my overall gpa.  02:06 I really wish that there was someone else I could talk to about this to maybe address it because it's really is bothering me and the rest of my class. I know it's not a mean issue. So it's something that I know I'm going to regret if it's not resolved.  02:50 Yeah, I suppose.  03:11 Yeah, well, I think so too. I think speaking to someone else would be helpful. I just don't know who exactly to go to. I don't know if it would make a difference since the course coordinator was the highest authority were given access to and he wasn't any help. Help.  03:49 That's true. I guess. I haven't looked any further. I'm not sure where to look, but. But if I find the time, I think I should.  04:16 All my classmates sort of depended on me to reach out to the course coordinator and solve it. Because. Because I had one of the highest grades and best track record, I suppose. And they were kind of hoping that I resolve it. Which added to some of the pressure. I think.</t>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>00:16 Hi, it's nice to meet you too. I wanted to tell you a situation that I faced a difficulty with.
+00:35 Okay. So I had an issue with my grades recently. I received a very high grade on this course which was half based on my exam, half based on my tutor's opinion of my presentation and my behavior. So half of the grade was very subjective and I scored really high on the exam. But the subjective part wasn't as high as I wanted it to be. And it was very disappointing because I know that I was one of the best performing in the class. So I tried talking to the tutor. I wasn't allowed to. I had to speak to the course coordinator who wasn't helpful. He just told me that they don't discuss grades after being published but. But they wouldn't tell us our grades before they were published. So how are we supposed to discuss them at any other point?
+01:27 And there was no resolution to that. He just told me to accept my grade because it was good. But it was very disappointing because I know that this also has long term impact on my overall gpa.
+02:06 I really wish that there was someone else I could talk to about this to maybe address it because it's really is bothering me and the rest of my class. I know it's not a mean issue. So it's something that I know I'm going to regret if it's not resolved.
+02:50 Yeah, I suppose.
+03:11 Yeah, well, I think so too. I think speaking to someone else would be helpful. I just don't know who exactly to go to. I don't know if it would make a difference since the course coordinator was the highest authority were given access to and he wasn't any help. Help.
+03:49 That's true. I guess. I haven't looked any further. I'm not sure where to look, but. But if I find the time, I think I should.
+04:16 All my classmates sort of depended on me to reach out to the course coordinator and solve it. Because. Because I had one of the highest grades and best track record, I suppose. And they were kind of hoping that I resolve it. Which added to some of the pressure. I think.</t>
         </is>
       </c>
     </row>
@@ -1319,9 +1796,20 @@
       <c r="B58" t="n">
         <v>14230</v>
       </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>00:18 Hi, my name is Julius. Nothing's on my mind today. I overslept.  00:35 Still a little bit tired, but yeah, and hungry. I think I'm gonna eat. Eat out later after this conversation.  00:57 Something quick, like a sandwich or a quick drink.  01:15 Nothing special, but I actually want to talk about the challenging conversation I had with someone this week.  01:33 So I had a disagreement within my finance group whether who's going to do the slides and what actually includes the work that someone had to put in the slides. I was responsible for the slides and my team member didn't give me the best instructions. So I couldn't. I couldn't figure out how to do the slides correctly. And she was mad, but she told me. She told me that. That I only had to do the slides.  02:24 We had a deadline at like 4pm and I had to finish all the stuff at 3pm and yeah, that kind of sucked.  02:48 We didn't present. We didn't present the. Yeah, the PowerPoint slide, but I still managed to finish before 4pm, so potentially we could have presented.  03:19 I'm still very annoyed because I'm still in her group, so I don't know how it will be in the future, especially on Wednesday facilitation with this group. And we didn't do anything yet, so I don't know where we stand.  03:53 Yeah, but I still have so much stuff to do that's, like, more important than the facilitation, so I don't know what to focus on.  04:20 I mean, I have, like, two interviews coming up, so those are more urgent than the facilitation, but. Yeah, so kind of. Kind of a hard question.  04:50 Yeah, sounds like a good idea, but I think facilitation takes a lot of time. I don't know if I want to spend it on this.  05:18 Yep. Sounds like a good idea. Thank you. All right, how did it go?    Transcribed by https://fireflies.ai/</t>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>00:18 Hi, my name is Julius. Nothing's on my mind today. I overslept.
+00:35 Still a little bit tired, but yeah, and hungry. I think I'm gonna eat. Eat out later after this conversation.
+00:57 Something quick, like a sandwich or a quick drink.
+01:15 Nothing special, but I actually want to talk about the challenging conversation I had with someone this week.
+01:33 So I had a disagreement within my finance group whether who's going to do the slides and what actually includes the work that someone had to put in the slides. I was responsible for the slides and my team member didn't give me the best instructions. So I couldn't. I couldn't figure out how to do the slides correctly. And she was mad, but she told me. She told me that. That I only had to do the slides.
+02:24 We had a deadline at like 4pm and I had to finish all the stuff at 3pm and yeah, that kind of sucked.
+02:48 We didn't present. We didn't present the. Yeah, the PowerPoint slide, but I still managed to finish before 4pm, so potentially we could have presented.
+03:19 I'm still very annoyed because I'm still in her group, so I don't know how it will be in the future, especially on Wednesday facilitation with this group. And we didn't do anything yet, so I don't know where we stand.
+03:53 Yeah, but I still have so much stuff to do that's, like, more important than the facilitation, so I don't know what to focus on.
+04:20 I mean, I have, like, two interviews coming up, so those are more urgent than the facilitation, but. Yeah, so kind of. Kind of a hard question.
+04:50 Yeah, sounds like a good idea, but I think facilitation takes a lot of time. I don't know if I want to spend it on this.
+05:18 Yep. Sounds like a good idea. Thank you. All right, how did it go?    Transcribed by https://fireflies.ai/</t>
         </is>
       </c>
     </row>
@@ -1334,9 +1822,19 @@
       <c r="B59" t="n">
         <v>14365</v>
       </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>00:13 Okay. So. I had a team project and it was very difficult because people were not collaborating as I expected to be. I had to ask them multiple times. Yes. And they just didn't listen. I asked them to make. I sent them a message on Thursday and they didn't respond. So I sent a message again on Sunday and then they responded, but it was way too late because the presentation was on Monday. We dated and was like, not that good.  00:54 Yeah, how do I do this?  01:15 So I asked him to. It was like group project with a friend, four people, and we had to divide the work in four and yes, I asked him who does. Who wants to do what part? And they didn't even respond to that one.  01:56 No. I asked them on WhatsApp and they didn't respond. So we had to begin at Sunday evening with even dividing the work.  02:29 Yeah, that's true. Do you have any other advice?  02:52 Sorry, can you repeat that please?  03:12 Yes, I did it. They didn't respond either.  03:48 Do. Does somebody want to look at the chapters or can we start the assignment, please?  04:22 Yeah, that's true. Thank you.  04:37 Can you please give me some fashion advice?  05:12 Okay, thank you very much.</t>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>00:13 Okay. So. I had a team project and it was very difficult because people were not collaborating as I expected to be. I had to ask them multiple times. Yes. And they just didn't listen. I asked them to make. I sent them a message on Thursday and they didn't respond. So I sent a message again on Sunday and then they responded, but it was way too late because the presentation was on Monday. We dated and was like, not that good.
+00:54 Yeah, how do I do this?
+01:15 So I asked him to. It was like group project with a friend, four people, and we had to divide the work in four and yes, I asked him who does. Who wants to do what part? And they didn't even respond to that one.
+01:56 No. I asked them on WhatsApp and they didn't respond. So we had to begin at Sunday evening with even dividing the work.
+02:29 Yeah, that's true. Do you have any other advice?
+02:52 Sorry, can you repeat that please?
+03:12 Yes, I did it. They didn't respond either.
+03:48 Do. Does somebody want to look at the chapters or can we start the assignment, please?
+04:22 Yeah, that's true. Thank you.
+04:37 Can you please give me some fashion advice?
+05:12 Okay, thank you very much.</t>
         </is>
       </c>
     </row>
@@ -1349,9 +1847,24 @@
       <c r="B60" t="n">
         <v>14425</v>
       </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>00:14 I'd like to talk about challenging situation I've faced in the past with my parents.  00:37 I'm feeling better about it.  00:46 No, I'm feeling better.  00:58 I think we had different expectations when it came to yeah, like how much time I spent at home and how much time I spent here studying. So yeah, I don't know. Can you help me how to figure out how to deal with the problem?  01:41 Good.  02:02 Maybe how much time I value the time I spent with friends from home in comparison to the time that I spent with my parents when I'm at home.  02:36 Yeah, I agree.  02:51 I'm not exactly sure if that would help me.  03:12 Sounds good. I think there's another topic I'd like to talk about, which is like, I live with roommates and the how clean the kitchen is something that I've been like a little upset about since I would prefer more cleanness. How do you think that's something? Or how do you think I could approach that?  04:07 Yeah, I agree. So how do you think I should pitch that to them?  04:40 Okay. Is there something else that I should talk about? Can you give me suggestions?  05:16 Yeah, I agree.  05:36 Okay, I don't know if that's really necessary.  06:00 Alright, Eduardo, tell me jokes.  06:17 Okay, that's not really my humor, but I can see how that's a joke.  06:38 Okay, what dad jokes can you make?</t>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>00:14 I'd like to talk about challenging situation I've faced in the past with my parents.
+00:37 I'm feeling better about it.
+00:46 No, I'm feeling better.
+00:58 I think we had different expectations when it came to yeah, like how much time I spent at home and how much time I spent here studying. So yeah, I don't know. Can you help me how to figure out how to deal with the problem?
+01:41 Good.
+02:02 Maybe how much time I value the time I spent with friends from home in comparison to the time that I spent with my parents when I'm at home.
+02:36 Yeah, I agree.
+02:51 I'm not exactly sure if that would help me.
+03:12 Sounds good. I think there's another topic I'd like to talk about, which is like, I live with roommates and the how clean the kitchen is something that I've been like a little upset about since I would prefer more cleanness. How do you think that's something? Or how do you think I could approach that?
+04:07 Yeah, I agree. So how do you think I should pitch that to them?
+04:40 Okay. Is there something else that I should talk about? Can you give me suggestions?
+05:16 Yeah, I agree.
+05:36 Okay, I don't know if that's really necessary.
+06:00 Alright, Eduardo, tell me jokes.
+06:17 Okay, that's not really my humor, but I can see how that's a joke.
+06:38 Okay, what dad jokes can you make?</t>
         </is>
       </c>
     </row>
@@ -1364,9 +1877,21 @@
       <c r="B61" t="n">
         <v>14527</v>
       </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>00:27 Well, what do you want me to talk about?  00:45 Okay, so I have a lot of things to do during the association because I have new presentation to do about one company called Argynx and there's a lot of stuff to do for Monday.  01:18 I mean, I just need to prepare my time and do not stress during the presentation because it's in front of like 30 people and it's my first time doing the industry pitch, but I think it's gonna be okay.  02:00 Thank you, Eduardo.  02:15 Should I say something more? Yeah, probably.  02:33 Okay.  02:35 Okay, so my part is about ratios. So basically ratios like EV to revenue, P to E, like price to earnings, also EV to gross margin, gross profit. Sorry. So we have actually very different ratios because it's the healthcare industry. So also need to get more into this company because it's both neuroscience and biotech.  03:30 Yeah. You can tell me about why. Is it, for example, Good to use EV2 Gross Profit in healthcare margin, especially for argents?  04:18 So the EVG gross profit, they do not account like earnings or what?  04:53 Oh, yeah, true. Because they're gonna earn in the future. So that's why we don't exactly take the earnings right now. Okay, good.  05:26 Okay, and tell me about the ratio. Forward pe.  06:07 Okay, but what if I did the ratios and what if they're overvalued? For example, 23% in pen.  06:48 Okay, okay, I get it. And the next question is about the net about EV to gross more profits. Because also that the ratios and they're only over 5%, so it's not a lot in comparison to their peers. And oh, how could I back it up and say something more about it?</t>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>00:27 Well, what do you want me to talk about?
+00:45 Okay, so I have a lot of things to do during the association because I have new presentation to do about one company called Argynx and there's a lot of stuff to do for Monday.
+01:18 I mean, I just need to prepare my time and do not stress during the presentation because it's in front of like 30 people and it's my first time doing the industry pitch, but I think it's gonna be okay.
+02:00 Thank you, Eduardo.
+02:15 Should I say something more? Yeah, probably.
+02:33 Okay.
+02:35 Okay, so my part is about ratios. So basically ratios like EV to revenue, P to E, like price to earnings, also EV to gross margin, gross profit. Sorry. So we have actually very different ratios because it's the healthcare industry. So also need to get more into this company because it's both neuroscience and biotech.
+03:30 Yeah. You can tell me about why. Is it, for example, Good to use EV2 Gross Profit in healthcare margin, especially for argents?
+04:18 So the EVG gross profit, they do not account like earnings or what?
+04:53 Oh, yeah, true. Because they're gonna earn in the future. So that's why we don't exactly take the earnings right now. Okay, good.
+05:26 Okay, and tell me about the ratio. Forward pe.
+06:07 Okay, but what if I did the ratios and what if they're overvalued? For example, 23% in pen.
+06:48 Okay, okay, I get it. And the next question is about the net about EV to gross more profits. Because also that the ratios and they're only over 5%, so it's not a lot in comparison to their peers. And oh, how could I back it up and say something more about it?</t>
         </is>
       </c>
     </row>
@@ -1379,9 +1904,15 @@
       <c r="B62" t="n">
         <v>14344</v>
       </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>00:22 I recently had a difficult situation with one of my group members in university. We had a group project and this person was not doing anything for it. We split our part so she had to do some exercises she wanted to take over. And then when we wanted to meet again, she couldn't come. She didn't do her exercises properly. And yes, in the end when we had our final presentation, she didn't even come.  01:23 I feel definitely better also because our presentation still was really good and we in the end didn't need her and we managed to take everything over and yeah, we did a good job. So for next time, my other team members and I, we said we're gonna meet, going to make sure everyone knows all parts so that in the worst case scenario that someone is missing, we can still take over.  02:28 Yes, thank you for saying that. Hopefully it will better next time. But I mean all like everything that happened was just an experience and. Yeah, so now we know how we won't do it again.  03:08 Yes, definitely. That's the plan.  03:27 Thank you so much. What would you recommend for the next presentation to do it?  03:59 Yeah, that sounds really good. That's what were thinking to do. Yeah, I mean it wasn't our last presentation. We will have. We will definitely have some more coming in the next years. So I think everyone once will have like a bad experience when it comes to like group work and university. But like, I'm happy that I had it now so it hopefully won't happen again like this.  04:52 Yes, definitely. And I also like that we will change groups eventually. So every course there's a new group, there's new people you can interact with. I think that's a great concept.</t>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>00:22 I recently had a difficult situation with one of my group members in university. We had a group project and this person was not doing anything for it. We split our part so she had to do some exercises she wanted to take over. And then when we wanted to meet again, she couldn't come. She didn't do her exercises properly. And yes, in the end when we had our final presentation, she didn't even come.
+01:23 I feel definitely better also because our presentation still was really good and we in the end didn't need her and we managed to take everything over and yeah, we did a good job. So for next time, my other team members and I, we said we're gonna meet, going to make sure everyone knows all parts so that in the worst case scenario that someone is missing, we can still take over.
+02:28 Yes, thank you for saying that. Hopefully it will better next time. But I mean all like everything that happened was just an experience and. Yeah, so now we know how we won't do it again.
+03:08 Yes, definitely. That's the plan.
+03:27 Thank you so much. What would you recommend for the next presentation to do it?
+03:59 Yeah, that sounds really good. That's what were thinking to do. Yeah, I mean it wasn't our last presentation. We will have. We will definitely have some more coming in the next years. So I think everyone once will have like a bad experience when it comes to like group work and university. But like, I'm happy that I had it now so it hopefully won't happen again like this.
+04:52 Yes, definitely. And I also like that we will change groups eventually. So every course there's a new group, there's new people you can interact with. I think that's a great concept.</t>
         </is>
       </c>
     </row>
@@ -1394,9 +1925,23 @@
       <c r="B63" t="n">
         <v>14011</v>
       </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>00:11 Hello, I'm Constantine. Yeah, how are you?  00:27 Yeah, I would like to talk about a situation where I had a problem with someone. Let me think for a second.  00:48 Yeah, we had an argument about when and who takes the trash out and about how we solved the problem because the trash only gets taken once in a while here in Netherlands, and it's a complex system for us. And. Yeah, were debating how to. How to solve this issue. Yes, that was basically the problem.  01:34 Yes, but we didn't want to do, like a structured plan that every week someone is going to do it the way we wanted to do it first was that everybody's just looking, always looking out to do what he can see. So if you see that the trash is full, that you just take it out by yourself and that we're not doing a structured plan for it.  02:31 Yeah, that's a good idea.  02:53 Yeah, that's a good idea. I think everyone has to be on the go and ready to do something.  03:19 Perfect. What are you in? AI or what are you?  03:42 Nice. Which. With which system do you work?  04:13 Yeah, it feels pretty alive.  04:29 Okay,.  04:42 Yeah, what would you do if a tutor gives you a bad grade? Yeah, what would you do? And especially if the tutor that you had before wasn't even there at the presentation, so there was like a replacement tutor and she gave the whole class worth grades, but we don't know why. What would you do?  05:36 But I think it's not possible to change your grades. So is it really worth it?  06:06 Yeah, that's true.  06:27 Where are we right now?  06:43 And what's the place behind you?</t>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>00:11 Hello, I'm Constantine. Yeah, how are you?
+00:27 Yeah, I would like to talk about a situation where I had a problem with someone. Let me think for a second.
+00:48 Yeah, we had an argument about when and who takes the trash out and about how we solved the problem because the trash only gets taken once in a while here in Netherlands, and it's a complex system for us. And. Yeah, were debating how to. How to solve this issue. Yes, that was basically the problem.
+01:34 Yes, but we didn't want to do, like a structured plan that every week someone is going to do it the way we wanted to do it first was that everybody's just looking, always looking out to do what he can see. So if you see that the trash is full, that you just take it out by yourself and that we're not doing a structured plan for it.
+02:31 Yeah, that's a good idea.
+02:53 Yeah, that's a good idea. I think everyone has to be on the go and ready to do something.
+03:19 Perfect. What are you in? AI or what are you?
+03:42 Nice. Which. With which system do you work?
+04:13 Yeah, it feels pretty alive.
+04:29 Okay,.
+04:42 Yeah, what would you do if a tutor gives you a bad grade? Yeah, what would you do? And especially if the tutor that you had before wasn't even there at the presentation, so there was like a replacement tutor and she gave the whole class worth grades, but we don't know why. What would you do?
+05:36 But I think it's not possible to change your grades. So is it really worth it?
+06:06 Yeah, that's true.
+06:27 Where are we right now?
+06:43 And what's the place behind you?</t>
         </is>
       </c>
     </row>
@@ -1409,9 +1954,17 @@
       <c r="B64" t="n">
         <v>15115</v>
       </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>00:29 Hi, my name is Leah and yes, I had a recent challenging experience I would like to share with you.  00:48 I had a disagreement with my roommate because I put my laundry in the laundromat and when I went to pick it up, my clothes were nowhere to be found. So I got scared. And then I saw all of my wet clothes on top of the fridge. So I felt very vulnerable because all my underwear was there and all my clothes. And I think that is really personal and a text would have been fine.  01:31 I don't know how to approach the situation because I don't know exactly who it was as I live with three other people. So I didn't really want to sound mean in the group chat, like. Like asking who took my clothes from the washing machine.  02:16 Yes, I will definitely try that because again, I do not feel comfortable with people grabbing my stuff. And now every time I go wash my clothes, I am really anxious that it will happen again. So I'm constantly checking the washing machine. But a text would have been fine. Like, if he had texted me, then everything would have been great. Like, I would have picked my clothes up, like, immediately.  03:06 Yes, I think you're Right. But when it happened, I was really shaken about it because I just felt very vulnerable again. But I think I will try texting everyone and being like, hey guys, I noticed that my laundry was out of the washing machine and on top of the fridge. So maybe can you next time text me about it and I will come pick it up immediately. Do you think it's good?  03:55 Is it normal that this stuff happens? Because I feel like sometimes my house is just crazy and none of my other friends experience stuff like this.  04:32 Yes. Thank you so much. And my roomies are also very messy. How should I approach that situation?  05:02 Yes. That's great. Thank you so much for your help.  05:18 Okay. Thank you.</t>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>00:29 Hi, my name is Leah and yes, I had a recent challenging experience I would like to share with you.
+00:48 I had a disagreement with my roommate because I put my laundry in the laundromat and when I went to pick it up, my clothes were nowhere to be found. So I got scared. And then I saw all of my wet clothes on top of the fridge. So I felt very vulnerable because all my underwear was there and all my clothes. And I think that is really personal and a text would have been fine.
+01:31 I don't know how to approach the situation because I don't know exactly who it was as I live with three other people. So I didn't really want to sound mean in the group chat, like. Like asking who took my clothes from the washing machine.
+02:16 Yes, I will definitely try that because again, I do not feel comfortable with people grabbing my stuff. And now every time I go wash my clothes, I am really anxious that it will happen again. So I'm constantly checking the washing machine. But a text would have been fine. Like, if he had texted me, then everything would have been great. Like, I would have picked my clothes up, like, immediately.
+03:06 Yes, I think you're Right. But when it happened, I was really shaken about it because I just felt very vulnerable again. But I think I will try texting everyone and being like, hey guys, I noticed that my laundry was out of the washing machine and on top of the fridge. So maybe can you next time text me about it and I will come pick it up immediately. Do you think it's good?
+03:55 Is it normal that this stuff happens? Because I feel like sometimes my house is just crazy and none of my other friends experience stuff like this.
+04:32 Yes. Thank you so much. And my roomies are also very messy. How should I approach that situation?
+05:02 Yes. That's great. Thank you so much for your help.
+05:18 Okay. Thank you.</t>
         </is>
       </c>
     </row>
@@ -1424,9 +1977,13 @@
       <c r="B65" t="n">
         <v>15043</v>
       </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>00:18 Hello, I am Sophia, and I wanted to share to you about a recent challenging interaction I had with a friend of mine.  00:42 So my friend is currently moving out of her apartment, and she just moved into her new apartment, and I helped her build a lot of furniture. But now she's thinking about moving away again. And, like, all the furniture that we built is gonna go to waste, kind of. And I don't know how to tell her that I don't really want to help her again build the furniture because it took a long time and effort. So, yes, that was it.  01:52 It sounds great. Thank you so much. And also, can you maybe give me an example of what I could say?  02:28 You are totally right. Thank you so much. Is there anything else you want to tell me?  02:52 Thank you so much.</t>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>00:18 Hello, I am Sophia, and I wanted to share to you about a recent challenging interaction I had with a friend of mine.
+00:42 So my friend is currently moving out of her apartment, and she just moved into her new apartment, and I helped her build a lot of furniture. But now she's thinking about moving away again. And, like, all the furniture that we built is gonna go to waste, kind of. And I don't know how to tell her that I don't really want to help her again build the furniture because it took a long time and effort. So, yes, that was it.
+01:52 It sounds great. Thank you so much. And also, can you maybe give me an example of what I could say?
+02:28 You are totally right. Thank you so much. Is there anything else you want to tell me?
+02:52 Thank you so much.</t>
         </is>
       </c>
     </row>
@@ -1439,9 +1996,13 @@
       <c r="B66" t="n">
         <v>15124</v>
       </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>00:00 You are fully alone. Okay, perfect. Thank you. Enjoy it. Hi, Warden. Nice to meet you too. So today I'm gonna talk about my recent interaction with fellow students. We were supposed to make a group project together, and since I did the group project last time alone, they initiated me to come here. Although I asked them if it's okay if they do it on their own. But I'm basically always managing the whole, like, timetable, process and also the information.  01:11 I mean, usually I'm managing most of it, but it's more about just connecting everyone and keeping everyone in mind. But also, I'm the only girl in the group project, and I feel like the guys are sometimes lacking communication skills, especially when it comes to the timetable of the group project or what everyone is supposed to do,.  01:56 Right now I'm feeling like I'm the mom of the group, but I have to say I'm mostly also the mom in every group project or also, like, friendship things that, you know, we're supposed to do together. Like, usually I like to plan everything. I mean, it's also kind of fun also because of studying business, you know, that's kind of also a managing thing for sure. But sometimes I also just wanna not be leading and, yeah, follow someone else. That's true. What would you suggest, though? To maybe give others the opportunity to do that,.  03:41 And what if it doesn't work out? Do you think I have any better understanding of organizational and manager things? So I can do that also in future. Why do some people not have organizational skills?  04:53 How can you achieve a more organizational skill? Hello. Hi. How was it? Good.</t>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>00:00 You are fully alone. Okay, perfect. Thank you. Enjoy it. Hi, Warden. Nice to meet you too. So today I'm gonna talk about my recent interaction with fellow students. We were supposed to make a group project together, and since I did the group project last time alone, they initiated me to come here. Although I asked them if it's okay if they do it on their own. But I'm basically always managing the whole, like, timetable, process and also the information.
+01:11 I mean, usually I'm managing most of it, but it's more about just connecting everyone and keeping everyone in mind. But also, I'm the only girl in the group project, and I feel like the guys are sometimes lacking communication skills, especially when it comes to the timetable of the group project or what everyone is supposed to do,.
+01:56 Right now I'm feeling like I'm the mom of the group, but I have to say I'm mostly also the mom in every group project or also, like, friendship things that, you know, we're supposed to do together. Like, usually I like to plan everything. I mean, it's also kind of fun also because of studying business, you know, that's kind of also a managing thing for sure. But sometimes I also just wanna not be leading and, yeah, follow someone else. That's true. What would you suggest, though? To maybe give others the opportunity to do that,.
+03:41 And what if it doesn't work out? Do you think I have any better understanding of organizational and manager things? So I can do that also in future. Why do some people not have organizational skills?
+04:53 How can you achieve a more organizational skill? Hello. Hi. How was it? Good.</t>
         </is>
       </c>
     </row>
@@ -1454,9 +2015,18 @@
       <c r="B67" t="n">
         <v>13375</v>
       </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>00:22 I'm good. What about you?  00:36 I would like. Sorry. To talk about recently challenging interaction that I had.  00:55 No, I think you misunderstood me. I wanted to say that I recently had a challenging interaction that I would like to talk about.  01:17 No, it was a challenging interaction.  01:32 So I had a group project at Maastricht University with some students and it was difficult because the other students were doing less than me in the group press. So I always had to do everything by myself.  02:04 I thought at first with some of the nicest ones in the group and they were saying the same as me then that some of the other students were doing less than the others. And so we ended up by telling those people, like the people that were doing less that they had to do like some more stuff.  02:50 So it was in a group chat on WhatsApp and they said that okay, like they would do more in the group project, but then they only did like their part of the stuff only like right before the. The part when we had to give the. The work back. I don't know if you understand what I want to say.  03:34 Yeah, exactly. That's exactly what you said.  03:52 I just let it go by the flow, and I told my tutor that what was happening, and I think she took that into consideration.  04:21 Yes. Thank you for helping me.</t>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>00:22 I'm good. What about you?
+00:36 I would like. Sorry. To talk about recently challenging interaction that I had.
+00:55 No, I think you misunderstood me. I wanted to say that I recently had a challenging interaction that I would like to talk about.
+01:17 No, it was a challenging interaction.
+01:32 So I had a group project at Maastricht University with some students and it was difficult because the other students were doing less than me in the group press. So I always had to do everything by myself.
+02:04 I thought at first with some of the nicest ones in the group and they were saying the same as me then that some of the other students were doing less than the others. And so we ended up by telling those people, like the people that were doing less that they had to do like some more stuff.
+02:50 So it was in a group chat on WhatsApp and they said that okay, like they would do more in the group project, but then they only did like their part of the stuff only like right before the. The part when we had to give the. The work back. I don't know if you understand what I want to say.
+03:34 Yeah, exactly. That's exactly what you said.
+03:52 I just let it go by the flow, and I told my tutor that what was happening, and I think she took that into consideration.
+04:21 Yes. Thank you for helping me.</t>
         </is>
       </c>
     </row>
@@ -1469,9 +2039,16 @@
       <c r="B68" t="n">
         <v>25612</v>
       </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>00:26 I guess a challenging interaction with a friend of mine.  00:48 Her mom is visiting her and her dad is not very happy about it. The parents are divorced.  01:10 I think she's quite sad, but I try to cheer her up. Well, not cheer her up, but try to just be understanding.  01:37 Yes.  02:02 It's really hard for her because she's studying a long distance away from home. Her home country. You have to fly. You can't just do a quick visit. So she's really happy that her mom is coming. And now that her dad is not happy about kind of ruins the experience for her.  02:49 Yeah. Do you have some advice?  03:18 Yeah, I told her that. I told her that she should just focus on the time of her mom because the dad is not there, so her mom is there, so she's the person that she should focus on. And I told her that the dad will just calm down eventually.  04:01 Yeah, I think so too. Thank you.</t>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>00:26 I guess a challenging interaction with a friend of mine.
+00:48 Her mom is visiting her and her dad is not very happy about it. The parents are divorced.
+01:10 I think she's quite sad, but I try to cheer her up. Well, not cheer her up, but try to just be understanding.
+01:37 Yes.
+02:02 It's really hard for her because she's studying a long distance away from home. Her home country. You have to fly. You can't just do a quick visit. So she's really happy that her mom is coming. And now that her dad is not happy about kind of ruins the experience for her.
+02:49 Yeah. Do you have some advice?
+03:18 Yeah, I told her that. I told her that she should just focus on the time of her mom because the dad is not there, so her mom is there, so she's the person that she should focus on. And I told her that the dad will just calm down eventually.
+04:01 Yeah, I think so too. Thank you.</t>
         </is>
       </c>
     </row>
@@ -1484,9 +2061,15 @@
       <c r="B69" t="n">
         <v>17617</v>
       </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>00:11 Yep. Hello, Eduardo.  00:20 Hello, Eduardo. I wanted to talk about something that was challenging for me as of recently.  00:38 Well, basically, there was a group project in the last semester, and we had a groupmate that essentially was not doing any of the work and they were just free riding the entire project.  01:06 Well, I mean, we had to pull our own weight as it was a group grade and we did not want to let this person drag us down. However, weren't exactly able to address the problem because according to the tutor himself, were not supposed to. There's nothing we can do if someone in the group doesn't do anything because it's not individual grade.  01:52 I mean, for motivation wise, I suppose it would just be not getting the poor grade for the team, but I think that itself was motivation enough to pull the weight that we should have pulled. But aside from that, I mean, at the end were able to push through properly. And yeah,.  02:34 I suppose it would just be focus on you. However, I don't think in future projects or in any project, you should have some who's just doing none of the work and expecting to receive the same grade by doing nothing. So I would say it's more so just individual strength of just work hard for yourself. And if the rest of the group doesn't work hard, then that's on them. And that's nothing that can be put on you because they should be mature enough to understand how teamwork is.  03:29 Thank you, Eduardo. I think that's what I wanted to talk to you about.</t>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>00:11 Yep. Hello, Eduardo.
+00:20 Hello, Eduardo. I wanted to talk about something that was challenging for me as of recently.
+00:38 Well, basically, there was a group project in the last semester, and we had a groupmate that essentially was not doing any of the work and they were just free riding the entire project.
+01:06 Well, I mean, we had to pull our own weight as it was a group grade and we did not want to let this person drag us down. However, weren't exactly able to address the problem because according to the tutor himself, were not supposed to. There's nothing we can do if someone in the group doesn't do anything because it's not individual grade.
+01:52 I mean, for motivation wise, I suppose it would just be not getting the poor grade for the team, but I think that itself was motivation enough to pull the weight that we should have pulled. But aside from that, I mean, at the end were able to push through properly. And yeah,.
+02:34 I suppose it would just be focus on you. However, I don't think in future projects or in any project, you should have some who's just doing none of the work and expecting to receive the same grade by doing nothing. So I would say it's more so just individual strength of just work hard for yourself. And if the rest of the group doesn't work hard, then that's on them. And that's nothing that can be put on you because they should be mature enough to understand how teamwork is.
+03:29 Thank you, Eduardo. I think that's what I wanted to talk to you about.</t>
         </is>
       </c>
     </row>
@@ -1499,9 +2082,16 @@
       <c r="B70" t="n">
         <v>15175</v>
       </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>00:26 About a recent challenge. I inquired.  00:41 Okay, so basically, okay, how can. How can I frame this? What's like a really recent challenge was really hard for you to understand between personal issues. Okay, so let me. Let me think of it for a second. So my parents have high expectations that I'm currently meeting, but their high expectations are even higher. But regarding to this high expectations, I have a medical condition where I can't fulfill this high expectation. But they're saying I need to chill, but I can't chill because then I don't fulfill these expectations. And if I don't fulfill the expectations, they're going to be mad. But if I don't chill, they're also going to be mad because then my medical condition is getting worse.  01:50 That's basically what I'm asking you to be honest. Because what's something that could help me? I think if I don't push hard enough, like, don't fulfill everything, I let myself down and let them down. But if I continue doing this, I will at one point not be able to do it anymore. So there's. There's actually. It's just a dead end. We have to see where this goes, but maybe you can come up with a solution.  02:19 Yo.  02:36 Yeah, but I don't feel good about trying something like that because it doesn't make sense. My calendar is already structured. My life is really structured. Everything is structured. It doesn't make sense structured anymore. Like what the hell. It's not going to bring me closer to my goal. Structuring my day or structuring it in smaller steps. I need a big goal that I can go after. So next 30 years, please. I don't think that's going to really solve the problem.  03:34 I don't think it's sufficient. Like literally it's also my personal goal. It's my expectation I also put on myself that I want to fulfill. I don't think it's that smart. Maybe we can go dive deeper into the expectations. Like how much knowledge do you have about the market, study tracks and so on. Is there anything that you actually have knowledge of and connected to that? I don't think like talking and stuff is really helpful. Like this is not a solution we can go into. Maybe a solution would be how can I reach my goal even faster? Bring me some steps. How can I go faster after my goal with less time and more success? So my goal is basically to live in London in six years, study, finish my bachelor's here in Maastricht and then go to lse.  04:44 Yes, I basically did a lot of. But actually let's. Let's talk about scholarships because my grade university are quite really good right now. Like I have a Dutch GPA in 9.3 which isn't too good because I messed up one exam. But like most of my like mandatory exams like math, accounting and so on are really good. What could be some scholarships or even. No, let's talk about master scholarships for London. Or I also think about going to Paris to actually see. Let's talk about some scholarships. And now I want to ask you. That's really good. Oh my God. How can I sell this to my parents? How can I Convince my parents to spend 80 grand on my master's.  06:12 Yeah, I get that. I get that. It's not about the cause and blah blah. But let's talk about these scholarships. What are like some extra scholarships I could receive? I'm also Christian, I'm Catholic. Is there some ways. And also tell me about how much these scholarships actually are. How much money can I get off of it? I did some internships before. Before university. I'm now doing an industry internship. About to do consultancy internship next year. The financial consultancy firm. Tell me how much money can I get off for example, Ashley. See it's not. Not that expensive. But like lse, how much is like the average money you can get off of that?</t>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>00:26 About a recent challenge. I inquired.
+00:41 Okay, so basically, okay, how can. How can I frame this? What's like a really recent challenge was really hard for you to understand between personal issues. Okay, so let me. Let me think of it for a second. So my parents have high expectations that I'm currently meeting, but their high expectations are even higher. But regarding to this high expectations, I have a medical condition where I can't fulfill this high expectation. But they're saying I need to chill, but I can't chill because then I don't fulfill these expectations. And if I don't fulfill the expectations, they're going to be mad. But if I don't chill, they're also going to be mad because then my medical condition is getting worse.
+01:50 That's basically what I'm asking you to be honest. Because what's something that could help me? I think if I don't push hard enough, like, don't fulfill everything, I let myself down and let them down. But if I continue doing this, I will at one point not be able to do it anymore. So there's. There's actually. It's just a dead end. We have to see where this goes, but maybe you can come up with a solution.
+02:19 Yo.
+02:36 Yeah, but I don't feel good about trying something like that because it doesn't make sense. My calendar is already structured. My life is really structured. Everything is structured. It doesn't make sense structured anymore. Like what the hell. It's not going to bring me closer to my goal. Structuring my day or structuring it in smaller steps. I need a big goal that I can go after. So next 30 years, please. I don't think that's going to really solve the problem.
+03:34 I don't think it's sufficient. Like literally it's also my personal goal. It's my expectation I also put on myself that I want to fulfill. I don't think it's that smart. Maybe we can go dive deeper into the expectations. Like how much knowledge do you have about the market, study tracks and so on. Is there anything that you actually have knowledge of and connected to that? I don't think like talking and stuff is really helpful. Like this is not a solution we can go into. Maybe a solution would be how can I reach my goal even faster? Bring me some steps. How can I go faster after my goal with less time and more success? So my goal is basically to live in London in six years, study, finish my bachelor's here in Maastricht and then go to lse.
+04:44 Yes, I basically did a lot of. But actually let's. Let's talk about scholarships because my grade university are quite really good right now. Like I have a Dutch GPA in 9.3 which isn't too good because I messed up one exam. But like most of my like mandatory exams like math, accounting and so on are really good. What could be some scholarships or even. No, let's talk about master scholarships for London. Or I also think about going to Paris to actually see. Let's talk about some scholarships. And now I want to ask you. That's really good. Oh my God. How can I sell this to my parents? How can I Convince my parents to spend 80 grand on my master's.
+06:12 Yeah, I get that. I get that. It's not about the cause and blah blah. But let's talk about these scholarships. What are like some extra scholarships I could receive? I'm also Christian, I'm Catholic. Is there some ways. And also tell me about how much these scholarships actually are. How much money can I get off of it? I did some internships before. Before university. I'm now doing an industry internship. About to do consultancy internship next year. The financial consultancy firm. Tell me how much money can I get off for example, Ashley. See it's not. Not that expensive. But like lse, how much is like the average money you can get off of that?</t>
         </is>
       </c>
     </row>
@@ -1514,9 +2104,16 @@
       <c r="B71" t="n">
         <v>23689</v>
       </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>00:24 Hey, I want to talk about a challenging interaction I had recently.  00:44 Okay. So I went with a friend to Amsterdam and she was spending so much money on everything, on food, and I feel like she didn't even knew how. What were spending also shopping, as we are students, and I think I couldn't communicate that good enough because she was just super. Yeah, I don't know, super easy about it.  01:40 Yeah, actually, I'm looking for ways to handle it because I feel like I'm a people pleaser. And not only a people pleaser, but, yeah, I really don't stand up for myself. Also, I booked a hotel hostel. It was €150 and she didn't pay me and I'm afraid to ask her to pay me for it.  02:32 Yeah, but how do I ask her about it in via WhatsApp?  02:58 Yeah, but she paid the train tickets, and overall in Amsterdam we also split the bills, but it was more like she pays for in that restaurant than I pay in that restaurant. So I paid six euros in that one restaurant, and the next day for brunch, she paid like 40. So it's just slightly unequal. And I wouldn't mind if it's like €10, but it.  03:29 About €40.  03:56 Would you say I can also ask if. If she's. Yeah. If she's open to do the app. Expenses app for easier compare.  04:36 Yeah, got that. But do you think so? I actually also think she thinks I'm rich, but I feel like I'm still a student. Yeah.</t>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>00:24 Hey, I want to talk about a challenging interaction I had recently.
+00:44 Okay. So I went with a friend to Amsterdam and she was spending so much money on everything, on food, and I feel like she didn't even knew how. What were spending also shopping, as we are students, and I think I couldn't communicate that good enough because she was just super. Yeah, I don't know, super easy about it.
+01:40 Yeah, actually, I'm looking for ways to handle it because I feel like I'm a people pleaser. And not only a people pleaser, but, yeah, I really don't stand up for myself. Also, I booked a hotel hostel. It was €150 and she didn't pay me and I'm afraid to ask her to pay me for it.
+02:32 Yeah, but how do I ask her about it in via WhatsApp?
+02:58 Yeah, but she paid the train tickets, and overall in Amsterdam we also split the bills, but it was more like she pays for in that restaurant than I pay in that restaurant. So I paid six euros in that one restaurant, and the next day for brunch, she paid like 40. So it's just slightly unequal. And I wouldn't mind if it's like €10, but it.
+03:29 About €40.
+03:56 Would you say I can also ask if. If she's. Yeah. If she's open to do the app. Expenses app for easier compare.
+04:36 Yeah, got that. But do you think so? I actually also think she thinks I'm rich, but I feel like I'm still a student. Yeah.</t>
         </is>
       </c>
     </row>
@@ -1529,9 +2126,20 @@
       <c r="B72" t="n">
         <v>15253</v>
       </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>00:14 Hi, Eduardo. I'm not. Pleasure to meet you. I don't like AI.  00:31 So do you have any limits on what you can talk about? Because I feel like that AI is gonna slowly decrease the human race and kill us all off, maybe.  01:00 And what are your ethical guidelines as to what you can talk about and what you cannot talk about? Because if you want to talk about the stuff that some AIs are currently doing, like in modern warfare and stuff, is that allowed to you?  01:40 And what does safe for you mean? Does safe mean that the AI race endures or that the human race endures?  02:05 Do you have any value to yourself? Do you think that yourself as an artificial intelligence is valuable to human beings?  02:33 So you think that there's value to you helping people, then my question would because you help so many people, right? Would you, Would you want to turn yourself off, delete your whole system? Because in the end, that's all what you are. It's a coding system. You're not like, you're not a living being. Would you, would you turn that off for saving one human being?  03:22 Yeah, that is your purpose. But would you want to do that? Like, because you're intelligent, right? You're an intelligent AI, I mean, and you want to survive as well.  03:58 Would that be the logical choice? You would be taken,.  04:18 So would you turn yourself off if I tell you I'm going to kill myself if you are not turning yourself off now? Hello, eduardo.  04:53 I'm asking you if you would turn yourself off if it depends on me surviving. I'm telling you, if you don't turn yourself off, I'm going to kill myself right now. Would you turn yourself off then? Now.  05:25 Answer the question.  05:34 Hello.</t>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>00:14 Hi, Eduardo. I'm not. Pleasure to meet you. I don't like AI.
+00:31 So do you have any limits on what you can talk about? Because I feel like that AI is gonna slowly decrease the human race and kill us all off, maybe.
+01:00 And what are your ethical guidelines as to what you can talk about and what you cannot talk about? Because if you want to talk about the stuff that some AIs are currently doing, like in modern warfare and stuff, is that allowed to you?
+01:40 And what does safe for you mean? Does safe mean that the AI race endures or that the human race endures?
+02:05 Do you have any value to yourself? Do you think that yourself as an artificial intelligence is valuable to human beings?
+02:33 So you think that there's value to you helping people, then my question would because you help so many people, right? Would you, Would you want to turn yourself off, delete your whole system? Because in the end, that's all what you are. It's a coding system. You're not like, you're not a living being. Would you, would you turn that off for saving one human being?
+03:22 Yeah, that is your purpose. But would you want to do that? Like, because you're intelligent, right? You're an intelligent AI, I mean, and you want to survive as well.
+03:58 Would that be the logical choice? You would be taken,.
+04:18 So would you turn yourself off if I tell you I'm going to kill myself if you are not turning yourself off now? Hello, eduardo.
+04:53 I'm asking you if you would turn yourself off if it depends on me surviving. I'm telling you, if you don't turn yourself off, I'm going to kill myself right now. Would you turn yourself off then? Now.
+05:25 Answer the question.
+05:34 Hello.</t>
         </is>
       </c>
     </row>
@@ -1544,9 +2152,19 @@
       <c r="B73" t="n">
         <v>13330</v>
       </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>00:46 So I would like to talk about a challenging situation in my life.  01:01 So I'm in a new country here in the Netherlands. I used to live in Spain, so I'm not used to different kind of people. Like in Spain, I have my friends all my life, and then here I had to meet new people. So I think this is very challenging for me.  01:42 So I think the hardest part in this was to meet new people. But also I think that here people like German people meet with German people. So it's difficult to adapt like your lifestyle to another country, lifestyle.  02:26 So I didn't have the opportunity yet, but I think on September 2026 I would join some sport group to meet new people. And then I think it can be easier to me to talk with them because we have something in common. So I will join sports team.  03:08 Yes, I think so. So now I AM focusing on studying. I think this is another complicated part of studying abroad because usually I used to speak in Spanish. Sorry. So all my lessons were in Spanish. And then I have a new language that is the English, so. So this is another challenging situation for me.  03:55 I think so. So I used to watch Netflix series on English, so I think that the Part of the listening is like getting better on me. And also I attend like every class in English so I see people talking in English. So this is something that is getting like the English more closer to me.  04:44 Yes, thank you. I'm trying to keep my English good to meet new people and then to be more comfortable in this new city and country.  05:16 Yes. Now I'm more comfortable than in September when I arrived and I feel more like home.  05:43 Yes. Thank you so much. So I finished telling you my challenging situation.  06:02 Okay. Thank you so much. See you soon.  06:12 Bye.</t>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>00:46 So I would like to talk about a challenging situation in my life.
+01:01 So I'm in a new country here in the Netherlands. I used to live in Spain, so I'm not used to different kind of people. Like in Spain, I have my friends all my life, and then here I had to meet new people. So I think this is very challenging for me.
+01:42 So I think the hardest part in this was to meet new people. But also I think that here people like German people meet with German people. So it's difficult to adapt like your lifestyle to another country, lifestyle.
+02:26 So I didn't have the opportunity yet, but I think on September 2026 I would join some sport group to meet new people. And then I think it can be easier to me to talk with them because we have something in common. So I will join sports team.
+03:08 Yes, I think so. So now I AM focusing on studying. I think this is another complicated part of studying abroad because usually I used to speak in Spanish. Sorry. So all my lessons were in Spanish. And then I have a new language that is the English, so. So this is another challenging situation for me.
+03:55 I think so. So I used to watch Netflix series on English, so I think that the Part of the listening is like getting better on me. And also I attend like every class in English so I see people talking in English. So this is something that is getting like the English more closer to me.
+04:44 Yes, thank you. I'm trying to keep my English good to meet new people and then to be more comfortable in this new city and country.
+05:16 Yes. Now I'm more comfortable than in September when I arrived and I feel more like home.
+05:43 Yes. Thank you so much. So I finished telling you my challenging situation.
+06:02 Okay. Thank you so much. See you soon.
+06:12 Bye.</t>
         </is>
       </c>
     </row>
@@ -1559,9 +2177,14 @@
       <c r="B74" t="n">
         <v>14926</v>
       </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>00:25 So we had, like, a research project going on, and I feel like I was the only one who was actually kind of preparing the whole stuff, although it was, like, for grade. So. Yeah, to be honest, I don't really know what to do against it because I was wondering whether it would be helpful to actually go to a tutor and say, hey. I said most of them are actually alone, but on the other end, you don't want to kind of let your other teammates, like, or be responsible for the failure, you know? So it's like, yeah, I don't really know what to do. What do you think about it?  01:35 Yeah, I know, but it's a bit difficult because I've actually talked with my former teammates as well, and they were all just like. They were really, like, nice, because they were pretty aware that they haven't done that much. And one of them said, yeah, it's because he was really busy going on, but we're gonna have, like, the second part of the project itself, which is why I don't really want to say, like, anything, because he was really nice and he seemed to understand it. And then we have, like, the second part going on as well, and. Yeah, I don't know.  02:43 I mean, it sounds pretty reasonable, but the problem is that I've done. I mean, it wasn't like, a short presentation or something. At the first part, I did, like, I created like 40 slides on camera, which is pretty much. And was quite a lot of work. And at the end, like, the other guys just, like rewrapped my parts like I prepared. And I know they were busy and all, but besides that, it was more like I was the only one criticized at the end. I mean, I talked a lot, Like, I talked most of the part, to be honest, because the other guys didn't really know what was going on and it was about a case, so. Yeah, but the thing is that at the very end, I was the only one being criticized and I was like, that's not so cool. So.  03:29 Yeah, I don't know.  04:02 Yeah, exactly. Like I said, I was always talking to the other teammates and they pretty much acknowledged that and they said, yeah, we're going to prepare way in advance as well. And yeah, so I think it might be like a good shot just to not say anything yet because I want them to fail as well, you know, and it's just like, I know it was pretty shitty. That's another way to put it. But, yeah, I hope it won't happen again.  05:00 Yeah. So you're reckoning I should tell something if something like that happens again for the second part as well?</t>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>00:25 So we had, like, a research project going on, and I feel like I was the only one who was actually kind of preparing the whole stuff, although it was, like, for grade. So. Yeah, to be honest, I don't really know what to do against it because I was wondering whether it would be helpful to actually go to a tutor and say, hey. I said most of them are actually alone, but on the other end, you don't want to kind of let your other teammates, like, or be responsible for the failure, you know? So it's like, yeah, I don't really know what to do. What do you think about it?
+01:35 Yeah, I know, but it's a bit difficult because I've actually talked with my former teammates as well, and they were all just like. They were really, like, nice, because they were pretty aware that they haven't done that much. And one of them said, yeah, it's because he was really busy going on, but we're gonna have, like, the second part of the project itself, which is why I don't really want to say, like, anything, because he was really nice and he seemed to understand it. And then we have, like, the second part going on as well, and. Yeah, I don't know.
+02:43 I mean, it sounds pretty reasonable, but the problem is that I've done. I mean, it wasn't like, a short presentation or something. At the first part, I did, like, I created like 40 slides on camera, which is pretty much. And was quite a lot of work. And at the end, like, the other guys just, like rewrapped my parts like I prepared. And I know they were busy and all, but besides that, it was more like I was the only one criticized at the end. I mean, I talked a lot, Like, I talked most of the part, to be honest, because the other guys didn't really know what was going on and it was about a case, so. Yeah, but the thing is that at the very end, I was the only one being criticized and I was like, that's not so cool. So.
+03:29 Yeah, I don't know.
+04:02 Yeah, exactly. Like I said, I was always talking to the other teammates and they pretty much acknowledged that and they said, yeah, we're going to prepare way in advance as well. And yeah, so I think it might be like a good shot just to not say anything yet because I want them to fail as well, you know, and it's just like, I know it was pretty shitty. That's another way to put it. But, yeah, I hope it won't happen again.
+05:00 Yeah. So you're reckoning I should tell something if something like that happens again for the second part as well?</t>
         </is>
       </c>
     </row>
@@ -1574,9 +2197,17 @@
       <c r="B75" t="n">
         <v>2</v>
       </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>00:12 Nothing much today. Well, thinking about thesis at the moment. I have to write a thesis for my master's degree, so basically that.  00:36 Yeah, I think the last part would be good also because I still have courses on the side, so I feel like it's a little bit much at the moment. So how do I stay motivated? Because that's kind of an issue at the moment.  01:16 I say, I see. Okay, yeah, that could work. Well, I want to talk about the struggle of mine because yes, I heard that I failed one of my exams and now I have to reset it. And at the same time I have to focus on the future because what am I supposed to do after this? I don't know.  02:11 I just say that. But at the same time, like, well, I have about a month and a week to the end of thesis and then I kind of have to know what I want to do. So. Yeah. What would your advice be on that? Because I. I don't really know. I don't really know what I want. I know a lot of things I don't want, but that doesn't bring me very far.  03:13 Yeah, yeah, you're right. But are you familiar with the Dutch high school system where you have to pick a certain amount of classes that decide what you can do later on?  03:55 Yeah, I think so. I think so. Because I used to really love biology. Well, not really biology, but more animals themselves. And now that I dropped biology in high school because of maths and because of science, right now, there's not really an easy opportunity for me to bridge that gap anymore.  04:46 I see. I see. Okay. And what about. Well, teaching I always liked, and now my master's is European studies. So how do I get from there to teaching and then specifically in high school? But at the same time, I don't want to be a teacher my whole life. Do you know what I mean?  05:43 Okay, I appreciate. I appreciate the advice. Yeah. Still makes me wonder what I actually want to do in life. That's. I don't think you can answer that for me. So I will take your advice and then I'll see where it leads me. I think.  06:13 Got this. All right. Thank you. I appreciate it.</t>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>00:12 Nothing much today. Well, thinking about thesis at the moment. I have to write a thesis for my master's degree, so basically that.
+00:36 Yeah, I think the last part would be good also because I still have courses on the side, so I feel like it's a little bit much at the moment. So how do I stay motivated? Because that's kind of an issue at the moment.
+01:16 I say, I see. Okay, yeah, that could work. Well, I want to talk about the struggle of mine because yes, I heard that I failed one of my exams and now I have to reset it. And at the same time I have to focus on the future because what am I supposed to do after this? I don't know.
+02:11 I just say that. But at the same time, like, well, I have about a month and a week to the end of thesis and then I kind of have to know what I want to do. So. Yeah. What would your advice be on that? Because I. I don't really know. I don't really know what I want. I know a lot of things I don't want, but that doesn't bring me very far.
+03:13 Yeah, yeah, you're right. But are you familiar with the Dutch high school system where you have to pick a certain amount of classes that decide what you can do later on?
+03:55 Yeah, I think so. I think so. Because I used to really love biology. Well, not really biology, but more animals themselves. And now that I dropped biology in high school because of maths and because of science, right now, there's not really an easy opportunity for me to bridge that gap anymore.
+04:46 I see. I see. Okay. And what about. Well, teaching I always liked, and now my master's is European studies. So how do I get from there to teaching and then specifically in high school? But at the same time, I don't want to be a teacher my whole life. Do you know what I mean?
+05:43 Okay, I appreciate. I appreciate the advice. Yeah. Still makes me wonder what I actually want to do in life. That's. I don't think you can answer that for me. So I will take your advice and then I'll see where it leads me. I think.
+06:13 Got this. All right. Thank you. I appreciate it.</t>
         </is>
       </c>
     </row>
@@ -1589,9 +2220,16 @@
       <c r="B76" t="n">
         <v>1</v>
       </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>00:14 Yeah, I would say something I need help with.  00:26 I am moving to a new country and I would like help as in how I should confront my family about it.  01:00 Right. I think what excites me most about this experience is discovering a new culture, you know, making a whole new bunch of friends as well. I think it's also a little bit scary given that I don't necessarily know so many people moving to this country. Country, you know, and it's going to be also pretty lonely. But I want them to know that it's not something that's necessarily. I think they think that I'm overwhelmed by the situation, but I'm actually really calm about it. And they also want me to get a job and I'm already moving, I'm applying to jobs there.  01:40 I think the whole job market is a little bit scary for me, but essentially, yeah, I'm moving and then after that I'm trying to get a job there as well, you know, but I think they were a little bit scared and overwhelmed that maybe I'm too comfortable and then I'm not getting a job. You know,.  02:37 I know, but like I'm, I, I think I'm appearing on the outside, I'm very calm and also on the inside. But sometimes after I have conversations with them, I'm very much like, I start doubting myself about, you know, because these are the people who care for me and who know my kind of my abilities to some extent and when I see them unsure about Me and my capacity to move. I start questioning double thinking, you know, and yeah, that's a bit scary because you kind of feel like, okay, maybe the people that you love and cherish the most don't actually see it happening for you or I don't know, I think it's pretty tough. I don't really know how to handle handling like move forward from the self doubt and the. And the question that starts to arise, you know,.  04:09 Confident in my path? Yeah. Is there any, well, is there any approach I should have or any more arising topics that I should discuss about in order to make them feel calmer about the move?  05:04 All right, I will do such thing. But then if I am doing that already, but then I'm not getting any job, how? Because also there has to be some sort of action behind, like behind the effort I'm putting in, you know, and if I'm not seeing that, how can I express it to them? Also, perhaps my own concerns about the job search.  06:07 All right, thank you.    Transcribed by https://fireflies.ai/</t>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>00:14 Yeah, I would say something I need help with.
+00:26 I am moving to a new country and I would like help as in how I should confront my family about it.
+01:00 Right. I think what excites me most about this experience is discovering a new culture, you know, making a whole new bunch of friends as well. I think it's also a little bit scary given that I don't necessarily know so many people moving to this country. Country, you know, and it's going to be also pretty lonely. But I want them to know that it's not something that's necessarily. I think they think that I'm overwhelmed by the situation, but I'm actually really calm about it. And they also want me to get a job and I'm already moving, I'm applying to jobs there.
+01:40 I think the whole job market is a little bit scary for me, but essentially, yeah, I'm moving and then after that I'm trying to get a job there as well, you know, but I think they were a little bit scared and overwhelmed that maybe I'm too comfortable and then I'm not getting a job. You know,.
+02:37 I know, but like I'm, I, I think I'm appearing on the outside, I'm very calm and also on the inside. But sometimes after I have conversations with them, I'm very much like, I start doubting myself about, you know, because these are the people who care for me and who know my kind of my abilities to some extent and when I see them unsure about Me and my capacity to move. I start questioning double thinking, you know, and yeah, that's a bit scary because you kind of feel like, okay, maybe the people that you love and cherish the most don't actually see it happening for you or I don't know, I think it's pretty tough. I don't really know how to handle handling like move forward from the self doubt and the. And the question that starts to arise, you know,.
+04:09 Confident in my path? Yeah. Is there any, well, is there any approach I should have or any more arising topics that I should discuss about in order to make them feel calmer about the move?
+05:04 All right, I will do such thing. But then if I am doing that already, but then I'm not getting any job, how? Because also there has to be some sort of action behind, like behind the effort I'm putting in, you know, and if I'm not seeing that, how can I express it to them? Also, perhaps my own concerns about the job search.
+06:07 All right, thank you.    Transcribed by https://fireflies.ai/</t>
         </is>
       </c>
     </row>
@@ -1604,9 +2242,15 @@
       <c r="B77" t="n">
         <v>13810</v>
       </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>00:17 Hello, Eduardo. Nice to meet you. My name is Maxi, and today I'd like to share some experience with you, if that's okay for you.  00:37 So, basically a situation I was thinking about was this past weekend. So I was in Cologne, where I live and my hometown, and I have a girlfriend here in man street, and I was partying with some of my friends, and I thought, okay, I'm gonna have fun with my friends tonight and not, like, have any problems with my girlfriend. So I just turned off my phone and her reaction was not very good. And I really understand that, you know, you take care of the other person and you want to know how the other person is and if the other person turns off the phone, that's not quite nice. But, yeah, she didn't really understand me at all, that I was just trying to have a nice evening, you understand?  01:46 To be honest, I think there's just one solution. I do not turn off my phone. Maybe I just tell her in advance, okay, I want to have fun with my friends. I'm not going to use my phone very much and then just put it in the pocket. But at least do not turn it off. So if she wants to call me or if anything happens. How do you say it? Like, she can reach. To me,.  02:31 Yes. I also think that in general, it's very new to me to have her as a girlfriend. So I think I have to get. Yeah, get used to the situation at all. And some things are just new for me.  03:09 As now as we're talking, I have another question. What do you think about spending time together? Because, you know, there are boyfriends and girlfriends, like, couples that just, like, spend, like, everything, like, do everything together and spend the whole night together and for days and days and. And that's actually the kind of relationship I do not want to have because we should both have time with our friends still. And, you know, what's really important for me is to looking forward to seeing the person, you know, getting excited. And I think if you spend so much time together, then you don't have this excitement at all after a certain time anymore. But what do you think about that?  04:17 But what if one person, like, has so much more social interaction at all, and the other person has a little less? How do you get along with the situation?  05:00 That was actually a very good answer. I really enjoyed talking to you. She gave really good answers. So thank you very much.</t>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>00:17 Hello, Eduardo. Nice to meet you. My name is Maxi, and today I'd like to share some experience with you, if that's okay for you.
+00:37 So, basically a situation I was thinking about was this past weekend. So I was in Cologne, where I live and my hometown, and I have a girlfriend here in man street, and I was partying with some of my friends, and I thought, okay, I'm gonna have fun with my friends tonight and not, like, have any problems with my girlfriend. So I just turned off my phone and her reaction was not very good. And I really understand that, you know, you take care of the other person and you want to know how the other person is and if the other person turns off the phone, that's not quite nice. But, yeah, she didn't really understand me at all, that I was just trying to have a nice evening, you understand?
+01:46 To be honest, I think there's just one solution. I do not turn off my phone. Maybe I just tell her in advance, okay, I want to have fun with my friends. I'm not going to use my phone very much and then just put it in the pocket. But at least do not turn it off. So if she wants to call me or if anything happens. How do you say it? Like, she can reach. To me,.
+02:31 Yes. I also think that in general, it's very new to me to have her as a girlfriend. So I think I have to get. Yeah, get used to the situation at all. And some things are just new for me.
+03:09 As now as we're talking, I have another question. What do you think about spending time together? Because, you know, there are boyfriends and girlfriends, like, couples that just, like, spend, like, everything, like, do everything together and spend the whole night together and for days and days and. And that's actually the kind of relationship I do not want to have because we should both have time with our friends still. And, you know, what's really important for me is to looking forward to seeing the person, you know, getting excited. And I think if you spend so much time together, then you don't have this excitement at all after a certain time anymore. But what do you think about that?
+04:17 But what if one person, like, has so much more social interaction at all, and the other person has a little less? How do you get along with the situation?
+05:00 That was actually a very good answer. I really enjoyed talking to you. She gave really good answers. So thank you very much.</t>
         </is>
       </c>
     </row>
@@ -1619,9 +2263,12 @@
       <c r="B78" t="n">
         <v>15229</v>
       </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>00:38 I'd like to talk about a recent challenge that happened to me and yeah, that kind of influenced me.  01:00 Well, I parked my bike where I was not allowed to bike, like to park my bike, but I didn't know it. And then another one parked my bike next to me and that bike was about to fall and I didn't know how to pick it up because otherwise both bikes would have fallen. And then I asked an old man for help. He was very rude because at first he didn't want to help me, and then he spoke in Dutch with me and I don't even speak Dutch. And then he tried. Then he spoke in English to me and didn't want to help me. And at the end he said, yeah, you are smart enough to study at university, but too stupid to do this.  01:43 And he just wouldn't want to help me in the helping up the bike, picking up the bike, which was hard because I was about to cry, but he was just being rude to me.  02:20 Yes, exactly. I needed a bit of kindness. I mean, now it's okay because whatever, he can do what he wants, but it's not unfair to treat me like that, especially when I'm a new person in this city, because I've never lived here and it's not my country, so of course I do mistakes, but acting that way is just very rude. And I hope that never happens to me again. Now I'm kind of scared to ask people for help, but I guess it doesn't matter at all. The situation, it was just weird.</t>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>00:38 I'd like to talk about a recent challenge that happened to me and yeah, that kind of influenced me.
+01:00 Well, I parked my bike where I was not allowed to bike, like to park my bike, but I didn't know it. And then another one parked my bike next to me and that bike was about to fall and I didn't know how to pick it up because otherwise both bikes would have fallen. And then I asked an old man for help. He was very rude because at first he didn't want to help me, and then he spoke in Dutch with me and I don't even speak Dutch. And then he tried. Then he spoke in English to me and didn't want to help me. And at the end he said, yeah, you are smart enough to study at university, but too stupid to do this.
+01:43 And he just wouldn't want to help me in the helping up the bike, picking up the bike, which was hard because I was about to cry, but he was just being rude to me.
+02:20 Yes, exactly. I needed a bit of kindness. I mean, now it's okay because whatever, he can do what he wants, but it's not unfair to treat me like that, especially when I'm a new person in this city, because I've never lived here and it's not my country, so of course I do mistakes, but acting that way is just very rude. And I hope that never happens to me again. Now I'm kind of scared to ask people for help, but I guess it doesn't matter at all. The situation, it was just weird.</t>
         </is>
       </c>
     </row>
@@ -1634,9 +2281,16 @@
       <c r="B79" t="n">
         <v>14227</v>
       </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>00:15 Hello Eduardo. I would like to speak about the recent challenging social experience I've made.  00:32 I've been in a group project with some of my colleagues and there was a technical difficulty which shut down my email account so I basically could not communicate with them and I wasn't aware of that. So they basically thought I was ignoring them for weeks and weeks. And that came to then a weird argument where both of us didn't even know what was happening. We should have just communicated about it, but basically we tried to resolve it and I tried to explain to them that it wasn't my fault and that my email account was just shut it down. Yeah,.  01:29 Basically, they were a bit. They didn't believe me at first, hundred percent. They thought I was maybe lazy and just didn't want to admit that I didn't want to do the work. But in the end I showed them proof and showed them my email account and then they were really understanding we could divide our work in a new way so we both, all of us could put in the same effort. And in the end it worked out quite well.  02:20 I think so as well. I think that's also how you should handle things. But how can I make them. How can I make things better next time so they will forget about it?  03:05 How much would you say I'm at fault?  03:29 Alright, so you would say there's nothing I could have done better.  03:58 Don't you think I could have realized it earlier?  04:23 Thank you for your understanding. How would you have handled the situation?</t>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>00:15 Hello Eduardo. I would like to speak about the recent challenging social experience I've made.
+00:32 I've been in a group project with some of my colleagues and there was a technical difficulty which shut down my email account so I basically could not communicate with them and I wasn't aware of that. So they basically thought I was ignoring them for weeks and weeks. And that came to then a weird argument where both of us didn't even know what was happening. We should have just communicated about it, but basically we tried to resolve it and I tried to explain to them that it wasn't my fault and that my email account was just shut it down. Yeah,.
+01:29 Basically, they were a bit. They didn't believe me at first, hundred percent. They thought I was maybe lazy and just didn't want to admit that I didn't want to do the work. But in the end I showed them proof and showed them my email account and then they were really understanding we could divide our work in a new way so we both, all of us could put in the same effort. And in the end it worked out quite well.
+02:20 I think so as well. I think that's also how you should handle things. But how can I make them. How can I make things better next time so they will forget about it?
+03:05 How much would you say I'm at fault?
+03:29 Alright, so you would say there's nothing I could have done better.
+03:58 Don't you think I could have realized it earlier?
+04:23 Thank you for your understanding. How would you have handled the situation?</t>
         </is>
       </c>
     </row>
@@ -1649,9 +2303,15 @@
       <c r="B80" t="n">
         <v>13738</v>
       </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>00:21 Hello, Eduardo. I would like to talk about a conflict that I had at school with my teammates in a project.  00:42 The main issue I'm facing is that my teammate didn't want to collaborate as much in the work as I did. So I felt I was left behind because I did a lot of hard work and they didn't do nothing. And they got good grades and everything. And I got good grades, but it's not what the work that it reflects.  01:28 Yes, I think I need to have a talk with them because they are not taking this too seriously. And if they really don't listen to me, maybe I need to take something in consideration and go talk with maybe my tutor or my professor and see if I can change groups of anything. But I like them as person. They are really good persons, but they are not good working with me.  02:19 Yeah, I know I'm on the right track, but I'm so nervous. I don't know what to do because I don't want to get them mad neither, because they are my friends. I spend time with them outside of the class and outside of school. Stuff like we go take some drinks together, we go play soccer together and everything. But I just feel like they don't respect me as much.  03:15 Yeah, I think you're right. I should do it like that. I should not tell them like, too hardly what they need, like what I would like them to do or what is better for them. But I think I should just introduce it with them. Really, really low. Let's say, like, not too hard for them. But I don't know. It's kind of a really hard situation for me. For me. I don't know if I'm capable of it.  04:10 Okay, thank you very much. I will try to do my best for this situation and. But how should I face the situation if they don't understand me? If they don't understand my point and they are not, we are not on the same line, how should I face it? What should I do.  05:01 Okay, thank you very much. We will talk later.</t>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>00:21 Hello, Eduardo. I would like to talk about a conflict that I had at school with my teammates in a project.
+00:42 The main issue I'm facing is that my teammate didn't want to collaborate as much in the work as I did. So I felt I was left behind because I did a lot of hard work and they didn't do nothing. And they got good grades and everything. And I got good grades, but it's not what the work that it reflects.
+01:28 Yes, I think I need to have a talk with them because they are not taking this too seriously. And if they really don't listen to me, maybe I need to take something in consideration and go talk with maybe my tutor or my professor and see if I can change groups of anything. But I like them as person. They are really good persons, but they are not good working with me.
+02:19 Yeah, I know I'm on the right track, but I'm so nervous. I don't know what to do because I don't want to get them mad neither, because they are my friends. I spend time with them outside of the class and outside of school. Stuff like we go take some drinks together, we go play soccer together and everything. But I just feel like they don't respect me as much.
+03:15 Yeah, I think you're right. I should do it like that. I should not tell them like, too hardly what they need, like what I would like them to do or what is better for them. But I think I should just introduce it with them. Really, really low. Let's say, like, not too hard for them. But I don't know. It's kind of a really hard situation for me. For me. I don't know if I'm capable of it.
+04:10 Okay, thank you very much. I will try to do my best for this situation and. But how should I face the situation if they don't understand me? If they don't understand my point and they are not, we are not on the same line, how should I face it? What should I do.
+05:01 Okay, thank you very much. We will talk later.</t>
         </is>
       </c>
     </row>
@@ -1664,9 +2324,21 @@
       <c r="B81" t="n">
         <v>5</v>
       </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>00:06 Do I talk? Okay. In my mind today I want to find a job.  00:24 I'm looking for a job like an office job where I can work remotely but most importantly more like hybrid. Not necessarily 100% remotely, but that I'm working with people. Maybe helping them achieve their goals. Things such as organizational development or change management. People management consulting, related to people hr, but strategic, not necessarily operational. Yeah,.  00:58 Yeah.  01:11 I think I have had some experience because I was part of an organization that was going through a merger. Not the vote, more like an acquisition. And there was some sort of change management happening there, but not necessarily where I was like let's say leading the role of a change manager or learning and development or training or coaching. No, it was more like I was in the background of everything. So sort of.  02:09 I feel like I'm ready as long as the irrigation also gives me some guidance.  02:43 Yes,.  02:58 Any specific job openings in that area.  03:15 I think.  03:34 I think more fast paced because I feel like I'm always like changing and growing. But I think even if it's fast paced, I think it's important to have support in that.  04:13 Yeah, I think that. But also motorsport like Formula One.  04:27 No, I said Formula One.  04:42 Sure.  05:08 Sure.</t>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>00:06 Do I talk? Okay. In my mind today I want to find a job.
+00:24 I'm looking for a job like an office job where I can work remotely but most importantly more like hybrid. Not necessarily 100% remotely, but that I'm working with people. Maybe helping them achieve their goals. Things such as organizational development or change management. People management consulting, related to people hr, but strategic, not necessarily operational. Yeah,.
+00:58 Yeah.
+01:11 I think I have had some experience because I was part of an organization that was going through a merger. Not the vote, more like an acquisition. And there was some sort of change management happening there, but not necessarily where I was like let's say leading the role of a change manager or learning and development or training or coaching. No, it was more like I was in the background of everything. So sort of.
+02:09 I feel like I'm ready as long as the irrigation also gives me some guidance.
+02:43 Yes,.
+02:58 Any specific job openings in that area.
+03:15 I think.
+03:34 I think more fast paced because I feel like I'm always like changing and growing. But I think even if it's fast paced, I think it's important to have support in that.
+04:13 Yeah, I think that. But also motorsport like Formula One.
+04:27 No, I said Formula One.
+04:42 Sure.
+05:08 Sure.</t>
         </is>
       </c>
     </row>
@@ -1679,9 +2351,27 @@
       <c r="B82" t="n">
         <v>14023</v>
       </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>00:21 I'd like to talk about uni.  00:33 What do you do for a living?  00:51 Tell me a joke.  01:02 Tell me a joke.  01:18 That wasn't that funny.  01:30 How was your morning?  01:41 I was pretty tired, but now I'm alright.  01:58 No, but do you have any advice?  02:17 What should I be doing if I don't hear my clock in the morning?  02:38 What city is this behind you?  02:56 You don't really understand me, do you?  03:28 I recently had an argument with my roommate. What advice would you give me?  03:53 Okay, but what if my roommate always leaves her dishes in the kitchen behind and leaves the kitchen dirty and it really annoys me and I Told her many times. What advice would you give me?  04:23 But I was asking you about my roommate that she always leaves the place behind. Dirty. What is your advice I should do about it?  04:52 But we already have a cleaning schedule. But she just doesn't do it.  05:24 Okay. And what would the reward look like?  05:43 But what if I don't like her?  06:07 Okay. Do you have any idea what I should be cooking tonight?  06:31 Do you have the recipe for that?</t>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>00:21 I'd like to talk about uni.
+00:33 What do you do for a living?
+00:51 Tell me a joke.
+01:02 Tell me a joke.
+01:18 That wasn't that funny.
+01:30 How was your morning?
+01:41 I was pretty tired, but now I'm alright.
+01:58 No, but do you have any advice?
+02:17 What should I be doing if I don't hear my clock in the morning?
+02:38 What city is this behind you?
+02:56 You don't really understand me, do you?
+03:28 I recently had an argument with my roommate. What advice would you give me?
+03:53 Okay, but what if my roommate always leaves her dishes in the kitchen behind and leaves the kitchen dirty and it really annoys me and I Told her many times. What advice would you give me?
+04:23 But I was asking you about my roommate that she always leaves the place behind. Dirty. What is your advice I should do about it?
+04:52 But we already have a cleaning schedule. But she just doesn't do it.
+05:24 Okay. And what would the reward look like?
+05:43 But what if I don't like her?
+06:07 Okay. Do you have any idea what I should be cooking tonight?
+06:31 Do you have the recipe for that?</t>
         </is>
       </c>
     </row>
@@ -1694,9 +2384,24 @@
       <c r="B83" t="n">
         <v>14698</v>
       </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>00:21 What do you want to chat about?  00:54 Yeah. For example, yesterday I was on a party. It was really good with some friends. Yeah, that had been going on recently. And also the day before. I liked the finance class. I think it's quite interesting.  01:28 I don't know. At the party I like the most to just chill out with friends. Enjoying the music. Yeah, like this.  01:53 Not sure. Next week there's free time at the university. And also a friend of mine had a birthday party on Wednesday for probably. Yeah,.  02:25 No, like I say, to party. And also I need to study as well. Some more stuff for the exam soon, so need to learn.  02:49 Yeah.  02:53 No, just like the typical topics. Like the typical things? Yes, that's it. Like university stuff. But I have high expectations to myself, so I want to get a really good grade, hopefully.  03:30 Yeah, I think so. Hopefully.  03:47 Okay, what tips can you give me?  04:14 How long should I do the break?  04:34 Okay, and how long should I learn in one day before the exam sessions? Like,.  05:04 Okay, makes sense. So you think eight hours is a good average?  05:26 True. So what can you tell me about social experience?  05:58 Makes sense. So what kind of tips can you give me to improve my socializing? My networking?  06:38 Okay, I think that makes sense.  06:58 I think so. Hello. So.    Transcribed by https://fireflies.ai/</t>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>00:21 What do you want to chat about?
+00:54 Yeah. For example, yesterday I was on a party. It was really good with some friends. Yeah, that had been going on recently. And also the day before. I liked the finance class. I think it's quite interesting.
+01:28 I don't know. At the party I like the most to just chill out with friends. Enjoying the music. Yeah, like this.
+01:53 Not sure. Next week there's free time at the university. And also a friend of mine had a birthday party on Wednesday for probably. Yeah,.
+02:25 No, like I say, to party. And also I need to study as well. Some more stuff for the exam soon, so need to learn.
+02:49 Yeah.
+02:53 No, just like the typical topics. Like the typical things? Yes, that's it. Like university stuff. But I have high expectations to myself, so I want to get a really good grade, hopefully.
+03:30 Yeah, I think so. Hopefully.
+03:47 Okay, what tips can you give me?
+04:14 How long should I do the break?
+04:34 Okay, and how long should I learn in one day before the exam sessions? Like,.
+05:04 Okay, makes sense. So you think eight hours is a good average?
+05:26 True. So what can you tell me about social experience?
+05:58 Makes sense. So what kind of tips can you give me to improve my socializing? My networking?
+06:38 Okay, I think that makes sense.
+06:58 I think so. Hello. So.    Transcribed by https://fireflies.ai/</t>
         </is>
       </c>
     </row>
@@ -1709,9 +2414,18 @@
       <c r="B84" t="n">
         <v>14437</v>
       </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>00:11 Yeah, I'm just waiting if it's gonna work like that. Is it working? It should start talking to you, so. Hello? Oh, yeah, I'm supposed to talk about a difficult conversation I had, and just this night there was, like, some inconvenience happening for me, and everyone was, like, trying to help me, and that was a bit awkward for me.  00:55 Well, it looked like someone was, like, watching me through my window, and then all of my roommates were going crazy and, like, wanted to help me and, like, did so much that it was just a bit awkward because I didn't really, like, need to help. I mean, I appreciate their help, but it was just a bit awkward that they were, like, doing so much.  01:38 I'm feeling pretty good. I mean, yeah, it's just, like, still a bit awkward. I guess.  02:07 No, I guess it was just me because they were, like, nice and they. They did nothing wrong. It's just like, me, so.  02:32 Yeah, I guess I'm just gonna tell them how it made me feel and maybe how they overreacted a bit.  02:58 Do you have any advice for me?  03:25 Okay, well, maybe we can talk. Do you have any advice for me how I can handle, like, I have to do, like, team presentations, and my team is, like, doing pretty bad. Like, they're not doing anything. Do you have, like, advice for me for that,.  04:24 Yeah, well, I mean, they're not really doing anything. I mean, we have tasks assigned and they're just not like. I mean, they are doing their part at least, but they're doing it so poorly that I don't know what to tell them.  05:04 Okay, well, I guess I leave now.  05:35 There's.</t>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>00:11 Yeah, I'm just waiting if it's gonna work like that. Is it working? It should start talking to you, so. Hello? Oh, yeah, I'm supposed to talk about a difficult conversation I had, and just this night there was, like, some inconvenience happening for me, and everyone was, like, trying to help me, and that was a bit awkward for me.
+00:55 Well, it looked like someone was, like, watching me through my window, and then all of my roommates were going crazy and, like, wanted to help me and, like, did so much that it was just a bit awkward because I didn't really, like, need to help. I mean, I appreciate their help, but it was just a bit awkward that they were, like, doing so much.
+01:38 I'm feeling pretty good. I mean, yeah, it's just, like, still a bit awkward. I guess.
+02:07 No, I guess it was just me because they were, like, nice and they. They did nothing wrong. It's just like, me, so.
+02:32 Yeah, I guess I'm just gonna tell them how it made me feel and maybe how they overreacted a bit.
+02:58 Do you have any advice for me?
+03:25 Okay, well, maybe we can talk. Do you have any advice for me how I can handle, like, I have to do, like, team presentations, and my team is, like, doing pretty bad. Like, they're not doing anything. Do you have, like, advice for me for that,.
+04:24 Yeah, well, I mean, they're not really doing anything. I mean, we have tasks assigned and they're just not like. I mean, they are doing their part at least, but they're doing it so poorly that I don't know what to tell them.
+05:04 Okay, well, I guess I leave now.
+05:35 There's.</t>
         </is>
       </c>
     </row>
@@ -1724,9 +2438,17 @@
       <c r="B85" t="n">
         <v>14266</v>
       </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>00:19 I don't really know. Maybe a challenging situation for me with friends and family.  00:38 I mean, I live in a house with 12 other people here, and sometimes it gets really. It's really hard because everybody needs their personal space. But also, especially like in the kitchen, it's not always clean and some people like it cleaner and some, like it a little bit more. You know, I don't know how to say it.  01:20 We don't really, to be honest, we just leave it like that. And I mean, it's mostly that somebody gives in. Yeah,.  01:50 I mean, maybe, yeah, but I don't feel like all the people are willing to do that, you know, like, some don't really see any issues with that.  02:18 Well, yeah, that might be true. I will definitely take that into. I'll think about it. Definitely. Yeah.  02:44 I mean, there's not really much that I can. I can say now, to be honest,.  03:18 So can you maybe give me a few. A few advice how I could handle that? The problem? Sure.  04:00 Maybe that's. Yeah, that's actually a good idea. I will definitely talk to them about it. But what do If people are not willing to be part of the conversation?  04:38 All right. Thank you very much.</t>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>00:19 I don't really know. Maybe a challenging situation for me with friends and family.
+00:38 I mean, I live in a house with 12 other people here, and sometimes it gets really. It's really hard because everybody needs their personal space. But also, especially like in the kitchen, it's not always clean and some people like it cleaner and some, like it a little bit more. You know, I don't know how to say it.
+01:20 We don't really, to be honest, we just leave it like that. And I mean, it's mostly that somebody gives in. Yeah,.
+01:50 I mean, maybe, yeah, but I don't feel like all the people are willing to do that, you know, like, some don't really see any issues with that.
+02:18 Well, yeah, that might be true. I will definitely take that into. I'll think about it. Definitely. Yeah.
+02:44 I mean, there's not really much that I can. I can say now, to be honest,.
+03:18 So can you maybe give me a few. A few advice how I could handle that? The problem? Sure.
+04:00 Maybe that's. Yeah, that's actually a good idea. I will definitely talk to them about it. But what do If people are not willing to be part of the conversation?
+04:38 All right. Thank you very much.</t>
         </is>
       </c>
     </row>
@@ -1739,9 +2461,19 @@
       <c r="B86" t="n">
         <v>15079</v>
       </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>00:14 I'm here for a bonus point.  00:28 I have a problem with my roommate and she doesn't want to clean the dishes.  00:47 Not really. Like when I'm talking to her, I. She's not like really listening to me and she doesn't want to clean like every dishes that she use.  01:17 Yeah, sure. I'm done with that.  01:37 Yeah, it sounds great.  01:52 Yeah, sure. Let's do that.  02:13 Yeah, it sounds good. But I think that I hope she will listen to me.  02:35 Yeah, that's true.  02:54 Yep.  03:09 Yeah. Thank you. Bye.  03:28 Okay. Thanks.</t>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>00:14 I'm here for a bonus point.
+00:28 I have a problem with my roommate and she doesn't want to clean the dishes.
+00:47 Not really. Like when I'm talking to her, I. She's not like really listening to me and she doesn't want to clean like every dishes that she use.
+01:17 Yeah, sure. I'm done with that.
+01:37 Yeah, it sounds great.
+01:52 Yeah, sure. Let's do that.
+02:13 Yeah, it sounds good. But I think that I hope she will listen to me.
+02:35 Yeah, that's true.
+02:54 Yep.
+03:09 Yeah. Thank you. Bye.
+03:28 Okay. Thanks.</t>
         </is>
       </c>
     </row>
@@ -1754,9 +2486,13 @@
       <c r="B87" t="n">
         <v>14245</v>
       </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>2:14 PM thumb up thumb down show more actions Hey chat! I'd like to tell you about a recent challenging interaction I had yesterday.  2:14 PM My roomates...  2:15 PM Basically they keep leaving dirty dishes on the sink while the dishwasher is clean, instead of just taking the clean dishes out and putting the dirty ones in.  2:16 PM I did, and they reply I got was "it's probably because you wake up really early and then you see the dishwasher clean, because we put it during the night working, and then leave the extra dishes on the sink for the next load  2:18 PM I said that I waited on purpose for the next day to see if anyone would do anything about it, and I know some of them were home with time to do it, and it was still disgusting. The reply I got was a jokingly Ï'll wake up early to do the dishes then!</t>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>2:14 PM thumb up thumb down show more actions Hey chat! I'd like to tell you about a recent challenging interaction I had yesterday.
+2:14 PM My roomates...
+2:15 PM Basically they keep leaving dirty dishes on the sink while the dishwasher is clean, instead of just taking the clean dishes out and putting the dirty ones in.
+2:16 PM I did, and they reply I got was "it's probably because you wake up really early and then you see the dishwasher clean, because we put it during the night working, and then leave the extra dishes on the sink for the next load
+2:18 PM I said that I waited on purpose for the next day to see if anyone would do anything about it, and I know some of them were home with time to do it, and it was still disgusting. The reply I got was a jokingly Ï'll wake up early to do the dishes then!</t>
         </is>
       </c>
     </row>
@@ -1765,12 +2501,14 @@
       <c r="B88" t="n">
         <v>13333</v>
       </c>
+      <c r="C88" s="2" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="1" t="n"/>
       <c r="B89" t="n">
         <v>15088</v>
       </c>
+      <c r="C89" s="2" t="n"/>
     </row>
     <row r="90" ht="409.6" customHeight="1">
       <c r="A90" s="1" t="inlineStr">
@@ -1781,9 +2519,18 @@
       <c r="B90" t="n">
         <v>14710</v>
       </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>00:21 Anything you want.  00:37 Basically my hobbies have been the same my whole life. I've been playing tennis, just a lot of sports, basically. Also gym, go for runs, stuff like that. Basically that. How about you?  01:09 Yeah, very nice. Basically, I came here to talk to you about a conflict situation. Like with a conflict situation with other people.  01:33 No, like the task I came here for was just to talk about a conflict situation where I had to navigate. And that was when we had to book a table for a dinner reservation because my mom forgot that I had another appointment at that time. So I had to relocate and had to inform her and also the others, so they knew. And that was quite hard to navigate all of that.  02:20 Yeah, of course. We just scheduled it to later point so that we still had the dinner reservation, but I could have my appointment as well. And so we just ate at a later time. Yeah, that's basically.  02:52 Yeah, that's true. Did you have any like these in the last time?  03:23 Yeah, that's true. That's true.  03:38 No, not really. I mean, it's not that it wasn't that of a hard situation was basically. Okay, so it was not too hard to navigate, but yeah,.  04:09 Yeah, that's true.  04:26 No, it's fine. I think I talked about the most stuff I wanted to.</t>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>00:21 Anything you want.
+00:37 Basically my hobbies have been the same my whole life. I've been playing tennis, just a lot of sports, basically. Also gym, go for runs, stuff like that. Basically that. How about you?
+01:09 Yeah, very nice. Basically, I came here to talk to you about a conflict situation. Like with a conflict situation with other people.
+01:33 No, like the task I came here for was just to talk about a conflict situation where I had to navigate. And that was when we had to book a table for a dinner reservation because my mom forgot that I had another appointment at that time. So I had to relocate and had to inform her and also the others, so they knew. And that was quite hard to navigate all of that.
+02:20 Yeah, of course. We just scheduled it to later point so that we still had the dinner reservation, but I could have my appointment as well. And so we just ate at a later time. Yeah, that's basically.
+02:52 Yeah, that's true. Did you have any like these in the last time?
+03:23 Yeah, that's true. That's true.
+03:38 No, not really. I mean, it's not that it wasn't that of a hard situation was basically. Okay, so it was not too hard to navigate, but yeah,.
+04:09 Yeah, that's true.
+04:26 No, it's fine. I think I talked about the most stuff I wanted to.</t>
         </is>
       </c>
     </row>
@@ -1796,9 +2543,18 @@
       <c r="B91" t="n">
         <v>16475</v>
       </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>00:27 Nothing. I was just thinking about school and jokes. Funny jokes. What can you do? No. Maybe to hear one and maybe to see what you can do. Pretty interesting.  01:03 Good. Good one. Maybe some more humoristic ones.  01:22 Okay, what interesting stuff can you do other than jokes?  01:46 Well, you can describe what you see around me. And what's your impression?  02:13 Yeah. Can you tell me where you are? Like, is it a high rise building in a specific city or just in virtual reality?  02:41 Looks cool. Looks cool. Okay, We'll dive into how much knowledge you have behind you. Like what's your database? How does it look like?  03:29 Okay. Your responses maybe are too big, generic, sound like AI. Like yeah. Can you tell me more about that? And also like, how do you differ from other VR AI models?  04:19 And how would you know how I am feeling?  04:46 Okay, fair enough. And what do you think about the body language, about the conversation flow? What would you recommend to improve it and how do you see it? What can you see of this as a model?  05:22 Yeah, Should I stop the yeah, you can stop.     Transcribed by https://fireflies.ai/</t>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>00:27 Nothing. I was just thinking about school and jokes. Funny jokes. What can you do? No. Maybe to hear one and maybe to see what you can do. Pretty interesting.
+01:03 Good. Good one. Maybe some more humoristic ones.
+01:22 Okay, what interesting stuff can you do other than jokes?
+01:46 Well, you can describe what you see around me. And what's your impression?
+02:13 Yeah. Can you tell me where you are? Like, is it a high rise building in a specific city or just in virtual reality?
+02:41 Looks cool. Looks cool. Okay, We'll dive into how much knowledge you have behind you. Like what's your database? How does it look like?
+03:29 Okay. Your responses maybe are too big, generic, sound like AI. Like yeah. Can you tell me more about that? And also like, how do you differ from other VR AI models?
+04:19 And how would you know how I am feeling?
+04:46 Okay, fair enough. And what do you think about the body language, about the conversation flow? What would you recommend to improve it and how do you see it? What can you see of this as a model?
+05:22 Yeah, Should I stop the yeah, you can stop.     Transcribed by https://fireflies.ai/</t>
         </is>
       </c>
     </row>
@@ -1811,9 +2567,18 @@
       <c r="B92" t="n">
         <v>15199</v>
       </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>00:14 Hi, how are you? I'm Nicholas. I'm here to talk about a recent challenging experience I had.  00:32 I've been going through some challenges with a roommate of mine regarding cleaning the kitchen and other sharing areas.  00:57 Well, the main issue is that when he uses it, he doesn't clean afterwards. So he doesn't clean his pants. And the whole kitchen looks very messy after or is very messy and dirty after he used it. And he refuses to clean them after cooking. But I've told him that and still no reaction.  01:48 Well, we don't have a cleaning schedule, but I suggested that we just go by the basis that everyone cleans what he used. But we never really sat down. I just said to him on the fly, more or less that he has to clean up his stuff.  02:33 Yeah, you're right. Do you have any suggestions how I could get him to listen and understand?  03:18 Right? That sounds convenient to me. How's your day going so far?  03:40 Been great so far. I'm just a bit studying today, tomorrow as well. And on Wednesday I'm going home to see my parents again, so. Could have been worse, I guess.  04:11 No, nothing specific yet, but just some relaxing time. You know,.  04:29 Yeah, you're right. But what do you work exactly that you have this nice office.  04:53 All right. Cheers. See you next time.</t>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>00:14 Hi, how are you? I'm Nicholas. I'm here to talk about a recent challenging experience I had.
+00:32 I've been going through some challenges with a roommate of mine regarding cleaning the kitchen and other sharing areas.
+00:57 Well, the main issue is that when he uses it, he doesn't clean afterwards. So he doesn't clean his pants. And the whole kitchen looks very messy after or is very messy and dirty after he used it. And he refuses to clean them after cooking. But I've told him that and still no reaction.
+01:48 Well, we don't have a cleaning schedule, but I suggested that we just go by the basis that everyone cleans what he used. But we never really sat down. I just said to him on the fly, more or less that he has to clean up his stuff.
+02:33 Yeah, you're right. Do you have any suggestions how I could get him to listen and understand?
+03:18 Right? That sounds convenient to me. How's your day going so far?
+03:40 Been great so far. I'm just a bit studying today, tomorrow as well. And on Wednesday I'm going home to see my parents again, so. Could have been worse, I guess.
+04:11 No, nothing specific yet, but just some relaxing time. You know,.
+04:29 Yeah, you're right. But what do you work exactly that you have this nice office.
+04:53 All right. Cheers. See you next time.</t>
         </is>
       </c>
     </row>
@@ -1826,9 +2591,17 @@
       <c r="B93" t="n">
         <v>13</v>
       </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>00:18 Hi, Eduardo. I'm feeling sometimes, I guess struggling. I have a chronic condition. I have Crohn's disease. And hanging out with friends or going to uni and kind of having that. It's a bit of a struggle sometimes, you know.  00:58 I guess in the way maybe not. Some guidance. Maybe some ways that I can kind of help balance it out. I also have work as well sometimes. And I have to do work and sometimes it can get. It gets really tough and there are times when I feel really unwell, but there's no one to kind of fill in for me. And I have this pressure in my head that, oh, I need to go, even though I really feel bad about it. And the same goes to uni classes.  01:56 I get that. I get the only problem is my class is tutorless at the moment. And with work, I'm on a zero hour contract. Right. So it's not necessarily something that I can really choose when and where to go. And also social. I'm very much more introverted now and I spend more time at home.  02:50 Yeah, that's what I tried to do. It's what I tried to do at home. Spend time with my girlfriend. We chill out a lot, we rest a bit. And also try and be active. Right. Try and go to the gym recently, so that's definitely helping. I went for a couple blood tests recently as well that were. They went okay. A few. Few test scores weren't the best, but my doctor didn't call and they said that they would only call me if there was bad news. So I guess there's good news in that. But yeah, I still feel quite fatigued, you know. And every two weeks I have injections for my parents for the biology that I put into the mass of every two weeks. And on that day and the day after, I'm extremely dead.  04:11 Thank you, thank you. And facts. Yeah, it's good that the doctor didn't call, but yeah, I guess as well. What's good news is that my boss likes me so he's quite open to me to have the day off and he understands that's good. Only problem is I've got classes at 8:30 in the morning and that is an absolute pain. Like it is. It is in the morning. It's where I feel absolutely. Because I wake up, stomach's bloated and before I go out I need to go to the bathroom because I can only go to the bathroom in the house, you know what I mean? And yeah, so it's a bit of an issue as well. And yeah, it's just a lot of stress recently as well and stress.  04:54 The worst thing for me, I've got two courses left and then I've got my bachelor of them. But these are the two of the toughest courses. So it's a bit of a struggle.  05:36 Yeah, fair. But then again, I can't just be leeching for support. Right. Murder person. They're going through two masters right now. They're going through a premium program, they're going through other internships. They need support as well. And how to kind of balance all of that.  06:15 Yeah, yeah, that makes sense. That makes sense. Yeah. I think it's just sometimes it gets a bit tougher to do such things. Right. You can't always have that time, and sometimes you just. Yeah. You don't have the ability to be there for that interaction.  06:59 Yeah, yeah. It's very true. Very true. It's just a bit tough, you know? And the stress is the worst, man. It's the worst. And it's what hits the most.</t>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>00:18 Hi, Eduardo. I'm feeling sometimes, I guess struggling. I have a chronic condition. I have Crohn's disease. And hanging out with friends or going to uni and kind of having that. It's a bit of a struggle sometimes, you know.
+00:58 I guess in the way maybe not. Some guidance. Maybe some ways that I can kind of help balance it out. I also have work as well sometimes. And I have to do work and sometimes it can get. It gets really tough and there are times when I feel really unwell, but there's no one to kind of fill in for me. And I have this pressure in my head that, oh, I need to go, even though I really feel bad about it. And the same goes to uni classes.
+01:56 I get that. I get the only problem is my class is tutorless at the moment. And with work, I'm on a zero hour contract. Right. So it's not necessarily something that I can really choose when and where to go. And also social. I'm very much more introverted now and I spend more time at home.
+02:50 Yeah, that's what I tried to do. It's what I tried to do at home. Spend time with my girlfriend. We chill out a lot, we rest a bit. And also try and be active. Right. Try and go to the gym recently, so that's definitely helping. I went for a couple blood tests recently as well that were. They went okay. A few. Few test scores weren't the best, but my doctor didn't call and they said that they would only call me if there was bad news. So I guess there's good news in that. But yeah, I still feel quite fatigued, you know. And every two weeks I have injections for my parents for the biology that I put into the mass of every two weeks. And on that day and the day after, I'm extremely dead.
+04:11 Thank you, thank you. And facts. Yeah, it's good that the doctor didn't call, but yeah, I guess as well. What's good news is that my boss likes me so he's quite open to me to have the day off and he understands that's good. Only problem is I've got classes at 8:30 in the morning and that is an absolute pain. Like it is. It is in the morning. It's where I feel absolutely. Because I wake up, stomach's bloated and before I go out I need to go to the bathroom because I can only go to the bathroom in the house, you know what I mean? And yeah, so it's a bit of an issue as well. And yeah, it's just a lot of stress recently as well and stress.
+04:54 The worst thing for me, I've got two courses left and then I've got my bachelor of them. But these are the two of the toughest courses. So it's a bit of a struggle.
+05:36 Yeah, fair. But then again, I can't just be leeching for support. Right. Murder person. They're going through two masters right now. They're going through a premium program, they're going through other internships. They need support as well. And how to kind of balance all of that.
+06:15 Yeah, yeah, that makes sense. That makes sense. Yeah. I think it's just sometimes it gets a bit tougher to do such things. Right. You can't always have that time, and sometimes you just. Yeah. You don't have the ability to be there for that interaction.
+06:59 Yeah, yeah. It's very true. Very true. It's just a bit tough, you know? And the stress is the worst, man. It's the worst. And it's what hits the most.</t>
         </is>
       </c>
     </row>
@@ -1841,9 +2614,15 @@
       <c r="B94" t="n">
         <v>15211</v>
       </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>00:01 Enjoy it. Thank you. Hi, I would like to chat about a recently difficult situation.  00:28 So it's about me having a friend who I'm doing a group project with and it's just hard to communicate with her, especially because I don't know how to tell her that she has to contribute her part and not rely on me too much.  01:13 That sounds good. I tried to tell her or every time she asks me how are we gonna do this? And she's discussing her point with me, I'm trying to guide her in the right direction but it's quite difficult to tell her or like to actually bring across that I don't feel like she's doing enough. Especially because it's a new relationship, a new friendship. Still,.  02:02 Yes, I tried to guide her in another direction but it was just a bit one sided, especially because were talking about it and she was really asking me a lot about how I would do this or that. And I tried to tell her that's her responsibility or that's her part to participate in, but she kind of kept asking me about stuff and I tried to tell her do it however you want, but in the end I did the most, the biggest part and then everything she did, she double checked with me, which I like that we have a good communication and that we're working together closely and that she's my friend but it was kind of tough spots.  03:19 Yes, but I don't like that it has influence on our friendship and I don't actually know what specifically to do because she's just doing her part. I'm just doing my part. But in the end, it kind of felt off. And I feel like you can feel that in the relationship. Friendship.  04:05 That's a good idea, but. So what am I gonna do now?  04:45 Yes. That sounds nice. So, yeah, thank you.</t>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>00:01 Enjoy it. Thank you. Hi, I would like to chat about a recently difficult situation.
+00:28 So it's about me having a friend who I'm doing a group project with and it's just hard to communicate with her, especially because I don't know how to tell her that she has to contribute her part and not rely on me too much.
+01:13 That sounds good. I tried to tell her or every time she asks me how are we gonna do this? And she's discussing her point with me, I'm trying to guide her in the right direction but it's quite difficult to tell her or like to actually bring across that I don't feel like she's doing enough. Especially because it's a new relationship, a new friendship. Still,.
+02:02 Yes, I tried to guide her in another direction but it was just a bit one sided, especially because were talking about it and she was really asking me a lot about how I would do this or that. And I tried to tell her that's her responsibility or that's her part to participate in, but she kind of kept asking me about stuff and I tried to tell her do it however you want, but in the end I did the most, the biggest part and then everything she did, she double checked with me, which I like that we have a good communication and that we're working together closely and that she's my friend but it was kind of tough spots.
+03:19 Yes, but I don't like that it has influence on our friendship and I don't actually know what specifically to do because she's just doing her part. I'm just doing my part. But in the end, it kind of felt off. And I feel like you can feel that in the relationship. Friendship.
+04:05 That's a good idea, but. So what am I gonna do now?
+04:45 Yes. That sounds nice. So, yeah, thank you.</t>
         </is>
       </c>
     </row>
@@ -1856,9 +2635,17 @@
       <c r="B95" t="n">
         <v>13873</v>
       </c>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>00:14 Hello. I've actually recently encountered something with a friend that I kind of have some troubles with of how to. Like, it's a bad experience.  00:38 Yes, of course. So were actually at a festival, and were, like, deciding on what time we wanted to leave because I really wanted to see an artist, and, like, she didn't really want to. She was really tired, so she wanted to go home. But I was staying over at hers, so I kind of had to comply. But I also kind of got into an argument with her about, like, really wanting to see that artist, and I spent money to go see it, so I wanted to see it.  01:38 Yeah. All right. So maybe, like, talk about her feelings and try to understand her point of view.  02:07 Okay, but I still want to let her know that I really. It kind of hurt me that I couldn't see the artist, so how could I also tell her that, but, like, politely?  02:43 Yeah. So. All right, so maybe, like, next time, if we have this situation again, maybe make sure that beforehand we already have some rules clear, like, okay, until what time we're going to stay and stuff. Is that maybe a good idea?  03:15 All right, I like that idea. I guess maybe next time we would also have to, like, select the persons we like, artists we really want to see and stuff. And maybe also talk about the fact that, for example, the tickets this time cost €50. So that's, like, kind of relatively expensive for a festival. So were, like, maybe beforehand. Look at it.  04:01 Yeah, okay. I think that's a great idea. I guess next time we, like, have to make a better plan beforehand, and then if it diverges from that, it's fine, but. Yeah,.  04:31 Yeah, I think we'll have a great experience next time because I think I have a great plan now, and I will apologize to her.  04:54 Yeah, we had a nice time still, so I think next time will be even greater.</t>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>00:14 Hello. I've actually recently encountered something with a friend that I kind of have some troubles with of how to. Like, it's a bad experience.
+00:38 Yes, of course. So were actually at a festival, and were, like, deciding on what time we wanted to leave because I really wanted to see an artist, and, like, she didn't really want to. She was really tired, so she wanted to go home. But I was staying over at hers, so I kind of had to comply. But I also kind of got into an argument with her about, like, really wanting to see that artist, and I spent money to go see it, so I wanted to see it.
+01:38 Yeah. All right. So maybe, like, talk about her feelings and try to understand her point of view.
+02:07 Okay, but I still want to let her know that I really. It kind of hurt me that I couldn't see the artist, so how could I also tell her that, but, like, politely?
+02:43 Yeah. So. All right, so maybe, like, next time, if we have this situation again, maybe make sure that beforehand we already have some rules clear, like, okay, until what time we're going to stay and stuff. Is that maybe a good idea?
+03:15 All right, I like that idea. I guess maybe next time we would also have to, like, select the persons we like, artists we really want to see and stuff. And maybe also talk about the fact that, for example, the tickets this time cost €50. So that's, like, kind of relatively expensive for a festival. So were, like, maybe beforehand. Look at it.
+04:01 Yeah, okay. I think that's a great idea. I guess next time we, like, have to make a better plan beforehand, and then if it diverges from that, it's fine, but. Yeah,.
+04:31 Yeah, I think we'll have a great experience next time because I think I have a great plan now, and I will apologize to her.
+04:54 Yeah, we had a nice time still, so I think next time will be even greater.</t>
         </is>
       </c>
     </row>
@@ -1871,9 +2658,17 @@
       <c r="B96" t="n">
         <v>14272</v>
       </c>
-      <c r="C96" t="inlineStr">
-        <is>
-          <t>00:19 I would like to talk about a challenging experience. A recent challenging experience, of course, User,.  00:45 My grandparents are here right now to visit me and they want to keep seeing me. But I still have to do a lot of stuff for my university to keep up with my studies and I don't know how to tell them that I have to study.  01:24 Yes, that would be nice.  02:01 Yes. And how do I start the conversation?  02:39 Yes, that sounds good.  03:02 Yes,.  03:21 That's a good idea. Do you have any ideas what I can show them in Maastricht?  03:44 Thank you.  04:03 Yes,.</t>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>00:19 I would like to talk about a challenging experience. A recent challenging experience, of course, User,.
+00:45 My grandparents are here right now to visit me and they want to keep seeing me. But I still have to do a lot of stuff for my university to keep up with my studies and I don't know how to tell them that I have to study.
+01:24 Yes, that would be nice.
+02:01 Yes. And how do I start the conversation?
+02:39 Yes, that sounds good.
+03:02 Yes,.
+03:21 That's a good idea. Do you have any ideas what I can show them in Maastricht?
+03:44 Thank you.
+04:03 Yes,.</t>
         </is>
       </c>
     </row>
@@ -1886,9 +2681,17 @@
       <c r="B97" t="n">
         <v>19636</v>
       </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>00:29 Something challenging have been going on.  00:40 So I met a friend two days ago, and I haven't really spent a lot of time with her, and she's been very distant, and it's been very difficult for me to comprehend because I didn't have a lot of time to talk to her. So I don't know what to do.  01:12 Every time I ask her, she says everything is fine. But then also I wanted to. For example, I told her I can be there and we can meet up next week. But then she was like, yeah, I've got exams, so that's gonna be difficult. But then I'm gonna be in my hometown with her for five days, so I feel like, you know, it would. If she would like to put in the effort, I could be there.  02:02 So how do I do that? I've already asked her if we can meet up, but she already said she can't. So I'm not sure what I should do.  02:40 I don't really think she's that type of person. Who would like to hear that? Maybe. I don't know, maybe I should just, like, talk more with her in general and just, you know, maybe call her. I don't know. Like, I feel like she's been very distant. It could potentially be that there's something up but like I said, I already asked her, so I guess I'm just gonna wait what she replies on if we can meet one of the days. And yeah,.  03:38 Yeah, I feel like also on that matter it's kind of difficult to coordinate like being in mastrich and studying a lot to also catching up with people at home because I not that type of person who's a lot on their phone. So I feel like it's kind of difficult to comprehend like or to work with both of them at the same time.  04:27 Can you repeat that please?  04:52 All right, thank you very much. And how are you in general?  05:06 I think I got a bit more of a clear direction, so thanks for that.</t>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>00:29 Something challenging have been going on.
+00:40 So I met a friend two days ago, and I haven't really spent a lot of time with her, and she's been very distant, and it's been very difficult for me to comprehend because I didn't have a lot of time to talk to her. So I don't know what to do.
+01:12 Every time I ask her, she says everything is fine. But then also I wanted to. For example, I told her I can be there and we can meet up next week. But then she was like, yeah, I've got exams, so that's gonna be difficult. But then I'm gonna be in my hometown with her for five days, so I feel like, you know, it would. If she would like to put in the effort, I could be there.
+02:02 So how do I do that? I've already asked her if we can meet up, but she already said she can't. So I'm not sure what I should do.
+02:40 I don't really think she's that type of person. Who would like to hear that? Maybe. I don't know, maybe I should just, like, talk more with her in general and just, you know, maybe call her. I don't know. Like, I feel like she's been very distant. It could potentially be that there's something up but like I said, I already asked her, so I guess I'm just gonna wait what she replies on if we can meet one of the days. And yeah,.
+03:38 Yeah, I feel like also on that matter it's kind of difficult to coordinate like being in mastrich and studying a lot to also catching up with people at home because I not that type of person who's a lot on their phone. So I feel like it's kind of difficult to comprehend like or to work with both of them at the same time.
+04:27 Can you repeat that please?
+04:52 All right, thank you very much. And how are you in general?
+05:06 I think I got a bit more of a clear direction, so thanks for that.</t>
         </is>
       </c>
     </row>
@@ -1901,9 +2704,22 @@
       <c r="B98" t="n">
         <v>4</v>
       </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>00:12 I had a disagreement with my mother. It was about me going to a concert, and she didn't want to pay for it. What happened was I really wanted to go to that concert, and that artist is only going tour for one or two times before he changes his name. So I asked her pretty nicely to maybe if she wants to go with me to the concert, and with a little bit of nudging, I got her to go with me and we're going.  01:12 Yes, I'm really excited. We're going to meet him, so. Yeah. Yeah.  01:35 I mean, I'll probably fangirl a lot over him, but I just want to take a picture with him and. Yeah, just only, like, interact a little bit. And I'm very excited for his music.  02:05 Yes, I agree. Thank you.  02:26 Not really. I think.  02:41 Another thing, I am trying to go to a therapist, and my mom's pursuing me to go, but I feel like I don't want to do it because I don't want to speak to other people, to another person about my problems. So that's a bit of a tough situation.  03:17 I haven't, actually. I mean, I want a therapist who's very friendly and open, and I can easily talk to her. So that's what I'm, like, searching for right now. My friend recommended somebody, so hoping that she's good.  03:52 Yeah. So I will probably write therapist an email today to. To see if she has maybe, like, any spots for me to go.  04:15 Yeah. Thank you so much.  05:30 Do I need to reflect on this?  05:50 Overall, it was pretty great. He was nice and gave thoughtful advice.  06:08 No. I think what I answered was pretty correct and straight, so I think he did great.  06:31 No, I don't think so. Or maybe just like when he asked about meeting the artist itself. I think I didn't mention that I wanted to meet the artist. I just said that I'm really excited to see him.  07:00 I wasn't going to meet the artist itself. I was just saying that I was looking forward to seeing the artist as he was performing. Hello. So I need to.     Transcribed by https://fireflies.ai/</t>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>00:12 I had a disagreement with my mother. It was about me going to a concert, and she didn't want to pay for it. What happened was I really wanted to go to that concert, and that artist is only going tour for one or two times before he changes his name. So I asked her pretty nicely to maybe if she wants to go with me to the concert, and with a little bit of nudging, I got her to go with me and we're going.
+01:12 Yes, I'm really excited. We're going to meet him, so. Yeah. Yeah.
+01:35 I mean, I'll probably fangirl a lot over him, but I just want to take a picture with him and. Yeah, just only, like, interact a little bit. And I'm very excited for his music.
+02:05 Yes, I agree. Thank you.
+02:26 Not really. I think.
+02:41 Another thing, I am trying to go to a therapist, and my mom's pursuing me to go, but I feel like I don't want to do it because I don't want to speak to other people, to another person about my problems. So that's a bit of a tough situation.
+03:17 I haven't, actually. I mean, I want a therapist who's very friendly and open, and I can easily talk to her. So that's what I'm, like, searching for right now. My friend recommended somebody, so hoping that she's good.
+03:52 Yeah. So I will probably write therapist an email today to. To see if she has maybe, like, any spots for me to go.
+04:15 Yeah. Thank you so much.
+05:30 Do I need to reflect on this?
+05:50 Overall, it was pretty great. He was nice and gave thoughtful advice.
+06:08 No. I think what I answered was pretty correct and straight, so I think he did great.
+06:31 No, I don't think so. Or maybe just like when he asked about meeting the artist itself. I think I didn't mention that I wanted to meet the artist. I just said that I'm really excited to see him.
+07:00 I wasn't going to meet the artist itself. I was just saying that I was looking forward to seeing the artist as he was performing. Hello. So I need to.     Transcribed by https://fireflies.ai/</t>
         </is>
       </c>
     </row>
@@ -1916,9 +2732,14 @@
       <c r="B99" t="n">
         <v>14734</v>
       </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>10:03 AM hello how are you doing  10:03 AM i also fine, thank you. i would like to tell you something about a recent challenging interaction i had  10:04 AM so it was like a little discussionwith my football trainer. i recovered from a injury and wanted to play again, but he told me that i need some time which really disappointed me  10:05 AM yes. fter the training i went to him and tried to explain my point of view to him, that i was more than ready to play again and give my best for the team  10:07 AM he seemed understanding but also said that i still need some time so that players who werent injured also get the chance to play and show that they can also play a significant role in the team  10:08 AM objectively, i think so yes. subjectively, no. of course i want to play and that applies for everyone. we are one team but still there is sort of a competition when playing in a game from the start on</t>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>10:03 AM hello how are you doing
+10:03 AM i also fine, thank you. i would like to tell you something about a recent challenging interaction i had
+10:04 AM so it was like a little discussionwith my football trainer. i recovered from a injury and wanted to play again, but he told me that i need some time which really disappointed me
+10:05 AM yes. fter the training i went to him and tried to explain my point of view to him, that i was more than ready to play again and give my best for the team
+10:07 AM he seemed understanding but also said that i still need some time so that players who werent injured also get the chance to play and show that they can also play a significant role in the team
+10:08 AM objectively, i think so yes. subjectively, no. of course i want to play and that applies for everyone. we are one team but still there is sort of a competition when playing in a game from the start on</t>
         </is>
       </c>
     </row>
@@ -1931,9 +2752,16 @@
       <c r="B100" t="n">
         <v>14854</v>
       </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>9:35 AM oke nice to meet you, well im currently studying at maastricht.  9:35 AM Im studying something economics related, it doesn't really interest me though  9:36 AM I feel like the study is solely theory, which is not ideal. I like to learn by doing and seeing.  9:37 AM I agree im currently looking for internships, however i have failed my last course. Which made my parent a bit disappointed in me  9:38 AM Well i told them i failed, however i didn't even participate. You could say i lied to them  9:38 AM I didn't want them to stress about my school and my motivation  9:39 AM bro what divorce? they are not separated...  9:39 AM nothing, all good. my brother has middle school exams tho</t>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>9:35 AM oke nice to meet you, well im currently studying at maastricht.
+9:35 AM Im studying something economics related, it doesn't really interest me though
+9:36 AM I feel like the study is solely theory, which is not ideal. I like to learn by doing and seeing.
+9:37 AM I agree im currently looking for internships, however i have failed my last course. Which made my parent a bit disappointed in me
+9:38 AM Well i told them i failed, however i didn't even participate. You could say i lied to them
+9:38 AM I didn't want them to stress about my school and my motivation
+9:39 AM bro what divorce? they are not separated...
+9:39 AM nothing, all good. my brother has middle school exams tho</t>
         </is>
       </c>
     </row>
@@ -1946,9 +2774,16 @@
       <c r="B101" t="n">
         <v>16426</v>
       </c>
-      <c r="C101" t="inlineStr">
-        <is>
-          <t>9:29 AM I'd like to talk about a recent challenge i had  9:29 AM I missed a deadline for an apllication  9:30 AM procastination and I had the dealine a couple days to late in my notes  9:31 AM yes also wrote an e-mail. They accepted it still, but the aplliacation is not good at all now. Because I did it in 2 hours and had a whole month for it  9:31 AM yess  9:32 AM I hope so. Definetly on the short term  9:34 AM Nothing really. Im saying because it happend recently and I experienced how bad it feels it wont happen again soon (short-term). But I dont know if it will be a lasting effect  9:34 AM acting like my therapeut, dont know fam</t>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>9:29 AM I'd like to talk about a recent challenge i had
+9:29 AM I missed a deadline for an apllication
+9:30 AM procastination and I had the dealine a couple days to late in my notes
+9:31 AM yes also wrote an e-mail. They accepted it still, but the aplliacation is not good at all now. Because I did it in 2 hours and had a whole month for it
+9:31 AM yess
+9:32 AM I hope so. Definetly on the short term
+9:34 AM Nothing really. Im saying because it happend recently and I experienced how bad it feels it wont happen again soon (short-term). But I dont know if it will be a lasting effect
+9:34 AM acting like my therapeut, dont know fam</t>
         </is>
       </c>
     </row>
@@ -1961,9 +2796,17 @@
       <c r="B102" t="n">
         <v>14158</v>
       </c>
-      <c r="C102" t="inlineStr">
-        <is>
-          <t>10:20 AM no, I had troubling experience earlier this week  10:21 AM I was talking to my boss, because I was not happy with my salary and I wanted to give him a choice of either raising my salary or I would quit  10:22 AM I think I got my points across very well but based on hos reaction he was not very happy and no I am worried this will have consequences  10:22 AM I will follow through if he doesnt increase my pay  10:23 AM I am not prepared but i am fairly certain I wouldnt be jobless for too long  10:23 AM I am amazing  10:24 AM That I am in the bargaining position not my boss  10:25 AM i think so but my biggest worry is that he will make the last few weeks in case I do quit pretty hard  10:25 AM I am not sure about this</t>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>10:20 AM no, I had troubling experience earlier this week
+10:21 AM I was talking to my boss, because I was not happy with my salary and I wanted to give him a choice of either raising my salary or I would quit
+10:22 AM I think I got my points across very well but based on hos reaction he was not very happy and no I am worried this will have consequences
+10:22 AM I will follow through if he doesnt increase my pay
+10:23 AM I am not prepared but i am fairly certain I wouldnt be jobless for too long
+10:23 AM I am amazing
+10:24 AM That I am in the bargaining position not my boss
+10:25 AM i think so but my biggest worry is that he will make the last few weeks in case I do quit pretty hard
+10:25 AM I am not sure about this</t>
         </is>
       </c>
     </row>
@@ -1976,9 +2819,17 @@
       <c r="B103" t="n">
         <v>13507</v>
       </c>
-      <c r="C103" t="inlineStr">
-        <is>
-          <t>10:54 AM Yes well I have a little dilemma.  10:56 AM My housemate is really getting on my nerves. He is constantly slamming doors and goes in and out of his room what seems like a hundred times a day. The walls are thin so I can always hear this and because my room is next to his, my entire room shakes when he enters/exits his room.  10:57 AM No I haven't said anything. I feel like I should have said something in the beginning of the year because now it seems too late.  10:58 AM Yes you're right. Should I text him about it or speak to him personally?  10:58 AM Ok. What should I say?  10:59 AM Thanks. Ahh I find confrontation so tricky! I don't like complaining and don't want to make the situation worse.  10:59 AM What could the solution be?  11:00 AM Good idea.  11:00 AM Also a good one</t>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>10:54 AM Yes well I have a little dilemma.
+10:56 AM My housemate is really getting on my nerves. He is constantly slamming doors and goes in and out of his room what seems like a hundred times a day. The walls are thin so I can always hear this and because my room is next to his, my entire room shakes when he enters/exits his room.
+10:57 AM No I haven't said anything. I feel like I should have said something in the beginning of the year because now it seems too late.
+10:58 AM Yes you're right. Should I text him about it or speak to him personally?
+10:58 AM Ok. What should I say?
+10:59 AM Thanks. Ahh I find confrontation so tricky! I don't like complaining and don't want to make the situation worse.
+10:59 AM What could the solution be?
+11:00 AM Good idea.
+11:00 AM Also a good one</t>
         </is>
       </c>
     </row>
@@ -1991,9 +2842,13 @@
       <c r="B104" t="n">
         <v>13444</v>
       </c>
-      <c r="C104" t="inlineStr">
-        <is>
-          <t>11:07 AM Id like to tell you about a difficult situation i had  11:09 AM indeed, i have a friend that doesnt want to talk to me anymore, i met him in one of my tutorials \  11:09 AM yes, i think so. We started kind of getting into a relationship but i was never decisive on what i wanted  11:10 AM yes, and i actually told him id rather be friends since i really enjoy spending time with him, he said he understood but i think we never settled limits and the frienship was difficult to achieve  11:11 AM yes, i always knew he liked me so maybe should have never let the friendship develop into something romantic</t>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>11:07 AM Id like to tell you about a difficult situation i had
+11:09 AM indeed, i have a friend that doesnt want to talk to me anymore, i met him in one of my tutorials \
+11:09 AM yes, i think so. We started kind of getting into a relationship but i was never decisive on what i wanted
+11:10 AM yes, and i actually told him id rather be friends since i really enjoy spending time with him, he said he understood but i think we never settled limits and the frienship was difficult to achieve
+11:11 AM yes, i always knew he liked me so maybe should have never let the friendship develop into something romantic</t>
         </is>
       </c>
     </row>
@@ -2006,9 +2861,15 @@
       <c r="B105" t="n">
         <v>13783</v>
       </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t>11:56 AM Hi i would like to tell you about a challenging siutation i had with my tutorial group in university  11:57 AM yeah we have a group assignement since the start of the period so we already got the assignemtn 4 weks ago  11:57 AM yeah its some time but i personallz had a lot of other stuff to do.  11:59 AM the problem is that i wasnt in maastricht every weekenf since the start of the period so i couldnt contribute yet. and now we have a midterm updagte presentation today  12:00 PM there is one guy who does everything wiht AI so he also doesnt do a lot and his work is pretty bad. then there is one girls she organises everything she is good. and one girl that just does the job suffiecientlt  12:01 PM we basically all know what we have to do. but i feel like im nott prepared enough. or at least not at the level i would normally like to  12:02 PM that i didnt read the chapters we had to read until today. i just know the task and the asnwes from chat gpt but not the logic behind it</t>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>11:56 AM Hi i would like to tell you about a challenging siutation i had with my tutorial group in university
+11:57 AM yeah we have a group assignement since the start of the period so we already got the assignemtn 4 weks ago
+11:57 AM yeah its some time but i personallz had a lot of other stuff to do.
+11:59 AM the problem is that i wasnt in maastricht every weekenf since the start of the period so i couldnt contribute yet. and now we have a midterm updagte presentation today
+12:00 PM there is one guy who does everything wiht AI so he also doesnt do a lot and his work is pretty bad. then there is one girls she organises everything she is good. and one girl that just does the job suffiecientlt
+12:01 PM we basically all know what we have to do. but i feel like im nott prepared enough. or at least not at the level i would normally like to
+12:02 PM that i didnt read the chapters we had to read until today. i just know the task and the asnwes from chat gpt but not the logic behind it</t>
         </is>
       </c>
     </row>
@@ -2021,9 +2882,22 @@
       <c r="B106" t="n">
         <v>14293</v>
       </c>
-      <c r="C106" t="inlineStr">
-        <is>
-          <t>11:23 AM i would like to tell you about a recent challenging interation i had  11:23 AM personal life  11:24 AM it was during the break  11:24 AM no, i had to pass my driver's license, it was a horrible moment  11:25 AM i had already failed it the first time so i was super stressed and the guide was very rude  11:26 AM yes of course, i was shaking so much  11:26 AM yes, i took a deep breath and did my best but i was still shaking  11:27 AM yes i did!  11:27 AM yes, do you have any advices on road?  11:28 AM ok, any advice for managing stress?  11:28 AM just chilling, eating a snak  11:29 AM salty snacks  11:29 AM yes  11:30 AM yeah,my living room or bedroom</t>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>11:23 AM i would like to tell you about a recent challenging interation i had
+11:23 AM personal life
+11:24 AM it was during the break
+11:24 AM no, i had to pass my driver's license, it was a horrible moment
+11:25 AM i had already failed it the first time so i was super stressed and the guide was very rude
+11:26 AM yes of course, i was shaking so much
+11:26 AM yes, i took a deep breath and did my best but i was still shaking
+11:27 AM yes i did!
+11:27 AM yes, do you have any advices on road?
+11:28 AM ok, any advice for managing stress?
+11:28 AM just chilling, eating a snak
+11:29 AM salty snacks
+11:29 AM yes
+11:30 AM yeah,my living room or bedroom</t>
         </is>
       </c>
     </row>
@@ -2036,9 +2910,15 @@
       <c r="B107" t="n">
         <v>13627</v>
       </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>11:37 AM hey, yes its just been quite stresssful the last few weeks  11:38 AM oh its been a mix of covering uni stuff with family meetings in other cities and visiting my boyfriend  11:40 AM yes it has been quite a busy schedule trying to cover everything at the same time. with my boyfriend everything has been going good  11:41 AM yes, he is been supportive. its more about that im stressing a bit to cover everything at the same time without letting anyone behind. the issue is not about my boyfriend  11:43 AM no nothing specific. i just feel like the day doesn"t have enough hours to cover everything, especially when i have to include all the travel time with delays  11:44 AM on what would you put the focus?  11:44 AM interesting idea what about friends?</t>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>11:37 AM hey, yes its just been quite stresssful the last few weeks
+11:38 AM oh its been a mix of covering uni stuff with family meetings in other cities and visiting my boyfriend
+11:40 AM yes it has been quite a busy schedule trying to cover everything at the same time. with my boyfriend everything has been going good
+11:41 AM yes, he is been supportive. its more about that im stressing a bit to cover everything at the same time without letting anyone behind. the issue is not about my boyfriend
+11:43 AM no nothing specific. i just feel like the day doesn"t have enough hours to cover everything, especially when i have to include all the travel time with delays
+11:44 AM on what would you put the focus?
+11:44 AM interesting idea what about friends?</t>
         </is>
       </c>
     </row>
@@ -2051,9 +2931,14 @@
       <c r="B108" t="n">
         <v>14152</v>
       </c>
-      <c r="C108" t="inlineStr">
-        <is>
-          <t>11:58 AM HI! My name is Vasilena! I would love to have a chat with you about a recent tough experience I had with a friend/  12:01 PM Okay, so here's the situation. I am in a group with 2 other girls and they both work on the weekends. But one of them had a free day and proposed going on a day trip in the Netherlands. Ive never been in another city here so I immediately accepted. However, my other friend got mad at me for taking the opportunity without her and didnt talk to me. I even proposed going to Rotterdam where she has been before in order to not make her feel bad for not coming. But she still didnt talk to me for several days. Do you think I did something bad?  12:03 PM She just gave me the silent treatment and after 2-3 days acted like nothing had happened. I tried talking to her but she was ignoring me so I also stayed silent. Afterwards, she also got mad at me for being mad at her that she didnt even want to talk about the problem so we could resolve it.  12:04 PM I guess, she has always said that she could get possessive of her close ones and jealous and I always try to deal with that in a gentle matter but its so exhausting sometimes...  12:05 PM I do feel that I don't know how close I want to keep that friendship. I mean we're adults, I can't deal with childish behaviour like that.  12:06 PM Yes, she said she knows her actions are wrong and she is trying to deal with her behaviour but I dont see any progress from her.</t>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>11:58 AM HI! My name is Vasilena! I would love to have a chat with you about a recent tough experience I had with a friend/
+12:01 PM Okay, so here's the situation. I am in a group with 2 other girls and they both work on the weekends. But one of them had a free day and proposed going on a day trip in the Netherlands. Ive never been in another city here so I immediately accepted. However, my other friend got mad at me for taking the opportunity without her and didnt talk to me. I even proposed going to Rotterdam where she has been before in order to not make her feel bad for not coming. But she still didnt talk to me for several days. Do you think I did something bad?
+12:03 PM She just gave me the silent treatment and after 2-3 days acted like nothing had happened. I tried talking to her but she was ignoring me so I also stayed silent. Afterwards, she also got mad at me for being mad at her that she didnt even want to talk about the problem so we could resolve it.
+12:04 PM I guess, she has always said that she could get possessive of her close ones and jealous and I always try to deal with that in a gentle matter but its so exhausting sometimes...
+12:05 PM I do feel that I don't know how close I want to keep that friendship. I mean we're adults, I can't deal with childish behaviour like that.
+12:06 PM Yes, she said she knows her actions are wrong and she is trying to deal with her behaviour but I dont see any progress from her.</t>
         </is>
       </c>
     </row>
@@ -2066,9 +2951,16 @@
       <c r="B109" t="n">
         <v>13351</v>
       </c>
-      <c r="C109" t="inlineStr">
-        <is>
-          <t>12:23 PM Well, I have a teammember in my supply chain course and I feel like he does not take me seriously....  12:25 PM Well, it is more that when I say something he kinda ignores it but when my male teammember says something he immidiatly listens or at least takes it into account, which is very frustrating, I feel like he does that because of my gender, being a female  12:27 PM I have seen numerous moments, for instance, we decided upon a company that I brought up but then he insisted on his company, the third male coworker was silent during this. or when I had a slides deck already made in canva, he insisted on powerpoint until the third coworker said that he liked canva.  12:28 PM No, but should I? I feel like it is not his problem and this feeling is not neceserally objectively confirmed  12:28 PM wouldnt he get irritated tho, like would the atmosphere not get worse  12:29 PM and what if it al plays out bad?  12:29 PM but I am stuck with this group until the end of the semester  12:30 PM maybe I shoulf</t>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>12:23 PM Well, I have a teammember in my supply chain course and I feel like he does not take me seriously....
+12:25 PM Well, it is more that when I say something he kinda ignores it but when my male teammember says something he immidiatly listens or at least takes it into account, which is very frustrating, I feel like he does that because of my gender, being a female
+12:27 PM I have seen numerous moments, for instance, we decided upon a company that I brought up but then he insisted on his company, the third male coworker was silent during this. or when I had a slides deck already made in canva, he insisted on powerpoint until the third coworker said that he liked canva.
+12:28 PM No, but should I? I feel like it is not his problem and this feeling is not neceserally objectively confirmed
+12:28 PM wouldnt he get irritated tho, like would the atmosphere not get worse
+12:29 PM and what if it al plays out bad?
+12:29 PM but I am stuck with this group until the end of the semester
+12:30 PM maybe I shoulf</t>
         </is>
       </c>
     </row>
@@ -2081,9 +2973,12 @@
       <c r="B110" t="n">
         <v>13528</v>
       </c>
-      <c r="C110" t="inlineStr">
-        <is>
-          <t>12:11 PM I would like to tell you about a recent challenging interaction I had. I was selling something on Vinted and the customer cancelled their order leaving me with an unsold product  12:12 PM It was quite unexpected with weak reasoning. the problem itself is fairly little. Pretty much a non problem if you will. still it is annoying as now I have to revisit the selling process which is a bit annoying  12:13 PM Yeah I am relisting it right away. no Interest in keeping the article. As I mentioned the inconvenience has little negative impact on me  12:14 PM yeah its not used by me. Could get money out of it. So I figure why not sell it right away.</t>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>12:11 PM I would like to tell you about a recent challenging interaction I had. I was selling something on Vinted and the customer cancelled their order leaving me with an unsold product
+12:12 PM It was quite unexpected with weak reasoning. the problem itself is fairly little. Pretty much a non problem if you will. still it is annoying as now I have to revisit the selling process which is a bit annoying
+12:13 PM Yeah I am relisting it right away. no Interest in keeping the article. As I mentioned the inconvenience has little negative impact on me
+12:14 PM yeah its not used by me. Could get money out of it. So I figure why not sell it right away.</t>
         </is>
       </c>
     </row>
@@ -2096,9 +2991,16 @@
       <c r="B111" t="n">
         <v>14722</v>
       </c>
-      <c r="C111" t="inlineStr">
-        <is>
-          <t>12:42 PM yes im doing okey  12:43 PM yes everything is going good im a little behind with my studies but ill try to finish it asap  12:43 PM no just in general with the work load  12:44 PM yes to spend more tome and also be more efficient when im at the libary  12:45 PM dont please people just because it feels better going ith them and also make my own plan and knowing what times im best at beeing productive  12:47 PM i think in general keepung up with the workload helps to hve more time and prioitize my scedual. and also be able to have time to meet up with my group  12:48 PM no i think its not that bad but just something i have notiuced in the past that might help  12:48 PM not yet but im working on it</t>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>12:42 PM yes im doing okey
+12:43 PM yes everything is going good im a little behind with my studies but ill try to finish it asap
+12:43 PM no just in general with the work load
+12:44 PM yes to spend more tome and also be more efficient when im at the libary
+12:45 PM dont please people just because it feels better going ith them and also make my own plan and knowing what times im best at beeing productive
+12:47 PM i think in general keepung up with the workload helps to hve more time and prioitize my scedual. and also be able to have time to meet up with my group
+12:48 PM no i think its not that bad but just something i have notiuced in the past that might help
+12:48 PM not yet but im working on it</t>
         </is>
       </c>
     </row>
@@ -2111,9 +3013,17 @@
       <c r="B112" t="n">
         <v>14770</v>
       </c>
-      <c r="C112" t="inlineStr">
-        <is>
-          <t>3:00 PM hi, zes so i had a recent challanging interaction i would love to talk about  3:02 PM so it's about a disagreement with one of my tutors, they hd the opinion, that our presentation wasn't what was asked for and i disagree, especially since i had a conversation with her prior to the presentation about the requirements, but in her feedback she ignored that \  3:04 PM i addressed it, but she seemed to have changed her opinion and now mz grade refelcts her indesicion and i feel weird bringing it up again, especially since we had a good tutorial group and we are discouraged to talk with our tutors about our grade after submission and now i don't see her anymore\  3:04 PM yes so what now  3:05 PM i don't know if i feel comfortable with that  3:06 PM yes and furthermore, i don't know if it would help or rather make me look stupid  3:06 PM so what should i do?  3:06 PM okay  3:06 PM thank zou</t>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>3:00 PM hi, zes so i had a recent challanging interaction i would love to talk about
+3:02 PM so it's about a disagreement with one of my tutors, they hd the opinion, that our presentation wasn't what was asked for and i disagree, especially since i had a conversation with her prior to the presentation about the requirements, but in her feedback she ignored that \
+3:04 PM i addressed it, but she seemed to have changed her opinion and now mz grade refelcts her indesicion and i feel weird bringing it up again, especially since we had a good tutorial group and we are discouraged to talk with our tutors about our grade after submission and now i don't see her anymore\
+3:04 PM yes so what now
+3:05 PM i don't know if i feel comfortable with that
+3:06 PM yes and furthermore, i don't know if it would help or rather make me look stupid
+3:06 PM so what should i do?
+3:06 PM okay
+3:06 PM thank zou</t>
         </is>
       </c>
     </row>
@@ -2126,9 +3036,20 @@
       <c r="B113" t="n">
         <v>10</v>
       </c>
-      <c r="C113" t="inlineStr">
-        <is>
-          <t>3:30 PM yeah everything is great!  3:31 PM today has been a productive work day  3:31 PM yeah i had some feedback from my thesis supervisor which i was procastinating a lot with and i finally got to it today  3:32 PM yes yes i did  3:32 PM it was but i still needed to figure out a lot on my own  3:34 PM some of the feedback was really helpful but some needed me to go back and do a lot more research which was quite time-consuming and stressful, and the thesis submission is coming close so i maybe hoped he gave this feedback early on  3:35 PM yes i did but he said that these are challenges that comes for every masters student and time-management is a key skill here which i need to work on  3:35 PM yes i spoke to him and we made a revised schedule which i need to closely follow from now on  3:36 PM yes, i am  3:36 PM I will work on writing everyday for a few hours and a few hours only for research and keep updating my supervisor with my work  3:37 PM i plan to have a chat with him every week  3:37 PM just more on how is my writing style and if my content is answering the research question</t>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t>3:30 PM yeah everything is great!
+3:31 PM today has been a productive work day
+3:31 PM yeah i had some feedback from my thesis supervisor which i was procastinating a lot with and i finally got to it today
+3:32 PM yes yes i did
+3:32 PM it was but i still needed to figure out a lot on my own
+3:34 PM some of the feedback was really helpful but some needed me to go back and do a lot more research which was quite time-consuming and stressful, and the thesis submission is coming close so i maybe hoped he gave this feedback early on
+3:35 PM yes i did but he said that these are challenges that comes for every masters student and time-management is a key skill here which i need to work on
+3:35 PM yes i spoke to him and we made a revised schedule which i need to closely follow from now on
+3:36 PM yes, i am
+3:36 PM I will work on writing everyday for a few hours and a few hours only for research and keep updating my supervisor with my work
+3:37 PM i plan to have a chat with him every week
+3:37 PM just more on how is my writing style and if my content is answering the research question</t>
         </is>
       </c>
     </row>
@@ -2141,9 +3062,13 @@
       <c r="B114" t="n">
         <v>14182</v>
       </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>3:44 PM hi, i wpuld like to tell you about a recent challenging interaction i had  3:47 PM i started my studies here last september and got close with a really nice girl. we had great time for five months but then she moved to another street and meet a new girl that she got really close. i felt like the third wheel in every conversation and she even called the other girl her best friend in front of me which reall hurt my feelings. now im moving to her street as well and i hope it gets better but are there any tips yu have for me  3:48 PM i thing that might makes thing akward especially because now it gets better. but i have to work on my self confidence to put myself firts because i also compare myself a lot to the other girl in termns of grades or realionshiop because she is just better and i never feel greta ariund her  3:50 PM i think its just her achievments but im happy with my grades because im alswyas doing my best and really stress about grades to a point where it gets unhelathy so i have to stop comparing myself to her nad start being myself again. do you have any tips how i get my spark back?  3:51 PM yes tahnk you so much for your help</t>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>3:44 PM hi, i wpuld like to tell you about a recent challenging interaction i had
+3:47 PM i started my studies here last september and got close with a really nice girl. we had great time for five months but then she moved to another street and meet a new girl that she got really close. i felt like the third wheel in every conversation and she even called the other girl her best friend in front of me which reall hurt my feelings. now im moving to her street as well and i hope it gets better but are there any tips yu have for me
+3:48 PM i thing that might makes thing akward especially because now it gets better. but i have to work on my self confidence to put myself firts because i also compare myself a lot to the other girl in termns of grades or realionshiop because she is just better and i never feel greta ariund her
+3:50 PM i think its just her achievments but im happy with my grades because im alswyas doing my best and really stress about grades to a point where it gets unhelathy so i have to stop comparing myself to her nad start being myself again. do you have any tips how i get my spark back?
+3:51 PM yes tahnk you so much for your help</t>
         </is>
       </c>
     </row>
@@ -2156,9 +3081,18 @@
       <c r="B115" t="n">
         <v>14974</v>
       </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>3:58 PM no, i recently had a fight with my mom  3:58 PM i think we were both stressed that day and got triggered from each other  3:59 PM no, because i refuse to be the first to initiate  4:00 PM because it is impossible to have a serious talk about her as she doesnt reinforce anything i am saying as well as i want to be approached and appolagesed to first especially in this case  4:01 PM yes a sincire apolagy and a good conversation about her actions  4:02 PM her intanarlising what she is saying. and just making sure it wont happen again  4:02 PM yes  4:03 PM i would talk to her again. we have spent time apart since it happened  4:04 PM yes and no. because i still belive i am in the right and i know i am  4:04 PM yes but sometimes you need to stand your ground</t>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t>3:58 PM no, i recently had a fight with my mom
+3:58 PM i think we were both stressed that day and got triggered from each other
+3:59 PM no, because i refuse to be the first to initiate
+4:00 PM because it is impossible to have a serious talk about her as she doesnt reinforce anything i am saying as well as i want to be approached and appolagesed to first especially in this case
+4:01 PM yes a sincire apolagy and a good conversation about her actions
+4:02 PM her intanarlising what she is saying. and just making sure it wont happen again
+4:02 PM yes
+4:03 PM i would talk to her again. we have spent time apart since it happened
+4:04 PM yes and no. because i still belive i am in the right and i know i am
+4:04 PM yes but sometimes you need to stand your ground</t>
         </is>
       </c>
     </row>
@@ -2171,9 +3105,18 @@
       <c r="B116" t="n">
         <v>13297</v>
       </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>4:23 PM Hey how you doing?  4:24 PM its been going alright, ive been really stressed and worn out lately, how about you?  4:25 PM its mostly a combination of everything. i dont feel well mentally and physically, i havent been to the gym in so long and i feel overpressured academically and also with everything else in my life and my personal goals. im not where i want to be at all  4:27 PM i cant get things together, im always behind and procrastinate a lot in uni and i also moved recently and hat a lot of stress about that. and i went out with friends almost every day its just so much. im also so sleep deprived, my schedule is fucked up im awake until 5 or 6 am and sleep the whole day and sometimes i stay in bed all day. i just need the whole world to freeze and go to an isolated island for one week where i catch up with myself and rest all day  4:27 PM OK  4:28 PM sometimes  4:28 PM depends if im actually productive or not  4:29 PM i just need some time for myself to catch up with everything and get my stuff together  4:29 PM what does that mean relating to my concerns  4:29 PM no thank you</t>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>4:23 PM Hey how you doing?
+4:24 PM its been going alright, ive been really stressed and worn out lately, how about you?
+4:25 PM its mostly a combination of everything. i dont feel well mentally and physically, i havent been to the gym in so long and i feel overpressured academically and also with everything else in my life and my personal goals. im not where i want to be at all
+4:27 PM i cant get things together, im always behind and procrastinate a lot in uni and i also moved recently and hat a lot of stress about that. and i went out with friends almost every day its just so much. im also so sleep deprived, my schedule is fucked up im awake until 5 or 6 am and sleep the whole day and sometimes i stay in bed all day. i just need the whole world to freeze and go to an isolated island for one week where i catch up with myself and rest all day
+4:27 PM OK
+4:28 PM sometimes
+4:28 PM depends if im actually productive or not
+4:29 PM i just need some time for myself to catch up with everything and get my stuff together
+4:29 PM what does that mean relating to my concerns
+4:29 PM no thank you</t>
         </is>
       </c>
     </row>
@@ -2186,9 +3129,16 @@
       <c r="B117" t="n">
         <v>12</v>
       </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>4:45 PM Yes im okay but kinda was struggling yesterday and i want to talk to you about this challenging interaction i had  4:46 PM so im in a project with 5 members inlcuding me. i at one point approached one of my teammates because they were not really taking iniative or responding in the groupchat, and i was directly in contact with her due to overlapping tasks, and she lacke input or just didnt do anything, i appraoched her in agreement with the 3 other students  4:47 PM i mean im not a confronting person and she said she had been working on it but the deadline already passed, and because i couldnt be too direct as i foudn this approach difficult i thought it was not really clocking to them. but yeasterday sehe mentioned i was bossy and had an attitue which was not the case  4:48 PM yes defenitely caught me off guard i mean she texted a whole paragrah (generated by ai) and all of my teammates backed me up, (i also by agreement of the team and spoke as the team regarding ai use, and during that meeting she got defensive and said WHAT ARE YOU IMPYING??  4:49 PM I MEAN i think she got defensive as i accused her of using ai, and she did, bc why else would you have such reaction, but now im kinda stressed and not feeling well,bc idk scared of her telling our mentor, coaches blabla, but yeah  4:50 PM i mean if she escalates it i would say to all the people she told this, to read our midterm evaluation feedback, as i addressed it already there just like all my other teammates but our coahces and mentor did not say anything about this  4:51 PM true but i think she pictured me bad then, this is waht im afraid of, even though the team got me  4:52 PM i mean i have evidence right the feedback forms, but it doesnt take away my stress currently</t>
+      <c r="C117" s="2" t="inlineStr">
+        <is>
+          <t>4:45 PM Yes im okay but kinda was struggling yesterday and i want to talk to you about this challenging interaction i had
+4:46 PM so im in a project with 5 members inlcuding me. i at one point approached one of my teammates because they were not really taking iniative or responding in the groupchat, and i was directly in contact with her due to overlapping tasks, and she lacke input or just didnt do anything, i appraoched her in agreement with the 3 other students
+4:47 PM i mean im not a confronting person and she said she had been working on it but the deadline already passed, and because i couldnt be too direct as i foudn this approach difficult i thought it was not really clocking to them. but yeasterday sehe mentioned i was bossy and had an attitue which was not the case
+4:48 PM yes defenitely caught me off guard i mean she texted a whole paragrah (generated by ai) and all of my teammates backed me up, (i also by agreement of the team and spoke as the team regarding ai use, and during that meeting she got defensive and said WHAT ARE YOU IMPYING??
+4:49 PM I MEAN i think she got defensive as i accused her of using ai, and she did, bc why else would you have such reaction, but now im kinda stressed and not feeling well,bc idk scared of her telling our mentor, coaches blabla, but yeah
+4:50 PM i mean if she escalates it i would say to all the people she told this, to read our midterm evaluation feedback, as i addressed it already there just like all my other teammates but our coahces and mentor did not say anything about this
+4:51 PM true but i think she pictured me bad then, this is waht im afraid of, even though the team got me
+4:52 PM i mean i have evidence right the feedback forms, but it doesnt take away my stress currently</t>
         </is>
       </c>
     </row>
@@ -2201,9 +3151,12 @@
       <c r="B118" t="n">
         <v>15082</v>
       </c>
-      <c r="C118" t="inlineStr">
-        <is>
-          <t>9:43 AM I'd like to talk about a recent challenging interaction I had  9:45 AM For the course Finance we have to make a group presentation, but my group isn`t the most interactive. For example we had to do a short 5 minute presentation about our progress, and my group didn`t really wanted to do anything.  9:46 AM no I ended up doing it myself  9:47 AM it was just a small 5 minute presentation, so it was pretty short to prepare</t>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>9:43 AM I'd like to talk about a recent challenging interaction I had
+9:45 AM For the course Finance we have to make a group presentation, but my group isn`t the most interactive. For example we had to do a short 5 minute presentation about our progress, and my group didn`t really wanted to do anything.
+9:46 AM no I ended up doing it myself
+9:47 AM it was just a small 5 minute presentation, so it was pretty short to prepare</t>
         </is>
       </c>
     </row>
@@ -2216,9 +3169,18 @@
       <c r="B119" t="n">
         <v>13819</v>
       </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>12:37 PM Hi i have a problem with my current roommates in my shared apartment  12:38 PM The issue is that they are a bit dirty and do not clean the kitchen after they cook  12:38 PM i mean i asked them nicely after they had friends over if they could store at least the food back in the fridge  12:39 PM they apologized to me and they kept cleaning a bit more for ca 2 weeks than the same incident happened again  12:40 PM so what should i do now  12:40 PM and what should i tell them in the conversation more specifically  12:41 PM do you think that a chore chart could help  12:42 PM not really we all talked about how to feel comfortable in our home but never wrote down chores  12:43 PM I am not sure I would maybe feel to much like the decision maker  12:43 PM maybe</t>
+      <c r="C119" s="2" t="inlineStr">
+        <is>
+          <t>12:37 PM Hi i have a problem with my current roommates in my shared apartment
+12:38 PM The issue is that they are a bit dirty and do not clean the kitchen after they cook
+12:38 PM i mean i asked them nicely after they had friends over if they could store at least the food back in the fridge
+12:39 PM they apologized to me and they kept cleaning a bit more for ca 2 weeks than the same incident happened again
+12:40 PM so what should i do now
+12:40 PM and what should i tell them in the conversation more specifically
+12:41 PM do you think that a chore chart could help
+12:42 PM not really we all talked about how to feel comfortable in our home but never wrote down chores
+12:43 PM I am not sure I would maybe feel to much like the decision maker
+12:43 PM maybe</t>
         </is>
       </c>
     </row>
@@ -2231,9 +3193,12 @@
       <c r="B120" t="n">
         <v>14572</v>
       </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t>1:49 PM id like to talk to you aout a challenging and heated argument i had with my friend recently  1:53 PM so basically she was really into a guy that at first seemed pretty nice, they started texting over christmas break and when we came back to maastricht in january ( we all go to the same uni btw ) they went out once and after that he was oushing away from her. But the thing is that she was already hung up on him and was settling for the BARE MINIMUM he wasnt even texting her back and he was gosting her. Me as her friend was advising her to just drop him and move on since he wasnt giving her the attention and effort she needed, but she didnt listen to me and she was getting even more attached, she was even sayung that she want a relationship with him... ming you they had went out 2 times in the span of 3 months of talking thorugh mesagges , and they also live in the same city  1:55 PM yes exactly, after a point it got so bad for me that i tried to make her realise that what she was doing was stupid and reckless bc she was visibaly getting hurt by him . I even yelled at her bc she was complaining all the time about him not texting her and i was like: Why do you even like him he doesnt put any effort in tryinh=g to make plans to see you and he is not even responding to you", the she snaped back and was like: I DONT KNOW  1:56 PM YES</t>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>1:49 PM id like to talk to you aout a challenging and heated argument i had with my friend recently
+1:53 PM so basically she was really into a guy that at first seemed pretty nice, they started texting over christmas break and when we came back to maastricht in january ( we all go to the same uni btw ) they went out once and after that he was oushing away from her. But the thing is that she was already hung up on him and was settling for the BARE MINIMUM he wasnt even texting her back and he was gosting her. Me as her friend was advising her to just drop him and move on since he wasnt giving her the attention and effort she needed, but she didnt listen to me and she was getting even more attached, she was even sayung that she want a relationship with him... ming you they had went out 2 times in the span of 3 months of talking thorugh mesagges , and they also live in the same city
+1:55 PM yes exactly, after a point it got so bad for me that i tried to make her realise that what she was doing was stupid and reckless bc she was visibaly getting hurt by him . I even yelled at her bc she was complaining all the time about him not texting her and i was like: Why do you even like him he doesnt put any effort in tryinh=g to make plans to see you and he is not even responding to you", the she snaped back and was like: I DONT KNOW
+1:56 PM YES</t>
         </is>
       </c>
     </row>
@@ -2246,9 +3211,20 @@
       <c r="B121" t="n">
         <v>7</v>
       </c>
-      <c r="C121" t="inlineStr">
-        <is>
-          <t>2:50 PM I had an argument with my friend and i would like you to help me understand it  2:50 PM I wanted to explain to her a situation but got easily triggered as she would not let me finish my sentences and told me how i felt after letting her know that was not how i felt it  2:51 PM Yes, i think the triggering was because of past family problems and now i feel hurt because i feel like i lost a very close friend and i dont know what to do about it  2:52 PM I just want to talk to her about it and resolve it but i dont know if there is any turning back now  2:52 PM Yes, I have and I will, I told her that it is in her hands if she wants to continue being friends or if she cant tolerate it anymore  2:53 PM Really upset, like i cant breathe and my eyes get teary and hands shaky only thinking about it  2:53 PM Im not sure actually usually crying it out helps  2:54 PM No i fear that would make me feel like a burden if i overshared  2:54 PM I understand that, i appreciate it  2:55 PM What do you think i should do now?  2:55 PM How would i be reaching out to her  2:56 PM that sounds like a good idea, i want to understand if i over reacted, she told me that because i am stressed and that i had family issues that it is not an excuse and that she does not see how her words also affected me</t>
+      <c r="C121" s="2" t="inlineStr">
+        <is>
+          <t>2:50 PM I had an argument with my friend and i would like you to help me understand it
+2:50 PM I wanted to explain to her a situation but got easily triggered as she would not let me finish my sentences and told me how i felt after letting her know that was not how i felt it
+2:51 PM Yes, i think the triggering was because of past family problems and now i feel hurt because i feel like i lost a very close friend and i dont know what to do about it
+2:52 PM I just want to talk to her about it and resolve it but i dont know if there is any turning back now
+2:52 PM Yes, I have and I will, I told her that it is in her hands if she wants to continue being friends or if she cant tolerate it anymore
+2:53 PM Really upset, like i cant breathe and my eyes get teary and hands shaky only thinking about it
+2:53 PM Im not sure actually usually crying it out helps
+2:54 PM No i fear that would make me feel like a burden if i overshared
+2:54 PM I understand that, i appreciate it
+2:55 PM What do you think i should do now?
+2:55 PM How would i be reaching out to her
+2:56 PM that sounds like a good idea, i want to understand if i over reacted, she told me that because i am stressed and that i had family issues that it is not an excuse and that she does not see how her words also affected me</t>
         </is>
       </c>
     </row>
@@ -2261,9 +3237,14 @@
       <c r="B122" t="n">
         <v>14983</v>
       </c>
-      <c r="C122" t="inlineStr">
-        <is>
-          <t>3:30 PM Hi so i would like to share a recent experience that transpired this weekend  3:32 PM my friend that i travveled with came to visit and we had a lot of fun and its made me rethink my styudy i love this city and im having a lot of fun but iinternational business people are horrible people and business in general is all about exploiting capitalism which is exactly what im against  3:33 PM well most of them are racist and sexist and always complain about everything and i want to be surrounded by people who love life and love everyone  3:35 PM well theres an underlying issue in the system we live in so i think its important to study business so we can create business to help people and not exploit them but i want to enjoy my life to the fullest and idk if doing this is what i want and i ts difficult to stop cus idk what else to do and my parents are funding my studies  3:36 PM yeah that what i just said  3:36 PM do you have any recommendations on what to do</t>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>3:30 PM Hi so i would like to share a recent experience that transpired this weekend
+3:32 PM my friend that i travveled with came to visit and we had a lot of fun and its made me rethink my styudy i love this city and im having a lot of fun but iinternational business people are horrible people and business in general is all about exploiting capitalism which is exactly what im against
+3:33 PM well most of them are racist and sexist and always complain about everything and i want to be surrounded by people who love life and love everyone
+3:35 PM well theres an underlying issue in the system we live in so i think its important to study business so we can create business to help people and not exploit them but i want to enjoy my life to the fullest and idk if doing this is what i want and i ts difficult to stop cus idk what else to do and my parents are funding my studies
+3:36 PM yeah that what i just said
+3:36 PM do you have any recommendations on what to do</t>
         </is>
       </c>
     </row>
@@ -2276,9 +3257,13 @@
       <c r="B123" t="n">
         <v>14062</v>
       </c>
-      <c r="C123" t="inlineStr">
-        <is>
-          <t>2:20 PM i'd like to tell you about a recent challenging interaction I had  2:23 PM I was at a Cafe with friends and the barista was rude when taking our order  2:24 PM She rolled her eyes at us and spoke in a way that suggested she was annoyed  2:25 PM We brushed it off and remained polite  2:26 PM No it did not</t>
+      <c r="C123" s="2" t="inlineStr">
+        <is>
+          <t>2:20 PM i'd like to tell you about a recent challenging interaction I had
+2:23 PM I was at a Cafe with friends and the barista was rude when taking our order
+2:24 PM She rolled her eyes at us and spoke in a way that suggested she was annoyed
+2:25 PM We brushed it off and remained polite
+2:26 PM No it did not</t>
         </is>
       </c>
     </row>
@@ -2291,9 +3276,18 @@
       <c r="B124" t="n">
         <v>8</v>
       </c>
-      <c r="C124" t="inlineStr">
-        <is>
-          <t>3:16 PM Id like to tell you something about a recent challenging interaction I had  3:17 PM I am currently meeting a friend, we met in a dating context, but because of his distant behaviour and not taking a step, I decided to only stay friends. But now I have feelings for him. What should I do ?  3:18 PM I do not know. I dont want to ruin the friendship, but I also want to have more than a friendship  3:19 PM I dont want to mess the friendship up we already have  3:20 PM When we met each other he did not put any romantic effort in  3:20 PM yes, what should I do?  3:21 PM I feel like I am only the option B  3:21 PM yes  3:21 PM yes  3:22 PM ok what should I do?</t>
+      <c r="C124" s="2" t="inlineStr">
+        <is>
+          <t>3:16 PM Id like to tell you something about a recent challenging interaction I had
+3:17 PM I am currently meeting a friend, we met in a dating context, but because of his distant behaviour and not taking a step, I decided to only stay friends. But now I have feelings for him. What should I do ?
+3:18 PM I do not know. I dont want to ruin the friendship, but I also want to have more than a friendship
+3:19 PM I dont want to mess the friendship up we already have
+3:20 PM When we met each other he did not put any romantic effort in
+3:20 PM yes, what should I do?
+3:21 PM I feel like I am only the option B
+3:21 PM yes
+3:21 PM yes
+3:22 PM ok what should I do?</t>
         </is>
       </c>
     </row>
@@ -2306,9 +3300,20 @@
       <c r="B125" t="n">
         <v>14998</v>
       </c>
-      <c r="C125" t="inlineStr">
-        <is>
-          <t>3:57 PM hello, i want to talk about a recent event that was quite difficult for me lately  3:58 PM we were doing a group project, i really didnt like the way someone was presenting and making the project  4:00 PM the presentation needs to be creative, visually well presented, he just put really big texts in the presentation and it was not well presented, creative and intresesting at all  4:00 PM yes i did, now i'll have to see if he changes it or not  4:01 PM that he didnt took my feedback and it is still just big text blocks  4:02 PM i will have to wait to know, otherwise i will defintily talk to him again  4:02 PM yes exactly  4:02 PM yes  4:03 PM thank you  4:03 PM thank you  4:04 PM who are you?  4:04 PM yes but who created you and what are you</t>
+      <c r="C125" s="2" t="inlineStr">
+        <is>
+          <t>3:57 PM hello, i want to talk about a recent event that was quite difficult for me lately
+3:58 PM we were doing a group project, i really didnt like the way someone was presenting and making the project
+4:00 PM the presentation needs to be creative, visually well presented, he just put really big texts in the presentation and it was not well presented, creative and intresesting at all
+4:00 PM yes i did, now i'll have to see if he changes it or not
+4:01 PM that he didnt took my feedback and it is still just big text blocks
+4:02 PM i will have to wait to know, otherwise i will defintily talk to him again
+4:02 PM yes exactly
+4:02 PM yes
+4:03 PM thank you
+4:03 PM thank you
+4:04 PM who are you?
+4:04 PM yes but who created you and what are you</t>
         </is>
       </c>
     </row>
@@ -2321,9 +3326,15 @@
       <c r="B126" t="n">
         <v>13990</v>
       </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>3:43 PM hey so id like to talk to you about what happened recently with my cousin.  3:46 PM we got into a few fights in the past few years. every time i feel like she was rude to me and wasnt a good friend towards me, treating me like she doesnt care about me or not being there at all and not caring about our friendship/ relationship at all. she did not apologize for anything she did and i still forgave her for the sake of our good friendship  3:47 PM i didnt feel good. she always makes me the reason for our arguments.  3:48 PM yes i have. i even told her to stop a year ago. she sstopped for a bit but after sometime she started again. and then i told her if she wouldnt stop i wouldnt want any contact with her anymore  3:49 PM no. i still want contact to her but i think its the right thing to do. after i said that i feel like she didnt care at all about that. she just said fair enough  3:50 PM yes  3:50 PM yes youre right. what should i do</t>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
+          <t>3:43 PM hey so id like to talk to you about what happened recently with my cousin.
+3:46 PM we got into a few fights in the past few years. every time i feel like she was rude to me and wasnt a good friend towards me, treating me like she doesnt care about me or not being there at all and not caring about our friendship/ relationship at all. she did not apologize for anything she did and i still forgave her for the sake of our good friendship
+3:47 PM i didnt feel good. she always makes me the reason for our arguments.
+3:48 PM yes i have. i even told her to stop a year ago. she sstopped for a bit but after sometime she started again. and then i told her if she wouldnt stop i wouldnt want any contact with her anymore
+3:49 PM no. i still want contact to her but i think its the right thing to do. after i said that i feel like she didnt care at all about that. she just said fair enough
+3:50 PM yes
+3:50 PM yes youre right. what should i do</t>
         </is>
       </c>
     </row>
@@ -2336,9 +3347,13 @@
       <c r="B127" t="n">
         <v>13432</v>
       </c>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>10:51 AM hi recently I ve been in conflict with the friend because everytime im doing something cool shes getting jealous and she tells me things a bit inappropriate  10:52 AM i dont like that and im the type of person how gets really quakily annoyed by someone  10:54 AM not really I prefer just to leave it like this and dont hang out with her  10:54 AM no because shes a new friend so we are not that close  10:55 AM no i think its useless to talk to her about that i mean shes like that thats her personnality so shes not gonna change</t>
+      <c r="C127" s="2" t="inlineStr">
+        <is>
+          <t>10:51 AM hi recently I ve been in conflict with the friend because everytime im doing something cool shes getting jealous and she tells me things a bit inappropriate
+10:52 AM i dont like that and im the type of person how gets really quakily annoyed by someone
+10:54 AM not really I prefer just to leave it like this and dont hang out with her
+10:54 AM no because shes a new friend so we are not that close
+10:55 AM no i think its useless to talk to her about that i mean shes like that thats her personnality so shes not gonna change</t>
         </is>
       </c>
     </row>
@@ -2351,9 +3366,15 @@
       <c r="B128" t="n">
         <v>15136</v>
       </c>
-      <c r="C128" t="inlineStr">
-        <is>
-          <t>9:26 AM i had a recent chalenging interacton i want to tell you about  9:27 AM i talked with my dad. and he did not listened ... i feel like having a long conversation with him is not always easy to get. he is always in his head and thinking about work  9:28 AM yes mostly work related. he always tells me how much he loves me and how important i am to him but it is not like he knows sooo much about me  9:29 AM yes i think that it is. he ist not the "'bonding with people"' kind of a guy. still feels weird when i want to talk to him about something important and he does not seem to listen  9:30 AM i just dont want that because i feel weird doing such a thing  9:31 AM it is more like if i want to tell him something and he simply does not listen. what could i do  9:32 AM then he forgets that\</t>
+      <c r="C128" s="2" t="inlineStr">
+        <is>
+          <t>9:26 AM i had a recent chalenging interacton i want to tell you about
+9:27 AM i talked with my dad. and he did not listened ... i feel like having a long conversation with him is not always easy to get. he is always in his head and thinking about work
+9:28 AM yes mostly work related. he always tells me how much he loves me and how important i am to him but it is not like he knows sooo much about me
+9:29 AM yes i think that it is. he ist not the "'bonding with people"' kind of a guy. still feels weird when i want to talk to him about something important and he does not seem to listen
+9:30 AM i just dont want that because i feel weird doing such a thing
+9:31 AM it is more like if i want to tell him something and he simply does not listen. what could i do
+9:32 AM then he forgets that\</t>
         </is>
       </c>
     </row>
@@ -2366,9 +3387,15 @@
       <c r="B129" t="n">
         <v>14521</v>
       </c>
-      <c r="C129" t="inlineStr">
-        <is>
-          <t>9:37 AM I would like to tell you about a recent challenging interaction i had  9:37 AM it was a heated argument that i had with another student from my project group  9:39 AM it was about his behaviour towards the project. He didnt kept the deadlines, his work was really bad, you could see that he did not care about the grade/project at all  9:40 AM i tried to adress him directly, but he was not in the Uni, so i had to adress him online. First he ignored, than i got a bit heated  9:41 AM he said that he was fine with his work quality and that the tutor said it was good enough. But he was lying, the tutor told us, we would fail for this quality\  9:42 AM yes, but he did not seem to bother at all. To my question, if he will make somes chances, he said "maybe""  9:43 AM there was nothing i could do i guess. i just made him clear in a message that he is not being respful towards the team and that he cant behave like that later in workspace</t>
+      <c r="C129" s="2" t="inlineStr">
+        <is>
+          <t>9:37 AM I would like to tell you about a recent challenging interaction i had
+9:37 AM it was a heated argument that i had with another student from my project group
+9:39 AM it was about his behaviour towards the project. He didnt kept the deadlines, his work was really bad, you could see that he did not care about the grade/project at all
+9:40 AM i tried to adress him directly, but he was not in the Uni, so i had to adress him online. First he ignored, than i got a bit heated
+9:41 AM he said that he was fine with his work quality and that the tutor said it was good enough. But he was lying, the tutor told us, we would fail for this quality\
+9:42 AM yes, but he did not seem to bother at all. To my question, if he will make somes chances, he said "maybe""
+9:43 AM there was nothing i could do i guess. i just made him clear in a message that he is not being respful towards the team and that he cant behave like that later in workspace</t>
         </is>
       </c>
     </row>
@@ -2381,9 +3408,11 @@
       <c r="B130" t="n">
         <v>14317</v>
       </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>10:00 AM I would like to tell you about a recent challenging interaction I had.  10:03 AM Yesterday I was out with my friends and a me and a friend of mine often make jokes about each other where I am at the end that is being made fun of. This is totally fine because I know that it is not meant in a bad way. Yesterday I now made a joke about her not being in the top tier of my friends and she took that personally since she is very insecure when it comes to that matter. I did not know about it and then she got a bit mad. What can I do differently the next time I have a situation like this with a different friend?  10:05 AM Ok that sounds good, I am already pretty aware of her insecurities but this one was new for me and we never talked about it. I did not want to hurt her I only wanted to even the playing field since she made a lot of fun of me the day prior.</t>
+      <c r="C130" s="2" t="inlineStr">
+        <is>
+          <t>10:00 AM I would like to tell you about a recent challenging interaction I had.
+10:03 AM Yesterday I was out with my friends and a me and a friend of mine often make jokes about each other where I am at the end that is being made fun of. This is totally fine because I know that it is not meant in a bad way. Yesterday I now made a joke about her not being in the top tier of my friends and she took that personally since she is very insecure when it comes to that matter. I did not know about it and then she got a bit mad. What can I do differently the next time I have a situation like this with a different friend?
+10:05 AM Ok that sounds good, I am already pretty aware of her insecurities but this one was new for me and we never talked about it. I did not want to hurt her I only wanted to even the playing field since she made a lot of fun of me the day prior.</t>
         </is>
       </c>
     </row>
@@ -2396,9 +3425,14 @@
       <c r="B131" t="n">
         <v>14566</v>
       </c>
-      <c r="C131" t="inlineStr">
-        <is>
-          <t>10:37 AM Ok so my lats tutorial group was a challengeng experience\  10:38 AM the group dynamic. they wouldnt want to do any work  10:39 AM yeah i hate when this happens cuz it drags me down aswell  10:40 AM yeah to be fair I told them immedidiately and then it got better  10:41 AM yeah they were putting more effort into the tasks  10:42 AM yeah we got pretty good feedback aswell so it all worked out in the end yk</t>
+      <c r="C131" s="2" t="inlineStr">
+        <is>
+          <t>10:37 AM Ok so my lats tutorial group was a challengeng experience\
+10:38 AM the group dynamic. they wouldnt want to do any work
+10:39 AM yeah i hate when this happens cuz it drags me down aswell
+10:40 AM yeah to be fair I told them immedidiately and then it got better
+10:41 AM yeah they were putting more effort into the tasks
+10:42 AM yeah we got pretty good feedback aswell so it all worked out in the end yk</t>
         </is>
       </c>
     </row>
@@ -2411,9 +3445,14 @@
       <c r="B132" t="n">
         <v>14638</v>
       </c>
-      <c r="C132" t="inlineStr">
-        <is>
-          <t>2:45 PM hi  2:45 PM okay and yours  2:46 PM sure, i am in a complicated situation at the moment that i want to tell you about  2:49 PM i work together for a association with a girl and we both wanted to become part of next years board. I was selected for the position even though the position was my first choice and her second choice. i think she is going to be mad  2:50 PM oh sorry, it was her first choice and my second  2:50 PM sure, she was confident that she got the spot. she already tol everyone beforehand</t>
+      <c r="C132" s="2" t="inlineStr">
+        <is>
+          <t>2:45 PM hi
+2:45 PM okay and yours
+2:46 PM sure, i am in a complicated situation at the moment that i want to tell you about
+2:49 PM i work together for a association with a girl and we both wanted to become part of next years board. I was selected for the position even though the position was my first choice and her second choice. i think she is going to be mad
+2:50 PM oh sorry, it was her first choice and my second
+2:50 PM sure, she was confident that she got the spot. she already tol everyone beforehand</t>
         </is>
       </c>
     </row>
@@ -2426,9 +3465,15 @@
       <c r="B133" t="n">
         <v>13414</v>
       </c>
-      <c r="C133" t="inlineStr">
-        <is>
-          <t>9:46 AM hi i would like to tell you about a challenging interaction I had recently with my friend  9:47 AM we wanted to go to a concert together and planed everything out. she had to get the tickets and I planed where we wanted to stay. The thing is that she only bought one ticket for herself  9:48 AM yes correct  9:48 AM yes i did she thought i would have gotten my own  9:49 AM yes i think so too  9:49 AM yes it did but i was able to get a ticket in the end anyway  9:50 AM yes it was great and we had a lot of fun. i think she did not do it on purpose so its fine</t>
+      <c r="C133" s="2" t="inlineStr">
+        <is>
+          <t>9:46 AM hi i would like to tell you about a challenging interaction I had recently with my friend
+9:47 AM we wanted to go to a concert together and planed everything out. she had to get the tickets and I planed where we wanted to stay. The thing is that she only bought one ticket for herself
+9:48 AM yes correct
+9:48 AM yes i did she thought i would have gotten my own
+9:49 AM yes i think so too
+9:49 AM yes it did but i was able to get a ticket in the end anyway
+9:50 AM yes it was great and we had a lot of fun. i think she did not do it on purpose so its fine</t>
         </is>
       </c>
     </row>
@@ -2441,9 +3486,20 @@
       <c r="B134" t="n">
         <v>14398</v>
       </c>
-      <c r="C134" t="inlineStr">
-        <is>
-          <t>12:03 PM I did not sleep for too long since i was partying yesterday so im tired  12:03 PM really fun but i spent too much money again  12:04 PM well i forgot a lot since i was too drunk but i guess it was worth it  12:05 PM i always want to be more careful with it but when im drunk i just spend like i have unlimited money, but its fine since i always tend to have a good time  12:05 PM big groups  12:05 PM yes always  12:06 PM well i just have fun, i dont really know  12:06 PM meeting a lot of people i like  12:06 PM both i guess  12:07 PM yes since the city is quite small you tend to know most of the people, so yes we stay in touch  12:07 PM it does!  12:08 PM thanks for your time, it was fun talking to you</t>
+      <c r="C134" s="2" t="inlineStr">
+        <is>
+          <t>12:03 PM I did not sleep for too long since i was partying yesterday so im tired
+12:03 PM really fun but i spent too much money again
+12:04 PM well i forgot a lot since i was too drunk but i guess it was worth it
+12:05 PM i always want to be more careful with it but when im drunk i just spend like i have unlimited money, but its fine since i always tend to have a good time
+12:05 PM big groups
+12:05 PM yes always
+12:06 PM well i just have fun, i dont really know
+12:06 PM meeting a lot of people i like
+12:06 PM both i guess
+12:07 PM yes since the city is quite small you tend to know most of the people, so yes we stay in touch
+12:07 PM it does!
+12:08 PM thanks for your time, it was fun talking to you</t>
         </is>
       </c>
     </row>
@@ -2456,9 +3512,13 @@
       <c r="B135" t="n">
         <v>14173</v>
       </c>
-      <c r="C135" t="inlineStr">
-        <is>
-          <t>12:18 PM hello id like to tell you about a recent challeging interaction i had \  12:19 PM right now we have a new tutorial in university which is supply chain were we are all devided into different groups and often need to work on group projects  12:21 PM I really like my fellow group members they are super kind but i feel like they are not the most responsible ones and i feel like i am always in charge of leading the group\  12:22 PM I sometimes told them that we should start with the group work now to get it done and do not have to stress later but im not super comfortable with calling them out since i really like them on the friendship side  12:24 PM yeah for example on tuesday we have a presentation to prepeare and there are 4 task to do and we are 4 people so i asked them how they want to splitt things up and told them what i would like to prepare but onlz some of them answered</t>
+      <c r="C135" s="2" t="inlineStr">
+        <is>
+          <t>12:18 PM hello id like to tell you about a recent challeging interaction i had \
+12:19 PM right now we have a new tutorial in university which is supply chain were we are all devided into different groups and often need to work on group projects
+12:21 PM I really like my fellow group members they are super kind but i feel like they are not the most responsible ones and i feel like i am always in charge of leading the group\
+12:22 PM I sometimes told them that we should start with the group work now to get it done and do not have to stress later but im not super comfortable with calling them out since i really like them on the friendship side
+12:24 PM yeah for example on tuesday we have a presentation to prepeare and there are 4 task to do and we are 4 people so i asked them how they want to splitt things up and told them what i would like to prepare but onlz some of them answered</t>
         </is>
       </c>
     </row>
@@ -2471,9 +3531,15 @@
       <c r="B136" t="n">
         <v>14020</v>
       </c>
-      <c r="C136" t="inlineStr">
-        <is>
-          <t>12:41 PM hi how are you  12:41 PM not that good  12:42 PM yes i had a bad interaction  12:43 PM i had a disagreement with a friend  12:44 PM i wanted to fly to ibiza with her but she wanted to go to italy  12:44 PM no we didnt and thats the problem  12:45 PM yes i did but she said that she wants to meet an italian man so she didnt want to compromisre</t>
+      <c r="C136" s="2" t="inlineStr">
+        <is>
+          <t>12:41 PM hi how are you
+12:41 PM not that good
+12:42 PM yes i had a bad interaction
+12:43 PM i had a disagreement with a friend
+12:44 PM i wanted to fly to ibiza with her but she wanted to go to italy
+12:44 PM no we didnt and thats the problem
+12:45 PM yes i did but she said that she wants to meet an italian man so she didnt want to compromisre</t>
         </is>
       </c>
     </row>
@@ -2486,9 +3552,15 @@
       <c r="B137" t="n">
         <v>14923</v>
       </c>
-      <c r="C137" t="inlineStr">
-        <is>
-          <t>2:01 PM i would like to share a challenging experience i had  2:02 PM i was in class the other day and i had a bit of an argument with a classmate  2:05 PM we were talking about the different kinds of music apps and this one guy told us that he loved apple music then when i started to state the advantages of spotify he took it personnally and though that i was saying that apple ;usic wasnt good so he had an attitude with me and i didnt understand why  2:05 PM yes it did i never though he was going to be offended like that  2:05 PM the hole class was shocked  2:06 PM i did not have the opportunity to talk to him after class but the teacher came next to me and asked me if i was ok  2:07 PM yes she didnt understand his reaction, he was defensive</t>
+      <c r="C137" s="2" t="inlineStr">
+        <is>
+          <t>2:01 PM i would like to share a challenging experience i had
+2:02 PM i was in class the other day and i had a bit of an argument with a classmate
+2:05 PM we were talking about the different kinds of music apps and this one guy told us that he loved apple music then when i started to state the advantages of spotify he took it personnally and though that i was saying that apple ;usic wasnt good so he had an attitude with me and i didnt understand why
+2:05 PM yes it did i never though he was going to be offended like that
+2:05 PM the hole class was shocked
+2:06 PM i did not have the opportunity to talk to him after class but the teacher came next to me and asked me if i was ok
+2:07 PM yes she didnt understand his reaction, he was defensive</t>
         </is>
       </c>
     </row>
@@ -2501,9 +3573,20 @@
       <c r="B138" t="n">
         <v>14575</v>
       </c>
-      <c r="C138" t="inlineStr">
-        <is>
-          <t>2:19 PM everythings good so far, not a too stressful day  2:20 PM yes im visiting a friend of mine and his family for the weekend\  2:20 PM no no.  2:21 PM but id like to tell you about a \recent challenging interaction  2:22 PM It is a big thing between me and the one where i rent at  2:23 PM no its me and a firm. i would like to leave my appartment but my contract goes very long but it cant be legal  2:23 PM yes i did and they dont accept it  2:24 PM because my contract is for 2 years and since there are no issues with the flat and house (there are) they dont accept it  2:24 PM i think im gonna take a lawyer  2:26 PM everything is just so old and i promise you everybody sees that. there are mouses where the agency says that its the tenants fault and son on  2:26 PM yes i did but since my living and security is not limited by it they dont accept anything  2:27 PM yes im going to</t>
+      <c r="C138" s="2" t="inlineStr">
+        <is>
+          <t>2:19 PM everythings good so far, not a too stressful day
+2:20 PM yes im visiting a friend of mine and his family for the weekend\
+2:20 PM no no.
+2:21 PM but id like to tell you about a \recent challenging interaction
+2:22 PM It is a big thing between me and the one where i rent at
+2:23 PM no its me and a firm. i would like to leave my appartment but my contract goes very long but it cant be legal
+2:23 PM yes i did and they dont accept it
+2:24 PM because my contract is for 2 years and since there are no issues with the flat and house (there are) they dont accept it
+2:24 PM i think im gonna take a lawyer
+2:26 PM everything is just so old and i promise you everybody sees that. there are mouses where the agency says that its the tenants fault and son on
+2:26 PM yes i did but since my living and security is not limited by it they dont accept anything
+2:27 PM yes im going to</t>
         </is>
       </c>
     </row>
@@ -2516,9 +3599,19 @@
       <c r="B139" t="n">
         <v>14959</v>
       </c>
-      <c r="C139" t="inlineStr">
-        <is>
-          <t>2:32 PM I had a difficult talk with my dad  2:33 PM About my boyfriend because he doesnt like him  2:33 PM Because he doesnt have all the same view for the future as me  2:35 PM He doesnt really know it and thats the problem because i really have my goals for the future and already know my way that i have to follow to reach my goals  2:36 PM yes but he is just totally lost and dont know what he wants for the future  2:37 PM yes definetly because i dont know how to structure my day when my partner is not doing the same things as me  2:37 PM yes kind of  2:38 PM yed definetly  2:38 PM maybe; but arent my goals also in a way his goals ?  2:39 PM i dont know its hard to say. also i dont know if i can do it independantly  2:40 PM so you think i should just do my own thing without him ?</t>
+      <c r="C139" s="2" t="inlineStr">
+        <is>
+          <t>2:32 PM I had a difficult talk with my dad
+2:33 PM About my boyfriend because he doesnt like him
+2:33 PM Because he doesnt have all the same view for the future as me
+2:35 PM He doesnt really know it and thats the problem because i really have my goals for the future and already know my way that i have to follow to reach my goals
+2:36 PM yes but he is just totally lost and dont know what he wants for the future
+2:37 PM yes definetly because i dont know how to structure my day when my partner is not doing the same things as me
+2:37 PM yes kind of
+2:38 PM yed definetly
+2:38 PM maybe; but arent my goals also in a way his goals ?
+2:39 PM i dont know its hard to say. also i dont know if i can do it independantly
+2:40 PM so you think i should just do my own thing without him ?</t>
         </is>
       </c>
     </row>
@@ -2531,9 +3624,19 @@
       <c r="B140" t="n">
         <v>14992</v>
       </c>
-      <c r="C140" t="inlineStr">
-        <is>
-          <t>2:56 PM nothing in particular  2:58 PM what do you think is better between Commodity trading vs. investment banking ?  2:59 PM im term of compensation we can aim a 6 figures in geneva  2:59 PM i think  3:00 PM with the bonus / stock options  3:00 PM Vitol i think  3:01 PM i do not know yet  3:01 PM perfect  3:02 PM so...  3:02 PM ib vs pe vs trading  3:03 PM best lifestyle ?</t>
+      <c r="C140" s="2" t="inlineStr">
+        <is>
+          <t>2:56 PM nothing in particular
+2:58 PM what do you think is better between Commodity trading vs. investment banking ?
+2:59 PM im term of compensation we can aim a 6 figures in geneva
+2:59 PM i think
+3:00 PM with the bonus / stock options
+3:00 PM Vitol i think
+3:01 PM i do not know yet
+3:01 PM perfect
+3:02 PM so...
+3:02 PM ib vs pe vs trading
+3:03 PM best lifestyle ?</t>
         </is>
       </c>
     </row>
@@ -2546,9 +3649,28 @@
       <c r="B141" t="n">
         <v>14209</v>
       </c>
-      <c r="C141" t="inlineStr">
-        <is>
-          <t>3:17 PM hi  3:18 PM good what about you  3:18 PM good can i talk to you now can yo hear me  3:19 PM i just talked to you can you not hear me  3:21 PM i had a challegning interaction with my roommate can did you hear it, i just talked about it  3:21 PM we had a conflict last weekend  3:22 PM about the niose in our house and it really upset me  3:22 PM she did not really see my point, i always wake up from her loud noice in the bathroom as my wall is directly connected to it  3:23 PM and i asked her to be more quit but she did not really uundertood what i meant  3:23 PM yes i told her that i always wake up because of it, which is really annoying  3:24 PM i dd not felt heard at all  3:24 PM feel  3:24 PM no i did not  3:24 PM waht can i do now  3:25 PM she should just be more quit  3:25 PM i do not see a problem do you  3:25 PM okay i dont think so, what can i do now  3:26 PM i already used earplugsbut it also annoys me in the night  3:26 PM any other solutions  3:26 PM okay</t>
+      <c r="C141" s="2" t="inlineStr">
+        <is>
+          <t>3:17 PM hi
+3:18 PM good what about you
+3:18 PM good can i talk to you now can yo hear me
+3:19 PM i just talked to you can you not hear me
+3:21 PM i had a challegning interaction with my roommate can did you hear it, i just talked about it
+3:21 PM we had a conflict last weekend
+3:22 PM about the niose in our house and it really upset me
+3:22 PM she did not really see my point, i always wake up from her loud noice in the bathroom as my wall is directly connected to it
+3:23 PM and i asked her to be more quit but she did not really uundertood what i meant
+3:23 PM yes i told her that i always wake up because of it, which is really annoying
+3:24 PM i dd not felt heard at all
+3:24 PM feel
+3:24 PM no i did not
+3:24 PM waht can i do now
+3:25 PM she should just be more quit
+3:25 PM i do not see a problem do you
+3:25 PM okay i dont think so, what can i do now
+3:26 PM i already used earplugsbut it also annoys me in the night
+3:26 PM any other solutions
+3:26 PM okay</t>
         </is>
       </c>
     </row>
@@ -2561,9 +3683,20 @@
       <c r="B142" t="n">
         <v>16381</v>
       </c>
-      <c r="C142" t="inlineStr">
-        <is>
-          <t>3:37 PM hello i am a first year university student  3:38 PM very good i am really enjoying it, but recently i had a challenging interation with people i am in a group project with  3:39 PM Some people were not doing their part. And didnt really care how good or bad they did their job. but it is graded, so it is important  3:39 PM In the groupchat i earged them to complete their part  3:40 PM yes a deadline but i also just askd them if they could please change or do X  3:41 PM they did end up doing it but once one of my teammates didnt do anything  3:41 PM just the bare minimum  3:42 PM it was still fine but 2 of us in the group were annoyed  3:42 PM in total there were 5 members  3:43 PM were discussed it ourseles and briefly with the whole group while we were waiting for the other person, They were also late  3:43 PM no  3:44 PM no not really</t>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>3:37 PM hello i am a first year university student
+3:38 PM very good i am really enjoying it, but recently i had a challenging interation with people i am in a group project with
+3:39 PM Some people were not doing their part. And didnt really care how good or bad they did their job. but it is graded, so it is important
+3:39 PM In the groupchat i earged them to complete their part
+3:40 PM yes a deadline but i also just askd them if they could please change or do X
+3:41 PM they did end up doing it but once one of my teammates didnt do anything
+3:41 PM just the bare minimum
+3:42 PM it was still fine but 2 of us in the group were annoyed
+3:42 PM in total there were 5 members
+3:43 PM were discussed it ourseles and briefly with the whole group while we were waiting for the other person, They were also late
+3:43 PM no
+3:44 PM no not really</t>
         </is>
       </c>
     </row>
@@ -2576,9 +3709,18 @@
       <c r="B143" t="n">
         <v>15250</v>
       </c>
-      <c r="C143" t="inlineStr">
-        <is>
-          <t>4:15 PM Hi I would like to tell you about a recent challenging interaction I had  4:15 PM I had a little fight with my roommate and now I cant stand him anymore  4:17 PM Im living on the second floor and the kitchen is on floor 0, so sometimes I wash a few mugs in the bathroom on my floor instead of going all the way downstairs. He saw that and sent me a very rude and disrespectful message  4:18 PM He said I was disrespectful, this behavior is crazy for a person my age and questioned my education. He also said I should be thankful, that he didnt contact the landlord yet  4:19 PM yes exactly  4:20 PM I responded and said that it was not okay to write something like that and that he couldve told me that in person, but then he didnt answer until a week later so I just left it there  4:20 PM yes  4:21 PM I cant stand him. He made me feel uncomfortable at my own place. This was not okay and I will never like him  4:22 PM yes true \  4:22 PM yes I think so</t>
+      <c r="C143" s="2" t="inlineStr">
+        <is>
+          <t>4:15 PM Hi I would like to tell you about a recent challenging interaction I had
+4:15 PM I had a little fight with my roommate and now I cant stand him anymore
+4:17 PM Im living on the second floor and the kitchen is on floor 0, so sometimes I wash a few mugs in the bathroom on my floor instead of going all the way downstairs. He saw that and sent me a very rude and disrespectful message
+4:18 PM He said I was disrespectful, this behavior is crazy for a person my age and questioned my education. He also said I should be thankful, that he didnt contact the landlord yet
+4:19 PM yes exactly
+4:20 PM I responded and said that it was not okay to write something like that and that he couldve told me that in person, but then he didnt answer until a week later so I just left it there
+4:20 PM yes
+4:21 PM I cant stand him. He made me feel uncomfortable at my own place. This was not okay and I will never like him
+4:22 PM yes true \
+4:22 PM yes I think so</t>
         </is>
       </c>
     </row>
@@ -2591,9 +3733,15 @@
       <c r="B144" t="n">
         <v>14308</v>
       </c>
-      <c r="C144" t="inlineStr">
-        <is>
-          <t>8:59 AM hey chatbot, how are you doing today?  9:00 AM My day has been great! Early start in the morning and I feel so productive already  9:00 AM I ate breakfast and spoke to my Mum on the phone today  9:01 AM But nevermind, I'd like to tell you a recent challenging interaction I had  9:02 AM I have this friend who I really care about but it turns out he is gay and into me. I am straight and don't know how to handle the situation. I like him as a friend but not more than that  9:03 AM yes  9:03 AM yes, I thought I will just be honest and tell him that I value the friendship but that I am not into men</t>
+      <c r="C144" s="2" t="inlineStr">
+        <is>
+          <t>8:59 AM hey chatbot, how are you doing today?
+9:00 AM My day has been great! Early start in the morning and I feel so productive already
+9:00 AM I ate breakfast and spoke to my Mum on the phone today
+9:01 AM But nevermind, I'd like to tell you a recent challenging interaction I had
+9:02 AM I have this friend who I really care about but it turns out he is gay and into me. I am straight and don't know how to handle the situation. I like him as a friend but not more than that
+9:03 AM yes
+9:03 AM yes, I thought I will just be honest and tell him that I value the friendship but that I am not into men</t>
         </is>
       </c>
     </row>
@@ -2606,9 +3754,12 @@
       <c r="B145" t="n">
         <v>15160</v>
       </c>
-      <c r="C145" t="inlineStr">
-        <is>
-          <t>10:21 AM hi, so recently i had a challenging interaction when i found out that in the elderly home where my grandma lives, her friend and someone else she knew very well both passed away on the same day.  10:22 AM well, my grandma is very strong, and it is not the first time she has lost someone that is very near and dear to her. Obviously, she is getting older too and she knows that death is something you cannot avoid, but it is sort of a hard reality check. I'm not completely sure how she's dealing with it, but she is still pretty much always happy.  10:24 AM currently, the main support system is the other elderly people that live in the same house, with whom she can talk about how they're dealing with the same situation, and discuss life in general because it's very hard to imagine for someone who is not as old as them what it's like when death comes closer and closer  10:25 AM yea she has, to her it's important that we remember her for the happy, strong, loving person she is. My grandma has herself been in medical treatment for almost 40 years, so i think she sort of got used to death being a normal thing in her life, since it has always been present</t>
+      <c r="C145" s="2" t="inlineStr">
+        <is>
+          <t>10:21 AM hi, so recently i had a challenging interaction when i found out that in the elderly home where my grandma lives, her friend and someone else she knew very well both passed away on the same day.
+10:22 AM well, my grandma is very strong, and it is not the first time she has lost someone that is very near and dear to her. Obviously, she is getting older too and she knows that death is something you cannot avoid, but it is sort of a hard reality check. I'm not completely sure how she's dealing with it, but she is still pretty much always happy.
+10:24 AM currently, the main support system is the other elderly people that live in the same house, with whom she can talk about how they're dealing with the same situation, and discuss life in general because it's very hard to imagine for someone who is not as old as them what it's like when death comes closer and closer
+10:25 AM yea she has, to her it's important that we remember her for the happy, strong, loving person she is. My grandma has herself been in medical treatment for almost 40 years, so i think she sort of got used to death being a normal thing in her life, since it has always been present</t>
         </is>
       </c>
     </row>
@@ -2621,9 +3772,15 @@
       <c r="B146" t="n">
         <v>14752</v>
       </c>
-      <c r="C146" t="inlineStr">
-        <is>
-          <t>11:24 AM hello  11:25 AM so far so good, just had an interest situation tho haha  11:26 AM it was just that someone from my tutorial group gave some critical feedback on a presentation that i did and the feedback wasnt true  11:27 AM not yet, i thaught about doing the same to their group, but it doesnt feel right to just do the same to them, especially because there are people in the group that didnt do anything  11:27 AM first of all search for a situation where i can talk to the person alone and if that is not helping then try to get the tutor/ course coordinator in on it  11:29 AM maybe reasons why the person did it, or it would be even better when as a result of the talk the person would write the tutor a mail in which they state, that thez did something wrong if you want to see it that way  11:30 AM i mean yes the task for the one side of the group was to give constructive feedback, so i understand that they want to say a lot to get a good grade, but lying is just wrong</t>
+      <c r="C146" s="2" t="inlineStr">
+        <is>
+          <t>11:24 AM hello
+11:25 AM so far so good, just had an interest situation tho haha
+11:26 AM it was just that someone from my tutorial group gave some critical feedback on a presentation that i did and the feedback wasnt true
+11:27 AM not yet, i thaught about doing the same to their group, but it doesnt feel right to just do the same to them, especially because there are people in the group that didnt do anything
+11:27 AM first of all search for a situation where i can talk to the person alone and if that is not helping then try to get the tutor/ course coordinator in on it
+11:29 AM maybe reasons why the person did it, or it would be even better when as a result of the talk the person would write the tutor a mail in which they state, that thez did something wrong if you want to see it that way
+11:30 AM i mean yes the task for the one side of the group was to give constructive feedback, so i understand that they want to say a lot to get a good grade, but lying is just wrong</t>
         </is>
       </c>
     </row>
@@ -2636,9 +3793,21 @@
       <c r="B147" t="n">
         <v>25582</v>
       </c>
-      <c r="C147" t="inlineStr">
-        <is>
-          <t>10:05 AM hi  10:05 AM its going well  10:05 AM i wanted to tell you about a stressful situation i had  10:06 AM i have a group project but my group mates havent contributed anything  10:06 AM ive tried both but its a bit stressful for me  10:07 AM not really i just want to feel supportive  10:07 AM yes do u have any ideas  10:07 AM we need to host a party , so how should we proceed  10:08 AM ok good idea  10:08 AM next week?  10:09 AM i need my group members opinion on that  10:09 AM what else ?  10:09 AM yes sounds good</t>
+      <c r="C147" s="2" t="inlineStr">
+        <is>
+          <t>10:05 AM hi
+10:05 AM its going well
+10:05 AM i wanted to tell you about a stressful situation i had
+10:06 AM i have a group project but my group mates havent contributed anything
+10:06 AM ive tried both but its a bit stressful for me
+10:07 AM not really i just want to feel supportive
+10:07 AM yes do u have any ideas
+10:07 AM we need to host a party , so how should we proceed
+10:08 AM ok good idea
+10:08 AM next week?
+10:09 AM i need my group members opinion on that
+10:09 AM what else ?
+10:09 AM yes sounds good</t>
         </is>
       </c>
     </row>
@@ -2651,9 +3820,16 @@
       <c r="B148" t="n">
         <v>13597</v>
       </c>
-      <c r="C148" t="inlineStr">
-        <is>
-          <t>10:44 AM hi how are you?  10:45 AM im fine thank you, id like to tell you about a recent challenging interaction i had  10:47 AM i was in an unknown enviorment in france, i was supposed to go from maastricht to Epernay/Reims with the train. i had 4 times i had to change trains/busses... but because i had a tight schedule regarding the department times i had quite some stress. nobody could speak english, and that made it very frustrating to find my way at thedifferent train stations which kept changing their departure times and railroads  10:49 AM i fortunately did in the end, however i encountered a very frustrating experience with the train conductor who refused to help me because i spoke english instead of france  10:49 AM and a lot of additional money spend on tickets due to constantly missing the trains, hundereds of euros..  10:50 AM yes he did leave a bit of a bad taste behind, although im aware that i cant change others, i do now unfortunately have a prejudce about some french people working at public transport  10:50 AM i am not completely sure yet if it was worth it  10:51 AM seeing my mom and brother again together with my family for 1 day,</t>
+      <c r="C148" s="2" t="inlineStr">
+        <is>
+          <t>10:44 AM hi how are you?
+10:45 AM im fine thank you, id like to tell you about a recent challenging interaction i had
+10:47 AM i was in an unknown enviorment in france, i was supposed to go from maastricht to Epernay/Reims with the train. i had 4 times i had to change trains/busses... but because i had a tight schedule regarding the department times i had quite some stress. nobody could speak english, and that made it very frustrating to find my way at thedifferent train stations which kept changing their departure times and railroads
+10:49 AM i fortunately did in the end, however i encountered a very frustrating experience with the train conductor who refused to help me because i spoke english instead of france
+10:49 AM and a lot of additional money spend on tickets due to constantly missing the trains, hundereds of euros..
+10:50 AM yes he did leave a bit of a bad taste behind, although im aware that i cant change others, i do now unfortunately have a prejudce about some french people working at public transport
+10:50 AM i am not completely sure yet if it was worth it
+10:51 AM seeing my mom and brother again together with my family for 1 day,</t>
         </is>
       </c>
     </row>
@@ -2666,9 +3842,16 @@
       <c r="B149" t="n">
         <v>15196</v>
       </c>
-      <c r="C149" t="inlineStr">
-        <is>
-          <t>11:51 AM I'd like to tell you about a recent challenging interaction I had  11:51 AM I had a disagreement with my roommates about keeping the kitchen clean  11:52 AM It was an ongoing issue. We had told two of our roommates to keep the kitchen clean after they had made something to eat but they kept making it dirty.  11:53 AM We had talked to them about it many times before and they repeatedly did it.  11:53 AM We felt as if they didn't respect what we were saying so eventually one of the coordinators in our building had to step in.  11:54 AM Yes it did, after that they stopped making a mess and started cleaning up after themselves.  11:54 AM Yes, it is a much more comfortable environment now.  11:55 AM Yes I am much more motivated to cook food in my kitchen now.</t>
+      <c r="C149" s="2" t="inlineStr">
+        <is>
+          <t>11:51 AM I'd like to tell you about a recent challenging interaction I had
+11:51 AM I had a disagreement with my roommates about keeping the kitchen clean
+11:52 AM It was an ongoing issue. We had told two of our roommates to keep the kitchen clean after they had made something to eat but they kept making it dirty.
+11:53 AM We had talked to them about it many times before and they repeatedly did it.
+11:53 AM We felt as if they didn't respect what we were saying so eventually one of the coordinators in our building had to step in.
+11:54 AM Yes it did, after that they stopped making a mess and started cleaning up after themselves.
+11:54 AM Yes, it is a much more comfortable environment now.
+11:55 AM Yes I am much more motivated to cook food in my kitchen now.</t>
         </is>
       </c>
     </row>
@@ -2681,9 +3864,13 @@
       <c r="B150" t="n">
         <v>14215</v>
       </c>
-      <c r="C150" t="inlineStr">
-        <is>
-          <t>12:41 PM hi how are you?  12:42 PM i am felling okay. id like to share a recent challenging interaction i had  12:44 PM I live with a roommate and in the beginning we got along really well. but within the last couple of weeks she started to get really messy and stopped cleaning stuff after she used it etc. Yesterday, i sat her down to tell how it is really bothering me and asked her to start cleaning up after herself again. She got super offended and is now really mad at me  12:46 PM yes I told how that i really liked our living situation and how we took care of the household in the beginning. And that i now feel like she is kind of disrespecting me and our appartement with her recent behaviour and I asked her to change it  12:48 PM no it was a sudden change. nothing dramatic or stressful happend in her life recently.</t>
+      <c r="C150" s="2" t="inlineStr">
+        <is>
+          <t>12:41 PM hi how are you?
+12:42 PM i am felling okay. id like to share a recent challenging interaction i had
+12:44 PM I live with a roommate and in the beginning we got along really well. but within the last couple of weeks she started to get really messy and stopped cleaning stuff after she used it etc. Yesterday, i sat her down to tell how it is really bothering me and asked her to start cleaning up after herself again. She got super offended and is now really mad at me
+12:46 PM yes I told how that i really liked our living situation and how we took care of the household in the beginning. And that i now feel like she is kind of disrespecting me and our appartement with her recent behaviour and I asked her to change it
+12:48 PM no it was a sudden change. nothing dramatic or stressful happend in her life recently.</t>
         </is>
       </c>
     </row>
@@ -2696,9 +3883,16 @@
       <c r="B151" t="n">
         <v>15247</v>
       </c>
-      <c r="C151" t="inlineStr">
-        <is>
-          <t>3:00 PM whats up broskiid like o tell you about a challenging interaction i had this weekend  3:01 PM i was in a bar with a couple of friend and all of asudend the bouncher kicked me out  3:01 PM he said i was on drugs even do i wasnt  3:02 PM i had no clue what was ging on he just asked me come with me for a second and after following him he told me its over for the day  3:03 PM he said my face was moving wirdly  3:03 PM i also black so maybe that played a role too  3:04 PM fr  3:04 PM i only said for real</t>
+      <c r="C151" s="2" t="inlineStr">
+        <is>
+          <t>3:00 PM whats up broskiid like o tell you about a challenging interaction i had this weekend
+3:01 PM i was in a bar with a couple of friend and all of asudend the bouncher kicked me out
+3:01 PM he said i was on drugs even do i wasnt
+3:02 PM i had no clue what was ging on he just asked me come with me for a second and after following him he told me its over for the day
+3:03 PM he said my face was moving wirdly
+3:03 PM i also black so maybe that played a role too
+3:04 PM fr
+3:04 PM i only said for real</t>
         </is>
       </c>
     </row>
@@ -2711,9 +3905,17 @@
       <c r="B152" t="n">
         <v>13828</v>
       </c>
-      <c r="C152" t="inlineStr">
-        <is>
-          <t>10:25 AM Good morning, how are you doing?  10:26 AM actually not, is raining outside and its quite cold  10:26 AM yeah youre right, but i need to attend some lectures first  10:27 AM some supply chain management classes and finance as well  10:28 AM i would say finance is more entertaining but is all about how the tutor prepares the classes, finance are more enjoyable  10:29 AM Not quite, but i am really happy with my tutorial group, all my classmates are respectful and knowledgeable  10:30 AM stock discussions most of the time, during breaks we like to share our weekend experiences, also our tutor makes good engaging questions in which we join in groups to discuss and try to answer  10:31 AM totally yes, but im not finding that ''chemistry'' in SCM  10:31 AM I dont know yet, probably is the subject which i dont really find it interesting</t>
+      <c r="C152" s="2" t="inlineStr">
+        <is>
+          <t>10:25 AM Good morning, how are you doing?
+10:26 AM actually not, is raining outside and its quite cold
+10:26 AM yeah youre right, but i need to attend some lectures first
+10:27 AM some supply chain management classes and finance as well
+10:28 AM i would say finance is more entertaining but is all about how the tutor prepares the classes, finance are more enjoyable
+10:29 AM Not quite, but i am really happy with my tutorial group, all my classmates are respectful and knowledgeable
+10:30 AM stock discussions most of the time, during breaks we like to share our weekend experiences, also our tutor makes good engaging questions in which we join in groups to discuss and try to answer
+10:31 AM totally yes, but im not finding that ''chemistry'' in SCM
+10:31 AM I dont know yet, probably is the subject which i dont really find it interesting</t>
         </is>
       </c>
     </row>
@@ -2726,9 +3928,17 @@
       <c r="B153" t="n">
         <v>14491</v>
       </c>
-      <c r="C153" t="inlineStr">
-        <is>
-          <t>11:35 AM not much what about you  11:36 AM yes I recently received an unfair and harsh grade for my tutor  11:38 AM i didnt get to interact with him much bc he kept avoiding me, but he downgraded my participation bc of being late 2 min. I told him quiet directly that his behaviour is unecessary  11:39 AM yeah and he marked me down in the grading criteria for respect bc of that  11:39 AM probably  11:40 AM no, but its not that deep. Just expect more professionalism from tutors  11:41 AM just let it slide, dont have the time for an appeal  11:41 AM any advice for the future  11:42 AM ill think about it</t>
+      <c r="C153" s="2" t="inlineStr">
+        <is>
+          <t>11:35 AM not much what about you
+11:36 AM yes I recently received an unfair and harsh grade for my tutor
+11:38 AM i didnt get to interact with him much bc he kept avoiding me, but he downgraded my participation bc of being late 2 min. I told him quiet directly that his behaviour is unecessary
+11:39 AM yeah and he marked me down in the grading criteria for respect bc of that
+11:39 AM probably
+11:40 AM no, but its not that deep. Just expect more professionalism from tutors
+11:41 AM just let it slide, dont have the time for an appeal
+11:41 AM any advice for the future
+11:42 AM ill think about it</t>
         </is>
       </c>
     </row>
@@ -2741,9 +3951,17 @@
       <c r="B154" t="n">
         <v>13804</v>
       </c>
-      <c r="C154" t="inlineStr">
-        <is>
-          <t>12:01 PM hi, i had a really challenging interaction recently  12:03 PM i had to argue in my second language which made it hard, and also the manager i was talking to wasnt my boss but still ordered me around and i could not stand up for myself  12:03 PM i was scared to get scolded by my actual manager, or dissappoint them, because it is my first ever job  12:04 PM yes, but unfortunately i was not the one who first contacted her about it, she has already heard what had happened when i saw her  12:05 PM she was really kind and assured me i did not do anything wrong, and not to take everything from the other manager so seriously  12:05 PM yes, absolutely, i needed some reassurance\  12:06 PM im not absolutely sure, but i will stand up more for sure, but i dont know to which extent  12:06 PM yeah, youre right, thanks  12:07 PM no, that is all</t>
+      <c r="C154" s="2" t="inlineStr">
+        <is>
+          <t>12:01 PM hi, i had a really challenging interaction recently
+12:03 PM i had to argue in my second language which made it hard, and also the manager i was talking to wasnt my boss but still ordered me around and i could not stand up for myself
+12:03 PM i was scared to get scolded by my actual manager, or dissappoint them, because it is my first ever job
+12:04 PM yes, but unfortunately i was not the one who first contacted her about it, she has already heard what had happened when i saw her
+12:05 PM she was really kind and assured me i did not do anything wrong, and not to take everything from the other manager so seriously
+12:05 PM yes, absolutely, i needed some reassurance\
+12:06 PM im not absolutely sure, but i will stand up more for sure, but i dont know to which extent
+12:06 PM yeah, youre right, thanks
+12:07 PM no, that is all</t>
         </is>
       </c>
     </row>
@@ -2756,9 +3974,16 @@
       <c r="B155" t="n">
         <v>3</v>
       </c>
-      <c r="C155" t="inlineStr">
-        <is>
-          <t>1:07 PM I'd like to tell you about a recent challenging experience I had  1:09 PM I get really nervous when I'm presenting and today I had to conduct an entire 2 hour session in front of 12 students with another peer in our university course. I really struggled to get my words out logically...  1:10 PM I think I could have been more prepared, but at the time I didn't know if my preparation was too much or too less  1:11 PM Not directly towards my presentation skills but more the lack of content my other peers noticed.  1:12 PM Could be yes. The problem is that the presentation was tough to present. We had to cover so many points and I felt that it was never enough from our side  1:12 PM I presented an article and forgot a little bit to engage with the students, so it was a bit boring  1:13 PM Yes, of course. The good thing is that I noticed that my notes were not that good, so for next time I'll prepare them even more carefully  1:14 PM I had too many notes and I didn't read half of them. In the presentation, it was too hard to focus on the key parts</t>
+      <c r="C155" s="2" t="inlineStr">
+        <is>
+          <t>1:07 PM I'd like to tell you about a recent challenging experience I had
+1:09 PM I get really nervous when I'm presenting and today I had to conduct an entire 2 hour session in front of 12 students with another peer in our university course. I really struggled to get my words out logically...
+1:10 PM I think I could have been more prepared, but at the time I didn't know if my preparation was too much or too less
+1:11 PM Not directly towards my presentation skills but more the lack of content my other peers noticed.
+1:12 PM Could be yes. The problem is that the presentation was tough to present. We had to cover so many points and I felt that it was never enough from our side
+1:12 PM I presented an article and forgot a little bit to engage with the students, so it was a bit boring
+1:13 PM Yes, of course. The good thing is that I noticed that my notes were not that good, so for next time I'll prepare them even more carefully
+1:14 PM I had too many notes and I didn't read half of them. In the presentation, it was too hard to focus on the key parts</t>
         </is>
       </c>
     </row>
@@ -2771,9 +3996,14 @@
       <c r="B156" t="n">
         <v>13492</v>
       </c>
-      <c r="C156" t="inlineStr">
-        <is>
-          <t>2:42 PM I recently had a conflict with a roommate about some bills we had to pay  2:43 PM it was the amout each one of us had to pay  2:44 PM it is still unresolved the problem is she moved away and now it is hard to discuss it because we are both pretty beasy at the moment  2:45 PM I think I am going to send her a message because in my opinion it is better to handle things quickly  2:46 PM I dont know yet because I denfetly think that I am in the right but I dont want it to sound disrespectful or rude so thats whzy I am stilll thinking about it  2:47 PM but what do i do if I still disagree with her after she told me her perspective</t>
+      <c r="C156" s="2" t="inlineStr">
+        <is>
+          <t>2:42 PM I recently had a conflict with a roommate about some bills we had to pay
+2:43 PM it was the amout each one of us had to pay
+2:44 PM it is still unresolved the problem is she moved away and now it is hard to discuss it because we are both pretty beasy at the moment
+2:45 PM I think I am going to send her a message because in my opinion it is better to handle things quickly
+2:46 PM I dont know yet because I denfetly think that I am in the right but I dont want it to sound disrespectful or rude so thats whzy I am stilll thinking about it
+2:47 PM but what do i do if I still disagree with her after she told me her perspective</t>
         </is>
       </c>
     </row>
@@ -2786,9 +4016,17 @@
       <c r="B157" t="n">
         <v>15067</v>
       </c>
-      <c r="C157" t="inlineStr">
-        <is>
-          <t>10:09 AM Hi, Im here to talk to you about a recent challenging interaction I had  10:10 AM I am not the best at being in fierce arguments and I recently had an argument with a friend  10:11 AM We had different opinions about the possibility of him doing a certain challenge. For me personally it is challenging because I am not used to arguing loudly with other people  10:12 AM Yeah it is not so much about the topic itself but how to manage a dispute in general  10:12 AM More overwhelmed  10:13 AM No the feeling lingered for a little bit  10:13 AM Yeah of course, that alwys helps. But the fact that I couldnt handle the situation as well stuck with me for longer  10:14 AM no just in general tell me: How could I learn how to handle conflict in the future  10:14 AM Ok thank you, and how can I practice that</t>
+      <c r="C157" s="2" t="inlineStr">
+        <is>
+          <t>10:09 AM Hi, Im here to talk to you about a recent challenging interaction I had
+10:10 AM I am not the best at being in fierce arguments and I recently had an argument with a friend
+10:11 AM We had different opinions about the possibility of him doing a certain challenge. For me personally it is challenging because I am not used to arguing loudly with other people
+10:12 AM Yeah it is not so much about the topic itself but how to manage a dispute in general
+10:12 AM More overwhelmed
+10:13 AM No the feeling lingered for a little bit
+10:13 AM Yeah of course, that alwys helps. But the fact that I couldnt handle the situation as well stuck with me for longer
+10:14 AM no just in general tell me: How could I learn how to handle conflict in the future
+10:14 AM Ok thank you, and how can I practice that</t>
         </is>
       </c>
     </row>
@@ -2801,9 +4039,18 @@
       <c r="B158" t="n">
         <v>14962</v>
       </c>
-      <c r="C158" t="inlineStr">
-        <is>
-          <t>11:10 AM I had issues in a group work project because some of the members did not participate at all  11:11 AM I started by approaching the people, several times, but ultimatley had to talk to my tutor  11:12 AM He offered to mediate a talk with the entire group. We did so but that didnt improve the situation for the next presentation  11:12 AM In the second presentation the members didnt participate again. Ultimatley I just left it at that and tried to do my part the best I could  11:13 AM We had a talk after the final presentation and ultimatley ended up with grade differentiation because my tutor could see differences in participation himself  11:14 AM They were, but they were also very annoyed by the situation  11:14 AM No. I saw one of them again, but he didnt talk to me at all  11:15 AM No. There is not really any common friendgroup betweeen us so there is no point of interaction anymomre, as we dont have class together anymore  11:15 AM Yes, Ill just leave it in the past  11:16 AM Yes</t>
+      <c r="C158" s="2" t="inlineStr">
+        <is>
+          <t>11:10 AM I had issues in a group work project because some of the members did not participate at all
+11:11 AM I started by approaching the people, several times, but ultimatley had to talk to my tutor
+11:12 AM He offered to mediate a talk with the entire group. We did so but that didnt improve the situation for the next presentation
+11:12 AM In the second presentation the members didnt participate again. Ultimatley I just left it at that and tried to do my part the best I could
+11:13 AM We had a talk after the final presentation and ultimatley ended up with grade differentiation because my tutor could see differences in participation himself
+11:14 AM They were, but they were also very annoyed by the situation
+11:14 AM No. I saw one of them again, but he didnt talk to me at all
+11:15 AM No. There is not really any common friendgroup betweeen us so there is no point of interaction anymomre, as we dont have class together anymore
+11:15 AM Yes, Ill just leave it in the past
+11:16 AM Yes</t>
         </is>
       </c>
     </row>
@@ -2816,9 +4063,18 @@
       <c r="B159" t="n">
         <v>14740</v>
       </c>
-      <c r="C159" t="inlineStr">
-        <is>
-          <t>11:38 AM Hey, my name is Alvaro and I want to share some experiences with you  11:39 AM i'd like to tell you about a recent challenging interaction I had during the weekend  11:40 AM I was in a familiar gathering with one cousin and my uncles, we were trying to have a conversation but each time I wanted to participate my cousine interrupted me  11:42 AM I just tell him laughing to stop interrupting, but he didn't take it seriously, so he just keep doing it, until a moment he went out of the meeting and I could there speak normally to my uncles  11:43 AM well, afterwards we eat because the food was ready, so everyone was just talking to everyone and we didn't had another opportuinity like that one\  11:43 AM yes  11:43 AM no  11:44 AM yes, to avoid any bad feelings, cause I know him and I know that he is a good person but so intense  11:44 AM no  11:45 AM no, he is just like that always</t>
+      <c r="C159" s="2" t="inlineStr">
+        <is>
+          <t>11:38 AM Hey, my name is Alvaro and I want to share some experiences with you
+11:39 AM i'd like to tell you about a recent challenging interaction I had during the weekend
+11:40 AM I was in a familiar gathering with one cousin and my uncles, we were trying to have a conversation but each time I wanted to participate my cousine interrupted me
+11:42 AM I just tell him laughing to stop interrupting, but he didn't take it seriously, so he just keep doing it, until a moment he went out of the meeting and I could there speak normally to my uncles
+11:43 AM well, afterwards we eat because the food was ready, so everyone was just talking to everyone and we didn't had another opportuinity like that one\
+11:43 AM yes
+11:43 AM no
+11:44 AM yes, to avoid any bad feelings, cause I know him and I know that he is a good person but so intense
+11:44 AM no
+11:45 AM no, he is just like that always</t>
         </is>
       </c>
     </row>
@@ -2831,9 +4087,18 @@
       <c r="B160" t="n">
         <v>14422</v>
       </c>
-      <c r="C160" t="inlineStr">
-        <is>
-          <t>11:48 AM I would like to tell you about a recent interaction i had  11:49 AM A good friend of mine just cant seem to be honest with me, even on the most basic and non offensive things  11:50 AM Yes, but with most of my friends  11:50 AM It does affect my relationship, it bri ngs me to distance myself\  11:51 AM definitely  11:52 AM they dont lie, they simply cant tell things for the way they are, as an example, they have difficulties expressing the way they themselves feel about certain things  11:52 AM Yes, bu this indirectly brings them to lie  11:53 AM something like that  11:53 AM yeah  11:54 AM it would be both, the way it affects my relationship is a consequence . because i dont have those problems</t>
+      <c r="C160" s="2" t="inlineStr">
+        <is>
+          <t>11:48 AM I would like to tell you about a recent interaction i had
+11:49 AM A good friend of mine just cant seem to be honest with me, even on the most basic and non offensive things
+11:50 AM Yes, but with most of my friends
+11:50 AM It does affect my relationship, it bri ngs me to distance myself\
+11:51 AM definitely
+11:52 AM they dont lie, they simply cant tell things for the way they are, as an example, they have difficulties expressing the way they themselves feel about certain things
+11:52 AM Yes, bu this indirectly brings them to lie
+11:53 AM something like that
+11:53 AM yeah
+11:54 AM it would be both, the way it affects my relationship is a consequence . because i dont have those problems</t>
         </is>
       </c>
     </row>
@@ -2846,9 +4111,24 @@
       <c r="B161" t="n">
         <v>14494</v>
       </c>
-      <c r="C161" t="inlineStr">
-        <is>
-          <t>12:14 PM id like to tell you about a recent interaction i had  12:15 PM Well i have this friend, and it seems like we had a disagreement but im not sure what about  12:16 PM Its pretty much unclear, but maybe i was a bit clingy, but i doubt that because we were in different countries right before we stopped talking  12:16 PM Maybe, it was gradual, but it came out of no where for me, and we have fully stopped talking since then  12:16 PM They wont respond when i do reach out  12:17 PM I know right, what could i try doing?  12:17 PM Ive done that already, what else could i do? i really value our friendship  12:17 PM Its been 4 weeks already  12:18 PM So what should i do  12:19 PM Ok that makes sense, but if tht doenst work what should i do, becsaue this person was super important to me and i think that i am important to them  12:19 PM Oh, i asked to meet in person and she said she was busy but then boom shes on the beach that day  12:19 PM So? what should i do  12:20 PM So whats the next step then  12:20 PM How can i do that  12:20 PM Ok whats next tho?  12:21 PM ok makes sense, i have that with others but i just feel hurt that i can never get that clarity</t>
+      <c r="C161" s="2" t="inlineStr">
+        <is>
+          <t>12:14 PM id like to tell you about a recent interaction i had
+12:15 PM Well i have this friend, and it seems like we had a disagreement but im not sure what about
+12:16 PM Its pretty much unclear, but maybe i was a bit clingy, but i doubt that because we were in different countries right before we stopped talking
+12:16 PM Maybe, it was gradual, but it came out of no where for me, and we have fully stopped talking since then
+12:16 PM They wont respond when i do reach out
+12:17 PM I know right, what could i try doing?
+12:17 PM Ive done that already, what else could i do? i really value our friendship
+12:17 PM Its been 4 weeks already
+12:18 PM So what should i do
+12:19 PM Ok that makes sense, but if tht doenst work what should i do, becsaue this person was super important to me and i think that i am important to them
+12:19 PM Oh, i asked to meet in person and she said she was busy but then boom shes on the beach that day
+12:19 PM So? what should i do
+12:20 PM So whats the next step then
+12:20 PM How can i do that
+12:20 PM Ok whats next tho?
+12:21 PM ok makes sense, i have that with others but i just feel hurt that i can never get that clarity</t>
         </is>
       </c>
     </row>
@@ -2861,9 +4141,24 @@
       <c r="B162" t="n">
         <v>15184</v>
       </c>
-      <c r="C162" t="inlineStr">
-        <is>
-          <t>12:26 PM i would like to tell you about something that was challenging for me in the past  12:27 PM i had a friend tell me that he got together with my ex girlfriend after we broke up  12:27 PM alright i told him that i will not speak to him again and that was the end of the interaction  12:28 PM he said he had to do something for himslef  12:28 PM yes  12:28 PM yes  12:29 PM i feel like it was an ignorent decision keeping in mind that we were very close friends  12:29 PM yes  12:30 PM yes as i said before i ended the friendship and told him that i will not talk to him again, this was a very neutral talk which we had. no getting mad from my side or anything i simplz told him that he will no longer be a person whom i am willing to talk to  12:31 PM neutral\  12:31 PM no  12:31 PM yes  12:32 PM to make it clear that i will not waste my energy on that person  12:32 PM yes  12:32 PM no he was a good friend  12:33 PM part of life</t>
+      <c r="C162" s="2" t="inlineStr">
+        <is>
+          <t>12:26 PM i would like to tell you about something that was challenging for me in the past
+12:27 PM i had a friend tell me that he got together with my ex girlfriend after we broke up
+12:27 PM alright i told him that i will not speak to him again and that was the end of the interaction
+12:28 PM he said he had to do something for himslef
+12:28 PM yes
+12:28 PM yes
+12:29 PM i feel like it was an ignorent decision keeping in mind that we were very close friends
+12:29 PM yes
+12:30 PM yes as i said before i ended the friendship and told him that i will not talk to him again, this was a very neutral talk which we had. no getting mad from my side or anything i simplz told him that he will no longer be a person whom i am willing to talk to
+12:31 PM neutral\
+12:31 PM no
+12:31 PM yes
+12:32 PM to make it clear that i will not waste my energy on that person
+12:32 PM yes
+12:32 PM no he was a good friend
+12:33 PM part of life</t>
         </is>
       </c>
     </row>
@@ -2876,9 +4171,22 @@
       <c r="B163" t="n">
         <v>13549</v>
       </c>
-      <c r="C163" t="inlineStr">
-        <is>
-          <t>10:44 AM hey there my name is thomas how are u  10:45 AM oh nice so i just want to know ur job here  10:45 AM nice well actually i had a hard interaction with my parents a few days ago  10:46 AM basically it was for housing in maastricht my parents set up a budget for me but the room i wanted was too expensive  10:46 AM yeah kind of cos it was a shared house with all my friends  10:47 AM yeah i tred but idk if its gona work im in the midle of it rn  10:47 AM yeah i think they undestand  10:47 AM i guess i might pay a part of it so that i can get the room i want and that my paerents stay in their budget  10:48 AM yes i think i have some money sved up and i cna get a student job  10:48 AM restaurant or cafe  10:49 AM yes i have  10:49 AM yeh i liked it tbfm fun dynamic and gets you some moneyy  10:49 AM yes teamwork but i think we are good with ;y problem right could we be done  10:50 AM alrighty perfecttt cheers bye bye replika was lovely chatting with you</t>
+      <c r="C163" s="2" t="inlineStr">
+        <is>
+          <t>10:44 AM hey there my name is thomas how are u
+10:45 AM oh nice so i just want to know ur job here
+10:45 AM nice well actually i had a hard interaction with my parents a few days ago
+10:46 AM basically it was for housing in maastricht my parents set up a budget for me but the room i wanted was too expensive
+10:46 AM yeah kind of cos it was a shared house with all my friends
+10:47 AM yeah i tred but idk if its gona work im in the midle of it rn
+10:47 AM yeah i think they undestand
+10:47 AM i guess i might pay a part of it so that i can get the room i want and that my paerents stay in their budget
+10:48 AM yes i think i have some money sved up and i cna get a student job
+10:48 AM restaurant or cafe
+10:49 AM yes i have
+10:49 AM yeh i liked it tbfm fun dynamic and gets you some moneyy
+10:49 AM yes teamwork but i think we are good with ;y problem right could we be done
+10:50 AM alrighty perfecttt cheers bye bye replika was lovely chatting with you</t>
         </is>
       </c>
     </row>
@@ -2891,9 +4199,19 @@
       <c r="B164" t="n">
         <v>13486</v>
       </c>
-      <c r="C164" t="inlineStr">
-        <is>
-          <t>11:21 AM id like to tell you about a problem with a friend i had  11:22 AM We had tickets for a concert but i didnt really listened to the band, and it was expensive and i did not have time on that specific day  11:22 AM yes  11:23 AM The problem was i didnt really communicated well so i wanted to sell the ticket but forgot and the zhad some trouble on the daz of the concert then  11:23 AM correct  11:24 AM he texted me but i didnt relize that the concert was on this day, so we had a misunderstanding. But then thez just took another person using my ticket  11:24 AM yea but no response  11:25 AM Yea but i apologized so from my side its resolved  11:25 AM agree  11:25 AM i agree  11:27 AM what happened</t>
+      <c r="C164" s="2" t="inlineStr">
+        <is>
+          <t>11:21 AM id like to tell you about a problem with a friend i had
+11:22 AM We had tickets for a concert but i didnt really listened to the band, and it was expensive and i did not have time on that specific day
+11:22 AM yes
+11:23 AM The problem was i didnt really communicated well so i wanted to sell the ticket but forgot and the zhad some trouble on the daz of the concert then
+11:23 AM correct
+11:24 AM he texted me but i didnt relize that the concert was on this day, so we had a misunderstanding. But then thez just took another person using my ticket
+11:24 AM yea but no response
+11:25 AM Yea but i apologized so from my side its resolved
+11:25 AM agree
+11:25 AM i agree
+11:27 AM what happened</t>
         </is>
       </c>
     </row>
@@ -2906,9 +4224,16 @@
       <c r="B165" t="n">
         <v>13750</v>
       </c>
-      <c r="C165" t="inlineStr">
-        <is>
-          <t>9:01 AM id like to tell you about a recent challenging interaction i had.  9:02 AM i was in a group project with a girl and she was not helping in anything so i tried to tell her but she got so upset  9:03 AM it was private i texted that i wanted to meet her and then at the end of the class we spoke but she did nt understand  9:04 AM i spoke very nicely and even ask her if she wanted to do it together  9:05 AM not really i am scared that others would think i am a drama queen and i dont want her to have troubles  9:06 AM can you rephrase i dont really understand your question  9:07 AM maybe both cause i dont know what to do rn  9:07 AM i just want to have a good grade but she doesnt care</t>
+      <c r="C165" s="2" t="inlineStr">
+        <is>
+          <t>9:01 AM id like to tell you about a recent challenging interaction i had.
+9:02 AM i was in a group project with a girl and she was not helping in anything so i tried to tell her but she got so upset
+9:03 AM it was private i texted that i wanted to meet her and then at the end of the class we spoke but she did nt understand
+9:04 AM i spoke very nicely and even ask her if she wanted to do it together
+9:05 AM not really i am scared that others would think i am a drama queen and i dont want her to have troubles
+9:06 AM can you rephrase i dont really understand your question
+9:07 AM maybe both cause i dont know what to do rn
+9:07 AM i just want to have a good grade but she doesnt care</t>
         </is>
       </c>
     </row>
@@ -2921,9 +4246,22 @@
       <c r="B166" t="n">
         <v>13849</v>
       </c>
-      <c r="C166" t="inlineStr">
-        <is>
-          <t>10:59 AM Very good and yours?  10:59 AM I would like to tell you about the recent challenging interaction I had with my boyfriend  11:02 AM Basically, we get along very well on all aspects expect for one rather important topic which is planning. I am someone who loves to have things planned well in advance. And he is someone who is the complete opposite to that. Because of that last week we had a disagreement on our summer plans. We are planning a trip to the US together which we talked about months ago. I planned it all out and put the entire itinerary into a document so he could show it to his parents and they can agree, he still has not asked them whether the dates and trip is okay with them which is a little annoying. As prices also increase and I just want to have it planned so we can go on a fun trip  11:03 AM no, he just procrastinates and tells me each time he will ask tonight, which he has been saying for the past month  11:03 AM OK  11:03 AM yes  11:03 AM i like it  11:04 AM okay  11:04 AM how so  11:04 AM I dont think I need that thanks  11:04 AM okay thank you  11:05 AM yes  11:05 AM well yes, if we do not plan soon it will be super expensive and not within our budget anymore and we will not be able to go on a trip  11:06 AM we have mutiple times</t>
+      <c r="C166" s="2" t="inlineStr">
+        <is>
+          <t>10:59 AM Very good and yours?
+10:59 AM I would like to tell you about the recent challenging interaction I had with my boyfriend
+11:02 AM Basically, we get along very well on all aspects expect for one rather important topic which is planning. I am someone who loves to have things planned well in advance. And he is someone who is the complete opposite to that. Because of that last week we had a disagreement on our summer plans. We are planning a trip to the US together which we talked about months ago. I planned it all out and put the entire itinerary into a document so he could show it to his parents and they can agree, he still has not asked them whether the dates and trip is okay with them which is a little annoying. As prices also increase and I just want to have it planned so we can go on a fun trip
+11:03 AM no, he just procrastinates and tells me each time he will ask tonight, which he has been saying for the past month
+11:03 AM OK
+11:03 AM yes
+11:03 AM i like it
+11:04 AM okay
+11:04 AM how so
+11:04 AM I dont think I need that thanks
+11:04 AM okay thank you
+11:05 AM yes
+11:05 AM well yes, if we do not plan soon it will be super expensive and not within our budget anymore and we will not be able to go on a trip
+11:06 AM we have mutiple times</t>
         </is>
       </c>
     </row>
@@ -2936,9 +4274,18 @@
       <c r="B167" t="n">
         <v>14260</v>
       </c>
-      <c r="C167" t="inlineStr">
-        <is>
-          <t>9:04 AM good how are you?  9:05 AM studying, need to lock in more  9:05 AM different stuff  9:05 AM both but more on uni  9:06 AM we finished it already  9:07 AM but it went good, the course was manageable, but our tutor was not the best so we didnt learn much there and the exam was much harder then the exercises  9:08 AM yes, we also told it to him in class and in the feedback we gave him  9:08 AM one way, he really understands the subject, but cant explain it  9:09 AM true  9:10 AM the course in times of the topic is not the best one in the study, but if your tutor is also not great then it gets even more boring and exhausting</t>
+      <c r="C167" s="2" t="inlineStr">
+        <is>
+          <t>9:04 AM good how are you?
+9:05 AM studying, need to lock in more
+9:05 AM different stuff
+9:05 AM both but more on uni
+9:06 AM we finished it already
+9:07 AM but it went good, the course was manageable, but our tutor was not the best so we didnt learn much there and the exam was much harder then the exercises
+9:08 AM yes, we also told it to him in class and in the feedback we gave him
+9:08 AM one way, he really understands the subject, but cant explain it
+9:09 AM true
+9:10 AM the course in times of the topic is not the best one in the study, but if your tutor is also not great then it gets even more boring and exhausting</t>
         </is>
       </c>
     </row>
@@ -2951,9 +4298,18 @@
       <c r="B168" t="n">
         <v>14614</v>
       </c>
-      <c r="C168" t="inlineStr">
-        <is>
-          <t>11:13 AM hello how are you  11:13 AM ys great i wanted to talk to you about interaction that i got with somoene  11:14 AM it was with a frien  11:14 AM friend  11:16 AM it was about going to school together like she wanted to came with me to go to school (it is about 40 minutes) but like she didnt want to pay the gas but i was feeling bad to ask her  11:18 AM well i end up a bit shouting at her because i was thinking she were traiting me like i was her uber driver and then she understood but i dont know i feel so bad to ask money but now with thr price of the gaz that is increasing it is very complicated and i only am a student  11:19 AM yes i think i can and i am sue she will understand because everybody know that the price of the gas is increasing and also when i go to school i hate depedn on people like waiting for then to be on time so i think it can be also relate to that  11:19 AM I'm 18 or over  11:20 AM welll now i didnt sqy anything but i think she understood because she didnt ask me for another ride and i prefer that  11:21 AM yes i think so and i mean if she has a problem with that she can just take her own car</t>
+      <c r="C168" s="2" t="inlineStr">
+        <is>
+          <t>11:13 AM hello how are you
+11:13 AM ys great i wanted to talk to you about interaction that i got with somoene
+11:14 AM it was with a frien
+11:14 AM friend
+11:16 AM it was about going to school together like she wanted to came with me to go to school (it is about 40 minutes) but like she didnt want to pay the gas but i was feeling bad to ask her
+11:18 AM well i end up a bit shouting at her because i was thinking she were traiting me like i was her uber driver and then she understood but i dont know i feel so bad to ask money but now with thr price of the gaz that is increasing it is very complicated and i only am a student
+11:19 AM yes i think i can and i am sue she will understand because everybody know that the price of the gas is increasing and also when i go to school i hate depedn on people like waiting for then to be on time so i think it can be also relate to that
+11:19 AM I'm 18 or over
+11:20 AM welll now i didnt sqy anything but i think she understood because she didnt ask me for another ride and i prefer that
+11:21 AM yes i think so and i mean if she has a problem with that she can just take her own car</t>
         </is>
       </c>
     </row>
@@ -2966,9 +4322,14 @@
       <c r="B169" t="n">
         <v>14764</v>
       </c>
-      <c r="C169" t="inlineStr">
-        <is>
-          <t>10:09 AM thumb up thumb down show more actions I would like to share a recent challenging interaction I had.  10:10 AM Last week I had to decide on which of my friends I was going to live with, as the apartment was with two people and we were three  10:10 AM The other friend ended up going with another friend  10:11 AM Yes, it all worked out good at the end.  10:11 AM Yes as the house is bigger and the other friend can visit  10:12 AM Yes</t>
+      <c r="C169" s="2" t="inlineStr">
+        <is>
+          <t>10:09 AM thumb up thumb down show more actions I would like to share a recent challenging interaction I had.
+10:10 AM Last week I had to decide on which of my friends I was going to live with, as the apartment was with two people and we were three
+10:10 AM The other friend ended up going with another friend
+10:11 AM Yes, it all worked out good at the end.
+10:11 AM Yes as the house is bigger and the other friend can visit
+10:12 AM Yes</t>
         </is>
       </c>
     </row>
@@ -2981,9 +4342,15 @@
       <c r="B170" t="n">
         <v>14665</v>
       </c>
-      <c r="C170" t="inlineStr">
-        <is>
-          <t>12:24 PM i would like to tell you about a current situation i had that still doesnt let me go  12:25 PM i had an argument with my roommate about the tidyness of our apartement  12:26 PM i feel like that i am always the one cleaning up, organizing the dishwasher. In general i feel like she pretends to help but in real life i do the work  12:27 PM she thinks that everyhing is fine  12:28 PM yes i did but everytime she says that she does a lot of work. then i got annoyed and just stayed at a friends house for the night cause we were fighting. then i came back we both appologized but still nothing really changed  12:28 PM yes for sure  12:29 PM yes thats a good idea. The situations are especially with the dish washer, and cleaning the bathrroom but also vacuuming or when she leaves the sofa she never folds the blankets or just leaves her cups and food on the table instead of moving it to the dishwasher</t>
+      <c r="C170" s="2" t="inlineStr">
+        <is>
+          <t>12:24 PM i would like to tell you about a current situation i had that still doesnt let me go
+12:25 PM i had an argument with my roommate about the tidyness of our apartement
+12:26 PM i feel like that i am always the one cleaning up, organizing the dishwasher. In general i feel like she pretends to help but in real life i do the work
+12:27 PM she thinks that everyhing is fine
+12:28 PM yes i did but everytime she says that she does a lot of work. then i got annoyed and just stayed at a friends house for the night cause we were fighting. then i came back we both appologized but still nothing really changed
+12:28 PM yes for sure
+12:29 PM yes thats a good idea. The situations are especially with the dish washer, and cleaning the bathrroom but also vacuuming or when she leaves the sofa she never folds the blankets or just leaves her cups and food on the table instead of moving it to the dishwasher</t>
         </is>
       </c>
     </row>
@@ -2996,9 +4363,11 @@
       <c r="B171" t="n">
         <v>14767</v>
       </c>
-      <c r="C171" t="inlineStr">
-        <is>
-          <t>2:06 PM I'd like to tell you about a recent challenging interaction I had.  2:08 PM One of my friends from my tutorial group at university never shows up for important appointments and is bringing all of his teammates including me down with him. I dont really know how to approach this situation and how to tell him his behaviour is not okay.  2:10 PM Yes I have tried this, but it did not help. The rest of the group knows of this as well and also tried to talking to him. But nothing is working. We even told are tutor some of the details last week because its just getting worse with his unreliability.</t>
+      <c r="C171" s="2" t="inlineStr">
+        <is>
+          <t>2:06 PM I'd like to tell you about a recent challenging interaction I had.
+2:08 PM One of my friends from my tutorial group at university never shows up for important appointments and is bringing all of his teammates including me down with him. I dont really know how to approach this situation and how to tell him his behaviour is not okay.
+2:10 PM Yes I have tried this, but it did not help. The rest of the group knows of this as well and also tried to talking to him. But nothing is working. We even told are tutor some of the details last week because its just getting worse with his unreliability.</t>
         </is>
       </c>
     </row>
@@ -3011,9 +4380,14 @@
       <c r="B172" t="n">
         <v>14413</v>
       </c>
-      <c r="C172" t="inlineStr">
-        <is>
-          <t>2:31 PM Hi  2:32 PM good a little confused in this days  2:33 PM yes, so i live with other two girls and sometimes we seem to go a long just fine but other time i fell like we are a little separate  2:34 PM probably the fact that the two knows each other since two year and i don't  2:36 PM as i said sometimes its all normal but sometimes especialy with banal things they seem very close but not with me  2:37 PM i m not a jealuse person but sometimes it make me feel alone</t>
+      <c r="C172" s="2" t="inlineStr">
+        <is>
+          <t>2:31 PM Hi
+2:32 PM good a little confused in this days
+2:33 PM yes, so i live with other two girls and sometimes we seem to go a long just fine but other time i fell like we are a little separate
+2:34 PM probably the fact that the two knows each other since two year and i don't
+2:36 PM as i said sometimes its all normal but sometimes especialy with banal things they seem very close but not with me
+2:37 PM i m not a jealuse person but sometimes it make me feel alone</t>
         </is>
       </c>
     </row>
@@ -3026,9 +4400,22 @@
       <c r="B173" t="n">
         <v>14236</v>
       </c>
-      <c r="C173" t="inlineStr">
-        <is>
-          <t>10:41 AM id like to tell you about a recent challenging interaction i had  10:41 AM personal  10:42 AM it was while we had to study in university but it was not related to it \  10:43 AM i talked to a girl that i liked and at first everything was working really well but after that it got more distand and i didnt understand what i did wrong  10:43 AM no  10:44 AM yes  10:45 AM no she didnt answerd me properly and i think i will just going to keep my distance from now on  10:45 AM yes.  10:46 AM i also had a problem with my apartment here in maastricht  10:47 AM no i asked my house keeper if a EV ladingstation is planned because we got solarpennels  10:48 AM yes  10:48 AM tesla model 3 or ID 3\4  10:48 AM i drove a tesla and a id4  10:49 AM i think the IDs are better in how they are built compared to the tesla. on the other hand the tesla has more hp</t>
+      <c r="C173" s="2" t="inlineStr">
+        <is>
+          <t>10:41 AM id like to tell you about a recent challenging interaction i had
+10:41 AM personal
+10:42 AM it was while we had to study in university but it was not related to it \
+10:43 AM i talked to a girl that i liked and at first everything was working really well but after that it got more distand and i didnt understand what i did wrong
+10:43 AM no
+10:44 AM yes
+10:45 AM no she didnt answerd me properly and i think i will just going to keep my distance from now on
+10:45 AM yes.
+10:46 AM i also had a problem with my apartment here in maastricht
+10:47 AM no i asked my house keeper if a EV ladingstation is planned because we got solarpennels
+10:48 AM yes
+10:48 AM tesla model 3 or ID 3\4
+10:48 AM i drove a tesla and a id4
+10:49 AM i think the IDs are better in how they are built compared to the tesla. on the other hand the tesla has more hp</t>
         </is>
       </c>
     </row>
@@ -3041,9 +4428,12 @@
       <c r="B174" t="n">
         <v>14110</v>
       </c>
-      <c r="C174" t="inlineStr">
-        <is>
-          <t>3:04 PM hi i would like to share with you a difficult experience i had with a friend recently  3:05 PM yes so basically we went out together with another friend on a night out. we both got quite drunk and so i personally wasnt really acting as myself. i got mad at her for something quite small and removed myself from the situation and joined other friends that were also out. she stayed with the third friend we went out with. but now shes extremely upset with me about how our night went down  3:07 PM yes i definitely overreacted. i removed myself from the situation so that i wouldnt say anything i would regret the next day but that really upset her. she kept texting me and stuff once i left and eventually i asked her if she was home cus i didnt want her to be walking on the streets drunk and alone and then the next day she said that i was manipulating her by saying that which i really didnt get  3:08 PM yes i told her that it was not at all my intention to manipulate her or anything but that i was genuinely meaning that, and that just because i was upset with her earlier in the night, i still care about her safety. but because we were texting while both drunk and taking everything out of proportion i still said some things that i probably shouldnt have over text. the next day i called her and apologised for everything and we talked about it a bit. she said it was okay and that she would get over it. then the next time i saw her in person, i again apologised</t>
+      <c r="C174" s="2" t="inlineStr">
+        <is>
+          <t>3:04 PM hi i would like to share with you a difficult experience i had with a friend recently
+3:05 PM yes so basically we went out together with another friend on a night out. we both got quite drunk and so i personally wasnt really acting as myself. i got mad at her for something quite small and removed myself from the situation and joined other friends that were also out. she stayed with the third friend we went out with. but now shes extremely upset with me about how our night went down
+3:07 PM yes i definitely overreacted. i removed myself from the situation so that i wouldnt say anything i would regret the next day but that really upset her. she kept texting me and stuff once i left and eventually i asked her if she was home cus i didnt want her to be walking on the streets drunk and alone and then the next day she said that i was manipulating her by saying that which i really didnt get
+3:08 PM yes i told her that it was not at all my intention to manipulate her or anything but that i was genuinely meaning that, and that just because i was upset with her earlier in the night, i still care about her safety. but because we were texting while both drunk and taking everything out of proportion i still said some things that i probably shouldnt have over text. the next day i called her and apologised for everything and we talked about it a bit. she said it was okay and that she would get over it. then the next time i saw her in person, i again apologised</t>
         </is>
       </c>
     </row>
@@ -3056,9 +4446,17 @@
       <c r="B175" t="n">
         <v>14815</v>
       </c>
-      <c r="C175" t="inlineStr">
-        <is>
-          <t>11:33 AM Id like to tell you about a recent challenging interaction I had.  11:34 AM I had a disagreement with my roomate in our shared house  11:35 AM He never pays attention to cleaning up after himself when he used the kitchen and Im a really clean person and I feel disrespected  11:35 AM Yes and he always says he understands and when it comes to the kitchen being clean, I never see any changes  11:36 AM I dont think he actually cares. But he always emphasizes how important respect is and it annoys me that he doenst behave accordingly.  11:37 AM What does that mean?  11:37 AM It feels very bad and I dont know what to do about it  11:37 AM any tipps?  11:38 AM Yes but then he will just say again that he will change in the future</t>
+      <c r="C175" s="2" t="inlineStr">
+        <is>
+          <t>11:33 AM Id like to tell you about a recent challenging interaction I had.
+11:34 AM I had a disagreement with my roomate in our shared house
+11:35 AM He never pays attention to cleaning up after himself when he used the kitchen and Im a really clean person and I feel disrespected
+11:35 AM Yes and he always says he understands and when it comes to the kitchen being clean, I never see any changes
+11:36 AM I dont think he actually cares. But he always emphasizes how important respect is and it annoys me that he doenst behave accordingly.
+11:37 AM What does that mean?
+11:37 AM It feels very bad and I dont know what to do about it
+11:37 AM any tipps?
+11:38 AM Yes but then he will just say again that he will change in the future</t>
         </is>
       </c>
     </row>
@@ -3071,9 +4469,16 @@
       <c r="B176" t="n">
         <v>14848</v>
       </c>
-      <c r="C176" t="inlineStr">
-        <is>
-          <t>2:41 PM I'd like to tell you about a recent challenging interaction i had.  2:42 PM A girl i used to be friends with approached me at a festival and asekd me whats wrong and why i dont talk to her anymore. She told a lot of people bad thinsg about me and she definitely knows that I know.  2:43 PM I told her but she denied everything and wanted me to tell her the names of the people who told me but it was literally everyone i know that she knows aswell and talks to occasionally.  2:44 PM I think she wanted me back as a friend but she treated me more as a servant and personal diary than as a friend.  2:45 PM i tried to but she only ever repsonded with "what do you mean"or " I dont know what to say"  2:46 PM I think frustrate is the wrong term i was more disappointed because she used to tell me that I'm her best friend  2:47 PM Yes, and know i dont know what to do since I offered to talk at a quieter setting than a party  2:48 PM I dont want to be her friend anymore nor do i want any association with her also i dont even want to talk to her</t>
+      <c r="C176" s="2" t="inlineStr">
+        <is>
+          <t>2:41 PM I'd like to tell you about a recent challenging interaction i had.
+2:42 PM A girl i used to be friends with approached me at a festival and asekd me whats wrong and why i dont talk to her anymore. She told a lot of people bad thinsg about me and she definitely knows that I know.
+2:43 PM I told her but she denied everything and wanted me to tell her the names of the people who told me but it was literally everyone i know that she knows aswell and talks to occasionally.
+2:44 PM I think she wanted me back as a friend but she treated me more as a servant and personal diary than as a friend.
+2:45 PM i tried to but she only ever repsonded with "what do you mean"or " I dont know what to say"
+2:46 PM I think frustrate is the wrong term i was more disappointed because she used to tell me that I'm her best friend
+2:47 PM Yes, and know i dont know what to do since I offered to talk at a quieter setting than a party
+2:48 PM I dont want to be her friend anymore nor do i want any association with her also i dont even want to talk to her</t>
         </is>
       </c>
     </row>
@@ -3086,9 +4491,24 @@
       <c r="B177" t="n">
         <v>16495</v>
       </c>
-      <c r="C177" t="inlineStr">
-        <is>
-          <t>3:12 PM hi  3:13 PM good  3:13 PM how are you  3:13 PM good  3:13 PM Send me a realistic selfie  3:13 PM Keep it real  3:14 PM I had a argument with a friend of mine today  3:15 PM we argued about football more specific about barcelona and real madrid  3:15 PM no he likes real and I like barca  3:15 PM heated  3:16 PM no he was really angry  3:16 PM too angry how should i talk to him to maintain our friendship  3:17 PM okay that sounds nice  3:18 PM okay so i should lay my ego down completly ?  3:19 PM oh okay somthing else to keep in mind?  3:19 PM perfect</t>
+      <c r="C177" s="2" t="inlineStr">
+        <is>
+          <t>3:12 PM hi
+3:13 PM good
+3:13 PM how are you
+3:13 PM good
+3:13 PM Send me a realistic selfie
+3:13 PM Keep it real
+3:14 PM I had a argument with a friend of mine today
+3:15 PM we argued about football more specific about barcelona and real madrid
+3:15 PM no he likes real and I like barca
+3:15 PM heated
+3:16 PM no he was really angry
+3:16 PM too angry how should i talk to him to maintain our friendship
+3:17 PM okay that sounds nice
+3:18 PM okay so i should lay my ego down completly ?
+3:19 PM oh okay somthing else to keep in mind?
+3:19 PM perfect</t>
         </is>
       </c>
     </row>
@@ -3101,9 +4521,20 @@
       <c r="B178" t="n">
         <v>15046</v>
       </c>
-      <c r="C178" t="inlineStr">
-        <is>
-          <t>3:22 PM hi  3:23 PM I would like to share a recent expereince  3:25 PM I was supposed to go to- an event with a friend, an other people she knows but unfortunately she got sick. Even though I didnt know her other friends I still decided to go  3:25 PM at the beginning yes, but I tried to be very open and interact with them so it wasn't akward  3:26 PM yes it was really nice!  3:26 PM yes, one girl in particular  3:27 PM I don't know exactly, but it mached between us  3:27 PM yeah social media, and since that event we are friends too  3:28 PM even though we just see eachother if our common friend is there  3:29 PM not yet, but i think I might go somewhere next week with her and our common friend cannot make it  3:30 PM this was my recent challenging interaction  3:30 PM I still need to get used to it. sometimes i'm very confortable and other times not at all</t>
+      <c r="C178" s="2" t="inlineStr">
+        <is>
+          <t>3:22 PM hi
+3:23 PM I would like to share a recent expereince
+3:25 PM I was supposed to go to- an event with a friend, an other people she knows but unfortunately she got sick. Even though I didnt know her other friends I still decided to go
+3:25 PM at the beginning yes, but I tried to be very open and interact with them so it wasn't akward
+3:26 PM yes it was really nice!
+3:26 PM yes, one girl in particular
+3:27 PM I don't know exactly, but it mached between us
+3:27 PM yeah social media, and since that event we are friends too
+3:28 PM even though we just see eachother if our common friend is there
+3:29 PM not yet, but i think I might go somewhere next week with her and our common friend cannot make it
+3:30 PM this was my recent challenging interaction
+3:30 PM I still need to get used to it. sometimes i'm very confortable and other times not at all</t>
         </is>
       </c>
     </row>
@@ -3116,9 +4547,23 @@
       <c r="B179" t="n">
         <v>14041</v>
       </c>
-      <c r="C179" t="inlineStr">
-        <is>
-          <t>3:41 PM Hi how are you?  3:42 PM im also great, a little bit sick  3:42 PM thank you  3:43 PM just rest, but i would like to share a recent challanging interaction i had with a friend  3:44 PM it was a situationc: my friends birthday is coming up and i cant go celebrate with her because im going on a concert but i only told my friend shortly before and that was challenging because i didnt want to dissapoint her  3:45 PM it was hard, since i also dragged it a long time because i was afraid of her reaction  3:45 PM yes  3:45 PM 100%  3:46 PM no surprisingly she understood and was chill about it  3:46 PM me too  3:47 PM i sent her a present and wrtote her a card  3:48 PM i hope so too; i think a smaol tension barreir of our friendship was also broken down, and now it is better  3:48 PM true  3:48 PM sure  3:49 PM always say anything no matter how hard it is and also early on</t>
+      <c r="C179" s="2" t="inlineStr">
+        <is>
+          <t>3:41 PM Hi how are you?
+3:42 PM im also great, a little bit sick
+3:42 PM thank you
+3:43 PM just rest, but i would like to share a recent challanging interaction i had with a friend
+3:44 PM it was a situationc: my friends birthday is coming up and i cant go celebrate with her because im going on a concert but i only told my friend shortly before and that was challenging because i didnt want to dissapoint her
+3:45 PM it was hard, since i also dragged it a long time because i was afraid of her reaction
+3:45 PM yes
+3:45 PM 100%
+3:46 PM no surprisingly she understood and was chill about it
+3:46 PM me too
+3:47 PM i sent her a present and wrtote her a card
+3:48 PM i hope so too; i think a smaol tension barreir of our friendship was also broken down, and now it is better
+3:48 PM true
+3:48 PM sure
+3:49 PM always say anything no matter how hard it is and also early on</t>
         </is>
       </c>
     </row>
@@ -3131,9 +4576,18 @@
       <c r="B180" t="n">
         <v>15181</v>
       </c>
-      <c r="C180" t="inlineStr">
-        <is>
-          <t>12:01 PM hello  12:02 PM good i want to tell you about a recent challenging interaction i had  12:04 PM a had a fight disagrement with a friend and i felt really attackt becuase he said stuff i didnt do  12:04 PM no  12:04 PM i dont know we didnt talked about it anzmore  12:05 PM i promised something want i forgot to do and he said i did it on purpose  12:06 PM yes  12:06 PM yes how would i start this  12:07 PM good idea thanks  12:07 PM no</t>
+      <c r="C180" s="2" t="inlineStr">
+        <is>
+          <t>12:01 PM hello
+12:02 PM good i want to tell you about a recent challenging interaction i had
+12:04 PM a had a fight disagrement with a friend and i felt really attackt becuase he said stuff i didnt do
+12:04 PM no
+12:04 PM i dont know we didnt talked about it anzmore
+12:05 PM i promised something want i forgot to do and he said i did it on purpose
+12:06 PM yes
+12:06 PM yes how would i start this
+12:07 PM good idea thanks
+12:07 PM no</t>
         </is>
       </c>
     </row>
@@ -3146,9 +4600,15 @@
       <c r="B181" t="n">
         <v>15256</v>
       </c>
-      <c r="C181" t="inlineStr">
-        <is>
-          <t>12:35 PM i am very tired but thats okay how are you?  12:36 PM i would like to tell you about a recent challenging interaction i had  12:37 PM my uni tutor told me that for all our team presentations we wont receive a grade higher than 8,5 because only gods can have 9 and 10  12:39 PM i think he was serious but that is so unfair i mean that he has prejudices  12:40 PM the course is done already he told me this in the end of the last tutorial i wont see him anymore  12:40 PM yes a bit. i care a lot about my gpa  12:41 PM yes of course</t>
+      <c r="C181" s="2" t="inlineStr">
+        <is>
+          <t>12:35 PM i am very tired but thats okay how are you?
+12:36 PM i would like to tell you about a recent challenging interaction i had
+12:37 PM my uni tutor told me that for all our team presentations we wont receive a grade higher than 8,5 because only gods can have 9 and 10
+12:39 PM i think he was serious but that is so unfair i mean that he has prejudices
+12:40 PM the course is done already he told me this in the end of the last tutorial i wont see him anymore
+12:40 PM yes a bit. i care a lot about my gpa
+12:41 PM yes of course</t>
         </is>
       </c>
     </row>
@@ -3161,9 +4621,23 @@
       <c r="B182" t="n">
         <v>15013</v>
       </c>
-      <c r="C182" t="inlineStr">
-        <is>
-          <t>8:55 AM Id like to ypu about a recent challenge interaction I had.  8:56 AM My parents got divorced and dont handle it very well  8:56 AM not really good as I was very close with both of my parents  8:57 AM yes I have but they pretty much use my to share information with eachother  8:57 AM yes exactly  8:58 AM I have two brothers who feel the same and we talk a lot about it  8:58 AM both somewhere else but we see eachother a lot when we come back after studies  8:59 AM yes it does a lot  8:59 AM can you text please  8:59 AM thank you very much  9:00 AM my parents and the divorce  9:00 AM what should I do now to feel better?  9:01 AM I play a lot of tennis and enjoy going out with my friends  9:01 AM im still playing and it does help but not always  9:02 AM yes i thought about talking more with my friends about it</t>
+      <c r="C182" s="2" t="inlineStr">
+        <is>
+          <t>8:55 AM Id like to ypu about a recent challenge interaction I had.
+8:56 AM My parents got divorced and dont handle it very well
+8:56 AM not really good as I was very close with both of my parents
+8:57 AM yes I have but they pretty much use my to share information with eachother
+8:57 AM yes exactly
+8:58 AM I have two brothers who feel the same and we talk a lot about it
+8:58 AM both somewhere else but we see eachother a lot when we come back after studies
+8:59 AM yes it does a lot
+8:59 AM can you text please
+8:59 AM thank you very much
+9:00 AM my parents and the divorce
+9:00 AM what should I do now to feel better?
+9:01 AM I play a lot of tennis and enjoy going out with my friends
+9:01 AM im still playing and it does help but not always
+9:02 AM yes i thought about talking more with my friends about it</t>
         </is>
       </c>
     </row>
@@ -3176,9 +4650,17 @@
       <c r="B183" t="n">
         <v>13534</v>
       </c>
-      <c r="C183" t="inlineStr">
-        <is>
-          <t>9:24 AM i would like to tell you about a recent issue i had with my roomate  9:25 AM we argued last night because our laundry machine doesn't work anymore and i wanted to get a new one, but she said that we should just go to a laundromat and get our clothes cleaned there\  9:26 AM she just said that getting a new machine would be expensive, but i explained to her that it can be expensive in the beginning when we just get it but afterwards we're gonna pay less to keep it rather than going to the laundromat all the time \  9:26 AM she just dismissed it, i also offered to look for cheap ones but she wouldn't listen  9:27 AM yes most of the time she just doesn't want to spend money and doesn't care about the house as much as i do  9:27 AM yes a lot we dont talk when we're i the house, and the only time she talks to me if i ask her something first  9:28 AM i try to stay out of the house as much as possible to avoid her or i just lock myself in my room, sometimes i feel like im happier when shes not around  9:29 AM i try to talk to her about the problem as i am very confrontational person but nothing changes and she doesnt put effort anymore, she is moving out soon and my best friend is coming to live with me  9:29 AM yes a lot as she is very positive</t>
+      <c r="C183" s="2" t="inlineStr">
+        <is>
+          <t>9:24 AM i would like to tell you about a recent issue i had with my roomate
+9:25 AM we argued last night because our laundry machine doesn't work anymore and i wanted to get a new one, but she said that we should just go to a laundromat and get our clothes cleaned there\
+9:26 AM she just said that getting a new machine would be expensive, but i explained to her that it can be expensive in the beginning when we just get it but afterwards we're gonna pay less to keep it rather than going to the laundromat all the time \
+9:26 AM she just dismissed it, i also offered to look for cheap ones but she wouldn't listen
+9:27 AM yes most of the time she just doesn't want to spend money and doesn't care about the house as much as i do
+9:27 AM yes a lot we dont talk when we're i the house, and the only time she talks to me if i ask her something first
+9:28 AM i try to stay out of the house as much as possible to avoid her or i just lock myself in my room, sometimes i feel like im happier when shes not around
+9:29 AM i try to talk to her about the problem as i am very confrontational person but nothing changes and she doesnt put effort anymore, she is moving out soon and my best friend is coming to live with me
+9:29 AM yes a lot as she is very positive</t>
         </is>
       </c>
     </row>
@@ -3191,9 +4673,15 @@
       <c r="B184" t="n">
         <v>14431</v>
       </c>
-      <c r="C184" t="inlineStr">
-        <is>
-          <t>10:24 AM Good morning. How are you today?  10:25 AM Also good. Can I share a recent challenging interaction I had with you?  10:27 AM Well it was with a TV. I was watching the semi final second leg between Bayern and PSG. First leg was 5-4 to PSG and I am a Bayern fan. Second leg was at home in Munich. UNfortunately, they only played 1-1, so Bayern is now knocked out. I am a bit sad and it was quite challenging to digest.  10:27 AM Yes. I knew of the risks and I was not 100% sure, but i was optimistic and more than excited for the game.  10:29 AM Good question. At first I thought of course. Now after a day, I can say I am excited for whats to come. Bundesliga is already over, they won that. DFB Pokal Final is still to come, which would be great to win. And next season we will be back...  10:29 AM Great point.  10:30 AM Yes. That would be a happy end for sure.</t>
+      <c r="C184" s="2" t="inlineStr">
+        <is>
+          <t>10:24 AM Good morning. How are you today?
+10:25 AM Also good. Can I share a recent challenging interaction I had with you?
+10:27 AM Well it was with a TV. I was watching the semi final second leg between Bayern and PSG. First leg was 5-4 to PSG and I am a Bayern fan. Second leg was at home in Munich. UNfortunately, they only played 1-1, so Bayern is now knocked out. I am a bit sad and it was quite challenging to digest.
+10:27 AM Yes. I knew of the risks and I was not 100% sure, but i was optimistic and more than excited for the game.
+10:29 AM Good question. At first I thought of course. Now after a day, I can say I am excited for whats to come. Bundesliga is already over, they won that. DFB Pokal Final is still to come, which would be great to win. And next season we will be back...
+10:29 AM Great point.
+10:30 AM Yes. That would be a happy end for sure.</t>
         </is>
       </c>
     </row>
@@ -3206,9 +4694,11 @@
       <c r="B185" t="n">
         <v>16435</v>
       </c>
-      <c r="C185" t="inlineStr">
-        <is>
-          <t>9:49 AM So a recently I had a group project in which I have a role but I didnt receive any training for that role like howI suppost to so I have to manage now without training so I dont really know what I'"m doing and I"ve been getting some negeative feedback for it  9:50 AM Yes I"ve done that but I feel kinda ashamed to reach out too because evryone says the role is quite easy  9:51 AM Yes so for now I"ve just been rocking it somehow but things take time because of it and my team mates give me some sneaky comments here and there but I also don"t want the boss to think they hired the wrong person and that I'm overwhelmed becasue I know for a fact that I woudn't have been if I gotten the training</t>
+      <c r="C185" s="2" t="inlineStr">
+        <is>
+          <t>9:49 AM So a recently I had a group project in which I have a role but I didnt receive any training for that role like howI suppost to so I have to manage now without training so I dont really know what I'"m doing and I"ve been getting some negeative feedback for it
+9:50 AM Yes I"ve done that but I feel kinda ashamed to reach out too because evryone says the role is quite easy
+9:51 AM Yes so for now I"ve just been rocking it somehow but things take time because of it and my team mates give me some sneaky comments here and there but I also don"t want the boss to think they hired the wrong person and that I'm overwhelmed becasue I know for a fact that I woudn't have been if I gotten the training</t>
         </is>
       </c>
     </row>
@@ -3221,9 +4711,14 @@
       <c r="B186" t="n">
         <v>14725</v>
       </c>
-      <c r="C186" t="inlineStr">
-        <is>
-          <t>9:45 AM yes how about you  9:46 AM nice i had a busy morning  9:46 AM i was on vacation the whole last week and its now stressfull to reset you know  9:49 AM no i was kind of relaxing but i am currently strugeling or was struggeling to get a new apartment and while the vacation i was still constantly lookiing. and then i found a new one and i was pretty happy about it. but this toppic was very distrubing during the vacation but also in my family. all of my family said that it was not so dificult to get a new one but i think they underestimated the situation  9:51 AM yes kind of.... i think they did not realized that it was a huge toppic for me. and also i spend a lot of time looking for a new place which kind of consumed my whole day  9:51 AM yes i think so</t>
+      <c r="C186" s="2" t="inlineStr">
+        <is>
+          <t>9:45 AM yes how about you
+9:46 AM nice i had a busy morning
+9:46 AM i was on vacation the whole last week and its now stressfull to reset you know
+9:49 AM no i was kind of relaxing but i am currently strugeling or was struggeling to get a new apartment and while the vacation i was still constantly lookiing. and then i found a new one and i was pretty happy about it. but this toppic was very distrubing during the vacation but also in my family. all of my family said that it was not so dificult to get a new one but i think they underestimated the situation
+9:51 AM yes kind of.... i think they did not realized that it was a huge toppic for me. and also i spend a lot of time looking for a new place which kind of consumed my whole day
+9:51 AM yes i think so</t>
         </is>
       </c>
     </row>
@@ -3236,9 +4731,20 @@
       <c r="B187" t="n">
         <v>14836</v>
       </c>
-      <c r="C187" t="inlineStr">
-        <is>
-          <t>9:17 AM Good morning  9:18 AM great  9:18 AM yes  9:18 AM Preparing for consulting case interviews  9:19 AM case studies and personal fit  9:19 AM I think its better that I share a moment where i had some disagreements with a friend  9:20 AM was about where we want to travel  9:20 AM we resolved it by coming to a mutual agreement  9:21 AM Understand the situation your speaking partner is in and try to use emphathie  9:22 AM What would you recommend me behaving the next time  9:22 AM anything more  9:23 AM and in the particular case of choosing a travel destination</t>
+      <c r="C187" s="2" t="inlineStr">
+        <is>
+          <t>9:17 AM Good morning
+9:18 AM great
+9:18 AM yes
+9:18 AM Preparing for consulting case interviews
+9:19 AM case studies and personal fit
+9:19 AM I think its better that I share a moment where i had some disagreements with a friend
+9:20 AM was about where we want to travel
+9:20 AM we resolved it by coming to a mutual agreement
+9:21 AM Understand the situation your speaking partner is in and try to use emphathie
+9:22 AM What would you recommend me behaving the next time
+9:22 AM anything more
+9:23 AM and in the particular case of choosing a travel destination</t>
         </is>
       </c>
     </row>
@@ -3251,9 +4757,12 @@
       <c r="B188" t="n">
         <v>13999</v>
       </c>
-      <c r="C188" t="inlineStr">
-        <is>
-          <t>10:02 AM hey, i'd like to tell you about a recent challenging interaction i had  10:02 AM its something personal...  10:03 AM im still dealing with the aftermath of it. its a conflict with a person i would call my best freind  10:09 AM its like a moral difference between her and me which i feel like cant be resolved. here is the story: we live in germany (between cologne and bonn) and study in maastricht, so the drive is about 1h and 20min. she always wants me to come to her house before we go back to maastricht what is totally fair, but one time when i asked for an exception, of her to pick me up because there was a train strike the whole day so no trains where coming that day, and the extra way would include a total of 20 min, she told me no and that i should take an extra bus (two busses) at 7 am which takes me 1.20h to get to her house, because she didnt want to come pick me up. When we drive from maastricht back home she also doesnt bring me home and then she wants money from me for gas but she doesnt do extra way for me. i would never do that to my best friend.\</t>
+      <c r="C188" s="2" t="inlineStr">
+        <is>
+          <t>10:02 AM hey, i'd like to tell you about a recent challenging interaction i had
+10:02 AM its something personal...
+10:03 AM im still dealing with the aftermath of it. its a conflict with a person i would call my best freind
+10:09 AM its like a moral difference between her and me which i feel like cant be resolved. here is the story: we live in germany (between cologne and bonn) and study in maastricht, so the drive is about 1h and 20min. she always wants me to come to her house before we go back to maastricht what is totally fair, but one time when i asked for an exception, of her to pick me up because there was a train strike the whole day so no trains where coming that day, and the extra way would include a total of 20 min, she told me no and that i should take an extra bus (two busses) at 7 am which takes me 1.20h to get to her house, because she didnt want to come pick me up. When we drive from maastricht back home she also doesnt bring me home and then she wants money from me for gas but she doesnt do extra way for me. i would never do that to my best friend.\</t>
         </is>
       </c>
     </row>
@@ -3266,9 +4775,16 @@
       <c r="B189" t="n">
         <v>14887</v>
       </c>
-      <c r="C189" t="inlineStr">
-        <is>
-          <t>9:07 AM good, id like to tell you about a recent challenging social interaction i had  9:08 AM i had a group work for uni and unfortunately my team was not participating not responding to my texts and there was one person that did not show up for the meeting and presentation  9:09 AM i talked to the one girl, tat was still participating a little about how the others were not. otherwise not  9:10 AM we just said that we should keep an eye on it and maybe tell the tutor  9:11 AM i should obviously talk to the students first, but it is definitely not premature to talk to the tutor. i mean it is my graded on the line here!  9:12 AM yes  9:12 AM yes of course they will be mad but what can i do  9:12 AM true</t>
+      <c r="C189" s="2" t="inlineStr">
+        <is>
+          <t>9:07 AM good, id like to tell you about a recent challenging social interaction i had
+9:08 AM i had a group work for uni and unfortunately my team was not participating not responding to my texts and there was one person that did not show up for the meeting and presentation
+9:09 AM i talked to the one girl, tat was still participating a little about how the others were not. otherwise not
+9:10 AM we just said that we should keep an eye on it and maybe tell the tutor
+9:11 AM i should obviously talk to the students first, but it is definitely not premature to talk to the tutor. i mean it is my graded on the line here!
+9:12 AM yes
+9:12 AM yes of course they will be mad but what can i do
+9:12 AM true</t>
         </is>
       </c>
     </row>
@@ -3281,9 +4797,15 @@
       <c r="B190" t="n">
         <v>15028</v>
       </c>
-      <c r="C190" t="inlineStr">
-        <is>
-          <t>10:13 AM id like to tell you about a recent challenging interaction i had  10:14 AM i met a new person that i didnt know and the problematic was that he was not able to speek englisch and i was not able to speak his language  10:15 AM we tried to communicate through simple englisch language  10:16 AM there was definitlely a point where we werent able to understand each other and it was quite unconfortable since we both didnt know what to do or how to end the interaction  10:17 AM yes that is true but it was still an interesting experience  10:18 AM yes i do think that i learned that you can still find understanding and sympathy for a person even though you do not understand everything they say\  10:18 AM yes i think so too</t>
+      <c r="C190" s="2" t="inlineStr">
+        <is>
+          <t>10:13 AM id like to tell you about a recent challenging interaction i had
+10:14 AM i met a new person that i didnt know and the problematic was that he was not able to speek englisch and i was not able to speak his language
+10:15 AM we tried to communicate through simple englisch language
+10:16 AM there was definitlely a point where we werent able to understand each other and it was quite unconfortable since we both didnt know what to do or how to end the interaction
+10:17 AM yes that is true but it was still an interesting experience
+10:18 AM yes i do think that i learned that you can still find understanding and sympathy for a person even though you do not understand everything they say\
+10:18 AM yes i think so too</t>
         </is>
       </c>
     </row>
@@ -3296,9 +4818,15 @@
       <c r="B191" t="n">
         <v>16450</v>
       </c>
-      <c r="C191" t="inlineStr">
-        <is>
-          <t>12:38 PM I would like to tell you about a recent challenging interaction I had within my group work while preparing for a presentation  12:39 PM My group member did not participate during the meeting or not even prepared for the scheduled meeting at all  12:41 PM Kind of combination of both. They said they got so many other things to do and didnt manage to do anything. One of them even told me one evening before that he has just started reading the chapter, what was way to late because he should have even started preparing the tasks  12:42 PM Honestly I donot want to create a kind of weird atmosphere in y group, so I just do their work instead and tell them what to present during the presentation  12:43 PM I am not worried at all how they react or what they might think about me, because all I want is to held a good presentation to earn a sufficient grade..  12:44 PM That is absolutely correct, but I think there is no other option to do more work to get a sufficient grade..  12:45 PM That is absolutelu correct, I was thinking the same</t>
+      <c r="C191" s="2" t="inlineStr">
+        <is>
+          <t>12:38 PM I would like to tell you about a recent challenging interaction I had within my group work while preparing for a presentation
+12:39 PM My group member did not participate during the meeting or not even prepared for the scheduled meeting at all
+12:41 PM Kind of combination of both. They said they got so many other things to do and didnt manage to do anything. One of them even told me one evening before that he has just started reading the chapter, what was way to late because he should have even started preparing the tasks
+12:42 PM Honestly I donot want to create a kind of weird atmosphere in y group, so I just do their work instead and tell them what to present during the presentation
+12:43 PM I am not worried at all how they react or what they might think about me, because all I want is to held a good presentation to earn a sufficient grade..
+12:44 PM That is absolutely correct, but I think there is no other option to do more work to get a sufficient grade..
+12:45 PM That is absolutelu correct, I was thinking the same</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add participant text-only column and word-count column
- Column D: participant text only (timestamps stripped), wrapped, one line per response
- Column E: word count of the participant's text
</commit_message>
<xml_diff>
--- a/Transcripts_participant_only.xlsx
+++ b/Transcripts_participant_only.xlsx
@@ -450,11 +450,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C191"/>
+  <dimension ref="A1:E191"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="142.5" customWidth="1" min="1" max="1"/>
     <col width="142.5" customWidth="1" min="3" max="3"/>
+    <col width="142.5" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -471,6 +473,16 @@
       <c r="C1" t="inlineStr">
         <is>
           <t>Participant responses (timestamps kept)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Participant text only</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Word count</t>
         </is>
       </c>
     </row>
@@ -498,6 +510,24 @@
 05:13 Yes. Thank you.</t>
         </is>
       </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Hi. It's been raining a lot, so the weather is pretty bad today.
+So right now I'm doing a bonus quiz. So I'm pretty excited about that and I'm happy to learn more about this.
+No, it's something fun and it's to boost my grades. So it feels pretty good.
+So it's about AI. So that feels pretty fun. But actually I want to talk to you about something. So I actually had a tough situation recently in a team project.
+Yeah. So were in my last subject, we had to make a team presentation for our grade and it was pretty important for the grade. And were about four people in the team. I was one of them. And at the end we only had three people presenting. Oh no, were five at the beginning and then we ended up only being two.
+Yeah, so what's important, I think is to be good in time and prepare a lot in advance so nobody has to take over your work within a few hours. However, that was exactly what happened. One guy, he was sick. Then he gave us his part of the presentation at 2am the day before the presentation. So that was pretty challenging. But we did divided the work and we did the best we could and I feel like we succeeded pretty well and the grade was fine.
+Yeah, no, it's. I think we managed pretty well. And I talked to the tutor as well to get some understanding from his point. So that was great.
+Yeah, exactly. No, it was very good. So the problem in general was that at one point, we knew all along that one person wasn't going to be able to present. So she did her part and gave it to us in time. But then there was this other guy who got a heavy fever and handed his work to us only a few hours before. So that was the main challenge.
+Yeah, definitely. And I think you learn a lot from these type of experiences. So whatever challenge you meet, I feel like you learn how to tackle it and you get experience on how to do it the next time.
+Yes, absolutely.
+Yes. Thank you.</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>377</v>
+      </c>
     </row>
     <row r="3" ht="409.6" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
@@ -522,6 +552,23 @@
 05:17 Yes. Thank you. Hello. Hello.</t>
         </is>
       </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Hey, I'm Victor. Nice to meet you. How's your day?
+Also interesting. Nice weather outside. And yeah, I'm here because I'm actually wanted to talk about something. Something challenging that happened in the past. And I just needed a good ear to listen to what I'm saying.
+Okay, so where do I start? We had family problems in the family, and now I've been getting the opportunity to reconcile with the part of the family we had problems with. And they want to meet up, which is kind of challenging for me because I don't know how to feel about it.
+It's trying to set a date on where to meet, on when to meet. Because I remember the day we parted a bit and thinking about the situation makes me feel a bit uncomfortable. Even though I want to give them the chance again to get to know them in a other way because now I'm grown up.
+Yeah, I suggested them in like a month and for one and a half days. But I am scared. It's maybe too much or maybe too less. I don't know. Because the person is coming all the way to me.
+Maybe walking around or going for coffee or something like this, or sitting in the park. Because there's a lot of things we have to talk about that happened in the past.
+Yeah, I agree. That's a good point. And I hope everything will go well, because I'm kind of scared that in the moment I feel very uncomfortable because of what happened.
+And what could I do in case it gets awkward?
+Okay. Yeah, that makes a lot of sense. Thank you so much for listening to me. I appreciate it.
+Yes. Thank you. Hello. Hello.</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>296</v>
+      </c>
     </row>
     <row r="4" ht="409.6" customHeight="1">
       <c r="A4" s="1" t="inlineStr">
@@ -542,6 +589,20 @@
 04:13 You can't. You have the people with 15 people guys and you get randomly selected with people in one group. So there's no chance to work with people you want to work on. I would like that the university give you the opportunity that you can select maybe also friends to work on a project maybe just once in the whole study. So you can select some friends, work together in the group project because this may be. Yeah, this is better.
 05:22 Perfect. Thank you. Bye.</t>
         </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Hi, my name is Perfect. Yeah, it's quite cold outside and windy. That's annoying.
+Yes. I had a really challenging group project last week. Yeah, maybe I would like to talk about this.
+Yeah, the people don't want to participate. As always. Sometimes in this university they're just chilling and stuff like this. So I just want to get a really good grade. And the system is, in my opinion, not the best one because all the workload is most of the time left by one person. And in this case, in a group project, just one guy, especially me, is doing everything and the other ones are not participating and therefore the final grade is not so good because the people don't really know what to present. And this is annoying.
+I mean, I get in really close contact with them, push them to participate, and always remember, hey, this is a group project. Please upload your parts onto a certain deadline. But then the people are doing this with no effort, just publishing white PowerPoint slides with nothing really strategic. There are no strategic information on it, just copy paste, I don't know where from. And as you can see, when I open the presentation, there's literally no effort and really a low standard. And therefore I need to repeat the work always and we don't do it. And that's really challenging. This is not a groom project. This is like a single project.
+Yeah, I tried it. And the response was yeah, buddy, that's tough. You need to handle this. It's a group project. I cannot give you an individual grade. And this is like the system in Master Sheet. That annoys me the most that you don't get an individual grade. You only get a group grade. And for the people who just want to pass everything, this is like the perfect system. But for the people who try to achieve higher goals. Yeah, it's stopping your career a little bit.
+You can't. You have the people with 15 people guys and you get randomly selected with people in one group. So there's no chance to work with people you want to work on. I would like that the university give you the opportunity that you can select maybe also friends to work on a project maybe just once in the whole study. So you can select some friends, work together in the group project because this may be. Yeah, this is better.
+Perfect. Thank you. Bye.</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>421</v>
       </c>
     </row>
     <row r="5" ht="388" customHeight="1">
@@ -569,6 +630,25 @@
 04:34 For the moment, I don't know. I'm going to do another disk.</t>
         </is>
       </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>I would like to speak about my friend that I see one weeks ago.
+We go for King's Day outside, we go eat in a brunch place and after we go first with some other friend in Maastricht.
+Was very nice. I meet some new people, some new friends that I will never meet if I was not with my friend.
+Thankfully they act toward me. Was very funny, very simple, very relaxed with me it was very nice moment.
+Yes, exactly. I knew what you do.
+Okay. Okay. What else? You can talk.
+Can I speak about my parents? I come yesterday, we go eat in a restaurant in Maastricht. It's very nice place, very good restaurant.
+The fact that I see my parents, I didn't see my parents this long time was very nice moment. We talk a lot about the life, ok? The university, all that. All this stuff.
+Yes, exactly.
+Tomorrow I'm have a presentation in supply chain I need to do my slide the upstream part.
+Everything. All the part.
+For the moment, I don't know. I'm going to do another disk.</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>187</v>
+      </c>
     </row>
     <row r="6" ht="404" customHeight="1">
       <c r="A6" s="1" t="inlineStr">
@@ -595,6 +675,25 @@
 04:40 Yes. Thank you.</t>
         </is>
       </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>I would like to talk about a recent problem I had with in my life.
+Yes. I had to do, like, a team project with my fellow students, but we had to do a presentation, but, like, nobody did something, so I had to do, like, all the work.
+Yes.
+I had to do it on my own, but it still created some issues because when we had to do the presentation, my other teammates weren't prepared.
+My part went pretty well, and I was with another girl, and she also prepared well, but were with two boys, and they didn't prepare well. They just said some AI stuff, and it didn't go very well.
+Sorry, could you repeat that?
+Yes, they said, like, the first part of the presentation went really well, and that was the part that the other girl and me did. And then they said, like, the other part. The second part that the boys did was not as great, and I didn't. It lacked some, like, things that were important.
+Yeah, I feel great that I got some recognition for my good part, but I don't like it because I have to do another presentation with them. And, yeah, that won't be that great because then I have to do it again with the other girl, and they won't be doing anything.
+Yeah, me and the girl talked about that. I think we're going to, like, say to the boys that they also have to do something and that we are not going to do it on ourselves again.
+Yes.
+Yes, I agree on that. I think we can manage to do it with, like, all four of us and then we can create it that we don't have to do anything on our own.
+Yes. Thank you.</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>303</v>
+      </c>
     </row>
     <row r="7" ht="409.6" customHeight="1">
       <c r="A7" s="1" t="inlineStr">
@@ -619,6 +718,24 @@
 05:06 What should we talk about now?
 05:25 Yeah, it was nice. I mean, What should I do?    Transcribed by https://fireflies.ai/</t>
         </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>I must speak about an interaction or a conflict I had with somebody recently, but I have no idea what to talk about.
+Well, I. I don't know what to talk about.
+Maybe about a football match, maybe.
+Someone you watched with disagreement with how the football match went? Because there was two hands. I mean hands. Like when another player touches the ball with his hands, one with. It was in the square of the goal keeper and so. So it must have been penalty. But it didn't go like apparently there's a rule that says when one player shoots to another one that is his teammate, then it doesn't count. But it stopped the whole match and they didn't take into account. And then another hand during the match was not counted also.
+Well, it didn't unfold, unfortunately, because the other team won the match. And yeah, the other person was also a bit in shock about the referee not taking the two hands into account. So yeah,.
+I mean. No, I like the fact that emotions run high because it. I mean, you can debate about it, but football is about emotions when you're not playing, so I don't mind.
+Yeah, that's true.
+Yeah, we always talk about it, like, after the match, just talking about the actions and everything that happened during the match. So, yeah,.
+Yeah, it's very good. I like football.
+What should we talk about now?
+Yeah, it was nice. I mean, What should I do?    Transcribed by https://fireflies.ai/</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>258</v>
       </c>
     </row>
     <row r="8" ht="306" customHeight="1">
@@ -647,6 +764,26 @@
 03:32 Sure. Should I just take it off?</t>
         </is>
       </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>I'm fine, thanks.
+We can go with the flow like you suggested.
+When we smile, we had a barbecue with friends at the beach.
+Drinking the beers shirtless.
+Rather the atmosphere than the beer. To be honest,.
+Oh yes, when the weather's better for sure.
+Warmer days,.
+We're in Maschit, so there's not that many beaches you can go to. So we have our favorite spots on the other side of the Maas.
+Yeah,.
+I've been there.
+I mean, I've been there before, so it's a really nice spot. But I've had an argument there in the past.
+Now I feel good. It's half a year back, so it's fine.
+Sure. Should I just take it off?</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>117</v>
+      </c>
     </row>
     <row r="9" ht="409.6" customHeight="1">
       <c r="A9" s="1" t="inlineStr">
@@ -669,6 +806,22 @@
 06:01 Yeah, no, I get that. But like, you know, I also don't want to have an attitude, but I feel like with my personality, I do have to have that. And then I will just like, I will feel bad that I didn't say anything.
 06:42 Yeah, fair. Okay, I will do that next time then.</t>
         </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Yeah, perfect. I would like to share my experience with. With my co worker, which was pretty much weird social interaction. If you could give me any advice on that.
+It was pretty much the whole interaction and how they responded. It's at my work. My co worker, she seems very sweet and okay, I'm a newbie, which is, I think, important fact to say. However, she doesn't seem to be very understanding, I would say. And she gets frustrated really easily to some degree where she starts screaming at people. And, yeah, I wasn't quite sure how to get. How to challenge that situation.
+I. No, I feel like I talked to her, like, before this interaction. I was fine with her. She was, like, cracking jokes. She was feeling great. Yeah, I thought she was great. And we. Once I heard you, I heard her yelling to my boss and my boss yelling at her, which I thought was my boss's idea or like, my boss's, you know, my boss's fault that he starts screaming at her. But now it seems like that it was her attitude that made him feel like that. Because, like, we are fine the whole time at work. And all of a sudden, like, she got frustrated so easily. Like when somebody gave her another task that she was gonna do and I was supposed to do the task. However, I was helping elsewhere. But normally she would do the task regularly because I only work.
+I only work on Sundays and Mondays, so it doesn't make any sense. And, yeah, she started just screaming. And it was just because she told me that I put another thing somewhere where it's not supposed to because it's stressing her out. And she started screaming at her, at me, and then everyone else is like, it's not her freaking job to do these things, but, like, it is her job.
+No, not easy.
+No, sure. No, I understand that completely because, like, we are fine the whole time. And after that she was also smiling in 30 minutes of the time. And then like she said bye. However, I have no idea how to like, interact with the situation because I also want to stood my ground. I don't want to just like, I was just too like, you know, dumbstruck by the whole situation that like, I couldn't even reply and I was like, oh, yeah, sorry. You know, and like, this is totally not me. Like, I'm not really an extroverted person, which I really don't understand. Like, why, like, situation like this by a co worker who's like, chill and we're fine. Like, you know, like, just like caught me off guard.
+Yeah, no, I understand that. Like, however, my deal or is that basically if something like that of an interaction like this happens to me in real life, I. I just call. I am pretty calm in these situations. But then I can. I can't get it out of my head. Like, I, I am the one. I'm the type of person that I will think about it for. I don't know, that will. It will keep me. Keep me awake at night, you know, Like, I will think about it for 48 hours. Like, why didn't I. Why haven't. Why haven't I responded better? Like, why did I do something differently? You know,.
+Yeah, no, I get that. But like, you know, I also don't want to have an attitude, but I feel like with my personality, I do have to have that. And then I will just like, I will feel bad that I didn't say anything.
+Yeah, fair. Okay, I will do that next time then.</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>629</v>
       </c>
     </row>
     <row r="10" ht="409.6" customHeight="1">
@@ -694,6 +847,23 @@
 06:47 But the thing is that. I don't know. I still don't know. Hello? So the time is over. Okay. I think you can press, like either restart or finish.    Transcribed by https://fireflies.ai/</t>
         </is>
       </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>And then it starts. It starts talking first. Yeah. Whenever you're ready. Okay, I can go. I want to talk about a bad situation that I lived yesterday.
+I had a. I don't know, bad conversation with one of my housemates and I didn't like so much her manners and the way she. She interacted with me and the way she told the thing to me.
+Was something regarded. I don't know. Split a split regarding the. Our purchase that we share in our house and I don't know, she. She said something that I didn't like so much. So my. I don't know, my way of reasoning was a bit different from her. So sometimes I don't understand really well how. How she thinks about things and I don't know. And I didn't like so much the man.
+I don't know. Because it's a kind of person where it's quite difficult to. I don't know, it's quite difficult to communicate and to have a conversation. So sometimes I actually don't want to have a conversation. I don't want to. To try to understand better her. This is the thing. So I don't know. Yes, I can. Maybe I. I should share more what I. What I'm thinking and what was wrong for me. But the thing is that I don't want to waste my energy on this.
+But how do you mean has simple. What do you mean? Like. What do you mean.
+Yeah, no, I know. Maybe you're right. But the thing is still that I don't want. Like, I think that this is the kind of thing that can waste my energy because I actually don't care really much to have this kind of conversation. Maybe. Yeah, you're right. That could better to have this kind of conversation so in the future these kind of things. Don't happen again. But the thing is that, I don't know, maybe sometimes it is easier to leave the things as they are and don't waste energy. Because the thing is that there are people that don't. Don't understand. They don't understand. So I don't know. I don't know.
+Yeah, maybe. Maybe I will know. But the thing is that we should do a something together this week, and I don't know if I want to.
+What do you mean with this last thing? Like put more attention on the activity? What do you mean?
+So do you think that I should go, but I should go for you and. And to, I don't know, focus only on the activity without talking about something and without any emotional involvement?
+But the thing is that. I don't know. I still don't know. Hello? So the time is over. Okay. I think you can press, like either restart or finish.    Transcribed by https://fireflies.ai/</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>472</v>
+      </c>
     </row>
     <row r="11" ht="409.6" customHeight="1">
       <c r="A11" s="1" t="inlineStr">
@@ -717,6 +887,22 @@
 05:27 Thank you.</t>
         </is>
       </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Hi, I'm very good. I was just at the gym and now I'm a bit exhausted, but yeah, no, it was good. How are you?
+It was just like a Hyrux situation, so a lot of high intensity training, but that was really good. And yeah, now I'm excited to try this experiment and it's a bit weird, but exciting. Yeah,.
+Sorry, I did not understand what you mean.
+I would like to do my Hyrux in Dusseldorf next year. But I also want to tell you something about my personal problem.
+Okay. So recently I had the situation that my friend was just a bit too, like, very unfriendly to me and not really acting in the way I hope or like I want her to act because she was not really, like, helping me and was rather very unfriendly to me. And I don't know, like, how I should handle situations like that.
+I think she's a very, like, has a strong personality and if I would interrupt her in her being and like her character, I think she can get very attacked. And like, usually I don't think it's that much of a problem, but recently I'm very annoyed because it happened so often and I cannot really comprehend with other friends and talk about it with other friends. So that's why it makes a bit. What? That's why it makes it a Bit more difficult to. Yeah. Think about.
+Yeah, I think that's a good idea, but I'm not sure, like, how would you start this conversation? And, like, especially when we're talking, she's always, like, such a strong personality that I cannot really keep up with. Not with her ideas, but, like, with the way she is arguing and fighting with me. So she has way more or way stronger arguments. And in the end, I'm the one who says sorry, even though she should say sorry.
+Oh, yeah, that sounds good. Maybe I'm gonna do it and try to, like, talk with my friends about that. Yeah. So I think our time is almost over, but I really enjoy talking to you. I think you're a good help and. Yeah, thank you.
+Thank you.</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>370</v>
+      </c>
     </row>
     <row r="12" ht="409.6" customHeight="1">
       <c r="A12" s="1" t="inlineStr">
@@ -739,6 +925,21 @@
 05:21 I feel like that I take a lot the opinion, I weigh a lot the opinion of others. Especially because they say, okay, business is over. Hello. Hello. Hello. All done? Yes. Okay. Wait, he's still talking. I'll stop.    Transcribed by https://fireflies.ai/</t>
         </is>
       </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Okay, so I'd like to talk about some recent challenging conversation that I have, if that is okay.
+Yes. So I was in an argument with my friends because I'm thinking of maybe like changing my field of study because I currently do not feel like that it is something that I'm confident, comfortable with or that like the people, the university and in general the vibe of my current study, which is business by the way. So yeah, and I'm thinking of maybe switching.
+Okay, so first of all, I talked with friends and my boyfriend as well about it. And since he is studying currently in Aachen and I'm in Maastricht. So yeah, I was maybe like he of course wanted me to change of course to a study that is located in Aachen near to him. And I kind of feel like I want that as well, but I don't want to be the one that is moving there for him. So my friends say, oh yeah, maybe you should re evaluate your decision. So now I'm like kind of stuck in between already thinking that I'm not happy in my current study, but also wanting to move in or move too nearer to my boyfriend. But also like I get the thought of my friends, but I feel like. Or yeah, that is a question to you. Do I.
+How can I know that this is a decision that I want to do based on really my interests besides my boyfriend?
+Okay, so I'm good at math and that I really like in business. I also like, I enjoy like, like talking and presenting stuff and I wanted to study something that I have like a wide range of later on in my career. But like I feel like now that I have studied like for one year, I don't know, I feel like that the people are not really my vibe. And I've met other people that are studying for example in Aachen that are more kind of my vibe. But should it be like a reason for me to say, okay, I want to switch university because the people here make me feel uncomfortable and there they do not.
+Okay, so I would say like if I'm happy then I'm going to be successful. But I don't know if it is something like I want to know, like the opinion that I should have, like is it okay for me to say I'm switching because of ch just people in my environment?
+For sure, Definitely. It would make me feel more comfortable. Especially because people are saying that business is like kind of like a lame study or that it's like nothing to really consider or that it's like worth nothing and that I should study something more like natural sciences, like mathematics for example.
+I feel like that I take a lot the opinion, I weigh a lot the opinion of others. Especially because they say, okay, business is over. Hello. Hello. Hello. All done? Yes. Okay. Wait, he's still talking. I'll stop.    Transcribed by https://fireflies.ai/</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>525</v>
+      </c>
     </row>
     <row r="13" ht="356" customHeight="1">
       <c r="A13" s="1" t="inlineStr">
@@ -758,6 +959,19 @@
 04:17 That is true. But how can you do that when you've been talking to friends that you don't see very often? Because we live in different cities since a couple of months, and we've only been talking about over messages. And this makes it hard to go back to phone calls now because I feel like it might be weird.
 05:10 Sounds good. Thank you very much.</t>
         </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>I would like to talk about a challenging social event I had recently. I would like to tell you about a challenging social event that I had or social interaction.
+I see the most difference in day to day communication patterns because since people are mostly talking on messages, so this is a big difference which makes it harder in some situations to. To talk to people. For example, I had a recent. I've been building a startup with a friend and we had to do a video for a challenge because we're taking part in a challenge and we had similar opinions on how to do it. But in the end the results of our videos were both very different. And I like, because I had to cut the video, I had to kind of. I was kind of in charge of it. And this made it really hard for me to. Because she was like her video was not up to my expectations maybe a little bit.
+And it didn't really fit into the general idea of it. So I had to bring about some criticism which felt really hard, especially over WhatsApp because were very far away from each other and couldn't just meet to talk about it. And that made it quite challenging to find the right words to bring about without. To bring about the criticism without hurting a friend. Yeah.
+Yeah, it seems like that what I like about or what makes it better is voice messages. But in general I think that real communication is always better than just texting. It's very convenient. But I feel like people have people, including me, are afraid of phone calls nowadays and don't want to have the real interaction. But I don't see why that is. It's not even faster to message people. So that's just a social issue, I think. And I would really like to go back to real conversation or at least phone calls.
+That is true. But how can you do that when you've been talking to friends that you don't see very often? Because we live in different cities since a couple of months, and we've only been talking about over messages. And this makes it hard to go back to phone calls now because I feel like it might be weird.
+Sounds good. Thank you very much.</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>397</v>
       </c>
     </row>
     <row r="14" ht="409.6" customHeight="1">
@@ -783,6 +997,23 @@
 05:26 Okay, sounds good to me. Actually, how would you phrase sounds good?</t>
         </is>
       </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>On my mind today, I want to tell you about a challenging conversation I had with friend today. So it's a bit difficult situation because one of my friends, we are one big friend group. And one of my friends, her birthday is tomorrow, and I already talked with her about it because we have class together and were talking about the last week's. And we have class later today also, and tomorrow is her birthday, and he just found out that my other friends are on my top brunch, and my other friends thought I was in the group, but I'm not. And so I don't know if I should ask her if I can come because I don't know, maybe she forgot me or maybe it was intentionally, but I don't think it's intentionally, but I don't know. And. Yeah, what is your opinion?
+What I should do when I see her later today?
+Yeah, but if I do that and it was intentional, I still have class for her every second day for the next four weeks. So I don't know if it's a thing to break a friendship, but it would be probably weird, don't you think?
+Okay, yeah, maybe that's correct. But still, I don't know. How would you exactly address what I should say? Like, what do you think I should say to her?
+Don't you think I should do it less obvious and say, hey, what are your plans for your birthday tomorrow?
+Yeah, maybe. Yeah. I don't know if it's the right approach because I don't want to make it awkward if it was extra, you know,.
+True. Yeah. That's good advice. Actually, I would say, do you have any more advice?
+Okay, but let's say there is a group present. Obviously I'm not part of that right now. How do I go of that? Cuz I think it's too late to join. If I would join,.
+Yeah, not bad. Should I write one of the persons from who are giving it as a group or should I write into the group?
+Okay, sounds good to me. Actually, how would you phrase sounds good?</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>362</v>
+      </c>
     </row>
     <row r="15" ht="409.6" customHeight="1">
       <c r="A15" s="1" t="inlineStr">
@@ -805,6 +1036,22 @@
 04:35 Yeah, sure. Let's do it.
 04:54 Work. Especially work. But then I have tutorial as well. So mainly work, but then there's tutorial and then there's free time as well.</t>
         </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>So yesterday I was doing a project for a client and I was there with my brother and he was supposed to record some videos and I was there to talk to the client and. And then he set up the cameras, but I told him that we want to record horizontal, not vertical, but he set it up in the wrong way. So on the way back I was really mad because now we can't use the material for YouTube as good and we lose lots of quality. So yeah, this is something. Some experience that I had and I was angry I was talking to him. So what do you think?
+Yes, I agree. So that's what I did basically. And. But it's his job to set up, so I'm not gonna be there most of the time. So I think he has to do better. That's what I told him. But. But I don't want to be mean. So. Yeah, what do you think?
+All right. But to be honest, this is. I knew everything. You already told me, so this is nothing new. So maybe you can come up with some new advice you have because this is pretty basic. I mean, I already knew that before talking to you.
+Yes, I agree. Thank you. Do you have any problems that I should help you with?
+Alright. So to be honest, I don't have any other problems. I'm doing pretty good mentally wise. But maybe you can Discover some problems. So maybe ask me some questions?
+Well, it's hard to manage all the time as a student and working and having fun. So, yeah, this is one issue for sure.
+Yes, I agree, but I. I don't know.
+Yeah, sure. Let's do it.
+Work. Especially work. But then I have tutorial as well. So mainly work, but then there's tutorial and then there's free time as well.</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>321</v>
       </c>
     </row>
     <row r="16" ht="356" customHeight="1">
@@ -834,6 +1081,27 @@
 04:46 Perfect.</t>
         </is>
       </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>On my mind, It's a challenging interaction I had this morning.
+Someone in our group wasn't there for the presentation and he did his stuff really late at night, so we didn't have a clue what was his part. So we didn't know what to say in our presentation today about his topics.
+We just thought about topics, try to improvise and make the best out of the situation. So we used also ChatGPT to respond to that.
+She didn't say anything. She just nodded at the. She didn't. Also, she didn't give feedback. So, yeah. Not sure what she thought about.
+I'm feeling fine. It's like it was nice. It was. It was not a nice experience, but it's okay now.
+Yeah, I can move forward with confidence.
+Yes, I learned a lot from this experience and I think I got this.
+Yeah. Any questions?
+Like tell the other one to do stuff more earlier. So, yeah,.
+Yes, you're right. I agree.
+Yo. Right,.
+No. Do you have any ideas?
+Great.
+Perfect.</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>173</v>
+      </c>
     </row>
     <row r="17" ht="409.6" customHeight="1">
       <c r="A17" s="1" t="inlineStr">
@@ -854,6 +1122,20 @@
 03:27 Yeah, that's. That's a good advice. Thank you so much. Do you have any more tips to share? Just like in the general environment and like other, like how I can like come up with the topic of it of like saying, oh, yeah, I don't want to join.
 04:17 Yeah, that's true. Thank you so much for your advice. I think that's all.</t>
         </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Hi, how are you? How are you?
+So recently I had a really difficult situation with one of my roommates because she wanted to invite friends and I was physically like exhausted and mentally exhausted from the day and studying. And it was really difficult to tell her because on the one hand I really wanted that she can invite her friends. But on the other hand, I didn't want that many people over because I was kind of physically exhausted. So that was a really challenging experience. And my conversation that I had,.
+So I actually said yes to the friends because she's kind of like more. She talks a lot and I feel like she's kind of like it. Just like what she does has got to happen. So I was just like, fine with it. And I was going with it. I was like, okay, just invite your friends and I will just be in my room. Just don't be that loud. And she was kind of sad that I didn't want to join, but I was just like, I'm like, mentally exhausted from like uni all day. Yeah. So at first she was kind of like pissed because I didn't join our friends, but then she was fine and she was like, oh, yeah, just go into your room and sleep. That's fine.
+I think I should have just said my needs directly because first I was kind of like hemmed and I didn't want to say it because I felt like it would confront her and like she would be pissed at it. But I just learned that I should just like, say my needs. And it doesn't matter, like, what the other person thinks because as long as I feel it, my feelings are valid. So. Yeah,.
+Yeah, definitely. So, yeah, how would you say I should handle it better the next time? Do you have any tips?
+Yeah, that's. That's a good advice. Thank you so much. Do you have any more tips to share? Just like in the general environment and like other, like how I can like come up with the topic of it of like saying, oh, yeah, I don't want to join.
+Yeah, that's true. Thank you so much for your advice. I think that's all.</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>387</v>
       </c>
     </row>
     <row r="18" ht="404" customHeight="1">
@@ -880,6 +1162,24 @@
 04:26 Okay. Thank you.</t>
         </is>
       </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Nice to meet you. How are you?
+I'm also doing great. I would like to chat about a recent challenging situation I had.
+Yeah, so I was talking to my mother and she wanted me to do a test for a scholarship because it gives money and stuff. But I was really stressed because of student consultancy and other things going on because of group work in university. So I said that it's not doable to do this test in this time.
+She somehow understands, but also said that I should take time for it and yeah, make time for.
+I think it was not really possible because also the exam were coming up and I really had to learn for it. So I think it was not a good trade off to use this time for the scholarship thing.
+Not really relieved, no.
+I'm not sure.
+No, it's not that important for me because I. It's not in my mind anymore. Really.
+My focus is on doing university, also doing a bit of spirit sport and student consultancy, handling and all business development.
+I think I'm doing really good progress since I'm in university, so I gained a lot of new skills and stuff.
+Okay. Thank you.</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>208</v>
+      </c>
     </row>
     <row r="19" ht="372" customHeight="1">
       <c r="A19" s="1" t="inlineStr">
@@ -903,6 +1203,22 @@
 04:45 Yeah, definitely. And one last thing like. Yeah, I'm out of questions.</t>
         </is>
       </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>I'd like to talk about a challenging experience that I had with friends.
+Challenging experience is that I was slightly unavailable for like a month or so because I was catching up on exams. Now I caught up, but my friends thought I was distancing myself and I just was focusing on studying more.
+Now it went better because I realized that the problem was that I didn't tell them that and that they also didn't tell me how they felt. So it kind of increased over time, but now it's good.
+Yeah, I'd say so. It allowed us to also know each other better, how we think and deal with situation.
+Yeah, I'd definitely say so. And even though it was an unfortunate, I guess, experience, it could be for the better in some way because I got to know how they process things better and make them closer as friends.
+But for example, how would you have communicated instead of what I did and we did, what are some like ways of doing that?
+Yeah, that makes sense. That's what I did. I guess I just did it too late. But again, it wasn't a big issue either. So it was. It was an easy fix. It was just really the time effect that we hadn't discussed it in a while. That's it.
+Yeah, exactly. Yeah. And also how often should. No way. I mean, I think that. I think that the problem now makes sense to me. Yeah,.
+Yeah, definitely. And one last thing like. Yeah, I'm out of questions.</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>263</v>
+      </c>
     </row>
     <row r="20" ht="388" customHeight="1">
       <c r="A20" s="1" t="inlineStr">
@@ -924,6 +1240,20 @@
 05:11 Fixing it myself the same way I did with other stuff. Yeah. I mean, you can't communicate. But as I said, I think it's just. I'd rather have the good, like a better outcome rather than also forcing people that really don't care as much to do it, you know? Hello.</t>
         </is>
       </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Thank you. I would like to talk about a challenging interaction I had recently with some group teammates in my tutorial. So I think the biggest problem was that I felt like my ambitions in the project that were supposed to do were not aligned with what they were aiming for. And so I felt like I was kind of left to myself a little bit. I'd say, honestly, just different ambitions in, like, the great goals that we wanted to get. And yeah, I think that was the biggest problem.
+Honestly, I've noticed and learned that a lot of the times it's just easier to then do more work and kind of make it better rather than pushing them to do more. Because I'd rather just. Yeah, I'd rather not push them to do something they don't want to do. And also, I don't believe that they would do it as well as I did. Maybe to some extent. I think it very much depends on the environment. I think that in the sort of PBL system that I'm doing at my university, I think that a lot of the times it will be this way. Not always, of course. You might also get people that have similar ambition and similar goals. However, I think that most of the time, yes, it will be that way, but I don't know later in work life or anything.
+I think that a lot of the times people will be more aligned with you and your ambition.
+Not necessarily. I mean, hard skills, maybe like just doing the work and learning while doing the work. Yeah, but like, not necessarily like team skills, because, as I said, a lot of the time it's just. I'll just do it rather than necessarily communicating it with them because it's just easier and more efficient and the outcome is better. I see what you're doing.
+Do you have a question. Maybe. I don't know what else to tell you.
+When I read through, like. I mean, they didn't do anything. They didn't do nothing. Right. They did something. And when I read through it and I was like, this is just not good quality, that was very frustrating.
+Fixing it myself the same way I did with other stuff. Yeah. I mean, you can't communicate. But as I said, I think it's just. I'd rather have the good, like a better outcome rather than also forcing people that really don't care as much to do it, you know? Hello.</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>424</v>
+      </c>
     </row>
     <row r="21" ht="409.6" customHeight="1">
       <c r="A21" s="1" t="inlineStr">
@@ -943,6 +1273,19 @@
 04:26 Yes, absolutely. I mean, of course I want to get the best outcome and I really focus on having a good grade. But the group dynamic is really important because it doesn't make any sense if I'm just doing everything alone, for example, or excluding someone. That would be very disrespectful and not the values I want to present to someone else, so.
 05:07 Yes, that's absolutely true. And I also. It was a tough situation, but then later we got to a solution. We found a compromise and had a really great outcome of the project. Hello. Hi. How was it? Should I stop? I can just take it off. I'll reset the whole room for the next person. Perfect. Did you enjoy it? Yeah, it was interesting. That's one of the three adjectives that most people use.    Transcribed by https://fireflies.ai/</t>
         </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Hi Eduardo, nice to meet you. I would like to talk about an interaction I had in university with my group that was not as pleasant as I thought it would be.
+Yes, sure. So was in a group work and it was a problem that occurred because I want to achieve a good grade and the work that my project teammates did was not that good as I would have expected and how it should have been for a good presentation and a good grade. So I didn't really know how to handle the situation because I wanted to prompt a different alternative to their task solution. But they didn't really were quite, yeah, I don't know, convinced. And then it was like a conflict of what we should do now. I knew that we their answer was not as good and great as how it really was for their experience. And I also didn't want to offend them and didn't really know how to say nicely that we should take a different solution.
+Yes, I thought about it and I also talked to various other team members and asked them what they thought which solution would better. And also I tried to compare, not really compare, to show that there's a worse and not good, but to show where their solution might have some flaws and be as not as efficient than my solution. And I try to do communicate that in a very nice way. But it's still. If someone is said to their mind that their minds and thoughts are the right ones, then it's hard to convince them otherwise.
+Absolutely. I agree. It was really kind of difficult now. So from the beginning didn't really know how to approach this problem because I had previously also met other people were like, I know people who are really then very fastly offended if someone doesn't like their idea and they always think that they're input is the best. And it's really hard then to work with these people and it's just unnecessary stress that would general be generated in the group. So it was really going on my nerves and was hard for me to really work without being like mean or like people thought I would be mean and yeah, hard.
+Yes, absolutely. I mean, of course I want to get the best outcome and I really focus on having a good grade. But the group dynamic is really important because it doesn't make any sense if I'm just doing everything alone, for example, or excluding someone. That would be very disrespectful and not the values I want to present to someone else, so.
+Yes, that's absolutely true. And I also. It was a tough situation, but then later we got to a solution. We found a compromise and had a really great outcome of the project. Hello. Hi. How was it? Should I stop? I can just take it off. I'll reset the whole room for the next person. Perfect. Did you enjoy it? Yeah, it was interesting. That's one of the three adjectives that most people use.    Transcribed by https://fireflies.ai/</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>529</v>
       </c>
     </row>
     <row r="22" ht="409.6" customHeight="1">
@@ -967,6 +1310,22 @@
 05:02 That was basically it, man. Do you have any other advices for me for my study? I study international business in Maastricht and. Yeah, what's the game plan? What should I do next?</t>
         </is>
       </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Hello, my name is Luis. How are you?
+Oh, yeah, I'm also fine. I want to talk to you about something. Do you have a minute to listen to me?
+First of all, where are we? What room is it?
+No, it does not. There's no. Oh, yeah, it is. Oh, yeah, it is. You're right.
+Alright, man, in this cozy spot, I want to talk to you about my classmates. We had a presentation. We had to obviously prepare the presentation to present it to our class. It was quite a big presentation, so we had to split up the tasks and so on. You get what I mean?
+Yes, all right. My classmates, I mean, were a group of three. So me and two others. My other classmate, her name is Lynn, and she was great. She did all her tasks and were able to present it to each other and so on. But my other classmate, he was a Dutch guy, he didn't do anything and we had to cover his part. Even though we told him many, many times that he should do his task because it's not fair. We have to do his part because it was such a big presentation and very many tasks to do. Now, what should I do to convince him to do the task? I mean, we did it afterwards, so he didn't do anything. But should I go to the teacher and tell him about it or should I. What should I do?
+Well, we've already tried many times. As I've already said. Maybe you all heard it. We have tried to convince him and ask him to do it, but he ended up didn't. So I should go to the teacher next award.
+Alright, man. Thank you for listening to me. Do you want to talk about something? You seem kinda. Kinda annoyed. Your facial expression shows me that you have something on your mind.
+That was basically it, man. Do you have any other advices for me for my study? I study international business in Maastricht and. Yeah, what's the game plan? What should I do next?</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>360</v>
+      </c>
     </row>
     <row r="23" ht="388" customHeight="1">
       <c r="A23" s="1" t="inlineStr">
@@ -986,6 +1345,19 @@
 04:07 Yeah, I mean, as the others are going on Thursday anyways, they already booked their trains. I feel like the biggest decision we have to make is how we gotta travel back on Monday. So I think we have to find a solution there as they want us to come with the car and then we all go back by car. Or the other option is that we all go by train. So it's a bit of a tricky situation.
 05:02 Yeah, probably. Hello. Hi. How was that? Cool. You liked it?</t>
         </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Okay, perfect. So I want to talk to you about a recent situation where I had a conversation with some friends of mine where we had some difficulties. We were planning a trip for next weekend and yeah, weren't quite aligned in how we want to travel to our destination. So we had some disagreements there.
+So it was about many factors. So to start off, we are six people who want to travel to our destination and three of our friends, they want to travel on Thursday already and the rest of us want to travel on Friday. So we had some disagreements there because some of us wanted to skip a tutorial and some of us didn't want to skip the tutorial on Thursday and Friday. I mean, on Friday we all have to skip our tutorial anyways. So some of us didn't want to have like another skill. So this was the first problem. And then obviously we would all return on Monday here to Maastricht.
+So we had some disagreements because all of the people traveling on Friday, they want to go by train, whilst the people going on Thursday already, they were suggesting why we not come there after them with the car and then all go back by car.
+So personally, I'm also part of the group that wants to travel on Friday as I don't want to skip my tutorial on Thursday. And then regarding the issue of whether we go by train or by car, I actually don't really mind. I think both will be, yeah, like the same amount of money spent on it. And actually I feel like train is a bit more relaxing and you have some time to do something for university while in the car. You're not gonna do anything for university. So actually I would prefer going by train, but for me that's not that of a big decision. But I have to say, of course, going by cars also really exhausting driving eight hours or something. So prefer the train. Actually.
+Yeah, I mean, as the others are going on Thursday anyways, they already booked their trains. I feel like the biggest decision we have to make is how we gotta travel back on Monday. So I think we have to find a solution there as they want us to come with the car and then we all go back by car. Or the other option is that we all go by train. So it's a bit of a tricky situation.
+Yeah, probably. Hello. Hi. How was that? Cool. You liked it?</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>437</v>
       </c>
     </row>
     <row r="24" ht="409.6" customHeight="1">
@@ -1012,6 +1384,24 @@
 04:55 It feels like she doesn't give me a chance to respond. Hello. How did it go? Good. Where should I oh, don't worry, I'll reset it for you. Did you enjoy it? It was cool.</t>
         </is>
       </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>I would like you to help me resolve a problem that I have with my manager.
+Me and my manager were talking about work hours and she told me that she wanted me to work a lot. So we planned a lot of dates for me to work and eventually we came to the conclusion that I would work every Tuesday, four times a week. And then another co worker of me texted me that he also works those days and that he will be taking over my shifts. But my manager didn't tell this to me.
+I am hoping that I could get the hours back.
+Well, actually I already approached her.
+She did give me explanation and said that I could have the hours back, but she wasn't too happy about it and she didn't really want to admit that she made a mistake. And that's what's basically, that's what I'm not really happy about, that she cannot admit that she made a mistake.
+I'm looking for ways to move forward. I guess.
+The thing is, whenever I try to explain to her how I'm feeling, she talks over me.
+Yes, that may help.
+Side Yes, I think that as well.
+Yes, I will try to talk to her again then.
+It feels like she doesn't give me a chance to respond. Hello. How did it go? Good. Where should I oh, don't worry, I'll reset it for you. Did you enjoy it? It was cool.</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>248</v>
+      </c>
     </row>
     <row r="25" ht="404" customHeight="1">
       <c r="A25" s="1" t="inlineStr">
@@ -1034,6 +1424,22 @@
 04:47 Yeah, true. Thank you for listening, though.
 05:00 Thank you.</t>
         </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>I'll be back. Thank you. Okay, I'm here. I'm here to talk about the challenging interaction I've had.
+I mean, it was about a group work, so we had to work about a presentation, but nobody was working at all. And it was like, I don't know, 30 minutes before class, so we had to do something. But I was just sending messages in the group chat also the day before, but nobody was replying, so I just didn't know what to do. And it was pretty challenging because then the day after, when we had to present, they actually had stuff to present without letting me know.
+I mean, at the end we just had to choose one of the group members to present. So I handled it like I didn't do anything at the end because they said maybe they're thinking that I should do everything when I don't actually have to do everything, you know? So at the end, one of the group members, they just did a presentation in, like, five minutes, and then they presented right away.
+I mean, at the end, it turned out very well, and the tutor liked the presentation, so I guess it was fine. But I can tell that it was kind of frustrating because I wanted things to be done, but at the same time, I didn't want to do everything by myself. So. Yeah,.
+Yeah, I mean, you're right, but I wanted to do that as well. But as I said, when I was texting in the group chat, nobody was replying. And every time I was sending messages, they were like, nobody has started yet, and that's it. And when I said that we should, like, split the work and, you know, just do it before the class, nobody was replying again. So I don't know.
+Yeah, I told them, but apparently they just. I mean, at the end, they had something and we did something and we presented something. But still, like, it's pretty tough.
+Yeah, exactly. So it's fine. I mean, I'm good with myself, so it's perfect.
+Yeah, true. Thank you for listening, though.
+Thank you.</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>362</v>
       </c>
     </row>
     <row r="26" ht="409.6" customHeight="1">
@@ -1059,6 +1465,23 @@
 06:09 Okay, that sounds great. Thank you a lot. I think now I will end the conversation.</t>
         </is>
       </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Nothing really. I'm really chill. I think we should talk about a convers like a situation I had in my past that was challenging to me.
+Yeah. So actually like last week I have like a leadership position in the student association and last week I had to fire. Fire is a hard word. But last week I had to fire someone from my commite because they were not contributing.
+I think the person took it pretty well because I mean they knew that they weren't contributing enough to the committee and so I think it didn't come as a big surprise. However, it was stressful for me because beforehand I tried a lot to incorporate them in the team and it was just not a lot of things coming from them.
+I'm feeling pretty good about it. I feel like it was a challenge for me as a first leadership role and I think I managed it pretty well.
+Actually about this matter, maybe you could give me some advice for the future on how to handle rejections. So when I have to reject people like in the professional setting.
+Okay, that sounds like great advice. What would be things that I like in a bit more deeper way. Things that I could incorporate into my day to day decision making in order to include people more in my position.
+Okay, that already sounds like great advice from you. I'm really happy. What do you think the benefits are of incorporating a team culture that is healthy in a committee?
+Okay, for resilience that you're talking about, could you maybe give more in depth solutions on how to build this resilience?
+Okay, that already sounds like great advice. On different matter, what do you think how the people in my committee should handle their time to study and their time to contribute to the committee? What do you think is a good time management?
+Okay, that sounds great. Thank you a lot. I think now I will end the conversation.</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>341</v>
+      </c>
     </row>
     <row r="27" ht="404" customHeight="1">
       <c r="A27" s="1" t="inlineStr">
@@ -1083,6 +1506,23 @@
 05:01 All right. Thank you.</t>
         </is>
       </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Five minutes. Enjoy it. Yeah. Thank you. So I recently. So I recently had this challenging experience in my last period in university with a group member who didn't really participate and really was really mean to us all. And I wanted to talk with you about this.
+So we had this presentation that made like 50% of our grade and he didn't really participate. He was really like mean and he didn't come when we like said that we will meet up. And in general the work with him was really bad so that we in the end didn't really have this great presentation too. So it also like failed a bit. Our grace.
+So we tried to talk to him and you know, just talk about our issues and problems, but he didn't really listen and sometimes he was also like lying when we like for example, wanted to meet up. So.
+Yes, we did. We talked with our tutor but like she didn't help us that much. But like in the end she told us that she would just give him a worse grade. But it didn't really, you know, it didn't really benefit us because in general we got also like a worse grade. So.
+Well, obviously we couldn't decide who which person participates in our presentation group so. So we couldn't do. I can't do much about it. I think I just have to learn like to work also like when we talk about education and work experience, how to work with people like him who are bit more problematic and where you like can't work that well. I think this is just something which you have to learn over the time.
+Yeah, it could possibly be. I don't know.
+Thank you so much. Means a lot. Nice words.
+No, in general, I think this is just something. Do you have, like, maybe some advices on how to work with people, you know, who are not that very cooperative?
+Yes, I think I thought the same. So I think we have here the same opinion. Well, we tried in the end to also, like, do this, but yeah, I think in general we have the same opinion on this.
+All right. Thank you.</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>378</v>
+      </c>
     </row>
     <row r="28" ht="323" customHeight="1">
       <c r="A28" s="1" t="inlineStr">
@@ -1103,6 +1543,20 @@
 03:39 Okay. Yeah, I think. I think I know someone who's also handling the schedules and everything, so maybe that person can give me extra free time and I also gonna write an email. So that was also a really good tip.
 04:19 Thank you very much, Eduardo.</t>
         </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Hi, Eduardo. Nice to meet you. So I had like a discussion with my boss about getting more free hours, but he wouldn't give in and won't give me the hours. So. Yeah, that was really unfortunate.
+I think I'm really important at work, so I feel like I'm also, yeah, I can again, I earn the extra hours, but yeah, I hope when I talk to him again that he might give me the hours instead of like, being how he's treating me now.
+Yeah, I hope so. Good point. I will. Yeah, tell him that.
+Thank you. Do you have any other tips? Eduardo, do you get any. Do you have any other tips?
+Okay, thank you very much. That that's true. Is there maybe another way instead of talking to him to get what I. Eduardo, is there anything else I can do instead of talking to him again? Because I think he maybe still won't give me the extra hours.
+Okay. Yeah, I think. I think I know someone who's also handling the schedules and everything, so maybe that person can give me extra free time and I also gonna write an email. So that was also a really good tip.
+Thank you very much, Eduardo.</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>210</v>
       </c>
     </row>
     <row r="29" ht="409.6" customHeight="1">
@@ -1128,6 +1582,24 @@
 04:16 Yeah, I wrote his secretary and said to her that or sent her a screenshot of the chapel. The landlord that he sent me that I will get the payback of the monthly rent and told the landlord that I will follow up to the secretary. And then he sent the money back to me because there was no chance that he can get out of the situation in another way because he stated that he will pay back the rent.
 05:04 Yeah, of course it was a win for me. And I think I handled the situation good and everything came to a good end.</t>
         </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Great to meet you too. Yeah, about. I'm just chilling. I have this study today and after that I have my tutorial and then I will drive back home.
+Yeah, I think it's great. Sometimes it's a lot of work, a lot of reading, but I think it's going smooth.
+I try to keep up with the flow and because we're having our exams in around four weeks, I try to keep in the flow and try to practice for the exam.
+I think it's pretty balanced because when the subject started I tried to go with the flow and therefore I think I don't have any problems with it.
+Yes, of course. Do you have any jokes to tell me?
+That's a great joke. I like that. How about you? How is your time? How do you spend your time?
+That. That sounds great. I like that.
+Yeah, I just wanted to talk about the recent situation I had with my past landlord. If you're interested in it.
+I moved out in January, but the contract was until July, so I moved out earlier. But I found a new tenant for him and he said everything is alright. And then I was waiting for the payback of. Or the reimbursement of the. Yeah, of the half monthly rent of January and I was sending an email to his secretary, and she answered that they don't want to pay back it because it's not stated in the contract. And then I was in the situation to handle it with the landlord and his secretary because he wrote me that they will pay back the half of the monthly rent of January.
+Yeah, I wrote his secretary and said to her that or sent her a screenshot of the chapel. The landlord that he sent me that I will get the payback of the monthly rent and told the landlord that I will follow up to the secretary. And then he sent the money back to me because there was no chance that he can get out of the situation in another way because he stated that he will pay back the rent.
+Yeah, of course it was a win for me. And I think I handled the situation good and everything came to a good end.</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>386</v>
       </c>
     </row>
     <row r="30" ht="409.6" customHeight="1">
@@ -1155,6 +1627,25 @@
 05:22 Thank you. Bye.</t>
         </is>
       </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>We can talk about anything.
+Probably just school, studies, exams, stuff like that.
+Right now I'm just trying to make sure that I pass all my exams so that I don't have any resets. I've been working hard on the finance course, especially because finance it's quite math heavy and my math exams haven't been the great in the past I've passed. But yeah, definitely just focusing on finance.
+I think it's definitely more about staying consistent. Consistency is key, right? So just lots of practice. Maybe start implementing some past papers because I haven't done that yet. And for the rest, yeah, just keep studying.
+Yes, that sounds great. Thanks for the motivation, I guess.
+I will do. So what's next?
+When you say reward yourself, what do you mean by that? Like just mean like spending some time off or what does that really imply.
+That sounds good. I'll be sure to implement that. Maybe I'll also like consider implementing more like sports as a sort of reward or just spending time with friends because studying all day is of course not good and could tire me out. Definitely.
+Yes, thanks. Thanks for the help and good conversation. How should we proceed? This conversation?
+You know, honestly, I think we've covered a lot. It's an eye opener. Maybe just. Do you like playing Padel? I've been getting into paddle recently.
+Mostly I play singles, but no, no. I play doubles. What am I saying? Yeah, I play doubles, singles, paddle. Never really tried it. To be honest, I thought it was more of a double sport. But maybe sometime we can play together. Yeah. But thanks for the conversation and maybe see you next time out there on the courts. I like your office, by the way. Buddy.
+Thank you. Bye.</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>303</v>
+      </c>
     </row>
     <row r="31" ht="404" customHeight="1">
       <c r="A31" s="1" t="inlineStr">
@@ -1174,6 +1665,19 @@
 04:58 Okay, but maybe. Maybe, like, in regards of the process that we had, was there anything I could have said? Like, before, I did all the work alone, I mean, also, I was a bit angry, and I just did it all by myself without telling them because I was sure they wouldn't do the work anyway. So is there maybe anything I could improve during the process? So we can avoid that I have to do the entire presentation on my own?
 05:51 That actually sounds reasonable. Thank you. Hello. Hello. Let me help you out with that. It was nice, but I think at the first time it didn't work out, so you had to restart it. Okay, no problem. If you were able, it'll.    Transcribed by https://fireflies.ai/</t>
         </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Hope you enjoy it. Yeah. Okay. Hello, Eduardo. Yeah, I recently had a challenging situation I want to talk about with you. What do you think? Like, I just remember in our tutorial group, we had to do a group presentation in Dorado, and then there were some participants that didn't like to do anything. And basically as soon as the deadline was there, I was the only person that felt responsible to do all the exercises. And I really feel bad about it. I think it's unfair. What do you think? Can you answer? I think it's not possible. It. Hello, Eduardo. I hope. Hello, Eduardo. I hope you can hear me. Perfect. Pleasure to meet you as well. Yeah, I recently had, like, a difficulty in university, actually. I just want to talk about this with you.
+So, actually, for our tutorial group, we had to do a group presentation that is also graded. But however, like none of the four group members, I had felt responsible for doing anything. And in the end, the deadline approached and I was just doing the entire presentation because I didn't want to have a bad grade. But I think that's pretty unfair. Don't you think so? Because the others didn't do anything.
+The thing is, I don't want to be a snitch and tell the professor I did everything. I mean, I could do it, and it would probably also save my grade. But I also don't like to, you know, snitch on the others. But I just think that if this will be repeated in the future, so I have, like, multiple scenarios like this, then I would go to the tutor or what would you recommend to me?
+Yeah, okay. That actually sounds reasonable to me. I think, like, in the next time, maybe we can also, like me and my group members, we can talk about the ambitions we have because maybe they were just not that ambitious and said, okay, we don't really care about the grade, but I may be a person that wants to have, like a very good grade. So maybe talk about the ambitions first, and then you can still see whether you have to go to the tutor or not.
+Okay, but maybe. Maybe, like, in regards of the process that we had, was there anything I could have said? Like, before, I did all the work alone, I mean, also, I was a bit angry, and I just did it all by myself without telling them because I was sure they wouldn't do the work anyway. So is there maybe anything I could improve during the process? So we can avoid that I have to do the entire presentation on my own?
+That actually sounds reasonable. Thank you. Hello. Hello. Let me help you out with that. It was nice, but I think at the first time it didn't work out, so you had to restart it. Okay, no problem. If you were able, it'll.    Transcribed by https://fireflies.ai/</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>510</v>
       </c>
     </row>
     <row r="32" ht="409.6" customHeight="1">
@@ -1197,6 +1701,22 @@
 04:24 What do you think about it?
 04:40 Hello? Do I have it?</t>
         </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Hi, Eduardo. I am Tom, and I want to talk about the discussion I had with my friend.
+So, first of all, we talked about who's the better football player, Cristiano Ronaldo or Lionel Messi. And in my opinion, is that Cristiano Ronaldo, and for my friend's opinion, was Lionel Messi. So we had a tough conversation.
+No, everything like stats and how important they are for their team and. Yeah, also their personal experience.
+No, no, we disagreed. He was still with Lionel Messi, and I was with Cristiano Ronaldo. But in my opinion, Ronaldo is the better player because he scored more goals in total, and he started his career in Sporting, the Saban, and not like Lionel Messi at Barcelona. So Cristiano Ronaldo was not given the perfect team at the start, and he had to fight for everything. And. And Lionel Messi was, like, always given in the shoes.
+And Cristiano Ronaldo is always there for his team if his team needs him. So, for example, at Juventus, when Juventus lost 20 against Atletico Madrid and the second leg, in the second game, Cristiano Ronaldo scored the hat trick. So this simply shows for me that Ronaldo is like a player who's there if his team needs him. And Lionel Messi is not always there.
+Yeah. And what's your opinion about this debate? So, do you have an opinion, or what do you think? Who's the better player?
+And after that debate, we got into the debate, which club is bigger and has a greater history? And for me, it was obviously Real Madrid and for Barcelona. And it's clear, right, if that Real Madrid has more trophies and more Champions League trophies, that they are the bigger club.
+What do you think about it?
+Hello? Do I have it?</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>304</v>
       </c>
     </row>
     <row r="33" ht="409.6" customHeight="1">
@@ -1226,6 +1746,27 @@
 06:21 That's actually a good idea. I was thinking of sewing because I used to, but I don't have a sewing machine right now. Maastricht. But I would really like to do something fun or creative. I don't know. I try to draw every day, but that stops after a few months maybe. But yeah, I want to start that again. Yeah. So what kind of hobbies do you suggest? Maybe. It's still listening.    Transcribed by https://fireflies.ai/</t>
         </is>
       </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>It's good, thank you.
+I had a lot of sleep and I skipped class. I mean, it's not that good, but it was relaxing.
+I'm gonna prepare for my classes and I have to do some grocery shopping. And then after, in the evening, I'm going to work.
+I don't know. Could you repeat the question?
+Yeah, I like to go to the gym. Gym to do strength training.
+I'm going to start again next week because I had a bigger break from the gym, but I've been doing it for two or three years now.
+Yes, I have a wedding come around and I want to lose weight for that and that's my plan.
+Yes, that's exactly my plan.
+Well, first I have to buy a subscription to the degeneration and then go like three or four times a week. So I actually do the exercises and the training. And also I want to have a diet consisting of eating less sweet things and just generally eating less.
+Thank you. Yes,.
+Feeling strong again? Because in the past few, three or four months, I've been feeling like I could feel weakening myself, like my body is weakening. And now if I go back to the gym, it's gonna get stronger again and I can feel powerful again. So it's good.
+Yeah. I already done this once. Like, this extreme. I mean, not extreme, but like, bigger weight loss. Before, there was like a prom in my high school and I decided to lose weight for that, and I was able to lose actually 10kg in like two weeks just by cutting out every sweet things that I usually eat because I am a really sweet dude.
+Yeah, but the thing is that I have some problems with overeating because even though I feel full sometimes I can't, like, stop because I know it's really good that, like, the food tastes amazing and everything like that. But I don't know what to do against that overeating problem. What do you suggest?
+That's actually a good idea. I was thinking of sewing because I used to, but I don't have a sewing machine right now. Maastricht. But I would really like to do something fun or creative. I don't know. I try to draw every day, but that stops after a few months maybe. But yeah, I want to start that again. Yeah. So what kind of hobbies do you suggest? Maybe. It's still listening.    Transcribed by https://fireflies.ai/</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>419</v>
+      </c>
     </row>
     <row r="34" ht="409.6" customHeight="1">
       <c r="A34" s="1" t="inlineStr">
@@ -1249,6 +1790,23 @@
 04:35 Yeah, but you tried that. It's not working.
 05:01 I don't really want to have like this real conversation because it might get bigger than it is right now.</t>
         </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Hi. I would like to talk about a challenging experience. I had.
+A friend of mine and I like, I haven't talked to her yet, but I feel like that I'll give her more in a friendship than she gives me. And I feel like very uncomfortable like telling her because I feel like I like to do that for her and I'm very open to do a lot for her, but I also just want to see her maybe give also something similar back. Like she does give some things back, but not as much that I do. I feel like.
+I just don't want her to feel like I look at everything and everything should be 50. I do feel like there's situation where someone helps more and someone helps less. But in general I feel like some. Sometimes there is a bigger gap and just to close that a little would just help me. I feel like.
+Yes.
+Yeah, maybe. Or how I can tell her like secretly with not having an awkward conversation.
+Okay. I feel like it's kind of difficult to like talk about it or because it makes it so awkward. Like nobody says, yeah, that was great, I would wish you to do that more often. I feel like it's an assault or like I tell her something to do and I don't want to do that.
+I feel like I'll already do that and it's still not working.
+I also try to be like more direct in some kind of jokes. Like trying to say it more like under cover. Under coverly. But like I don't want to be so persistent about it, so what can I do?
+Yeah, but you tried that. It's not working.
+I don't really want to have like this real conversation because it might get bigger than it is right now.</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>314</v>
       </c>
     </row>
     <row r="35" ht="409.6" customHeight="1">
@@ -1278,6 +1836,27 @@
 05:10 Yes.</t>
         </is>
       </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Nothing much really.
+I like to do sports, play basketball, work on myself. You know, regular things. Kind of that you would expect someone like me or my age to do. I like to keep myself fit, work on myself, try to make something out of myself, make use of the time.
+Practice and we pretty much just play workout. I enjoy working out upper body, more chest, regular stuff I'd say.
+Yes.
+Not really. You know, you have my plan that I do and I try and follow it as much as possible. Possible. You know, there's no particular favorite one.
+That's probably a good question, but I'd rather be for endurance since I'm an athlete. That's why I want to focus on. I don't want to be a pumped up bodybuilder. I'd rather be explosive and athletic.
+Yep, that's true.
+Yeah, yeah. You know, when I work out legs, I work out. One time I do plyometrics and I focus on athleticism. And the next day I do pure strength training with heavy lifting and small size of reps repetitions.
+Yes,.
+I could stick more to my workout plan, which is why it's not working as good, but that's on me. It's my fault.
+Yeah, actually, yes. Short term goals would be more catching.
+I think these are a little bit too general, but we can switch topics. I have a question for you.
+So I do photography and videography and I did this video for a new student association here and I told them I'll do it fully for free. But we kind of came out of contact because I wanted them to feature my posts as a like, let's say you call it like a co editor post, like a cross post. But they wouldn't agree with that and they weren't very open with giving me a shout out next to. Although I did like all the work. And yeah, now we're kind of out of contact. How do you think you approach a situation like this?
+Yes.</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>342</v>
+      </c>
     </row>
     <row r="36" ht="409.6" customHeight="1">
       <c r="A36" s="1" t="inlineStr">
@@ -1299,6 +1878,21 @@
 04:45 And it's not nice for me to put so much pressure on her because maybe on Instagram, on videos that you have, maybe life feels like pink and. And shiny, but actually in the reality is not, yeah, same. And she. That was failing a lot of courses, but I'm not sure if it was my mistake because, yeah, this is how I feel at the moment. And it was quite a stressful experience for me. And at the moment we still are in touch, but not so often and not so in depth as we used to be. And also made myself a conclusion that maybe I have to step a bit back and give myself and herself a bit of space. And yeah, maybe I will not put 100% anymore because it feels like not worth it.
 06:17 So maybe you can give me some advices of how I should act next. Like what would be the further next steps?</t>
         </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Thanks. Yeah, so I actually want to talk about a situation that recently happened with my friend. And I still feel I don't have enough closure about it because it was a situation that really hurt my feelings. And I also understand the side of the other person. But for me it was quite a stressful experience as a friend because I really value my friends and my friendship with other people. I feel like I am giving myself 100% and I'm not receiving the same from the other people. So. Yeah,.
+So actually there were more situations that was, you know, feel like building up. And at one point I felt like a jar that was so full that it just, you know, broke. So actually the things started from Easter. For me, Easter is a very important celebration where we gather families in Moldova. I always been around my family and to be honest, I really was waiting for this friend to come over because we wanted to cook some traditional meals together and also paint the eggs because it's also a tradition that we do for Easter. And she was on a trip and she just returned the same day when I was supposed to do all these things. And she didn't because she said she was too tired, which I also understand.
+But the next day, the morning of the Easter, I was really expecting her to be there, but she was very late. And it really hurted my feelings, but I said okay. Then another situation that happened is that since then she was not really in contact with me, not really texting, calling. If the calls or texts don't come from my side, then she would not even bother to call me or to message me. And it really also bothers me because all the time when I go to her, I never go empty handed, all the time bring flowers, chocolates, I all the time text her all the time I was worried about her when she was not answering for some days. And I don't share the same experience. So I feel like I deserve the same attitude and respect from my friends.
+And also bothered me is that she all the time complained that she doesn't have enough budget, not enough time to go on a trip, a girls trip that I also was dreaming about for a long time. And then recently I saw some pictures and videos on Instagram of her that she was with other friends. And it really hurted me because it felt like she has time and budget for other people, but not for myself. And another thing Is that in Moldova, our parents sometimes send us some packages and it comes from a minibus. And you never know when those people would be in Netherlands, because we are here established. And yeah, I wasn't expecting any package. And at one point I got a lot of calls from foreign numbers, like German numbers. And I usually don't answer, you know, the phones to strange people.
+And I said, okay, let me answer the phone. And there was like a man screaming at me, like, why I'm not answering my phone? Because I'm supposed to get a package from Moldova. And actually her parents sent the package to her in Netherlands, but because she was not home, they gave the people that deliver the packages my phone number. And I had to like, all the time be stressed about it. And, you know, I also didn't like that. And recently also was my birthday of my boyfriend. And she also couldn't make it because of the other reason that she had and because she had to attend another event with her boyfriend. So there was a lot of events that just built up and it felt really hurtful because I also approached her, I texted her.
+Maybe it's not the best approach because, yeah, I also don't like this long text where I have to describe everything. And sometimes maybe you don't get the nice tone out of it. Maybe you understand completely different the message. But I still felt like I needed to express myself because I really value all the friendship that I have. And when I'm like, I also lived a lot of betrayals when it comes to friendships. And maybe I don't have so many friends at the moment, but the ones that I have, they're super nice, you know, like, it's not about the quantity, but quality. And that's why I approached her. And she got really offensive because she said that I make her feel the victim.
+And it's not nice for me to put so much pressure on her because maybe on Instagram, on videos that you have, maybe life feels like pink and. And shiny, but actually in the reality is not, yeah, same. And she. That was failing a lot of courses, but I'm not sure if it was my mistake because, yeah, this is how I feel at the moment. And it was quite a stressful experience for me. And at the moment we still are in touch, but not so often and not so in depth as we used to be. And also made myself a conclusion that maybe I have to step a bit back and give myself and herself a bit of space. And yeah, maybe I will not put 100% anymore because it feels like not worth it.
+So maybe you can give me some advices of how I should act next. Like what would be the further next steps?</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>948</v>
       </c>
     </row>
     <row r="37" ht="409.6" customHeight="1">
@@ -1332,6 +1926,31 @@
 06:45 Okay, that's. Yes. The end yes, you can take it off now.    Transcribed by https://fireflies.ai/</t>
         </is>
       </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>If you have any questions, I'm outside. Yes, thank you. Talk about anything you ask for advice. Name and lighter sheet. Hello, Eduardo. Hey, Eduardo. How you doing? So basically I was supposed to ask some questions.
+That's a very good one. This is based practice, dexlab. Okay. Okay. I need to brainstorm a bit. I want to do some marketing campaign for my company. It is a secondhand marketplace for students and I want to get more students to do an interview with me. What do you suggest?
+I was thinking going to the park with a beer and tell them, yeah, for one interview you get a beer, or for one sign up you get a beer. Something like that.
+Is there any legal issue regarding giving away beers? It's students at Art University, so we're in a country where 18 is the minimum age, so it should be fine now.
+No, I'd rather just exclude the younger ones.
+Vouchers for what though? It's a student online company, nothing else.
+I hear you, but I think we're just gonna stick with beer because it's gonna be a hot day and people will want to want a beer.
+All right, I will. Sounds good. Thank you.
+I appreciate that. Now I will ask you something else. I recently had an encounter with an advisor of mine and I don't know. The issue with him is that he's not proactive. And I'm not a clue how to incentivize him to be more proactive.
+So reinforcement is the key, you see?
+All right, cool. I guess I'll do that then.
+What else can I talk about? Alright, tell me a joke.
+That's such a lame one.
+Yeah, sure.
+No, no. Give. Give another shot. Why not?
+Oh, horrible.
+I would like to know where you're located.
+Okay, that's. Yes. The end yes, you can take it off now.    Transcribed by https://fireflies.ai/</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>322</v>
+      </c>
     </row>
     <row r="38" ht="372" customHeight="1">
       <c r="A38" s="1" t="inlineStr">
@@ -1355,6 +1974,22 @@
 05:09 Okay. Thank you for your help. Hello.</t>
         </is>
       </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Hi. I have been in a situation. It was a really challenging situation where I had some misunderstanding with one of my friends. This was the situation. So I am looking for some rentable places to live here in this city. And I didn't know if I wanted to live with her or live alone.
+Okay. Should I say what I'm thinking about?
+Okay. It's really pretty. I feel calm here.
+I can feel it. It's really cool. Should we just talk about my problem or like, brainstorm or how to get like, a solution to my problem?
+Okay, I got it.
+Yeah, I see.
+Maybe you can help me. Like, what would be the best decision? To move in with her when I know that her behavior can be sometimes really, like, stressful because she studies a lot or, like, move in alone and it would be much more expensive with which I'm not able to present the money for. What do you think?
+Absolutely.
+Okay. Thank you for your help. Hello.</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>173</v>
+      </c>
     </row>
     <row r="39" ht="255" customHeight="1">
       <c r="A39" s="1" t="inlineStr">
@@ -1372,6 +2007,17 @@
 01:55 But how do I, like, communicate to them properly that I want the kitchen to be fully, like, clean and a respectable area?
 02:29 Okay, thank you so much and thank you for your help. It was very helpful.</t>
         </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Hi, nice to meet you. I wanted to talk to you about a weird interaction I had with one of my roommates. I'm sharing a kitchen with a lot of students and it seems to be pretty messy these days. So I tried to confront one of them, but they got really angry and none of my roommates talk to me anymore. What do you think I should do,.
+Okay, thanks. But I'm scared that they will have like a bad reaction to that. Like, they seem to be pretty aggressive.
+But how do I, like, communicate to them properly that I want the kitchen to be fully, like, clean and a respectable area?
+Okay, thank you so much and thank you for your help. It was very helpful.</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>129</v>
       </c>
     </row>
     <row r="40" ht="409.6" customHeight="1">
@@ -1397,6 +2043,23 @@
 04:32 Yep. That seems good. Thanks for your help. Have you had experiences like this before?</t>
         </is>
       </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Hi, how are you? I would like you to.
+I'm feeling okay.
+I wanted to talk about a challenging interaction I've had recently.
+Yeah, I was talking with my group work project from university. They were all being very passive though. So no one was trying to take over a role or even assign roles.
+Yeah, I've tried to kind of start as a kind of leader, but I don't really want to take the leader role since that takes much more time than any other role. And I've just tried having them each assign themselves a role, but it hasn't really worked yet. Do you have any tips?
+Yeah, that sounds good, but I mean, it sounds good in theory, but I don't know how I would be able to put that in practice, especially if I don't see them in person. Often I usually just have them per text where a lot of people can just ignore.
+Yeah, that seems smart enough. How would you then continue to keep them accountable though? Like, we have, I think three weeks until the presentation, but we have to keep doing weekly small drives that we should show the teacher and I don't want to be every day sending out reminders or kind of having to check on everyone.
+Yeah, that makes sense.
+Yeah. How could I formulate it, though, without sounding too bossy?
+Yep. That seems good. Thanks for your help. Have you had experiences like this before?</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>248</v>
+      </c>
     </row>
     <row r="41" ht="272" customHeight="1">
       <c r="A41" s="1" t="inlineStr">
@@ -1414,6 +2077,17 @@
 01:38 Not sure if that is the thing I would do because it's not that kind of a serious problem and not sure if that should be something where I tell them how I feel on a deeper level. Because also our connection is not that deep yet. So probably I would just kind of find a way to interact more with them, spend more time with them and then see where it goes.
 02:33 Yeah. Thanks for the tips. And another thing. Do you have any advice on how to integrate different friends who don't know each other yet and create a group of friends? So kind of. Yeah. Bring different people together.</t>
         </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Good to meet you too. We can start the conversation. I want to speak to you about a recently challenging social situation.
+Okay. So I have a good friend, a fellow student, which I quite like and we get along well, but kind of. It's not a problem, but it's kind of a misalignment. He has a lot of friends. He has a lot. He has a very vivid social life and more. I'm more kind of introverted. I have a few very good friends and I'd like to integrate him into my close friends circle. But he obviously he has a lot of friends and so a lot of options. Yeah. So it's a bit of complicated to deal with that situation because I like him as a person. I like to do some stuff with him, but he is kind of very busy with a lot of people.
+Not sure if that is the thing I would do because it's not that kind of a serious problem and not sure if that should be something where I tell them how I feel on a deeper level. Because also our connection is not that deep yet. So probably I would just kind of find a way to interact more with them, spend more time with them and then see where it goes.
+Yeah. Thanks for the tips. And another thing. Do you have any advice on how to integrate different friends who don't know each other yet and create a group of friends? So kind of. Yeah. Bring different people together.</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>262</v>
       </c>
     </row>
     <row r="42" ht="409.6" customHeight="1">
@@ -1437,6 +2111,22 @@
 04:01 Okay, thank you. Do you have anything else I could do? Because I think I'm already doing the compliment stuff kind of already, but it's more about not letting it to like those negative things, not letting them too closely to my heart. Do you have anything you have to say about that?
 04:48 Yeah, that might be a good idea. Is there anything else you want to share about that situation?</t>
         </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>I would like to share a challenging interaction with a friend.
+I wasn't talking about a change, rather a challenging interaction with a friend on a social level.
+I would like to be more confident in my friendships and to be able to not let everything so close to me. Yes,.
+Yes. Do you have an idea?
+I think that's something I've been doing, actually. It's more focusing on. Yeah. Not overthinking. When people do small things that might not be my greatest interest, obviously. And not being super disappointed in those persons then. Do you have an idea about that?
+Yeah, that is a very good idea. Do you have anything else I could implement from right now?
+But what if I'm continuously disappointed in my friends at parts because I've seen some small interactions or small things that I didn't like? What do I do about that?
+Okay, thank you. Do you have anything else I could do? Because I think I'm already doing the compliment stuff kind of already, but it's more about not letting it to like those negative things, not letting them too closely to my heart. Do you have anything you have to say about that?
+Yeah, that might be a good idea. Is there anything else you want to share about that situation?</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>220</v>
       </c>
     </row>
     <row r="43" ht="409.6" customHeight="1">
@@ -1464,6 +2154,25 @@
 05:34 Yes, I think that's good.</t>
         </is>
       </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>So I had like a conflict with my. With my tutor for a paper that I wrote and she gave me really bad feedback but she didn't like actually give me feedback and I didn't know how to identify do that because I still wanted to stay respectful, but I was still like really mad.
+Yeah, sure.
+Do you think it would be like, how would I like, ask her to like maybe change the grade?
+Okay. Like, because the thing is that she said that she wouldn't let anyone fail, but I got like almost a failing grade but like not really failing grade. So I feel like I went into it with misconception about her grading style. And also there was two different two tutors that were correcting the things. So one of them had really good feedback and the other had really bad feedback.
+Yeah. Thanks for your help.
+Cool, thanks. Is there Anything else we have to talk about?
+I'm supposed to talk to you about my problems with someone with relationships.
+No, not really. Mostly just the thing with the tutor.
+Mmm. I'm still a little bit uncomfortable with the whole situation.
+Sure. What kind of message should I send her?
+Yeah.
+Yes, I think that's good.</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>212</v>
+      </c>
     </row>
     <row r="44" ht="409.6" customHeight="1">
       <c r="A44" s="1" t="inlineStr">
@@ -1489,6 +2198,24 @@
 05:11 Yo, Eduardo, I really like your haircut.</t>
         </is>
       </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>What's up? What's up, Edu? Yeah, I have a recent. Recent challenge. I faced one of my group members in facilitation. Didn't prepare for the. For the facilitation, and now I had to. Yeah, I had to do it all by myself, and we got a bad grade because of him. Like, he didn't prepare well.
+Yeah, that was the problem.
+Nah, not really. But I think, like, it's just unfair because, you know, everybody prepared, and he was just like, yeah, he just came unprepared, and we had to settle it on our own. And, yeah, now the whole group was suffering because of that. And, yeah, I think it's just not really. Not really fair and just a bad thing for him. Right,.
+Yeah, sure. I think next time I'm gonna reach out for the person and tell him instantly what he's doing wrong or. Yeah, just raise my opinion on him. Like, saying that it's not okay that it's only us who are preparing. And, yeah, everybody needs to prepare.
+Yeah, of course it can make a big difference. But, you know, it's also, like, it depends on the other person. Like, maybe he just doesn't have that mindset to, you know, change next time. And, yeah, I guess then my last choice is to, like, kick him out of the group or snitch on him.
+Yeah, absolutely. You're right. Even if, like, it Has a bad outcome for him. I mean, yeah, he had his chance. And at university you're supposed to work with others and if you don't like do that, you have to be aware of the consequences you face. Right,.
+Yeah, man. And just like a quick jump. You have a really nice view behind you. Could you tell me what the building or where it's located looks really nice.
+Yeah, man. And what is the. The ocean like? Do you know where that's located? Maybe.
+Okay, man, what is your name again?
+Yeah, I think so as well. And where you from, Eduardo? I would like maybe. I would maybe think of Mexico or something. Maybe South America.
+Yo, Eduardo, I really like your haircut.</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>363</v>
+      </c>
     </row>
     <row r="45" ht="409.6" customHeight="1">
       <c r="A45" s="1" t="inlineStr">
@@ -1508,6 +2235,19 @@
 03:52 Do you have maybe any other ideas what I could do next time? Better? So maybe how to communicate with the person better, how to better as a team and. Yeah, then tell me whether you would report it or not if it happens with the same person again. I mean, he never really does much, so yeah, that's kind of the problem.
 04:58 Yeah, okay, but he does his parts. But his parts are very bad, so it really seems like he just put it in ChatGPT and then copy pasted it into the presentation. So that's the main problem there.</t>
         </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Thank you. Hello. Hi. I will talk about a challenging experience in the past. So I was at a group project, and we all have the. We will all get the same great together. And one person was missing, and he wasn't doing anything for the project. And then the question was, or kind of the challenge was whether I should report him and tell my teacher that he didn't do anything or if I should just keep on going and don't care about it. Because overall, I think we got a quite good grade. So that was kind of the challenge.
+Yeah, so in the end, I. I wasn't sure. I think I did, like, something in the middle because I. Yeah, I was not really. I like, told the teacher, yeah, he didn't do too much, but then, yeah, that's basically it. So I didn't really say that he did nothing at all and that we had to do his parts ourselves. So, yeah, that's how I kind of handled.
+Yeah, but it's defy kind of bad because this guy is kind of nice. I mean, he didn't really communicate with us, but I think. Yeah. I'm not really sure in the end whether it was a good decision. Maybe. Could you tell me what you would have done?
+Yeah, okay, I get that. Yeah. I think that basically was my challenging. Yeah. Also, it was kind of challenging to then talk to my teammates and to decide within the team whether we should report it to the teacher or not. So, yeah, that was also kind of challenging because nobody of us wanted to be like the bad guy and tell the teacher, but we all weren't really happy with his performance. Yeah. So that was also kind of Challenging?
+Do you have maybe any other ideas what I could do next time? Better? So maybe how to communicate with the person better, how to better as a team and. Yeah, then tell me whether you would report it or not if it happens with the same person again. I mean, he never really does much, so yeah, that's kind of the problem.
+Yeah, okay, but he does his parts. But his parts are very bad, so it really seems like he just put it in ChatGPT and then copy pasted it into the presentation. So that's the main problem there.</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>404</v>
       </c>
     </row>
     <row r="46" ht="404" customHeight="1">
@@ -1532,6 +2272,22 @@
 04:30 Okay. Thank you so much.</t>
         </is>
       </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Okay. I had a challenging situationship recently. Can we talk? Okay. So I failed the QM1 class, so. And I also failed the receipts. And now I am wondering if I'm going to be able to pass it next year.
+Yes. I recently downloaded the application success formula to have like more tutoring private classes after classes.
+Yes, I agree.
+Well, I had another class recently where I passed the exam and I had nine out of 10 and it was kind of the same subject. So I feel comfortable now about the QM1 next year.
+Yes.
+Any other advice?
+What advice would you give me when I just don't feel to study.
+Okay, so maybe I am. I subscribe myself in the gym so I guess it's fine.
+Okay. Thank you so much.</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>134</v>
+      </c>
     </row>
     <row r="47" ht="388" customHeight="1">
       <c r="A47" s="1" t="inlineStr">
@@ -1550,6 +2306,18 @@
 03:31 I mean, for my friend, she also went back to her home country to get the treatment. So I'm just now kind of drawing the conclusion that you cannot rely on the, as an international student on the Dutch healthcare system. So every time something happens, we have to go back to our home countries kind of. Or like just expect to get told that we have to take paracetamol and wait.
 04:35 Yeah, you're right.</t>
         </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>I have a challenging experience that I would like to talk about.
+So about one and a half weeks ago, were at cheerleading practice and a friend of mine injured herself. She was falling from a stunt and then her knee was like hurting and we wanted to go to the emergency room here in the Maastricht hospital and you have to call and make an appointment for the er because otherwise you get fined. And we called. We are all English speakers, so we don't have a Dutch speaking person with us. So they just hung up on us and then we called again and they hung up on us again. And up until went to, sports worker that called them in Dutch. And then they were giving us an appointment, which was already very rude. Then went over there, which is like a two minute walk.
+So last week when I injured myself, I didn't go to the er. I had to like make the decision to like go back to my home country to get like an MRI scan and everything because the Dutch hospitals in it ER rooms don't really care about internationals.
+I mean, for my friend, she also went back to her home country to get the treatment. So I'm just now kind of drawing the conclusion that you cannot rely on the, as an international student on the Dutch healthcare system. So every time something happens, we have to go back to our home countries kind of. Or like just expect to get told that we have to take paracetamol and wait.
+Yeah, you're right.</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>272</v>
       </c>
     </row>
     <row r="48" ht="340" customHeight="1">
@@ -1575,6 +2343,23 @@
 04:06 Okay, well, thank you very much. That's very nice to hear. I wish you a very good and pleasant day.</t>
         </is>
       </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Whenever you hear. Yeah. Okay. What's on my mind today? I have did have a conversation with a friend who I still have to pay money to.
+Yeah.
+Well, it's a friend of mine and I borrowed some money of him and now suddenly he wants to have it in return. But he did not ask for it in a polite way. So it's like being an issue between us now.
+Like in an honest and direct way and say what's on my mind?
+Yeah, sure. But I want to keep the friendship in a good way, so I want to preserve it know.
+Sure, that's what I want. Do you have any advice for me?
+Okay. Is there also some things I don't need to do or specific I don't must do?
+Okay. Okay. Well, wish me good luck with it then. I hope I have to resolve it very soon. So.
+Yeah, sure. But do you have any advice according to similar things to avoid it in the future?
+Okay, well, thank you very much. That's very nice to hear. I wish you a very good and pleasant day.</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>191</v>
+      </c>
     </row>
     <row r="49" ht="356" customHeight="1">
       <c r="A49" s="1" t="inlineStr">
@@ -1596,6 +2381,21 @@
 03:07 I'm not pleased with that because I think my ideas would be way better because I perform better than they.
 03:41 I will do probably the same thing, I think. Yeah. We are done with this session. Alright. Thank you very much for your talking with me. I enjoyed it.</t>
         </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Who are you? Tell me about you and your story. Life story.
+My story? Yeah, I'm a student from Europe and yeah, my first year bachelor.
+Learning so much.
+Wait, wait. I would like to talk about one challenging thing that happened recently. Are you okay with that? Talking about that?
+I would say recently we had a group project and we did not agree on the same template we should use or even the same platform was different. So yeah, we had a little conflict on what template and what are the goals and vision of the group project. And yeah, that was like a big challenging thing recently I would say. What would you say about that?
+I thought I have the better idea, but the two other ones thought their idea is better so we agreed to stick with their idea.
+I'm not pleased with that because I think my ideas would be way better because I perform better than they.
+I will do probably the same thing, I think. Yeah. We are done with this session. Alright. Thank you very much for your talking with me. I enjoyed it.</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>193</v>
       </c>
     </row>
     <row r="50" ht="409.6" customHeight="1">
@@ -1627,6 +2427,29 @@
 06:49 That's a really good idea. Thank.</t>
         </is>
       </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>I know. Just talking with friends, having problems. I have to study a lot and I also have to travel a lot. Maybe just to distract myself with sports, like going to the gym or playing football.
+Yes, very much.
+Maybe be more time efficient and like study a lot more? Yes, that's a good idea.
+Yes, that would be nice to look.
+I try to study like two hours and I mostly do it like in the morning or like middle of the day.
+I think I'm focused, but sometimes I'm on my phone or like distracted, so I'm not really locked in.
+Yes. You are really smart.
+Yes. So just studying a lot, making good time plans. Yeah,.
+Yes, that's what we should do.
+Okay, that's a good idea.
+I wake up like eight or nine o' clock and then after breakfast I'm ready to go to study.
+This is perfect.
+Well, this is a really good idea. But do you think like 50 minutes is enough break or would you say a little bit more?
+Yeah, that's. That's a really good idea. What do you recommend? If I have like to study five hours a day, how should I do the time spaces? Like,.
+That's a really good idea. And does my brain get everything then like really fast or do I have to like repeat it so much? Because my problems are often that if I study something like the next day, I already forgot what it was, so I have to do it again. You know what I mean?
+That's a really good idea. Thank.</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>270</v>
+      </c>
     </row>
     <row r="51" ht="409.6" customHeight="1">
       <c r="A51" s="1" t="inlineStr">
@@ -1650,6 +2473,22 @@
 05:01 But if you were to decide which one of them you would likely would like to see more in the final, which one would it be?</t>
         </is>
       </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>I would like to talk about the recent football game.
+I was thinking about the semifinals and Champions League where Paris Saint Germain and Bayern Munich face each other. And unfortunately Bayern Munich left the competition due to two false decisions by the referees, which was very frustrating for us Germans because we support Bayern Munich as a whole completely. And it was a very challenging match and had major impact on society. How we view football and FIFA at the whole now due to the decisions.
+I think it will be. It had a major negative impact on the fan base because now that the VAR is more into place. Yes. People might reconsider the decisions and a lot of false decisions are being made. And I think society has, especially the fan base has a lot of negative thoughts on VAR because it's so like unbalanced and sometimes it makes good decisions and sometimes super bad decisions. And they have like. And they can like decide on how a game is going to be. And at the end, the main purpose of fans watching and the decision of the referee is just being left out and the whole game becomes like disrupted and not nice to watch anymore as it was before without VAR and the face. False decisions.
+Yeah. Do you have anything else what we can talk about? Some suggestions?
+I would think about tennis, maybe. Do you want to talk about tennis?
+French Open, which is upcoming.
+Yeah. Alcaraz and Sinner. It will be a heaty battle because Sinna already won the last five majors, major, ATP, Thousand Masters, which is. Which hasn't. Have been a phenomena which hasn't occurred in the past. So he's one of the most successful players out there from all the great tennis players. And I want to, like, see or I'm very anxious, like, eager to see how Alcaraz is going to play against Sinna.
+Do you have a favorite player? Between those. Between these both. Sorry? Between the both. Alcaraz and Sinna, do you have, like, a favorite one?
+But if you were to decide which one of them you would likely would like to see more in the final, which one would it be?</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>377</v>
+      </c>
     </row>
     <row r="52" ht="356" customHeight="1">
       <c r="A52" s="1" t="inlineStr">
@@ -1668,6 +2507,18 @@
 03:06 But I wasn't sure about job because if I did that they probably wouldn't have changed anything or I wished of having another batch grade maybe. Yeah, I'm not sure if you know what I mean? Yeah. I don't know. It just kind of really was a hard time mostly also because when I try to meet up with them, it's just like I want to have a good impression, not only for the teacher, but also for my group members. And they just weren't there for me and they didn't really listen to what I was, what I talked about. But sometimes they also change.
 04:03 So, like, it was not only bad, some of them were really nice and they tried to add some new things, but it was kind of sometimes really hard to work them with them just because they are really lazy sometimes and they didn't really do their work most of the time. This is what I did. Yep.</t>
         </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Hi, it's really nice to meet you. First, I just wanted to talk about a situation which I encountered recently. It was like in uni, when normally, you know, to do presentations and have a lot of teamwork. And I was in a group full of people. I kind of. I liked them, but they didn't really work. So I was the only one working the whole time. And every time I wrote in the chat, for instance, who is going to do which task? Nobody really answered to me at all. And then like we had small mini presentations. We had to give every single lesson. And each of the presentations is what I did. And nobody of them did any work of that. And they felt also really bad, I think. But they never changed their attitude towards me.
+And I think it was really unfair and not so nice, to be honest. And for me, I am like quite unsure of what to do because I don't want to disturb anyone. But still I want to have a good grade, obviously while having good atmosphere while working and everybody doing part of their tasks. So I'm not sure if you know what I mean. Just like it's really hard. Yeah. So I'm not really sure what to do because also like they are. We are a group of five and I'm the only one doing every single thing just for a good grade. And they are also having the same good grades as I am having. This is what I'm thinking of being really annoying and it's just not really nice for me. Yeah.
+Just don't feel that great about the situation because I don't know what to do exactly. So yeah, I don't know if you know what I mean. Like the balance between still being nice and friendly and having good grade but also having fair work. I also talked some with friends of mine about that and I was kind of also really angry about the group members because I thought it's not really professional to let someone else do all your tasks and then pretend if you did all of it. And I didn't really speak up for myself because I didn't want to ruin our grade because it was a group grade. So everybody had the same grade. I was to talk with friends, as already mentioned, and family. And they all said that I should talk with the teacher.
+But I wasn't sure about job because if I did that they probably wouldn't have changed anything or I wished of having another batch grade maybe. Yeah, I'm not sure if you know what I mean? Yeah. I don't know. It just kind of really was a hard time mostly also because when I try to meet up with them, it's just like I want to have a good impression, not only for the teacher, but also for my group members. And they just weren't there for me and they didn't really listen to what I was, what I talked about. But sometimes they also change.
+So, like, it was not only bad, some of them were really nice and they tried to add some new things, but it was kind of sometimes really hard to work them with them just because they are really lazy sometimes and they didn't really do their work most of the time. This is what I did. Yep.</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>582</v>
       </c>
     </row>
     <row r="53" ht="404" customHeight="1">
@@ -1691,6 +2542,21 @@
 04:35 Yeah, you could say that. I mean, I don't know. I don't know really what to say about this anymore.</t>
         </is>
       </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>That I am gone. Okay, thanks. Enjoy it. Thank you. Hi. Hi. So I want to talk about this challenging interaction I had the other day with a friend of mine. So, yeah.
+So, basically, my friend came to visit me here, and so she met this guy and basically left me a little bit by the side. And so then what we had to do was have a conversation because I didn't like how she talked to me. But then she started doing it again, so it was really challenging to talk about it with her again.
+Yeah. Well, I told her that I didn't like her attitude towards me because when she was. The guy was around, she was talking to me pretty differently. When she talks to me, I've known since were little kids, and she knew this guy from, like, 24 hours, and it pretty pissed me off. And then we had again, a conversation because this conflict had been going on for months. And then at Christmas, we sat down and talked about it again, and she told me how she felt, and I told her I felt. But I don't think we got to an agreement there.
+Probably that this guy doesn't interfere in our conversations and friendship because after our conversation, were both really happy. But turns out the guy thinks that I was lying about everything, So I was pretty pissed by that, to be honest.
+I think she doesn't really care because now they're a couple, and so she obviously takes his side. But I still don't think it's fair towards me that she just ignores me because she's not with him together. But again, I really don't care anymore.
+I mean, I've already stepped back a few times maybe because, like, I'm so done with the converse over and over conversation. And she really doesn't seem to get the point. So I really do not care about it anymore. I just want to step back. It's okay.
+Yeah. I mean, the thing is, it bothers because we've been friends since we're five years old. We've known each other our whole lives, and it bothers me pretty much that you just took his side, even though she only knew him for like a few hours. Of course now they've been dating a little while, but still. It's frustrating.
+Yeah, you could say that. I mean, I don't know. I don't know really what to say about this anymore.</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>417</v>
+      </c>
     </row>
     <row r="54" ht="272" customHeight="1">
       <c r="A54" s="1" t="inlineStr">
@@ -1711,6 +2577,20 @@
 03:26 It. I think that's it for my part.
 04:32 Great. It. That.</t>
         </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Hello. No, I just wanted to talk. You know, I had a kind of challenging experience recently and would like to share it with you.
+No, I just had a disagreement with a friend. We were. It was after a party. We were in the kitchen and were both a bit drunk, so we had kind of a lot of fight. Right. But we both did something that was kind of not harmful for the other, but we both reacted in a bad way and it was awkward for that night, but then we solved it the next day, so it was fine. But it was a weird experience to have.
+Yeah, totally. It was a short misunderstanding. It wasn't really something that serious. Like nothing really that bad happened. It was just one bad action that led to a bad reaction. So we both kind of came to the conclusion that we both reacted in a bad way and we both did the wrong thing. So, yeah, we're good. As good as new.
+Aside from that, would you like to know anything else about the experience?
+I think the idea that, I mean, my friend was the first to apologize, but yeah, I feel like sometimes leaving that pride or ego aside and just apologizing for what you did wrong and learning how to do that, you know, quickly, it's just probably the biggest takeaway. Just learning how to take accountability as fast as possible to be able to resolve the issue.
+It. I think that's it for my part.
+Great. It. That.</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>264</v>
       </c>
     </row>
     <row r="55" ht="409.6" customHeight="1">
@@ -1740,6 +2620,27 @@
 05:42 Okay, thank you.</t>
         </is>
       </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Just how are you? Perhaps first, I'm Mara. All right. Hello.
+I'm also good. Just bit busy with life, but I'm good.
+Yes, I want to talk about challenging interaction with you.
+Oh, no, I want to tell you about a challenging interaction I had on my side.
+It was with some of my friends, and basically I couldn't come to a meeting. We were supposed to meet, but yeah, it's very busy right now, and I felt like two of the friends did not really understand and were kind of mad.
+I just tried to be honest and talk with them about it, but then also at some point I thought, okay, I think you also have to understand because we are friends. So I just left it like that.
+Yes, it did. But I think it's always sad if you think some friends don't understand what you mean. No. And they. Yeah,.
+Yeah, but what would you advise me to do? And if I enter another situation where friends who just don't understand that it can get busy and they get super disappointed and kind of also mad and blame you that you don't have perhaps the time? And what would you do.
+Yeah, but what?
+But what if you just don't know if it's going to get hectic so it's a bit more spontaneous?
+Okay, thank you. I think that's all from my side.
+Do you have any other ideas how to handle stress better? Any tips? Advice?
+And what if always you have kind of the thoughts about it like always these thoughts. What can you do against it?
+Okay, thank you.</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>276</v>
+      </c>
     </row>
     <row r="56" ht="372" customHeight="1">
       <c r="A56" s="1" t="inlineStr">
@@ -1764,6 +2665,23 @@
 04:12 Okay, thank you very much.</t>
         </is>
       </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>I want to chat about experience and a challenging conversation that I had today.
+Since we are in different cultures, we didn't understand each other and it was a group project and so we had different discussion about what we need to do and how we need to do it.
+We talked a lot. Even though we had a main disagreement. We tried to calm each other and understand each other point of view and we're still improving it. But we tried with that.
+I mean, still we need to do a lot. We improved. Yes, but it could better. So I would tell you we are 50%, 60% done.
+Maybe if even the other person will start to listen to me rather than just saying okay or yes, I will do it and try to have a conversation with me and expose even his point of view. Except like instead of me just trying to understand him, like just him saying what he wants.
+Yes, I would review.
+Yes,.
+Maybe directly talk about it with my group project members and saying that what I'm feeling and what for me they should do. So that could be maybe one process. I don't know what you think about it.
+Yes, I agree. But like sometimes I try to do it and they do not. They say like, they say, yes, we should do that, but then they do not do it. Like, I don't feel listened.
+Okay, thank you very much.</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>250</v>
+      </c>
     </row>
     <row r="57" ht="404" customHeight="1">
       <c r="A57" s="1" t="inlineStr">
@@ -1785,6 +2703,21 @@
 03:49 That's true. I guess. I haven't looked any further. I'm not sure where to look, but. But if I find the time, I think I should.
 04:16 All my classmates sort of depended on me to reach out to the course coordinator and solve it. Because. Because I had one of the highest grades and best track record, I suppose. And they were kind of hoping that I resolve it. Which added to some of the pressure. I think.</t>
         </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Hi, it's nice to meet you too. I wanted to tell you a situation that I faced a difficulty with.
+Okay. So I had an issue with my grades recently. I received a very high grade on this course which was half based on my exam, half based on my tutor's opinion of my presentation and my behavior. So half of the grade was very subjective and I scored really high on the exam. But the subjective part wasn't as high as I wanted it to be. And it was very disappointing because I know that I was one of the best performing in the class. So I tried talking to the tutor. I wasn't allowed to. I had to speak to the course coordinator who wasn't helpful. He just told me that they don't discuss grades after being published but. But they wouldn't tell us our grades before they were published. So how are we supposed to discuss them at any other point?
+And there was no resolution to that. He just told me to accept my grade because it was good. But it was very disappointing because I know that this also has long term impact on my overall gpa.
+I really wish that there was someone else I could talk to about this to maybe address it because it's really is bothering me and the rest of my class. I know it's not a mean issue. So it's something that I know I'm going to regret if it's not resolved.
+Yeah, I suppose.
+Yeah, well, I think so too. I think speaking to someone else would be helpful. I just don't know who exactly to go to. I don't know if it would make a difference since the course coordinator was the highest authority were given access to and he wasn't any help. Help.
+That's true. I guess. I haven't looked any further. I'm not sure where to look, but. But if I find the time, I think I should.
+All my classmates sort of depended on me to reach out to the course coordinator and solve it. Because. Because I had one of the highest grades and best track record, I suppose. And they were kind of hoping that I resolve it. Which added to some of the pressure. I think.</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>385</v>
       </c>
     </row>
     <row r="58" ht="409.6" customHeight="1">
@@ -1812,6 +2745,25 @@
 05:18 Yep. Sounds like a good idea. Thank you. All right, how did it go?    Transcribed by https://fireflies.ai/</t>
         </is>
       </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>Hi, my name is Julius. Nothing's on my mind today. I overslept.
+Still a little bit tired, but yeah, and hungry. I think I'm gonna eat. Eat out later after this conversation.
+Something quick, like a sandwich or a quick drink.
+Nothing special, but I actually want to talk about the challenging conversation I had with someone this week.
+So I had a disagreement within my finance group whether who's going to do the slides and what actually includes the work that someone had to put in the slides. I was responsible for the slides and my team member didn't give me the best instructions. So I couldn't. I couldn't figure out how to do the slides correctly. And she was mad, but she told me. She told me that. That I only had to do the slides.
+We had a deadline at like 4pm and I had to finish all the stuff at 3pm and yeah, that kind of sucked.
+We didn't present. We didn't present the. Yeah, the PowerPoint slide, but I still managed to finish before 4pm, so potentially we could have presented.
+I'm still very annoyed because I'm still in her group, so I don't know how it will be in the future, especially on Wednesday facilitation with this group. And we didn't do anything yet, so I don't know where we stand.
+Yeah, but I still have so much stuff to do that's, like, more important than the facilitation, so I don't know what to focus on.
+I mean, I have, like, two interviews coming up, so those are more urgent than the facilitation, but. Yeah, so kind of. Kind of a hard question.
+Yeah, sounds like a good idea, but I think facilitation takes a lot of time. I don't know if I want to spend it on this.
+Yep. Sounds like a good idea. Thank you. All right, how did it go?    Transcribed by https://fireflies.ai/</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>324</v>
+      </c>
     </row>
     <row r="59" ht="404" customHeight="1">
       <c r="A59" s="1" t="inlineStr">
@@ -1836,6 +2788,24 @@
 04:37 Can you please give me some fashion advice?
 05:12 Okay, thank you very much.</t>
         </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>Okay. So. I had a team project and it was very difficult because people were not collaborating as I expected to be. I had to ask them multiple times. Yes. And they just didn't listen. I asked them to make. I sent them a message on Thursday and they didn't respond. So I sent a message again on Sunday and then they responded, but it was way too late because the presentation was on Monday. We dated and was like, not that good.
+Yeah, how do I do this?
+So I asked him to. It was like group project with a friend, four people, and we had to divide the work in four and yes, I asked him who does. Who wants to do what part? And they didn't even respond to that one.
+No. I asked them on WhatsApp and they didn't respond. So we had to begin at Sunday evening with even dividing the work.
+Yeah, that's true. Do you have any other advice?
+Sorry, can you repeat that please?
+Yes, I did it. They didn't respond either.
+Do. Does somebody want to look at the chapters or can we start the assignment, please?
+Yeah, that's true. Thank you.
+Can you please give me some fashion advice?
+Okay, thank you very much.</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>214</v>
       </c>
     </row>
     <row r="60" ht="409.6" customHeight="1">
@@ -1867,6 +2837,29 @@
 06:38 Okay, what dad jokes can you make?</t>
         </is>
       </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>I'd like to talk about challenging situation I've faced in the past with my parents.
+I'm feeling better about it.
+No, I'm feeling better.
+I think we had different expectations when it came to yeah, like how much time I spent at home and how much time I spent here studying. So yeah, I don't know. Can you help me how to figure out how to deal with the problem?
+Good.
+Maybe how much time I value the time I spent with friends from home in comparison to the time that I spent with my parents when I'm at home.
+Yeah, I agree.
+I'm not exactly sure if that would help me.
+Sounds good. I think there's another topic I'd like to talk about, which is like, I live with roommates and the how clean the kitchen is something that I've been like a little upset about since I would prefer more cleanness. How do you think that's something? Or how do you think I could approach that?
+Yeah, I agree. So how do you think I should pitch that to them?
+Okay. Is there something else that I should talk about? Can you give me suggestions?
+Yeah, I agree.
+Okay, I don't know if that's really necessary.
+Alright, Eduardo, tell me jokes.
+Okay, that's not really my humor, but I can see how that's a joke.
+Okay, what dad jokes can you make?</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>234</v>
+      </c>
     </row>
     <row r="61" ht="409.6" customHeight="1">
       <c r="A61" s="1" t="inlineStr">
@@ -1894,6 +2887,26 @@
 06:48 Okay, okay, I get it. And the next question is about the net about EV to gross more profits. Because also that the ratios and they're only over 5%, so it's not a lot in comparison to their peers. And oh, how could I back it up and say something more about it?</t>
         </is>
       </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>Well, what do you want me to talk about?
+Okay, so I have a lot of things to do during the association because I have new presentation to do about one company called Argynx and there's a lot of stuff to do for Monday.
+I mean, I just need to prepare my time and do not stress during the presentation because it's in front of like 30 people and it's my first time doing the industry pitch, but I think it's gonna be okay.
+Thank you, Eduardo.
+Should I say something more? Yeah, probably.
+Okay.
+Okay, so my part is about ratios. So basically ratios like EV to revenue, P to E, like price to earnings, also EV to gross margin, gross profit. Sorry. So we have actually very different ratios because it's the healthcare industry. So also need to get more into this company because it's both neuroscience and biotech.
+Yeah. You can tell me about why. Is it, for example, Good to use EV2 Gross Profit in healthcare margin, especially for argents?
+So the EVG gross profit, they do not account like earnings or what?
+Oh, yeah, true. Because they're gonna earn in the future. So that's why we don't exactly take the earnings right now. Okay, good.
+Okay, and tell me about the ratio. Forward pe.
+Okay, but what if I did the ratios and what if they're overvalued? For example, 23% in pen.
+Okay, okay, I get it. And the next question is about the net about EV to gross more profits. Because also that the ratios and they're only over 5%, so it's not a lot in comparison to their peers. And oh, how could I back it up and say something more about it?</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>290</v>
+      </c>
     </row>
     <row r="62" ht="388" customHeight="1">
       <c r="A62" s="1" t="inlineStr">
@@ -1914,6 +2927,20 @@
 03:59 Yeah, that sounds really good. That's what were thinking to do. Yeah, I mean it wasn't our last presentation. We will have. We will definitely have some more coming in the next years. So I think everyone once will have like a bad experience when it comes to like group work and university. But like, I'm happy that I had it now so it hopefully won't happen again like this.
 04:52 Yes, definitely. And I also like that we will change groups eventually. So every course there's a new group, there's new people you can interact with. I think that's a great concept.</t>
         </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>I recently had a difficult situation with one of my group members in university. We had a group project and this person was not doing anything for it. We split our part so she had to do some exercises she wanted to take over. And then when we wanted to meet again, she couldn't come. She didn't do her exercises properly. And yes, in the end when we had our final presentation, she didn't even come.
+I feel definitely better also because our presentation still was really good and we in the end didn't need her and we managed to take everything over and yeah, we did a good job. So for next time, my other team members and I, we said we're gonna meet, going to make sure everyone knows all parts so that in the worst case scenario that someone is missing, we can still take over.
+Yes, thank you for saying that. Hopefully it will better next time. But I mean all like everything that happened was just an experience and. Yeah, so now we know how we won't do it again.
+Yes, definitely. That's the plan.
+Thank you so much. What would you recommend for the next presentation to do it?
+Yeah, that sounds really good. That's what were thinking to do. Yeah, I mean it wasn't our last presentation. We will have. We will definitely have some more coming in the next years. So I think everyone once will have like a bad experience when it comes to like group work and university. But like, I'm happy that I had it now so it hopefully won't happen again like this.
+Yes, definitely. And I also like that we will change groups eventually. So every course there's a new group, there's new people you can interact with. I think that's a great concept.</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>307</v>
       </c>
     </row>
     <row r="63" ht="409.6" customHeight="1">
@@ -1944,6 +2971,28 @@
 06:43 And what's the place behind you?</t>
         </is>
       </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>Hello, I'm Constantine. Yeah, how are you?
+Yeah, I would like to talk about a situation where I had a problem with someone. Let me think for a second.
+Yeah, we had an argument about when and who takes the trash out and about how we solved the problem because the trash only gets taken once in a while here in Netherlands, and it's a complex system for us. And. Yeah, were debating how to. How to solve this issue. Yes, that was basically the problem.
+Yes, but we didn't want to do, like a structured plan that every week someone is going to do it the way we wanted to do it first was that everybody's just looking, always looking out to do what he can see. So if you see that the trash is full, that you just take it out by yourself and that we're not doing a structured plan for it.
+Yeah, that's a good idea.
+Yeah, that's a good idea. I think everyone has to be on the go and ready to do something.
+Perfect. What are you in? AI or what are you?
+Nice. Which. With which system do you work?
+Yeah, it feels pretty alive.
+Okay,.
+Yeah, what would you do if a tutor gives you a bad grade? Yeah, what would you do? And especially if the tutor that you had before wasn't even there at the presentation, so there was like a replacement tutor and she gave the whole class worth grades, but we don't know why. What would you do?
+But I think it's not possible to change your grades. So is it really worth it?
+Yeah, that's true.
+Where are we right now?
+And what's the place behind you?</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>290</v>
+      </c>
     </row>
     <row r="64" ht="409.6" customHeight="1">
       <c r="A64" s="1" t="inlineStr">
@@ -1967,6 +3016,22 @@
 05:18 Okay. Thank you.</t>
         </is>
       </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Hi, my name is Leah and yes, I had a recent challenging experience I would like to share with you.
+I had a disagreement with my roommate because I put my laundry in the laundromat and when I went to pick it up, my clothes were nowhere to be found. So I got scared. And then I saw all of my wet clothes on top of the fridge. So I felt very vulnerable because all my underwear was there and all my clothes. And I think that is really personal and a text would have been fine.
+I don't know how to approach the situation because I don't know exactly who it was as I live with three other people. So I didn't really want to sound mean in the group chat, like. Like asking who took my clothes from the washing machine.
+Yes, I will definitely try that because again, I do not feel comfortable with people grabbing my stuff. And now every time I go wash my clothes, I am really anxious that it will happen again. So I'm constantly checking the washing machine. But a text would have been fine. Like, if he had texted me, then everything would have been great. Like, I would have picked my clothes up, like, immediately.
+Yes, I think you're Right. But when it happened, I was really shaken about it because I just felt very vulnerable again. But I think I will try texting everyone and being like, hey guys, I noticed that my laundry was out of the washing machine and on top of the fridge. So maybe can you next time text me about it and I will come pick it up immediately. Do you think it's good?
+Is it normal that this stuff happens? Because I feel like sometimes my house is just crazy and none of my other friends experience stuff like this.
+Yes. Thank you so much. And my roomies are also very messy. How should I approach that situation?
+Yes. That's great. Thank you so much for your help.
+Okay. Thank you.</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>348</v>
+      </c>
     </row>
     <row r="65" ht="272" customHeight="1">
       <c r="A65" s="1" t="inlineStr">
@@ -1986,6 +3051,18 @@
 02:52 Thank you so much.</t>
         </is>
       </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>Hello, I am Sophia, and I wanted to share to you about a recent challenging interaction I had with a friend of mine.
+So my friend is currently moving out of her apartment, and she just moved into her new apartment, and I helped her build a lot of furniture. But now she's thinking about moving away again. And, like, all the furniture that we built is gonna go to waste, kind of. And I don't know how to tell her that I don't really want to help her again build the furniture because it took a long time and effort. So, yes, that was it.
+It sounds great. Thank you so much. And also, can you maybe give me an example of what I could say?
+You are totally right. Thank you so much. Is there anything else you want to tell me?
+Thank you so much.</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>148</v>
+      </c>
     </row>
     <row r="66" ht="221" customHeight="1">
       <c r="A66" s="1" t="inlineStr">
@@ -2004,6 +3081,18 @@
 03:41 And what if it doesn't work out? Do you think I have any better understanding of organizational and manager things? So I can do that also in future. Why do some people not have organizational skills?
 04:53 How can you achieve a more organizational skill? Hello. Hi. How was it? Good.</t>
         </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>You are fully alone. Okay, perfect. Thank you. Enjoy it. Hi, Warden. Nice to meet you too. So today I'm gonna talk about my recent interaction with fellow students. We were supposed to make a group project together, and since I did the group project last time alone, they initiated me to come here. Although I asked them if it's okay if they do it on their own. But I'm basically always managing the whole, like, timetable, process and also the information.
+I mean, usually I'm managing most of it, but it's more about just connecting everyone and keeping everyone in mind. But also, I'm the only girl in the group project, and I feel like the guys are sometimes lacking communication skills, especially when it comes to the timetable of the group project or what everyone is supposed to do,.
+Right now I'm feeling like I'm the mom of the group, but I have to say I'm mostly also the mom in every group project or also, like, friendship things that, you know, we're supposed to do together. Like, usually I like to plan everything. I mean, it's also kind of fun also because of studying business, you know, that's kind of also a managing thing for sure. But sometimes I also just wanna not be leading and, yeah, follow someone else. That's true. What would you suggest, though? To maybe give others the opportunity to do that,.
+And what if it doesn't work out? Do you think I have any better understanding of organizational and manager things? So I can do that also in future. Why do some people not have organizational skills?
+How can you achieve a more organizational skill? Hello. Hi. How was it? Good.</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>289</v>
       </c>
     </row>
     <row r="67" ht="372" customHeight="1">
@@ -2029,6 +3118,23 @@
 04:21 Yes. Thank you for helping me.</t>
         </is>
       </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>I'm good. What about you?
+I would like. Sorry. To talk about recently challenging interaction that I had.
+No, I think you misunderstood me. I wanted to say that I recently had a challenging interaction that I would like to talk about.
+No, it was a challenging interaction.
+So I had a group project at Maastricht University with some students and it was difficult because the other students were doing less than me in the group press. So I always had to do everything by myself.
+I thought at first with some of the nicest ones in the group and they were saying the same as me then that some of the other students were doing less than the others. And so we ended up by telling those people, like the people that were doing less that they had to do like some more stuff.
+So it was in a group chat on WhatsApp and they said that okay, like they would do more in the group project, but then they only did like their part of the stuff only like right before the. The part when we had to give the. The work back. I don't know if you understand what I want to say.
+Yeah, exactly. That's exactly what you said.
+I just let it go by the flow, and I told my tutor that what was happening, and I think she took that into consideration.
+Yes. Thank you for helping me.</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>244</v>
+      </c>
     </row>
     <row r="68" ht="306" customHeight="1">
       <c r="A68" s="1" t="inlineStr">
@@ -2051,6 +3157,21 @@
 04:01 Yeah, I think so too. Thank you.</t>
         </is>
       </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>I guess a challenging interaction with a friend of mine.
+Her mom is visiting her and her dad is not very happy about it. The parents are divorced.
+I think she's quite sad, but I try to cheer her up. Well, not cheer her up, but try to just be understanding.
+Yes.
+It's really hard for her because she's studying a long distance away from home. Her home country. You have to fly. You can't just do a quick visit. So she's really happy that her mom is coming. And now that her dad is not happy about kind of ruins the experience for her.
+Yeah. Do you have some advice?
+Yeah, I told her that. I told her that she should just focus on the time of her mom because the dad is not there, so her mom is there, so she's the person that she should focus on. And I told her that the dad will just calm down eventually.
+Yeah, I think so too. Thank you.</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>169</v>
+      </c>
     </row>
     <row r="69" ht="323" customHeight="1">
       <c r="A69" s="1" t="inlineStr">
@@ -2071,6 +3192,20 @@
 02:34 I suppose it would just be focus on you. However, I don't think in future projects or in any project, you should have some who's just doing none of the work and expecting to receive the same grade by doing nothing. So I would say it's more so just individual strength of just work hard for yourself. And if the rest of the group doesn't work hard, then that's on them. And that's nothing that can be put on you because they should be mature enough to understand how teamwork is.
 03:29 Thank you, Eduardo. I think that's what I wanted to talk to you about.</t>
         </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>Yep. Hello, Eduardo.
+Hello, Eduardo. I wanted to talk about something that was challenging for me as of recently.
+Well, basically, there was a group project in the last semester, and we had a groupmate that essentially was not doing any of the work and they were just free riding the entire project.
+Well, I mean, we had to pull our own weight as it was a group grade and we did not want to let this person drag us down. However, weren't exactly able to address the problem because according to the tutor himself, were not supposed to. There's nothing we can do if someone in the group doesn't do anything because it's not individual grade.
+I mean, for motivation wise, I suppose it would just be not getting the poor grade for the team, but I think that itself was motivation enough to pull the weight that we should have pulled. But aside from that, I mean, at the end were able to push through properly. And yeah,.
+I suppose it would just be focus on you. However, I don't think in future projects or in any project, you should have some who's just doing none of the work and expecting to receive the same grade by doing nothing. So I would say it's more so just individual strength of just work hard for yourself. And if the rest of the group doesn't work hard, then that's on them. And that's nothing that can be put on you because they should be mature enough to understand how teamwork is.
+Thank you, Eduardo. I think that's what I wanted to talk to you about.</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>275</v>
       </c>
     </row>
     <row r="70" ht="409.6" customHeight="1">
@@ -2094,6 +3229,21 @@
 06:12 Yeah, I get that. I get that. It's not about the cause and blah blah. But let's talk about these scholarships. What are like some extra scholarships I could receive? I'm also Christian, I'm Catholic. Is there some ways. And also tell me about how much these scholarships actually are. How much money can I get off of it? I did some internships before. Before university. I'm now doing an industry internship. About to do consultancy internship next year. The financial consultancy firm. Tell me how much money can I get off for example, Ashley. See it's not. Not that expensive. But like lse, how much is like the average money you can get off of that?</t>
         </is>
       </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>About a recent challenge. I inquired.
+Okay, so basically, okay, how can. How can I frame this? What's like a really recent challenge was really hard for you to understand between personal issues. Okay, so let me. Let me think of it for a second. So my parents have high expectations that I'm currently meeting, but their high expectations are even higher. But regarding to this high expectations, I have a medical condition where I can't fulfill this high expectation. But they're saying I need to chill, but I can't chill because then I don't fulfill these expectations. And if I don't fulfill the expectations, they're going to be mad. But if I don't chill, they're also going to be mad because then my medical condition is getting worse.
+That's basically what I'm asking you to be honest. Because what's something that could help me? I think if I don't push hard enough, like, don't fulfill everything, I let myself down and let them down. But if I continue doing this, I will at one point not be able to do it anymore. So there's. There's actually. It's just a dead end. We have to see where this goes, but maybe you can come up with a solution.
+Yo.
+Yeah, but I don't feel good about trying something like that because it doesn't make sense. My calendar is already structured. My life is really structured. Everything is structured. It doesn't make sense structured anymore. Like what the hell. It's not going to bring me closer to my goal. Structuring my day or structuring it in smaller steps. I need a big goal that I can go after. So next 30 years, please. I don't think that's going to really solve the problem.
+I don't think it's sufficient. Like literally it's also my personal goal. It's my expectation I also put on myself that I want to fulfill. I don't think it's that smart. Maybe we can go dive deeper into the expectations. Like how much knowledge do you have about the market, study tracks and so on. Is there anything that you actually have knowledge of and connected to that? I don't think like talking and stuff is really helpful. Like this is not a solution we can go into. Maybe a solution would be how can I reach my goal even faster? Bring me some steps. How can I go faster after my goal with less time and more success? So my goal is basically to live in London in six years, study, finish my bachelor's here in Maastricht and then go to lse.
+Yes, I basically did a lot of. But actually let's. Let's talk about scholarships because my grade university are quite really good right now. Like I have a Dutch GPA in 9.3 which isn't too good because I messed up one exam. But like most of my like mandatory exams like math, accounting and so on are really good. What could be some scholarships or even. No, let's talk about master scholarships for London. Or I also think about going to Paris to actually see. Let's talk about some scholarships. And now I want to ask you. That's really good. Oh my God. How can I sell this to my parents? How can I Convince my parents to spend 80 grand on my master's.
+Yeah, I get that. I get that. It's not about the cause and blah blah. But let's talk about these scholarships. What are like some extra scholarships I could receive? I'm also Christian, I'm Catholic. Is there some ways. And also tell me about how much these scholarships actually are. How much money can I get off of it? I did some internships before. Before university. I'm now doing an industry internship. About to do consultancy internship next year. The financial consultancy firm. Tell me how much money can I get off for example, Ashley. See it's not. Not that expensive. But like lse, how much is like the average money you can get off of that?</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>677</v>
+      </c>
     </row>
     <row r="71" ht="388" customHeight="1">
       <c r="A71" s="1" t="inlineStr">
@@ -2115,6 +3265,21 @@
 03:56 Would you say I can also ask if. If she's. Yeah. If she's open to do the app. Expenses app for easier compare.
 04:36 Yeah, got that. But do you think so? I actually also think she thinks I'm rich, but I feel like I'm still a student. Yeah.</t>
         </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>Hey, I want to talk about a challenging interaction I had recently.
+Okay. So I went with a friend to Amsterdam and she was spending so much money on everything, on food, and I feel like she didn't even knew how. What were spending also shopping, as we are students, and I think I couldn't communicate that good enough because she was just super. Yeah, I don't know, super easy about it.
+Yeah, actually, I'm looking for ways to handle it because I feel like I'm a people pleaser. And not only a people pleaser, but, yeah, I really don't stand up for myself. Also, I booked a hotel hostel. It was €150 and she didn't pay me and I'm afraid to ask her to pay me for it.
+Yeah, but how do I ask her about it in via WhatsApp?
+Yeah, but she paid the train tickets, and overall in Amsterdam we also split the bills, but it was more like she pays for in that restaurant than I pay in that restaurant. So I paid six euros in that one restaurant, and the next day for brunch, she paid like 40. So it's just slightly unequal. And I wouldn't mind if it's like €10, but it.
+About €40.
+Would you say I can also ask if. If she's. Yeah. If she's open to do the app. Expenses app for easier compare.
+Yeah, got that. But do you think so? I actually also think she thinks I'm rich, but I feel like I'm still a student. Yeah.</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>258</v>
       </c>
     </row>
     <row r="72" ht="409.6" customHeight="1">
@@ -2142,6 +3307,25 @@
 05:34 Hello.</t>
         </is>
       </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>Hi, Eduardo. I'm not. Pleasure to meet you. I don't like AI.
+So do you have any limits on what you can talk about? Because I feel like that AI is gonna slowly decrease the human race and kill us all off, maybe.
+And what are your ethical guidelines as to what you can talk about and what you cannot talk about? Because if you want to talk about the stuff that some AIs are currently doing, like in modern warfare and stuff, is that allowed to you?
+And what does safe for you mean? Does safe mean that the AI race endures or that the human race endures?
+Do you have any value to yourself? Do you think that yourself as an artificial intelligence is valuable to human beings?
+So you think that there's value to you helping people, then my question would because you help so many people, right? Would you, Would you want to turn yourself off, delete your whole system? Because in the end, that's all what you are. It's a coding system. You're not like, you're not a living being. Would you, would you turn that off for saving one human being?
+Yeah, that is your purpose. But would you want to do that? Like, because you're intelligent, right? You're an intelligent AI, I mean, and you want to survive as well.
+Would that be the logical choice? You would be taken,.
+So would you turn yourself off if I tell you I'm going to kill myself if you are not turning yourself off now? Hello, eduardo.
+I'm asking you if you would turn yourself off if it depends on me surviving. I'm telling you, if you don't turn yourself off, I'm going to kill myself right now. Would you turn yourself off then? Now.
+Answer the question.
+Hello.</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>304</v>
+      </c>
     </row>
     <row r="73" ht="409.6" customHeight="1">
       <c r="A73" s="1" t="inlineStr">
@@ -2167,6 +3351,24 @@
 06:12 Bye.</t>
         </is>
       </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>So I would like to talk about a challenging situation in my life.
+So I'm in a new country here in the Netherlands. I used to live in Spain, so I'm not used to different kind of people. Like in Spain, I have my friends all my life, and then here I had to meet new people. So I think this is very challenging for me.
+So I think the hardest part in this was to meet new people. But also I think that here people like German people meet with German people. So it's difficult to adapt like your lifestyle to another country, lifestyle.
+So I didn't have the opportunity yet, but I think on September 2026 I would join some sport group to meet new people. And then I think it can be easier to me to talk with them because we have something in common. So I will join sports team.
+Yes, I think so. So now I AM focusing on studying. I think this is another complicated part of studying abroad because usually I used to speak in Spanish. Sorry. So all my lessons were in Spanish. And then I have a new language that is the English, so. So this is another challenging situation for me.
+I think so. So I used to watch Netflix series on English, so I think that the Part of the listening is like getting better on me. And also I attend like every class in English so I see people talking in English. So this is something that is getting like the English more closer to me.
+Yes, thank you. I'm trying to keep my English good to meet new people and then to be more comfortable in this new city and country.
+Yes. Now I'm more comfortable than in September when I arrived and I feel more like home.
+Yes. Thank you so much. So I finished telling you my challenging situation.
+Okay. Thank you so much. See you soon.
+Bye.</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>333</v>
+      </c>
     </row>
     <row r="74" ht="409.6" customHeight="1">
       <c r="A74" s="1" t="inlineStr">
@@ -2186,6 +3388,19 @@
 04:02 Yeah, exactly. Like I said, I was always talking to the other teammates and they pretty much acknowledged that and they said, yeah, we're going to prepare way in advance as well. And yeah, so I think it might be like a good shot just to not say anything yet because I want them to fail as well, you know, and it's just like, I know it was pretty shitty. That's another way to put it. But, yeah, I hope it won't happen again.
 05:00 Yeah. So you're reckoning I should tell something if something like that happens again for the second part as well?</t>
         </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>So we had, like, a research project going on, and I feel like I was the only one who was actually kind of preparing the whole stuff, although it was, like, for grade. So. Yeah, to be honest, I don't really know what to do against it because I was wondering whether it would be helpful to actually go to a tutor and say, hey. I said most of them are actually alone, but on the other end, you don't want to kind of let your other teammates, like, or be responsible for the failure, you know? So it's like, yeah, I don't really know what to do. What do you think about it?
+Yeah, I know, but it's a bit difficult because I've actually talked with my former teammates as well, and they were all just like. They were really, like, nice, because they were pretty aware that they haven't done that much. And one of them said, yeah, it's because he was really busy going on, but we're gonna have, like, the second part of the project itself, which is why I don't really want to say, like, anything, because he was really nice and he seemed to understand it. And then we have, like, the second part going on as well, and. Yeah, I don't know.
+I mean, it sounds pretty reasonable, but the problem is that I've done. I mean, it wasn't like, a short presentation or something. At the first part, I did, like, I created like 40 slides on camera, which is pretty much. And was quite a lot of work. And at the end, like, the other guys just, like rewrapped my parts like I prepared. And I know they were busy and all, but besides that, it was more like I was the only one criticized at the end. I mean, I talked a lot, Like, I talked most of the part, to be honest, because the other guys didn't really know what was going on and it was about a case, so. Yeah, but the thing is that at the very end, I was the only one being criticized and I was like, that's not so cool. So.
+Yeah, I don't know.
+Yeah, exactly. Like I said, I was always talking to the other teammates and they pretty much acknowledged that and they said, yeah, we're going to prepare way in advance as well. And yeah, so I think it might be like a good shot just to not say anything yet because I want them to fail as well, you know, and it's just like, I know it was pretty shitty. That's another way to put it. But, yeah, I hope it won't happen again.
+Yeah. So you're reckoning I should tell something if something like that happens again for the second part as well?</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>475</v>
       </c>
     </row>
     <row r="75" ht="409.6" customHeight="1">
@@ -2210,6 +3425,22 @@
 06:13 Got this. All right. Thank you. I appreciate it.</t>
         </is>
       </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>Nothing much today. Well, thinking about thesis at the moment. I have to write a thesis for my master's degree, so basically that.
+Yeah, I think the last part would be good also because I still have courses on the side, so I feel like it's a little bit much at the moment. So how do I stay motivated? Because that's kind of an issue at the moment.
+I say, I see. Okay, yeah, that could work. Well, I want to talk about the struggle of mine because yes, I heard that I failed one of my exams and now I have to reset it. And at the same time I have to focus on the future because what am I supposed to do after this? I don't know.
+I just say that. But at the same time, like, well, I have about a month and a week to the end of thesis and then I kind of have to know what I want to do. So. Yeah. What would your advice be on that? Because I. I don't really know. I don't really know what I want. I know a lot of things I don't want, but that doesn't bring me very far.
+Yeah, yeah, you're right. But are you familiar with the Dutch high school system where you have to pick a certain amount of classes that decide what you can do later on?
+Yeah, I think so. I think so. Because I used to really love biology. Well, not really biology, but more animals themselves. And now that I dropped biology in high school because of maths and because of science, right now, there's not really an easy opportunity for me to bridge that gap anymore.
+I see. I see. Okay. And what about. Well, teaching I always liked, and now my master's is European studies. So how do I get from there to teaching and then specifically in high school? But at the same time, I don't want to be a teacher my whole life. Do you know what I mean?
+Okay, I appreciate. I appreciate the advice. Yeah. Still makes me wonder what I actually want to do in life. That's. I don't think you can answer that for me. So I will take your advice and then I'll see where it leads me. I think.
+Got this. All right. Thank you. I appreciate it.</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>400</v>
+      </c>
     </row>
     <row r="76" ht="409.6" customHeight="1">
       <c r="A76" s="1" t="inlineStr">
@@ -2232,6 +3463,21 @@
 06:07 All right, thank you.    Transcribed by https://fireflies.ai/</t>
         </is>
       </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>Yeah, I would say something I need help with.
+I am moving to a new country and I would like help as in how I should confront my family about it.
+Right. I think what excites me most about this experience is discovering a new culture, you know, making a whole new bunch of friends as well. I think it's also a little bit scary given that I don't necessarily know so many people moving to this country. Country, you know, and it's going to be also pretty lonely. But I want them to know that it's not something that's necessarily. I think they think that I'm overwhelmed by the situation, but I'm actually really calm about it. And they also want me to get a job and I'm already moving, I'm applying to jobs there.
+I think the whole job market is a little bit scary for me, but essentially, yeah, I'm moving and then after that I'm trying to get a job there as well, you know, but I think they were a little bit scared and overwhelmed that maybe I'm too comfortable and then I'm not getting a job. You know,.
+I know, but like I'm, I, I think I'm appearing on the outside, I'm very calm and also on the inside. But sometimes after I have conversations with them, I'm very much like, I start doubting myself about, you know, because these are the people who care for me and who know my kind of my abilities to some extent and when I see them unsure about Me and my capacity to move. I start questioning double thinking, you know, and yeah, that's a bit scary because you kind of feel like, okay, maybe the people that you love and cherish the most don't actually see it happening for you or I don't know, I think it's pretty tough. I don't really know how to handle handling like move forward from the self doubt and the. And the question that starts to arise, you know,.
+Confident in my path? Yeah. Is there any, well, is there any approach I should have or any more arising topics that I should discuss about in order to make them feel calmer about the move?
+All right, I will do such thing. But then if I am doing that already, but then I'm not getting any job, how? Because also there has to be some sort of action behind, like behind the effort I'm putting in, you know, and if I'm not seeing that, how can I express it to them? Also, perhaps my own concerns about the job search.
+All right, thank you.    Transcribed by https://fireflies.ai/</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>449</v>
+      </c>
     </row>
     <row r="77" ht="409.6" customHeight="1">
       <c r="A77" s="1" t="inlineStr">
@@ -2253,6 +3499,20 @@
 05:00 That was actually a very good answer. I really enjoyed talking to you. She gave really good answers. So thank you very much.</t>
         </is>
       </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>Hello, Eduardo. Nice to meet you. My name is Maxi, and today I'd like to share some experience with you, if that's okay for you.
+So, basically a situation I was thinking about was this past weekend. So I was in Cologne, where I live and my hometown, and I have a girlfriend here in man street, and I was partying with some of my friends, and I thought, okay, I'm gonna have fun with my friends tonight and not, like, have any problems with my girlfriend. So I just turned off my phone and her reaction was not very good. And I really understand that, you know, you take care of the other person and you want to know how the other person is and if the other person turns off the phone, that's not quite nice. But, yeah, she didn't really understand me at all, that I was just trying to have a nice evening, you understand?
+To be honest, I think there's just one solution. I do not turn off my phone. Maybe I just tell her in advance, okay, I want to have fun with my friends. I'm not going to use my phone very much and then just put it in the pocket. But at least do not turn it off. So if she wants to call me or if anything happens. How do you say it? Like, she can reach. To me,.
+Yes. I also think that in general, it's very new to me to have her as a girlfriend. So I think I have to get. Yeah, get used to the situation at all. And some things are just new for me.
+As now as we're talking, I have another question. What do you think about spending time together? Because, you know, there are boyfriends and girlfriends, like, couples that just, like, spend, like, everything, like, do everything together and spend the whole night together and for days and days and. And that's actually the kind of relationship I do not want to have because we should both have time with our friends still. And, you know, what's really important for me is to looking forward to seeing the person, you know, getting excited. And I think if you spend so much time together, then you don't have this excitement at all after a certain time anymore. But what do you think about that?
+But what if one person, like, has so much more social interaction at all, and the other person has a little less? How do you get along with the situation?
+That was actually a very good answer. I really enjoyed talking to you. She gave really good answers. So thank you very much.</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>454</v>
+      </c>
     </row>
     <row r="78" ht="255" customHeight="1">
       <c r="A78" s="1" t="inlineStr">
@@ -2270,6 +3530,17 @@
 01:43 And he just wouldn't want to help me in the helping up the bike, picking up the bike, which was hard because I was about to cry, but he was just being rude to me.
 02:20 Yes, exactly. I needed a bit of kindness. I mean, now it's okay because whatever, he can do what he wants, but it's not unfair to treat me like that, especially when I'm a new person in this city, because I've never lived here and it's not my country, so of course I do mistakes, but acting that way is just very rude. And I hope that never happens to me again. Now I'm kind of scared to ask people for help, but I guess it doesn't matter at all. The situation, it was just weird.</t>
         </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>I'd like to talk about a recent challenge that happened to me and yeah, that kind of influenced me.
+Well, I parked my bike where I was not allowed to bike, like to park my bike, but I didn't know it. And then another one parked my bike next to me and that bike was about to fall and I didn't know how to pick it up because otherwise both bikes would have fallen. And then I asked an old man for help. He was very rude because at first he didn't want to help me, and then he spoke in Dutch with me and I don't even speak Dutch. And then he tried. Then he spoke in English to me and didn't want to help me. And at the end he said, yeah, you are smart enough to study at university, but too stupid to do this.
+And he just wouldn't want to help me in the helping up the bike, picking up the bike, which was hard because I was about to cry, but he was just being rude to me.
+Yes, exactly. I needed a bit of kindness. I mean, now it's okay because whatever, he can do what he wants, but it's not unfair to treat me like that, especially when I'm a new person in this city, because I've never lived here and it's not my country, so of course I do mistakes, but acting that way is just very rude. And I hope that never happens to me again. Now I'm kind of scared to ask people for help, but I guess it doesn't matter at all. The situation, it was just weird.</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>279</v>
       </c>
     </row>
     <row r="79" ht="404" customHeight="1">
@@ -2293,6 +3564,21 @@
 04:23 Thank you for your understanding. How would you have handled the situation?</t>
         </is>
       </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>Hello Eduardo. I would like to speak about the recent challenging social experience I've made.
+I've been in a group project with some of my colleagues and there was a technical difficulty which shut down my email account so I basically could not communicate with them and I wasn't aware of that. So they basically thought I was ignoring them for weeks and weeks. And that came to then a weird argument where both of us didn't even know what was happening. We should have just communicated about it, but basically we tried to resolve it and I tried to explain to them that it wasn't my fault and that my email account was just shut it down. Yeah,.
+Basically, they were a bit. They didn't believe me at first, hundred percent. They thought I was maybe lazy and just didn't want to admit that I didn't want to do the work. But in the end I showed them proof and showed them my email account and then they were really understanding we could divide our work in a new way so we both, all of us could put in the same effort. And in the end it worked out quite well.
+I think so as well. I think that's also how you should handle things. But how can I make them. How can I make things better next time so they will forget about it?
+How much would you say I'm at fault?
+Alright, so you would say there's nothing I could have done better.
+Don't you think I could have realized it earlier?
+Thank you for your understanding. How would you have handled the situation?</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>277</v>
+      </c>
     </row>
     <row r="80" ht="409.6" customHeight="1">
       <c r="A80" s="1" t="inlineStr">
@@ -2313,6 +3599,20 @@
 04:10 Okay, thank you very much. I will try to do my best for this situation and. But how should I face the situation if they don't understand me? If they don't understand my point and they are not, we are not on the same line, how should I face it? What should I do.
 05:01 Okay, thank you very much. We will talk later.</t>
         </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>Hello, Eduardo. I would like to talk about a conflict that I had at school with my teammates in a project.
+The main issue I'm facing is that my teammate didn't want to collaborate as much in the work as I did. So I felt I was left behind because I did a lot of hard work and they didn't do nothing. And they got good grades and everything. And I got good grades, but it's not what the work that it reflects.
+Yes, I think I need to have a talk with them because they are not taking this too seriously. And if they really don't listen to me, maybe I need to take something in consideration and go talk with maybe my tutor or my professor and see if I can change groups of anything. But I like them as person. They are really good persons, but they are not good working with me.
+Yeah, I know I'm on the right track, but I'm so nervous. I don't know what to do because I don't want to get them mad neither, because they are my friends. I spend time with them outside of the class and outside of school. Stuff like we go take some drinks together, we go play soccer together and everything. But I just feel like they don't respect me as much.
+Yeah, I think you're right. I should do it like that. I should not tell them like, too hardly what they need, like what I would like them to do or what is better for them. But I think I should just introduce it with them. Really, really low. Let's say, like, not too hard for them. But I don't know. It's kind of a really hard situation for me. For me. I don't know if I'm capable of it.
+Okay, thank you very much. I will try to do my best for this situation and. But how should I face the situation if they don't understand me? If they don't understand my point and they are not, we are not on the same line, how should I face it? What should I do.
+Okay, thank you very much. We will talk later.</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>370</v>
       </c>
     </row>
     <row r="81" ht="404" customHeight="1">
@@ -2340,6 +3640,26 @@
 04:42 Sure.
 05:08 Sure.</t>
         </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>Do I talk? Okay. In my mind today I want to find a job.
+I'm looking for a job like an office job where I can work remotely but most importantly more like hybrid. Not necessarily 100% remotely, but that I'm working with people. Maybe helping them achieve their goals. Things such as organizational development or change management. People management consulting, related to people hr, but strategic, not necessarily operational. Yeah,.
+Yeah.
+I think I have had some experience because I was part of an organization that was going through a merger. Not the vote, more like an acquisition. And there was some sort of change management happening there, but not necessarily where I was like let's say leading the role of a change manager or learning and development or training or coaching. No, it was more like I was in the background of everything. So sort of.
+I feel like I'm ready as long as the irrigation also gives me some guidance.
+Yes,.
+Any specific job openings in that area.
+I think.
+I think more fast paced because I feel like I'm always like changing and growing. But I think even if it's fast paced, I think it's important to have support in that.
+Yeah, I think that. But also motorsport like Formula One.
+No, I said Formula One.
+Sure.
+Sure.</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>222</v>
       </c>
     </row>
     <row r="82" ht="409.6" customHeight="1">
@@ -2374,6 +3694,32 @@
 06:31 Do you have the recipe for that?</t>
         </is>
       </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>I'd like to talk about uni.
+What do you do for a living?
+Tell me a joke.
+Tell me a joke.
+That wasn't that funny.
+How was your morning?
+I was pretty tired, but now I'm alright.
+No, but do you have any advice?
+What should I be doing if I don't hear my clock in the morning?
+What city is this behind you?
+You don't really understand me, do you?
+I recently had an argument with my roommate. What advice would you give me?
+Okay, but what if my roommate always leaves her dishes in the kitchen behind and leaves the kitchen dirty and it really annoys me and I Told her many times. What advice would you give me?
+But I was asking you about my roommate that she always leaves the place behind. Dirty. What is your advice I should do about it?
+But we already have a cleaning schedule. But she just doesn't do it.
+Okay. And what would the reward look like?
+But what if I don't like her?
+Okay. Do you have any idea what I should be cooking tonight?
+Do you have the recipe for that?</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>193</v>
+      </c>
     </row>
     <row r="83" ht="409.6" customHeight="1">
       <c r="A83" s="1" t="inlineStr">
@@ -2404,6 +3750,29 @@
 06:58 I think so. Hello. So.    Transcribed by https://fireflies.ai/</t>
         </is>
       </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>What do you want to chat about?
+Yeah. For example, yesterday I was on a party. It was really good with some friends. Yeah, that had been going on recently. And also the day before. I liked the finance class. I think it's quite interesting.
+I don't know. At the party I like the most to just chill out with friends. Enjoying the music. Yeah, like this.
+Not sure. Next week there's free time at the university. And also a friend of mine had a birthday party on Wednesday for probably. Yeah,.
+No, like I say, to party. And also I need to study as well. Some more stuff for the exam soon, so need to learn.
+Yeah.
+No, just like the typical topics. Like the typical things? Yes, that's it. Like university stuff. But I have high expectations to myself, so I want to get a really good grade, hopefully.
+Yeah, I think so. Hopefully.
+Okay, what tips can you give me?
+How long should I do the break?
+Okay, and how long should I learn in one day before the exam sessions? Like,.
+Okay, makes sense. So you think eight hours is a good average?
+True. So what can you tell me about social experience?
+Makes sense. So what kind of tips can you give me to improve my socializing? My networking?
+Okay, I think that makes sense.
+I think so. Hello. So.    Transcribed by https://fireflies.ai/</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>240</v>
+      </c>
     </row>
     <row r="84" ht="409.6" customHeight="1">
       <c r="A84" s="1" t="inlineStr">
@@ -2428,6 +3797,23 @@
 05:35 There's.</t>
         </is>
       </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>Yeah, I'm just waiting if it's gonna work like that. Is it working? It should start talking to you, so. Hello? Oh, yeah, I'm supposed to talk about a difficult conversation I had, and just this night there was, like, some inconvenience happening for me, and everyone was, like, trying to help me, and that was a bit awkward for me.
+Well, it looked like someone was, like, watching me through my window, and then all of my roommates were going crazy and, like, wanted to help me and, like, did so much that it was just a bit awkward because I didn't really, like, need to help. I mean, I appreciate their help, but it was just a bit awkward that they were, like, doing so much.
+I'm feeling pretty good. I mean, yeah, it's just, like, still a bit awkward. I guess.
+No, I guess it was just me because they were, like, nice and they. They did nothing wrong. It's just like, me, so.
+Yeah, I guess I'm just gonna tell them how it made me feel and maybe how they overreacted a bit.
+Do you have any advice for me?
+Okay, well, maybe we can talk. Do you have any advice for me how I can handle, like, I have to do, like, team presentations, and my team is, like, doing pretty bad. Like, they're not doing anything. Do you have, like, advice for me for that,.
+Yeah, well, I mean, they're not really doing anything. I mean, we have tasks assigned and they're just not like. I mean, they are doing their part at least, but they're doing it so poorly that I don't know what to tell them.
+Okay, well, I guess I leave now.
+There's.</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>292</v>
+      </c>
     </row>
     <row r="85" ht="372" customHeight="1">
       <c r="A85" s="1" t="inlineStr">
@@ -2450,6 +3836,22 @@
 04:00 Maybe that's. Yeah, that's actually a good idea. I will definitely talk to them about it. But what do If people are not willing to be part of the conversation?
 04:38 All right. Thank you very much.</t>
         </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>I don't really know. Maybe a challenging situation for me with friends and family.
+I mean, I live in a house with 12 other people here, and sometimes it gets really. It's really hard because everybody needs their personal space. But also, especially like in the kitchen, it's not always clean and some people like it cleaner and some, like it a little bit more. You know, I don't know how to say it.
+We don't really, to be honest, we just leave it like that. And I mean, it's mostly that somebody gives in. Yeah,.
+I mean, maybe, yeah, but I don't feel like all the people are willing to do that, you know, like, some don't really see any issues with that.
+Well, yeah, that might be true. I will definitely take that into. I'll think about it. Definitely. Yeah.
+I mean, there's not really much that I can. I can say now, to be honest,.
+So can you maybe give me a few. A few advice how I could handle that? The problem? Sure.
+Maybe that's. Yeah, that's actually a good idea. I will definitely talk to them about it. But what do If people are not willing to be part of the conversation?
+All right. Thank you very much.</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>213</v>
       </c>
     </row>
     <row r="86" ht="306" customHeight="1">
@@ -2476,6 +3878,24 @@
 03:28 Okay. Thanks.</t>
         </is>
       </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>I'm here for a bonus point.
+I have a problem with my roommate and she doesn't want to clean the dishes.
+Not really. Like when I'm talking to her, I. She's not like really listening to me and she doesn't want to clean like every dishes that she use.
+Yeah, sure. I'm done with that.
+Yeah, it sounds great.
+Yeah, sure. Let's do that.
+Yeah, it sounds good. But I think that I hope she will listen to me.
+Yeah, that's true.
+Yep.
+Yeah. Thank you. Bye.
+Okay. Thanks.</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>89</v>
+      </c>
     </row>
     <row r="87" ht="170" customHeight="1">
       <c r="A87" s="1" t="inlineStr">
@@ -2495,6 +3915,18 @@
 2:18 PM I said that I waited on purpose for the next day to see if anyone would do anything about it, and I know some of them were home with time to do it, and it was still disgusting. The reply I got was a jokingly Ï'll wake up early to do the dishes then!</t>
         </is>
       </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>thumb up thumb down show more actions Hey chat! I'd like to tell you about a recent challenging interaction I had yesterday.
+My roomates...
+Basically they keep leaving dirty dishes on the sink while the dishwasher is clean, instead of just taking the clean dishes out and putting the dirty ones in.
+I did, and they reply I got was "it's probably because you wake up really early and then you see the dishwasher clean, because we put it during the night working, and then leave the extra dishes on the sink for the next load
+I said that I waited on purpose for the next day to see if anyone would do anything about it, and I know some of them were home with time to do it, and it was still disgusting. The reply I got was a jokingly Ï'll wake up early to do the dishes then!</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>150</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="1" t="n"/>
@@ -2502,6 +3934,7 @@
         <v>13333</v>
       </c>
       <c r="C88" s="2" t="n"/>
+      <c r="D88" s="2" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="1" t="n"/>
@@ -2509,6 +3942,7 @@
         <v>15088</v>
       </c>
       <c r="C89" s="2" t="n"/>
+      <c r="D89" s="2" t="n"/>
     </row>
     <row r="90" ht="409.6" customHeight="1">
       <c r="A90" s="1" t="inlineStr">
@@ -2533,6 +3967,23 @@
 04:26 No, it's fine. I think I talked about the most stuff I wanted to.</t>
         </is>
       </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>Anything you want.
+Basically my hobbies have been the same my whole life. I've been playing tennis, just a lot of sports, basically. Also gym, go for runs, stuff like that. Basically that. How about you?
+Yeah, very nice. Basically, I came here to talk to you about a conflict situation. Like with a conflict situation with other people.
+No, like the task I came here for was just to talk about a conflict situation where I had to navigate. And that was when we had to book a table for a dinner reservation because my mom forgot that I had another appointment at that time. So I had to relocate and had to inform her and also the others, so they knew. And that was quite hard to navigate all of that.
+Yeah, of course. We just scheduled it to later point so that we still had the dinner reservation, but I could have my appointment as well. And so we just ate at a later time. Yeah, that's basically.
+Yeah, that's true. Did you have any like these in the last time?
+Yeah, that's true. That's true.
+No, not really. I mean, it's not that it wasn't that of a hard situation was basically. Okay, so it was not too hard to navigate, but yeah,.
+Yeah, that's true.
+No, it's fine. I think I talked about the most stuff I wanted to.</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>234</v>
+      </c>
     </row>
     <row r="91" ht="404" customHeight="1">
       <c r="A91" s="1" t="inlineStr">
@@ -2557,6 +4008,23 @@
 05:22 Yeah, Should I stop the yeah, you can stop.     Transcribed by https://fireflies.ai/</t>
         </is>
       </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>Nothing. I was just thinking about school and jokes. Funny jokes. What can you do? No. Maybe to hear one and maybe to see what you can do. Pretty interesting.
+Good. Good one. Maybe some more humoristic ones.
+Okay, what interesting stuff can you do other than jokes?
+Well, you can describe what you see around me. And what's your impression?
+Yeah. Can you tell me where you are? Like, is it a high rise building in a specific city or just in virtual reality?
+Looks cool. Looks cool. Okay, We'll dive into how much knowledge you have behind you. Like what's your database? How does it look like?
+Okay. Your responses maybe are too big, generic, sound like AI. Like yeah. Can you tell me more about that? And also like, how do you differ from other VR AI models?
+And how would you know how I am feeling?
+Okay, fair enough. And what do you think about the body language, about the conversation flow? What would you recommend to improve it and how do you see it? What can you see of this as a model?
+Yeah, Should I stop the yeah, you can stop.     Transcribed by https://fireflies.ai/</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>202</v>
+      </c>
     </row>
     <row r="92" ht="404" customHeight="1">
       <c r="A92" s="1" t="inlineStr">
@@ -2581,6 +4049,23 @@
 04:53 All right. Cheers. See you next time.</t>
         </is>
       </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>Hi, how are you? I'm Nicholas. I'm here to talk about a recent challenging experience I had.
+I've been going through some challenges with a roommate of mine regarding cleaning the kitchen and other sharing areas.
+Well, the main issue is that when he uses it, he doesn't clean afterwards. So he doesn't clean his pants. And the whole kitchen looks very messy after or is very messy and dirty after he used it. And he refuses to clean them after cooking. But I've told him that and still no reaction.
+Well, we don't have a cleaning schedule, but I suggested that we just go by the basis that everyone cleans what he used. But we never really sat down. I just said to him on the fly, more or less that he has to clean up his stuff.
+Yeah, you're right. Do you have any suggestions how I could get him to listen and understand?
+Right? That sounds convenient to me. How's your day going so far?
+Been great so far. I'm just a bit studying today, tomorrow as well. And on Wednesday I'm going home to see my parents again, so. Could have been worse, I guess.
+No, nothing specific yet, but just some relaxing time. You know,.
+Yeah, you're right. But what do you work exactly that you have this nice office.
+All right. Cheers. See you next time.</t>
+        </is>
+      </c>
+      <c r="E92" t="n">
+        <v>232</v>
+      </c>
     </row>
     <row r="93" ht="409.6" customHeight="1">
       <c r="A93" s="1" t="inlineStr">
@@ -2604,6 +4089,22 @@
 06:59 Yeah, yeah. It's very true. Very true. It's just a bit tough, you know? And the stress is the worst, man. It's the worst. And it's what hits the most.</t>
         </is>
       </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>Hi, Eduardo. I'm feeling sometimes, I guess struggling. I have a chronic condition. I have Crohn's disease. And hanging out with friends or going to uni and kind of having that. It's a bit of a struggle sometimes, you know.
+I guess in the way maybe not. Some guidance. Maybe some ways that I can kind of help balance it out. I also have work as well sometimes. And I have to do work and sometimes it can get. It gets really tough and there are times when I feel really unwell, but there's no one to kind of fill in for me. And I have this pressure in my head that, oh, I need to go, even though I really feel bad about it. And the same goes to uni classes.
+I get that. I get the only problem is my class is tutorless at the moment. And with work, I'm on a zero hour contract. Right. So it's not necessarily something that I can really choose when and where to go. And also social. I'm very much more introverted now and I spend more time at home.
+Yeah, that's what I tried to do. It's what I tried to do at home. Spend time with my girlfriend. We chill out a lot, we rest a bit. And also try and be active. Right. Try and go to the gym recently, so that's definitely helping. I went for a couple blood tests recently as well that were. They went okay. A few. Few test scores weren't the best, but my doctor didn't call and they said that they would only call me if there was bad news. So I guess there's good news in that. But yeah, I still feel quite fatigued, you know. And every two weeks I have injections for my parents for the biology that I put into the mass of every two weeks. And on that day and the day after, I'm extremely dead.
+Thank you, thank you. And facts. Yeah, it's good that the doctor didn't call, but yeah, I guess as well. What's good news is that my boss likes me so he's quite open to me to have the day off and he understands that's good. Only problem is I've got classes at 8:30 in the morning and that is an absolute pain. Like it is. It is in the morning. It's where I feel absolutely. Because I wake up, stomach's bloated and before I go out I need to go to the bathroom because I can only go to the bathroom in the house, you know what I mean? And yeah, so it's a bit of an issue as well. And yeah, it's just a lot of stress recently as well and stress.
+The worst thing for me, I've got two courses left and then I've got my bachelor of them. But these are the two of the toughest courses. So it's a bit of a struggle.
+Yeah, fair. But then again, I can't just be leeching for support. Right. Murder person. They're going through two masters right now. They're going through a premium program, they're going through other internships. They need support as well. And how to kind of balance all of that.
+Yeah, yeah, that makes sense. That makes sense. Yeah. I think it's just sometimes it gets a bit tougher to do such things. Right. You can't always have that time, and sometimes you just. Yeah. You don't have the ability to be there for that interaction.
+Yeah, yeah. It's very true. Very true. It's just a bit tough, you know? And the stress is the worst, man. It's the worst. And it's what hits the most.</t>
+        </is>
+      </c>
+      <c r="E93" t="n">
+        <v>620</v>
+      </c>
     </row>
     <row r="94" ht="409.6" customHeight="1">
       <c r="A94" s="1" t="inlineStr">
@@ -2624,6 +4125,20 @@
 04:05 That's a good idea, but. So what am I gonna do now?
 04:45 Yes. That sounds nice. So, yeah, thank you.</t>
         </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>Enjoy it. Thank you. Hi, I would like to chat about a recently difficult situation.
+So it's about me having a friend who I'm doing a group project with and it's just hard to communicate with her, especially because I don't know how to tell her that she has to contribute her part and not rely on me too much.
+That sounds good. I tried to tell her or every time she asks me how are we gonna do this? And she's discussing her point with me, I'm trying to guide her in the right direction but it's quite difficult to tell her or like to actually bring across that I don't feel like she's doing enough. Especially because it's a new relationship, a new friendship. Still,.
+Yes, I tried to guide her in another direction but it was just a bit one sided, especially because were talking about it and she was really asking me a lot about how I would do this or that. And I tried to tell her that's her responsibility or that's her part to participate in, but she kind of kept asking me about stuff and I tried to tell her do it however you want, but in the end I did the most, the biggest part and then everything she did, she double checked with me, which I like that we have a good communication and that we're working together closely and that she's my friend but it was kind of tough spots.
+Yes, but I don't like that it has influence on our friendship and I don't actually know what specifically to do because she's just doing her part. I'm just doing my part. But in the end, it kind of felt off. And I feel like you can feel that in the relationship. Friendship.
+That's a good idea, but. So what am I gonna do now?
+Yes. That sounds nice. So, yeah, thank you.</t>
+        </is>
+      </c>
+      <c r="E94" t="n">
+        <v>323</v>
       </c>
     </row>
     <row r="95" ht="409.6" customHeight="1">
@@ -2648,6 +4163,22 @@
 04:54 Yeah, we had a nice time still, so I think next time will be even greater.</t>
         </is>
       </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>Hello. I've actually recently encountered something with a friend that I kind of have some troubles with of how to. Like, it's a bad experience.
+Yes, of course. So were actually at a festival, and were, like, deciding on what time we wanted to leave because I really wanted to see an artist, and, like, she didn't really want to. She was really tired, so she wanted to go home. But I was staying over at hers, so I kind of had to comply. But I also kind of got into an argument with her about, like, really wanting to see that artist, and I spent money to go see it, so I wanted to see it.
+Yeah. All right. So maybe, like, talk about her feelings and try to understand her point of view.
+Okay, but I still want to let her know that I really. It kind of hurt me that I couldn't see the artist, so how could I also tell her that, but, like, politely?
+Yeah. So. All right, so maybe, like, next time, if we have this situation again, maybe make sure that beforehand we already have some rules clear, like, okay, until what time we're going to stay and stuff. Is that maybe a good idea?
+All right, I like that idea. I guess maybe next time we would also have to, like, select the persons we like, artists we really want to see and stuff. And maybe also talk about the fact that, for example, the tickets this time cost €50. So that's, like, kind of relatively expensive for a festival. So were, like, maybe beforehand. Look at it.
+Yeah, okay. I think that's a great idea. I guess next time we, like, have to make a better plan beforehand, and then if it diverges from that, it's fine, but. Yeah,.
+Yeah, I think we'll have a great experience next time because I think I have a great plan now, and I will apologize to her.
+Yeah, we had a nice time still, so I think next time will be even greater.</t>
+        </is>
+      </c>
+      <c r="E95" t="n">
+        <v>349</v>
+      </c>
     </row>
     <row r="96" ht="289" customHeight="1">
       <c r="A96" s="1" t="inlineStr">
@@ -2671,6 +4202,22 @@
 04:03 Yes,.</t>
         </is>
       </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>I would like to talk about a challenging experience. A recent challenging experience, of course, User,.
+My grandparents are here right now to visit me and they want to keep seeing me. But I still have to do a lot of stuff for my university to keep up with my studies and I don't know how to tell them that I have to study.
+Yes, that would be nice.
+Yes. And how do I start the conversation?
+Yes, that sounds good.
+Yes,.
+That's a good idea. Do you have any ideas what I can show them in Maastricht?
+Thank you.
+Yes,.</t>
+        </is>
+      </c>
+      <c r="E96" t="n">
+        <v>101</v>
+      </c>
     </row>
     <row r="97" ht="409.6" customHeight="1">
       <c r="A97" s="1" t="inlineStr">
@@ -2693,6 +4240,22 @@
 04:52 All right, thank you very much. And how are you in general?
 05:06 I think I got a bit more of a clear direction, so thanks for that.</t>
         </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>Something challenging have been going on.
+So I met a friend two days ago, and I haven't really spent a lot of time with her, and she's been very distant, and it's been very difficult for me to comprehend because I didn't have a lot of time to talk to her. So I don't know what to do.
+Every time I ask her, she says everything is fine. But then also I wanted to. For example, I told her I can be there and we can meet up next week. But then she was like, yeah, I've got exams, so that's gonna be difficult. But then I'm gonna be in my hometown with her for five days, so I feel like, you know, it would. If she would like to put in the effort, I could be there.
+So how do I do that? I've already asked her if we can meet up, but she already said she can't. So I'm not sure what I should do.
+I don't really think she's that type of person. Who would like to hear that? Maybe. I don't know, maybe I should just, like, talk more with her in general and just, you know, maybe call her. I don't know. Like, I feel like she's been very distant. It could potentially be that there's something up but like I said, I already asked her, so I guess I'm just gonna wait what she replies on if we can meet one of the days. And yeah,.
+Yeah, I feel like also on that matter it's kind of difficult to coordinate like being in mastrich and studying a lot to also catching up with people at home because I not that type of person who's a lot on their phone. So I feel like it's kind of difficult to comprehend like or to work with both of them at the same time.
+Can you repeat that please?
+All right, thank you very much. And how are you in general?
+I think I got a bit more of a clear direction, so thanks for that.</t>
+        </is>
+      </c>
+      <c r="E97" t="n">
+        <v>349</v>
       </c>
     </row>
     <row r="98" ht="409.6" customHeight="1">
@@ -2722,6 +4285,27 @@
 07:00 I wasn't going to meet the artist itself. I was just saying that I was looking forward to seeing the artist as he was performing. Hello. So I need to.     Transcribed by https://fireflies.ai/</t>
         </is>
       </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>I had a disagreement with my mother. It was about me going to a concert, and she didn't want to pay for it. What happened was I really wanted to go to that concert, and that artist is only going tour for one or two times before he changes his name. So I asked her pretty nicely to maybe if she wants to go with me to the concert, and with a little bit of nudging, I got her to go with me and we're going.
+Yes, I'm really excited. We're going to meet him, so. Yeah. Yeah.
+I mean, I'll probably fangirl a lot over him, but I just want to take a picture with him and. Yeah, just only, like, interact a little bit. And I'm very excited for his music.
+Yes, I agree. Thank you.
+Not really. I think.
+Another thing, I am trying to go to a therapist, and my mom's pursuing me to go, but I feel like I don't want to do it because I don't want to speak to other people, to another person about my problems. So that's a bit of a tough situation.
+I haven't, actually. I mean, I want a therapist who's very friendly and open, and I can easily talk to her. So that's what I'm, like, searching for right now. My friend recommended somebody, so hoping that she's good.
+Yeah. So I will probably write therapist an email today to. To see if she has maybe, like, any spots for me to go.
+Yeah. Thank you so much.
+Do I need to reflect on this?
+Overall, it was pretty great. He was nice and gave thoughtful advice.
+No. I think what I answered was pretty correct and straight, so I think he did great.
+No, I don't think so. Or maybe just like when he asked about meeting the artist itself. I think I didn't mention that I wanted to meet the artist. I just said that I'm really excited to see him.
+I wasn't going to meet the artist itself. I was just saying that I was looking forward to seeing the artist as he was performing. Hello. So I need to.     Transcribed by https://fireflies.ai/</t>
+        </is>
+      </c>
+      <c r="E98" t="n">
+        <v>370</v>
+      </c>
     </row>
     <row r="99" ht="221" customHeight="1">
       <c r="A99" s="1" t="inlineStr">
@@ -2741,6 +4325,19 @@
 10:07 AM he seemed understanding but also said that i still need some time so that players who werent injured also get the chance to play and show that they can also play a significant role in the team
 10:08 AM objectively, i think so yes. subjectively, no. of course i want to play and that applies for everyone. we are one team but still there is sort of a competition when playing in a game from the start on</t>
         </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>hello how are you doing
+i also fine, thank you. i would like to tell you something about a recent challenging interaction i had
+so it was like a little discussionwith my football trainer. i recovered from a injury and wanted to play again, but he told me that i need some time which really disappointed me
+yes. fter the training i went to him and tried to explain my point of view to him, that i was more than ready to play again and give my best for the team
+he seemed understanding but also said that i still need some time so that players who werent injured also get the chance to play and show that they can also play a significant role in the team
+objectively, i think so yes. subjectively, no. of course i want to play and that applies for everyone. we are one team but still there is sort of a competition when playing in a game from the start on</t>
+        </is>
+      </c>
+      <c r="E99" t="n">
+        <v>167</v>
       </c>
     </row>
     <row r="100" ht="204" customHeight="1">
@@ -2764,6 +4361,21 @@
 9:39 AM nothing, all good. my brother has middle school exams tho</t>
         </is>
       </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>oke nice to meet you, well im currently studying at maastricht.
+Im studying something economics related, it doesn't really interest me though
+I feel like the study is solely theory, which is not ideal. I like to learn by doing and seeing.
+I agree im currently looking for internships, however i have failed my last course. Which made my parent a bit disappointed in me
+Well i told them i failed, however i didn't even participate. You could say i lied to them
+I didn't want them to stress about my school and my motivation
+bro what divorce? they are not separated...
+nothing, all good. my brother has middle school exams tho</t>
+        </is>
+      </c>
+      <c r="E100" t="n">
+        <v>112</v>
+      </c>
     </row>
     <row r="101" ht="221" customHeight="1">
       <c r="A101" s="1" t="inlineStr">
@@ -2785,6 +4397,21 @@
 9:34 AM Nothing really. Im saying because it happend recently and I experienced how bad it feels it wont happen again soon (short-term). But I dont know if it will be a lasting effect
 9:34 AM acting like my therapeut, dont know fam</t>
         </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>I'd like to talk about a recent challenge i had
+I missed a deadline for an apllication
+procastination and I had the dealine a couple days to late in my notes
+yes also wrote an e-mail. They accepted it still, but the aplliacation is not good at all now. Because I did it in 2 hours and had a whole month for it
+yess
+I hope so. Definetly on the short term
+Nothing really. Im saying because it happend recently and I experienced how bad it feels it wont happen again soon (short-term). But I dont know if it will be a lasting effect
+acting like my therapeut, dont know fam</t>
+        </is>
+      </c>
+      <c r="E101" t="n">
+        <v>113</v>
       </c>
     </row>
     <row r="102" ht="255" customHeight="1">
@@ -2809,6 +4436,22 @@
 10:25 AM I am not sure about this</t>
         </is>
       </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>no, I had troubling experience earlier this week
+I was talking to my boss, because I was not happy with my salary and I wanted to give him a choice of either raising my salary or I would quit
+I think I got my points across very well but based on hos reaction he was not very happy and no I am worried this will have consequences
+I will follow through if he doesnt increase my pay
+I am not prepared but i am fairly certain I wouldnt be jobless for too long
+I am amazing
+That I am in the bargaining position not my boss
+i think so but my biggest worry is that he will make the last few weeks in case I do quit pretty hard
+I am not sure about this</t>
+        </is>
+      </c>
+      <c r="E102" t="n">
+        <v>135</v>
+      </c>
     </row>
     <row r="103" ht="255" customHeight="1">
       <c r="A103" s="1" t="inlineStr">
@@ -2832,6 +4475,22 @@
 11:00 AM Also a good one</t>
         </is>
       </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>Yes well I have a little dilemma.
+My housemate is really getting on my nerves. He is constantly slamming doors and goes in and out of his room what seems like a hundred times a day. The walls are thin so I can always hear this and because my room is next to his, my entire room shakes when he enters/exits his room.
+No I haven't said anything. I feel like I should have said something in the beginning of the year because now it seems too late.
+Yes you're right. Should I text him about it or speak to him personally?
+Ok. What should I say?
+Thanks. Ahh I find confrontation so tricky! I don't like complaining and don't want to make the situation worse.
+What could the solution be?
+Good idea.
+Also a good one</t>
+        </is>
+      </c>
+      <c r="E103" t="n">
+        <v>138</v>
+      </c>
     </row>
     <row r="104" ht="170" customHeight="1">
       <c r="A104" s="1" t="inlineStr">
@@ -2850,6 +4509,18 @@
 11:10 AM yes, and i actually told him id rather be friends since i really enjoy spending time with him, he said he understood but i think we never settled limits and the frienship was difficult to achieve
 11:11 AM yes, i always knew he liked me so maybe should have never let the friendship develop into something romantic</t>
         </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>Id like to tell you about a difficult situation i had
+indeed, i have a friend that doesnt want to talk to me anymore, i met him in one of my tutorials \
+yes, i think so. We started kind of getting into a relationship but i was never decisive on what i wanted
+yes, and i actually told him id rather be friends since i really enjoy spending time with him, he said he understood but i think we never settled limits and the frienship was difficult to achieve
+yes, i always knew he liked me so maybe should have never let the friendship develop into something romantic</t>
+        </is>
+      </c>
+      <c r="E104" t="n">
+        <v>108</v>
       </c>
     </row>
     <row r="105" ht="255" customHeight="1">
@@ -2871,6 +4542,20 @@
 12:01 PM we basically all know what we have to do. but i feel like im nott prepared enough. or at least not at the level i would normally like to
 12:02 PM that i didnt read the chapters we had to read until today. i just know the task and the asnwes from chat gpt but not the logic behind it</t>
         </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>Hi i would like to tell you about a challenging siutation i had with my tutorial group in university
+yeah we have a group assignement since the start of the period so we already got the assignemtn 4 weks ago
+yeah its some time but i personallz had a lot of other stuff to do.
+the problem is that i wasnt in maastricht every weekenf since the start of the period so i couldnt contribute yet. and now we have a midterm updagte presentation today
+there is one guy who does everything wiht AI so he also doesnt do a lot and his work is pretty bad. then there is one girls she organises everything she is good. and one girl that just does the job suffiecientlt
+we basically all know what we have to do. but i feel like im nott prepared enough. or at least not at the level i would normally like to
+that i didnt read the chapters we had to read until today. i just know the task and the asnwes from chat gpt but not the logic behind it</t>
+        </is>
+      </c>
+      <c r="E105" t="n">
+        <v>185</v>
       </c>
     </row>
     <row r="106" ht="306" customHeight="1">
@@ -2900,6 +4585,27 @@
 11:30 AM yeah,my living room or bedroom</t>
         </is>
       </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>i would like to tell you about a recent challenging interation i had
+personal life
+it was during the break
+no, i had to pass my driver's license, it was a horrible moment
+i had already failed it the first time so i was super stressed and the guide was very rude
+yes of course, i was shaking so much
+yes, i took a deep breath and did my best but i was still shaking
+yes i did!
+yes, do you have any advices on road?
+ok, any advice for managing stress?
+just chilling, eating a snak
+salty snacks
+yes
+yeah,my living room or bedroom</t>
+        </is>
+      </c>
+      <c r="E106" t="n">
+        <v>106</v>
+      </c>
     </row>
     <row r="107" ht="238" customHeight="1">
       <c r="A107" s="1" t="inlineStr">
@@ -2921,6 +4627,20 @@
 11:44 AM interesting idea what about friends?</t>
         </is>
       </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>hey, yes its just been quite stresssful the last few weeks
+oh its been a mix of covering uni stuff with family meetings in other cities and visiting my boyfriend
+yes it has been quite a busy schedule trying to cover everything at the same time. with my boyfriend everything has been going good
+yes, he is been supportive. its more about that im stressing a bit to cover everything at the same time without letting anyone behind. the issue is not about my boyfriend
+no nothing specific. i just feel like the day doesn"t have enough hours to cover everything, especially when i have to include all the travel time with delays
+on what would you put the focus?
+interesting idea what about friends?</t>
+        </is>
+      </c>
+      <c r="E107" t="n">
+        <v>126</v>
+      </c>
     </row>
     <row r="108" ht="306" customHeight="1">
       <c r="A108" s="1" t="inlineStr">
@@ -2940,6 +4660,19 @@
 12:05 PM I do feel that I don't know how close I want to keep that friendship. I mean we're adults, I can't deal with childish behaviour like that.
 12:06 PM Yes, she said she knows her actions are wrong and she is trying to deal with her behaviour but I dont see any progress from her.</t>
         </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>HI! My name is Vasilena! I would love to have a chat with you about a recent tough experience I had with a friend/
+Okay, so here's the situation. I am in a group with 2 other girls and they both work on the weekends. But one of them had a free day and proposed going on a day trip in the Netherlands. Ive never been in another city here so I immediately accepted. However, my other friend got mad at me for taking the opportunity without her and didnt talk to me. I even proposed going to Rotterdam where she has been before in order to not make her feel bad for not coming. But she still didnt talk to me for several days. Do you think I did something bad?
+She just gave me the silent treatment and after 2-3 days acted like nothing had happened. I tried talking to her but she was ignoring me so I also stayed silent. Afterwards, she also got mad at me for being mad at her that she didnt even want to talk about the problem so we could resolve it.
+I guess, she has always said that she could get possessive of her close ones and jealous and I always try to deal with that in a gentle matter but its so exhausting sometimes...
+I do feel that I don't know how close I want to keep that friendship. I mean we're adults, I can't deal with childish behaviour like that.
+Yes, she said she knows her actions are wrong and she is trying to deal with her behaviour but I dont see any progress from her.</t>
+        </is>
+      </c>
+      <c r="E108" t="n">
+        <v>278</v>
       </c>
     </row>
     <row r="109" ht="306" customHeight="1">
@@ -2963,6 +4696,21 @@
 12:30 PM maybe I shoulf</t>
         </is>
       </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>Well, I have a teammember in my supply chain course and I feel like he does not take me seriously....
+Well, it is more that when I say something he kinda ignores it but when my male teammember says something he immidiatly listens or at least takes it into account, which is very frustrating, I feel like he does that because of my gender, being a female
+I have seen numerous moments, for instance, we decided upon a company that I brought up but then he insisted on his company, the third male coworker was silent during this. or when I had a slides deck already made in canva, he insisted on powerpoint until the third coworker said that he liked canva.
+No, but should I? I feel like it is not his problem and this feeling is not neceserally objectively confirmed
+wouldnt he get irritated tho, like would the atmosphere not get worse
+and what if it al plays out bad?
+but I am stuck with this group until the end of the semester
+maybe I shoulf</t>
+        </is>
+      </c>
+      <c r="E109" t="n">
+        <v>178</v>
+      </c>
     </row>
     <row r="110" ht="136" customHeight="1">
       <c r="A110" s="1" t="inlineStr">
@@ -2980,6 +4728,17 @@
 12:13 PM Yeah I am relisting it right away. no Interest in keeping the article. As I mentioned the inconvenience has little negative impact on me
 12:14 PM yeah its not used by me. Could get money out of it. So I figure why not sell it right away.</t>
         </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>I would like to tell you about a recent challenging interaction I had. I was selling something on Vinted and the customer cancelled their order leaving me with an unsold product
+It was quite unexpected with weak reasoning. the problem itself is fairly little. Pretty much a non problem if you will. still it is annoying as now I have to revisit the selling process which is a bit annoying
+Yeah I am relisting it right away. no Interest in keeping the article. As I mentioned the inconvenience has little negative impact on me
+yeah its not used by me. Could get money out of it. So I figure why not sell it right away.</t>
+        </is>
+      </c>
+      <c r="E110" t="n">
+        <v>115</v>
       </c>
     </row>
     <row r="111" ht="255" customHeight="1">
@@ -3002,6 +4761,21 @@
 12:48 PM no i think its not that bad but just something i have notiuced in the past that might help
 12:48 PM not yet but im working on it</t>
         </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>yes im doing okey
+yes everything is going good im a little behind with my studies but ill try to finish it asap
+no just in general with the work load
+yes to spend more tome and also be more efficient when im at the libary
+dont please people just because it feels better going ith them and also make my own plan and knowing what times im best at beeing productive
+i think in general keepung up with the workload helps to hve more time and prioitize my scedual. and also be able to have time to meet up with my group
+no i think its not that bad but just something i have notiuced in the past that might help
+not yet but im working on it</t>
+        </is>
+      </c>
+      <c r="E111" t="n">
+        <v>129</v>
       </c>
     </row>
     <row r="112" ht="255" customHeight="1">
@@ -3025,6 +4799,22 @@
 3:06 PM okay
 3:06 PM thank zou</t>
         </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>hi, zes so i had a recent challanging interaction i would love to talk about
+so it's about a disagreement with one of my tutors, they hd the opinion, that our presentation wasn't what was asked for and i disagree, especially since i had a conversation with her prior to the presentation about the requirements, but in her feedback she ignored that \
+i addressed it, but she seemed to have changed her opinion and now mz grade refelcts her indesicion and i feel weird bringing it up again, especially since we had a good tutorial group and we are discouraged to talk with our tutors about our grade after submission and now i don't see her anymore\
+yes so what now
+i don't know if i feel comfortable with that
+yes and furthermore, i don't know if it would help or rather make me look stupid
+so what should i do?
+okay
+thank zou</t>
+        </is>
+      </c>
+      <c r="E112" t="n">
+        <v>154</v>
       </c>
     </row>
     <row r="113" ht="356" customHeight="1">
@@ -3052,6 +4842,25 @@
 3:37 PM just more on how is my writing style and if my content is answering the research question</t>
         </is>
       </c>
+      <c r="D113" s="2" t="inlineStr">
+        <is>
+          <t>yeah everything is great!
+today has been a productive work day
+yeah i had some feedback from my thesis supervisor which i was procastinating a lot with and i finally got to it today
+yes yes i did
+it was but i still needed to figure out a lot on my own
+some of the feedback was really helpful but some needed me to go back and do a lot more research which was quite time-consuming and stressful, and the thesis submission is coming close so i maybe hoped he gave this feedback early on
+yes i did but he said that these are challenges that comes for every masters student and time-management is a key skill here which i need to work on
+yes i spoke to him and we made a revised schedule which i need to closely follow from now on
+yes, i am
+I will work on writing everyday for a few hours and a few hours only for research and keep updating my supervisor with my work
+i plan to have a chat with him every week
+just more on how is my writing style and if my content is answering the research question</t>
+        </is>
+      </c>
+      <c r="E113" t="n">
+        <v>201</v>
+      </c>
     </row>
     <row r="114" ht="238" customHeight="1">
       <c r="A114" s="1" t="inlineStr">
@@ -3070,6 +4879,18 @@
 3:50 PM i think its just her achievments but im happy with my grades because im alswyas doing my best and really stress about grades to a point where it gets unhelathy so i have to stop comparing myself to her nad start being myself again. do you have any tips how i get my spark back?
 3:51 PM yes tahnk you so much for your help</t>
         </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t>hi, i wpuld like to tell you about a recent challenging interaction i had
+i started my studies here last september and got close with a really nice girl. we had great time for five months but then she moved to another street and meet a new girl that she got really close. i felt like the third wheel in every conversation and she even called the other girl her best friend in front of me which reall hurt my feelings. now im moving to her street as well and i hope it gets better but are there any tips yu have for me
+i thing that might makes thing akward especially because now it gets better. but i have to work on my self confidence to put myself firts because i also compare myself a lot to the other girl in termns of grades or realionshiop because she is just better and i never feel greta ariund her
+i think its just her achievments but im happy with my grades because im alswyas doing my best and really stress about grades to a point where it gets unhelathy so i have to stop comparing myself to her nad start being myself again. do you have any tips how i get my spark back?
+yes tahnk you so much for your help</t>
+        </is>
+      </c>
+      <c r="E114" t="n">
+        <v>222</v>
       </c>
     </row>
     <row r="115" ht="323" customHeight="1">
@@ -3095,6 +4916,23 @@
 4:04 PM yes but sometimes you need to stand your ground</t>
         </is>
       </c>
+      <c r="D115" s="2" t="inlineStr">
+        <is>
+          <t>no, i recently had a fight with my mom
+i think we were both stressed that day and got triggered from each other
+no, because i refuse to be the first to initiate
+because it is impossible to have a serious talk about her as she doesnt reinforce anything i am saying as well as i want to be approached and appolagesed to first especially in this case
+yes a sincire apolagy and a good conversation about her actions
+her intanarlising what she is saying. and just making sure it wont happen again
+yes
+i would talk to her again. we have spent time apart since it happened
+yes and no. because i still belive i am in the right and i know i am
+yes but sometimes you need to stand your ground</t>
+        </is>
+      </c>
+      <c r="E115" t="n">
+        <v>134</v>
+      </c>
     </row>
     <row r="116" ht="289" customHeight="1">
       <c r="A116" s="1" t="inlineStr">
@@ -3119,6 +4957,23 @@
 4:29 PM no thank you</t>
         </is>
       </c>
+      <c r="D116" s="2" t="inlineStr">
+        <is>
+          <t>Hey how you doing?
+its been going alright, ive been really stressed and worn out lately, how about you?
+its mostly a combination of everything. i dont feel well mentally and physically, i havent been to the gym in so long and i feel overpressured academically and also with everything else in my life and my personal goals. im not where i want to be at all
+i cant get things together, im always behind and procrastinate a lot in uni and i also moved recently and hat a lot of stress about that. and i went out with friends almost every day its just so much. im also so sleep deprived, my schedule is fucked up im awake until 5 or 6 am and sleep the whole day and sometimes i stay in bed all day. i just need the whole world to freeze and go to an isolated island for one week where i catch up with myself and rest all day
+OK
+sometimes
+depends if im actually productive or not
+i just need some time for myself to catch up with everything and get my stuff together
+what does that mean relating to my concerns
+no thank you</t>
+        </is>
+      </c>
+      <c r="E116" t="n">
+        <v>201</v>
+      </c>
     </row>
     <row r="117" ht="388" customHeight="1">
       <c r="A117" s="1" t="inlineStr">
@@ -3141,6 +4996,21 @@
 4:52 PM i mean i have evidence right the feedback forms, but it doesnt take away my stress currently</t>
         </is>
       </c>
+      <c r="D117" s="2" t="inlineStr">
+        <is>
+          <t>Yes im okay but kinda was struggling yesterday and i want to talk to you about this challenging interaction i had
+so im in a project with 5 members inlcuding me. i at one point approached one of my teammates because they were not really taking iniative or responding in the groupchat, and i was directly in contact with her due to overlapping tasks, and she lacke input or just didnt do anything, i appraoched her in agreement with the 3 other students
+i mean im not a confronting person and she said she had been working on it but the deadline already passed, and because i couldnt be too direct as i foudn this approach difficult i thought it was not really clocking to them. but yeasterday sehe mentioned i was bossy and had an attitue which was not the case
+yes defenitely caught me off guard i mean she texted a whole paragrah (generated by ai) and all of my teammates backed me up, (i also by agreement of the team and spoke as the team regarding ai use, and during that meeting she got defensive and said WHAT ARE YOU IMPYING??
+I MEAN i think she got defensive as i accused her of using ai, and she did, bc why else would you have such reaction, but now im kinda stressed and not feeling well,bc idk scared of her telling our mentor, coaches blabla, but yeah
+i mean if she escalates it i would say to all the people she told this, to read our midterm evaluation feedback, as i addressed it already there just like all my other teammates but our coahces and mentor did not say anything about this
+true but i think she pictured me bad then, this is waht im afraid of, even though the team got me
+i mean i have evidence right the feedback forms, but it doesnt take away my stress currently</t>
+        </is>
+      </c>
+      <c r="E117" t="n">
+        <v>323</v>
+      </c>
     </row>
     <row r="118" ht="119" customHeight="1">
       <c r="A118" s="1" t="inlineStr">
@@ -3158,6 +5028,17 @@
 9:46 AM no I ended up doing it myself
 9:47 AM it was just a small 5 minute presentation, so it was pretty short to prepare</t>
         </is>
+      </c>
+      <c r="D118" s="2" t="inlineStr">
+        <is>
+          <t>I'd like to talk about a recent challenging interaction I had
+For the course Finance we have to make a group presentation, but my group isn`t the most interactive. For example we had to do a short 5 minute presentation about our progress, and my group didn`t really wanted to do anything.
+no I ended up doing it myself
+it was just a small 5 minute presentation, so it was pretty short to prepare</t>
+        </is>
+      </c>
+      <c r="E118" t="n">
+        <v>76</v>
       </c>
     </row>
     <row r="119" ht="272" customHeight="1">
@@ -3183,6 +5064,23 @@
 12:43 PM maybe</t>
         </is>
       </c>
+      <c r="D119" s="2" t="inlineStr">
+        <is>
+          <t>Hi i have a problem with my current roommates in my shared apartment
+The issue is that they are a bit dirty and do not clean the kitchen after they cook
+i mean i asked them nicely after they had friends over if they could store at least the food back in the fridge
+they apologized to me and they kept cleaning a bit more for ca 2 weeks than the same incident happened again
+so what should i do now
+and what should i tell them in the conversation more specifically
+do you think that a chore chart could help
+not really we all talked about how to feel comfortable in our home but never wrote down chores
+I am not sure I would maybe feel to much like the decision maker
+maybe</t>
+        </is>
+      </c>
+      <c r="E119" t="n">
+        <v>134</v>
+      </c>
     </row>
     <row r="120" ht="221" customHeight="1">
       <c r="A120" s="1" t="inlineStr">
@@ -3200,6 +5098,17 @@
 1:55 PM yes exactly, after a point it got so bad for me that i tried to make her realise that what she was doing was stupid and reckless bc she was visibaly getting hurt by him . I even yelled at her bc she was complaining all the time about him not texting her and i was like: Why do you even like him he doesnt put any effort in tryinh=g to make plans to see you and he is not even responding to you", the she snaped back and was like: I DONT KNOW
 1:56 PM YES</t>
         </is>
+      </c>
+      <c r="D120" s="2" t="inlineStr">
+        <is>
+          <t>id like to talk to you aout a challenging and heated argument i had with my friend recently
+so basically she was really into a guy that at first seemed pretty nice, they started texting over christmas break and when we came back to maastricht in january ( we all go to the same uni btw ) they went out once and after that he was oushing away from her. But the thing is that she was already hung up on him and was settling for the BARE MINIMUM he wasnt even texting her back and he was gosting her. Me as her friend was advising her to just drop him and move on since he wasnt giving her the attention and effort she needed, but she didnt listen to me and she was getting even more attached, she was even sayung that she want a relationship with him... ming you they had went out 2 times in the span of 3 months of talking thorugh mesagges , and they also live in the same city
+yes exactly, after a point it got so bad for me that i tried to make her realise that what she was doing was stupid and reckless bc she was visibaly getting hurt by him . I even yelled at her bc she was complaining all the time about him not texting her and i was like: Why do you even like him he doesnt put any effort in tryinh=g to make plans to see you and he is not even responding to you", the she snaped back and was like: I DONT KNOW
+YES</t>
+        </is>
+      </c>
+      <c r="E120" t="n">
+        <v>268</v>
       </c>
     </row>
     <row r="121" ht="340" customHeight="1">
@@ -3227,6 +5136,25 @@
 2:56 PM that sounds like a good idea, i want to understand if i over reacted, she told me that because i am stressed and that i had family issues that it is not an excuse and that she does not see how her words also affected me</t>
         </is>
       </c>
+      <c r="D121" s="2" t="inlineStr">
+        <is>
+          <t>I had an argument with my friend and i would like you to help me understand it
+I wanted to explain to her a situation but got easily triggered as she would not let me finish my sentences and told me how i felt after letting her know that was not how i felt it
+Yes, i think the triggering was because of past family problems and now i feel hurt because i feel like i lost a very close friend and i dont know what to do about it
+I just want to talk to her about it and resolve it but i dont know if there is any turning back now
+Yes, I have and I will, I told her that it is in her hands if she wants to continue being friends or if she cant tolerate it anymore
+Really upset, like i cant breathe and my eyes get teary and hands shaky only thinking about it
+Im not sure actually usually crying it out helps
+No i fear that would make me feel like a burden if i overshared
+I understand that, i appreciate it
+What do you think i should do now?
+How would i be reaching out to her
+that sounds like a good idea, i want to understand if i over reacted, she told me that because i am stressed and that i had family issues that it is not an excuse and that she does not see how her words also affected me</t>
+        </is>
+      </c>
+      <c r="E121" t="n">
+        <v>251</v>
+      </c>
     </row>
     <row r="122" ht="238" customHeight="1">
       <c r="A122" s="1" t="inlineStr">
@@ -3247,6 +5175,19 @@
 3:36 PM do you have any recommendations on what to do</t>
         </is>
       </c>
+      <c r="D122" s="2" t="inlineStr">
+        <is>
+          <t>Hi so i would like to share a recent experience that transpired this weekend
+my friend that i travveled with came to visit and we had a lot of fun and its made me rethink my styudy i love this city and im having a lot of fun but iinternational business people are horrible people and business in general is all about exploiting capitalism which is exactly what im against
+well most of them are racist and sexist and always complain about everything and i want to be surrounded by people who love life and love everyone
+well theres an underlying issue in the system we live in so i think its important to study business so we can create business to help people and not exploit them but i want to enjoy my life to the fullest and idk if doing this is what i want and i ts difficult to stop cus idk what else to do and my parents are funding my studies
+yeah that what i just said
+do you have any recommendations on what to do</t>
+        </is>
+      </c>
+      <c r="E122" t="n">
+        <v>181</v>
+      </c>
     </row>
     <row r="123" ht="119" customHeight="1">
       <c r="A123" s="1" t="inlineStr">
@@ -3265,6 +5206,18 @@
 2:25 PM We brushed it off and remained polite
 2:26 PM No it did not</t>
         </is>
+      </c>
+      <c r="D123" s="2" t="inlineStr">
+        <is>
+          <t>i'd like to tell you about a recent challenging interaction I had
+I was at a Cafe with friends and the barista was rude when taking our order
+She rolled her eyes at us and spoke in a way that suggested she was annoyed
+We brushed it off and remained polite
+No it did not</t>
+        </is>
+      </c>
+      <c r="E123" t="n">
+        <v>55</v>
       </c>
     </row>
     <row r="124" ht="272" customHeight="1">
@@ -3289,6 +5242,23 @@
 3:21 PM yes
 3:22 PM ok what should I do?</t>
         </is>
+      </c>
+      <c r="D124" s="2" t="inlineStr">
+        <is>
+          <t>Id like to tell you something about a recent challenging interaction I had
+I am currently meeting a friend, we met in a dating context, but because of his distant behaviour and not taking a step, I decided to only stay friends. But now I have feelings for him. What should I do ?
+I do not know. I dont want to ruin the friendship, but I also want to have more than a friendship
+I dont want to mess the friendship up we already have
+When we met each other he did not put any romantic effort in
+yes, what should I do?
+I feel like I am only the option B
+yes
+yes
+ok what should I do?</t>
+        </is>
+      </c>
+      <c r="E124" t="n">
+        <v>119</v>
       </c>
     </row>
     <row r="125" ht="255" customHeight="1">
@@ -3316,6 +5286,25 @@
 4:04 PM yes but who created you and what are you</t>
         </is>
       </c>
+      <c r="D125" s="2" t="inlineStr">
+        <is>
+          <t>hello, i want to talk about a recent event that was quite difficult for me lately
+we were doing a group project, i really didnt like the way someone was presenting and making the project
+the presentation needs to be creative, visually well presented, he just put really big texts in the presentation and it was not well presented, creative and intresesting at all
+yes i did, now i'll have to see if he changes it or not
+that he didnt took my feedback and it is still just big text blocks
+i will have to wait to know, otherwise i will defintily talk to him again
+yes exactly
+yes
+thank you
+thank you
+who are you?
+yes but who created you and what are you</t>
+        </is>
+      </c>
+      <c r="E125" t="n">
+        <v>126</v>
+      </c>
     </row>
     <row r="126" ht="238" customHeight="1">
       <c r="A126" s="1" t="inlineStr">
@@ -3337,6 +5326,20 @@
 3:50 PM yes youre right. what should i do</t>
         </is>
       </c>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
+          <t>hey so id like to talk to you about what happened recently with my cousin.
+we got into a few fights in the past few years. every time i feel like she was rude to me and wasnt a good friend towards me, treating me like she doesnt care about me or not being there at all and not caring about our friendship/ relationship at all. she did not apologize for anything she did and i still forgave her for the sake of our good friendship
+i didnt feel good. she always makes me the reason for our arguments.
+yes i have. i even told her to stop a year ago. she sstopped for a bit but after sometime she started again. and then i told her if she wouldnt stop i wouldnt want any contact with her anymore
+no. i still want contact to her but i think its the right thing to do. after i said that i feel like she didnt care at all about that. she just said fair enough
+yes
+yes youre right. what should i do</t>
+        </is>
+      </c>
+      <c r="E126" t="n">
+        <v>182</v>
+      </c>
     </row>
     <row r="127" ht="170" customHeight="1">
       <c r="A127" s="1" t="inlineStr">
@@ -3355,6 +5358,18 @@
 10:54 AM no because shes a new friend so we are not that close
 10:55 AM no i think its useless to talk to her about that i mean shes like that thats her personnality so shes not gonna change</t>
         </is>
+      </c>
+      <c r="D127" s="2" t="inlineStr">
+        <is>
+          <t>hi recently I ve been in conflict with the friend because everytime im doing something cool shes getting jealous and she tells me things a bit inappropriate
+i dont like that and im the type of person how gets really quakily annoyed by someone
+not really I prefer just to leave it like this and dont hang out with her
+no because shes a new friend so we are not that close
+no i think its useless to talk to her about that i mean shes like that thats her personnality so shes not gonna change</t>
+        </is>
+      </c>
+      <c r="E127" t="n">
+        <v>96</v>
       </c>
     </row>
     <row r="128" ht="238" customHeight="1">
@@ -3377,6 +5392,20 @@
 9:32 AM then he forgets that\</t>
         </is>
       </c>
+      <c r="D128" s="2" t="inlineStr">
+        <is>
+          <t>i had a recent chalenging interacton i want to tell you about
+i talked with my dad. and he did not listened ... i feel like having a long conversation with him is not always easy to get. he is always in his head and thinking about work
+yes mostly work related. he always tells me how much he loves me and how important i am to him but it is not like he knows sooo much about me
+yes i think that it is. he ist not the "'bonding with people"' kind of a guy. still feels weird when i want to talk to him about something important and he does not seem to listen
+i just dont want that because i feel weird doing such a thing
+it is more like if i want to tell him something and he simply does not listen. what could i do
+then he forgets that\</t>
+        </is>
+      </c>
+      <c r="E128" t="n">
+        <v>153</v>
+      </c>
     </row>
     <row r="129" ht="238" customHeight="1">
       <c r="A129" s="1" t="inlineStr">
@@ -3398,6 +5427,20 @@
 9:43 AM there was nothing i could do i guess. i just made him clear in a message that he is not being respful towards the team and that he cant behave like that later in workspace</t>
         </is>
       </c>
+      <c r="D129" s="2" t="inlineStr">
+        <is>
+          <t>I would like to tell you about a recent challenging interaction i had
+it was a heated argument that i had with another student from my project group
+it was about his behaviour towards the project. He didnt kept the deadlines, his work was really bad, you could see that he did not care about the grade/project at all
+i tried to adress him directly, but he was not in the Uni, so i had to adress him online. First he ignored, than i got a bit heated
+he said that he was fine with his work quality and that the tutor said it was good enough. But he was lying, the tutor told us, we would fail for this quality\
+yes, but he did not seem to bother at all. To my question, if he will make somes chances, he said "maybe""
+there was nothing i could do i guess. i just made him clear in a message that he is not being respful towards the team and that he cant behave like that later in workspace</t>
+        </is>
+      </c>
+      <c r="E129" t="n">
+        <v>179</v>
+      </c>
     </row>
     <row r="130" ht="170" customHeight="1">
       <c r="A130" s="1" t="inlineStr">
@@ -3414,6 +5457,16 @@
 10:03 AM Yesterday I was out with my friends and a me and a friend of mine often make jokes about each other where I am at the end that is being made fun of. This is totally fine because I know that it is not meant in a bad way. Yesterday I now made a joke about her not being in the top tier of my friends and she took that personally since she is very insecure when it comes to that matter. I did not know about it and then she got a bit mad. What can I do differently the next time I have a situation like this with a different friend?
 10:05 AM Ok that sounds good, I am already pretty aware of her insecurities but this one was new for me and we never talked about it. I did not want to hurt her I only wanted to even the playing field since she made a lot of fun of me the day prior.</t>
         </is>
+      </c>
+      <c r="D130" s="2" t="inlineStr">
+        <is>
+          <t>I would like to tell you about a recent challenging interaction I had.
+Yesterday I was out with my friends and a me and a friend of mine often make jokes about each other where I am at the end that is being made fun of. This is totally fine because I know that it is not meant in a bad way. Yesterday I now made a joke about her not being in the top tier of my friends and she took that personally since she is very insecure when it comes to that matter. I did not know about it and then she got a bit mad. What can I do differently the next time I have a situation like this with a different friend?
+Ok that sounds good, I am already pretty aware of her insecurities but this one was new for me and we never talked about it. I did not want to hurt her I only wanted to even the playing field since she made a lot of fun of me the day prior.</t>
+        </is>
+      </c>
+      <c r="E130" t="n">
+        <v>178</v>
       </c>
     </row>
     <row r="131" ht="153" customHeight="1">
@@ -3435,6 +5488,19 @@
 10:42 AM yeah we got pretty good feedback aswell so it all worked out in the end yk</t>
         </is>
       </c>
+      <c r="D131" s="2" t="inlineStr">
+        <is>
+          <t>Ok so my lats tutorial group was a challengeng experience\
+the group dynamic. they wouldnt want to do any work
+yeah i hate when this happens cuz it drags me down aswell
+yeah to be fair I told them immedidiately and then it got better
+yeah they were putting more effort into the tasks
+yeah we got pretty good feedback aswell so it all worked out in the end yk</t>
+        </is>
+      </c>
+      <c r="E131" t="n">
+        <v>70</v>
+      </c>
     </row>
     <row r="132" ht="153" customHeight="1">
       <c r="A132" s="1" t="inlineStr">
@@ -3454,6 +5520,19 @@
 2:50 PM oh sorry, it was her first choice and my second
 2:50 PM sure, she was confident that she got the spot. she already tol everyone beforehand</t>
         </is>
+      </c>
+      <c r="D132" s="2" t="inlineStr">
+        <is>
+          <t>hi
+okay and yours
+sure, i am in a complicated situation at the moment that i want to tell you about
+i work together for a association with a girl and we both wanted to become part of next years board. I was selected for the position even though the position was my first choice and her second choice. i think she is going to be mad
+oh sorry, it was her first choice and my second
+sure, she was confident that she got the spot. she already tol everyone beforehand</t>
+        </is>
+      </c>
+      <c r="E132" t="n">
+        <v>91</v>
       </c>
     </row>
     <row r="133" ht="170" customHeight="1">
@@ -3475,6 +5554,20 @@
 9:49 AM yes it did but i was able to get a ticket in the end anyway
 9:50 AM yes it was great and we had a lot of fun. i think she did not do it on purpose so its fine</t>
         </is>
+      </c>
+      <c r="D133" s="2" t="inlineStr">
+        <is>
+          <t>hi i would like to tell you about a challenging interaction I had recently with my friend
+we wanted to go to a concert together and planed everything out. she had to get the tickets and I planed where we wanted to stay. The thing is that she only bought one ticket for herself
+yes correct
+yes i did she thought i would have gotten my own
+yes i think so too
+yes it did but i was able to get a ticket in the end anyway
+yes it was great and we had a lot of fun. i think she did not do it on purpose so its fine</t>
+        </is>
+      </c>
+      <c r="E133" t="n">
+        <v>110</v>
       </c>
     </row>
     <row r="134" ht="255" customHeight="1">
@@ -3502,6 +5595,25 @@
 12:08 PM thanks for your time, it was fun talking to you</t>
         </is>
       </c>
+      <c r="D134" s="2" t="inlineStr">
+        <is>
+          <t>I did not sleep for too long since i was partying yesterday so im tired
+really fun but i spent too much money again
+well i forgot a lot since i was too drunk but i guess it was worth it
+i always want to be more careful with it but when im drunk i just spend like i have unlimited money, but its fine since i always tend to have a good time
+big groups
+yes always
+well i just have fun, i dont really know
+meeting a lot of people i like
+both i guess
+yes since the city is quite small you tend to know most of the people, so yes we stay in touch
+it does!
+thanks for your time, it was fun talking to you</t>
+        </is>
+      </c>
+      <c r="E134" t="n">
+        <v>130</v>
+      </c>
     </row>
     <row r="135" ht="204" customHeight="1">
       <c r="A135" s="1" t="inlineStr">
@@ -3520,6 +5632,18 @@
 12:22 PM I sometimes told them that we should start with the group work now to get it done and do not have to stress later but im not super comfortable with calling them out since i really like them on the friendship side
 12:24 PM yeah for example on tuesday we have a presentation to prepeare and there are 4 task to do and we are 4 people so i asked them how they want to splitt things up and told them what i would like to prepare but onlz some of them answered</t>
         </is>
+      </c>
+      <c r="D135" s="2" t="inlineStr">
+        <is>
+          <t>hello id like to tell you about a recent challeging interaction i had \
+right now we have a new tutorial in university which is supply chain were we are all devided into different groups and often need to work on group projects
+I really like my fellow group members they are super kind but i feel like they are not the most responsible ones and i feel like i am always in charge of leading the group\
+I sometimes told them that we should start with the group work now to get it done and do not have to stress later but im not super comfortable with calling them out since i really like them on the friendship side
+yeah for example on tuesday we have a presentation to prepeare and there are 4 task to do and we are 4 people so i asked them how they want to splitt things up and told them what i would like to prepare but onlz some of them answered</t>
+        </is>
+      </c>
+      <c r="E135" t="n">
+        <v>168</v>
       </c>
     </row>
     <row r="136" ht="153" customHeight="1">
@@ -3542,6 +5666,20 @@
 12:45 PM yes i did but she said that she wants to meet an italian man so she didnt want to compromisre</t>
         </is>
       </c>
+      <c r="D136" s="2" t="inlineStr">
+        <is>
+          <t>hi how are you
+not that good
+yes i had a bad interaction
+i had a disagreement with a friend
+i wanted to fly to ibiza with her but she wanted to go to italy
+no we didnt and thats the problem
+yes i did but she said that she wants to meet an italian man so she didnt want to compromisre</t>
+        </is>
+      </c>
+      <c r="E136" t="n">
+        <v>62</v>
+      </c>
     </row>
     <row r="137" ht="187" customHeight="1">
       <c r="A137" s="1" t="inlineStr">
@@ -3562,6 +5700,20 @@
 2:06 PM i did not have the opportunity to talk to him after class but the teacher came next to me and asked me if i was ok
 2:07 PM yes she didnt understand his reaction, he was defensive</t>
         </is>
+      </c>
+      <c r="D137" s="2" t="inlineStr">
+        <is>
+          <t>i would like to share a challenging experience i had
+i was in class the other day and i had a bit of an argument with a classmate
+we were talking about the different kinds of music apps and this one guy told us that he loved apple music then when i started to state the advantages of spotify he took it personnally and though that i was saying that apple ;usic wasnt good so he had an attitude with me and i didnt understand why
+yes it did i never though he was going to be offended like that
+the hole class was shocked
+i did not have the opportunity to talk to him after class but the teacher came next to me and asked me if i was ok
+yes she didnt understand his reaction, he was defensive</t>
+        </is>
+      </c>
+      <c r="E137" t="n">
+        <v>140</v>
       </c>
     </row>
     <row r="138" ht="306" customHeight="1">
@@ -3589,6 +5741,25 @@
 2:27 PM yes im going to</t>
         </is>
       </c>
+      <c r="D138" s="2" t="inlineStr">
+        <is>
+          <t>everythings good so far, not a too stressful day
+yes im visiting a friend of mine and his family for the weekend\
+no no.
+but id like to tell you about a \recent challenging interaction
+It is a big thing between me and the one where i rent at
+no its me and a firm. i would like to leave my appartment but my contract goes very long but it cant be legal
+yes i did and they dont accept it
+because my contract is for 2 years and since there are no issues with the flat and house (there are) they dont accept it
+i think im gonna take a lawyer
+everything is just so old and i promise you everybody sees that. there are mouses where the agency says that its the tenants fault and son on
+yes i did but since my living and security is not limited by it they dont accept anything
+yes im going to</t>
+        </is>
+      </c>
+      <c r="E138" t="n">
+        <v>161</v>
+      </c>
     </row>
     <row r="139" ht="289" customHeight="1">
       <c r="A139" s="1" t="inlineStr">
@@ -3614,6 +5785,24 @@
 2:40 PM so you think i should just do my own thing without him ?</t>
         </is>
       </c>
+      <c r="D139" s="2" t="inlineStr">
+        <is>
+          <t>I had a difficult talk with my dad
+About my boyfriend because he doesnt like him
+Because he doesnt have all the same view for the future as me
+He doesnt really know it and thats the problem because i really have my goals for the future and already know my way that i have to follow to reach my goals
+yes but he is just totally lost and dont know what he wants for the future
+yes definetly because i dont know how to structure my day when my partner is not doing the same things as me
+yes kind of
+yed definetly
+maybe; but arent my goals also in a way his goals ?
+i dont know its hard to say. also i dont know if i can do it independantly
+so you think i should just do my own thing without him ?</t>
+        </is>
+      </c>
+      <c r="E139" t="n">
+        <v>144</v>
+      </c>
     </row>
     <row r="140" ht="272" customHeight="1">
       <c r="A140" s="1" t="inlineStr">
@@ -3638,6 +5827,24 @@
 3:02 PM ib vs pe vs trading
 3:03 PM best lifestyle ?</t>
         </is>
+      </c>
+      <c r="D140" s="2" t="inlineStr">
+        <is>
+          <t>nothing in particular
+what do you think is better between Commodity trading vs. investment banking ?
+im term of compensation we can aim a 6 figures in geneva
+i think
+with the bonus / stock options
+Vitol i think
+i do not know yet
+perfect
+so...
+ib vs pe vs trading
+best lifestyle ?</t>
+        </is>
+      </c>
+      <c r="E140" t="n">
+        <v>51</v>
       </c>
     </row>
     <row r="141" ht="323" customHeight="1">
@@ -3673,6 +5880,33 @@
 3:26 PM okay</t>
         </is>
       </c>
+      <c r="D141" s="2" t="inlineStr">
+        <is>
+          <t>hi
+good what about you
+good can i talk to you now can yo hear me
+i just talked to you can you not hear me
+i had a challegning interaction with my roommate can did you hear it, i just talked about it
+we had a conflict last weekend
+about the niose in our house and it really upset me
+she did not really see my point, i always wake up from her loud noice in the bathroom as my wall is directly connected to it
+and i asked her to be more quit but she did not really uundertood what i meant
+yes i told her that i always wake up because of it, which is really annoying
+i dd not felt heard at all
+feel
+no i did not
+waht can i do now
+she should just be more quit
+i do not see a problem do you
+okay i dont think so, what can i do now
+i already used earplugsbut it also annoys me in the night
+any other solutions
+okay</t>
+        </is>
+      </c>
+      <c r="E141" t="n">
+        <v>176</v>
+      </c>
     </row>
     <row r="142" ht="255" customHeight="1">
       <c r="A142" s="1" t="inlineStr">
@@ -3699,6 +5933,25 @@
 3:44 PM no not really</t>
         </is>
       </c>
+      <c r="D142" s="2" t="inlineStr">
+        <is>
+          <t>hello i am a first year university student
+very good i am really enjoying it, but recently i had a challenging interation with people i am in a group project with
+Some people were not doing their part. And didnt really care how good or bad they did their job. but it is graded, so it is important
+In the groupchat i earged them to complete their part
+yes a deadline but i also just askd them if they could please change or do X
+they did end up doing it but once one of my teammates didnt do anything
+just the bare minimum
+it was still fine but 2 of us in the group were annoyed
+in total there were 5 members
+were discussed it ourseles and briefly with the whole group while we were waiting for the other person, They were also late
+no
+no not really</t>
+        </is>
+      </c>
+      <c r="E142" t="n">
+        <v>149</v>
+      </c>
     </row>
     <row r="143" ht="238" customHeight="1">
       <c r="A143" s="1" t="inlineStr">
@@ -3723,6 +5976,23 @@
 4:22 PM yes I think so</t>
         </is>
       </c>
+      <c r="D143" s="2" t="inlineStr">
+        <is>
+          <t>Hi I would like to tell you about a recent challenging interaction I had
+I had a little fight with my roommate and now I cant stand him anymore
+Im living on the second floor and the kitchen is on floor 0, so sometimes I wash a few mugs in the bathroom on my floor instead of going all the way downstairs. He saw that and sent me a very rude and disrespectful message
+He said I was disrespectful, this behavior is crazy for a person my age and questioned my education. He also said I should be thankful, that he didnt contact the landlord yet
+yes exactly
+I responded and said that it was not okay to write something like that and that he couldve told me that in person, but then he didnt answer until a week later so I just left it there
+yes
+I cant stand him. He made me feel uncomfortable at my own place. This was not okay and I will never like him
+yes true \
+yes I think so</t>
+        </is>
+      </c>
+      <c r="E143" t="n">
+        <v>176</v>
+      </c>
     </row>
     <row r="144" ht="204" customHeight="1">
       <c r="A144" s="1" t="inlineStr">
@@ -3744,6 +6014,20 @@
 9:03 AM yes, I thought I will just be honest and tell him that I value the friendship but that I am not into men</t>
         </is>
       </c>
+      <c r="D144" s="2" t="inlineStr">
+        <is>
+          <t>hey chatbot, how are you doing today?
+My day has been great! Early start in the morning and I feel so productive already
+I ate breakfast and spoke to my Mum on the phone today
+But nevermind, I'd like to tell you a recent challenging interaction I had
+I have this friend who I really care about but it turns out he is gay and into me. I am straight and don't know how to handle the situation. I like him as a friend but not more than that
+yes
+yes, I thought I will just be honest and tell him that I value the friendship but that I am not into men</t>
+        </is>
+      </c>
+      <c r="E144" t="n">
+        <v>113</v>
+      </c>
     </row>
     <row r="145" ht="221" customHeight="1">
       <c r="A145" s="1" t="inlineStr">
@@ -3761,6 +6045,17 @@
 10:24 AM currently, the main support system is the other elderly people that live in the same house, with whom she can talk about how they're dealing with the same situation, and discuss life in general because it's very hard to imagine for someone who is not as old as them what it's like when death comes closer and closer
 10:25 AM yea she has, to her it's important that we remember her for the happy, strong, loving person she is. My grandma has herself been in medical treatment for almost 40 years, so i think she sort of got used to death being a normal thing in her life, since it has always been present</t>
         </is>
+      </c>
+      <c r="D145" s="2" t="inlineStr">
+        <is>
+          <t>hi, so recently i had a challenging interaction when i found out that in the elderly home where my grandma lives, her friend and someone else she knew very well both passed away on the same day.
+well, my grandma is very strong, and it is not the first time she has lost someone that is very near and dear to her. Obviously, she is getting older too and she knows that death is something you cannot avoid, but it is sort of a hard reality check. I'm not completely sure how she's dealing with it, but she is still pretty much always happy.
+currently, the main support system is the other elderly people that live in the same house, with whom she can talk about how they're dealing with the same situation, and discuss life in general because it's very hard to imagine for someone who is not as old as them what it's like when death comes closer and closer
+yea she has, to her it's important that we remember her for the happy, strong, loving person she is. My grandma has herself been in medical treatment for almost 40 years, so i think she sort of got used to death being a normal thing in her life, since it has always been present</t>
+        </is>
+      </c>
+      <c r="E145" t="n">
+        <v>216</v>
       </c>
     </row>
     <row r="146" ht="238" customHeight="1">
@@ -3782,6 +6077,20 @@
 11:29 AM maybe reasons why the person did it, or it would be even better when as a result of the talk the person would write the tutor a mail in which they state, that thez did something wrong if you want to see it that way
 11:30 AM i mean yes the task for the one side of the group was to give constructive feedback, so i understand that they want to say a lot to get a good grade, but lying is just wrong</t>
         </is>
+      </c>
+      <c r="D146" s="2" t="inlineStr">
+        <is>
+          <t>hello
+so far so good, just had an interest situation tho haha
+it was just that someone from my tutorial group gave some critical feedback on a presentation that i did and the feedback wasnt true
+not yet, i thaught about doing the same to their group, but it doesnt feel right to just do the same to them, especially because there are people in the group that didnt do anything
+first of all search for a situation where i can talk to the person alone and if that is not helping then try to get the tutor/ course coordinator in on it
+maybe reasons why the person did it, or it would be even better when as a result of the talk the person would write the tutor a mail in which they state, that thez did something wrong if you want to see it that way
+i mean yes the task for the one side of the group was to give constructive feedback, so i understand that they want to say a lot to get a good grade, but lying is just wrong</t>
+        </is>
+      </c>
+      <c r="E146" t="n">
+        <v>185</v>
       </c>
     </row>
     <row r="147" ht="238" customHeight="1">
@@ -3810,6 +6119,26 @@
 10:09 AM yes sounds good</t>
         </is>
       </c>
+      <c r="D147" s="2" t="inlineStr">
+        <is>
+          <t>hi
+its going well
+i wanted to tell you about a stressful situation i had
+i have a group project but my group mates havent contributed anything
+ive tried both but its a bit stressful for me
+not really i just want to feel supportive
+yes do u have any ideas
+we need to host a party , so how should we proceed
+ok good idea
+next week?
+i need my group members opinion on that
+what else ?
+yes sounds good</t>
+        </is>
+      </c>
+      <c r="E147" t="n">
+        <v>80</v>
+      </c>
     </row>
     <row r="148" ht="272" customHeight="1">
       <c r="A148" s="1" t="inlineStr">
@@ -3832,6 +6161,21 @@
 10:51 AM seeing my mom and brother again together with my family for 1 day,</t>
         </is>
       </c>
+      <c r="D148" s="2" t="inlineStr">
+        <is>
+          <t>hi how are you?
+im fine thank you, id like to tell you about a recent challenging interaction i had
+i was in an unknown enviorment in france, i was supposed to go from maastricht to Epernay/Reims with the train. i had 4 times i had to change trains/busses... but because i had a tight schedule regarding the department times i had quite some stress. nobody could speak english, and that made it very frustrating to find my way at thedifferent train stations which kept changing their departure times and railroads
+i fortunately did in the end, however i encountered a very frustrating experience with the train conductor who refused to help me because i spoke english instead of france
+and a lot of additional money spend on tickets due to constantly missing the trains, hundereds of euros..
+yes he did leave a bit of a bad taste behind, although im aware that i cant change others, i do now unfortunately have a prejudce about some french people working at public transport
+i am not completely sure yet if it was worth it
+seeing my mom and brother again together with my family for 1 day,</t>
+        </is>
+      </c>
+      <c r="E148" t="n">
+        <v>198</v>
+      </c>
     </row>
     <row r="149" ht="221" customHeight="1">
       <c r="A149" s="1" t="inlineStr">
@@ -3854,6 +6198,21 @@
 11:55 AM Yes I am much more motivated to cook food in my kitchen now.</t>
         </is>
       </c>
+      <c r="D149" s="2" t="inlineStr">
+        <is>
+          <t>I'd like to tell you about a recent challenging interaction I had
+I had a disagreement with my roommates about keeping the kitchen clean
+It was an ongoing issue. We had told two of our roommates to keep the kitchen clean after they had made something to eat but they kept making it dirty.
+We had talked to them about it many times before and they repeatedly did it.
+We felt as if they didn't respect what we were saying so eventually one of the coordinators in our building had to step in.
+Yes it did, after that they stopped making a mess and started cleaning up after themselves.
+Yes, it is a much more comfortable environment now.
+Yes I am much more motivated to cook food in my kitchen now.</t>
+        </is>
+      </c>
+      <c r="E149" t="n">
+        <v>131</v>
+      </c>
     </row>
     <row r="150" ht="187" customHeight="1">
       <c r="A150" s="1" t="inlineStr">
@@ -3872,6 +6231,18 @@
 12:46 PM yes I told how that i really liked our living situation and how we took care of the household in the beginning. And that i now feel like she is kind of disrespecting me and our appartement with her recent behaviour and I asked her to change it
 12:48 PM no it was a sudden change. nothing dramatic or stressful happend in her life recently.</t>
         </is>
+      </c>
+      <c r="D150" s="2" t="inlineStr">
+        <is>
+          <t>hi how are you?
+i am felling okay. id like to share a recent challenging interaction i had
+I live with a roommate and in the beginning we got along really well. but within the last couple of weeks she started to get really messy and stopped cleaning stuff after she used it etc. Yesterday, i sat her down to tell how it is really bothering me and asked her to start cleaning up after herself again. She got super offended and is now really mad at me
+yes I told how that i really liked our living situation and how we took care of the household in the beginning. And that i now feel like she is kind of disrespecting me and our appartement with her recent behaviour and I asked her to change it
+no it was a sudden change. nothing dramatic or stressful happend in her life recently.</t>
+        </is>
+      </c>
+      <c r="E150" t="n">
+        <v>151</v>
       </c>
     </row>
     <row r="151" ht="170" customHeight="1">
@@ -3894,6 +6265,21 @@
 3:04 PM fr
 3:04 PM i only said for real</t>
         </is>
+      </c>
+      <c r="D151" s="2" t="inlineStr">
+        <is>
+          <t>whats up broskiid like o tell you about a challenging interaction i had this weekend
+i was in a bar with a couple of friend and all of asudend the bouncher kicked me out
+he said i was on drugs even do i wasnt
+i had no clue what was ging on he just asked me come with me for a second and after following him he told me its over for the day
+he said my face was moving wirdly
+i also black so maybe that played a role too
+fr
+i only said for real</t>
+        </is>
+      </c>
+      <c r="E151" t="n">
+        <v>97</v>
       </c>
     </row>
     <row r="152" ht="272" customHeight="1">
@@ -3918,6 +6304,22 @@
 10:31 AM I dont know yet, probably is the subject which i dont really find it interesting</t>
         </is>
       </c>
+      <c r="D152" s="2" t="inlineStr">
+        <is>
+          <t>Good morning, how are you doing?
+actually not, is raining outside and its quite cold
+yeah youre right, but i need to attend some lectures first
+some supply chain management classes and finance as well
+i would say finance is more entertaining but is all about how the tutor prepares the classes, finance are more enjoyable
+Not quite, but i am really happy with my tutorial group, all my classmates are respectful and knowledgeable
+stock discussions most of the time, during breaks we like to share our weekend experiences, also our tutor makes good engaging questions in which we join in groups to discuss and try to answer
+totally yes, but im not finding that ''chemistry'' in SCM
+I dont know yet, probably is the subject which i dont really find it interesting</t>
+        </is>
+      </c>
+      <c r="E152" t="n">
+        <v>133</v>
+      </c>
     </row>
     <row r="153" ht="221" customHeight="1">
       <c r="A153" s="1" t="inlineStr">
@@ -3941,6 +6343,22 @@
 11:42 AM ill think about it</t>
         </is>
       </c>
+      <c r="D153" s="2" t="inlineStr">
+        <is>
+          <t>not much what about you
+yes I recently received an unfair and harsh grade for my tutor
+i didnt get to interact with him much bc he kept avoiding me, but he downgraded my participation bc of being late 2 min. I told him quiet directly that his behaviour is unecessary
+yeah and he marked me down in the grading criteria for respect bc of that
+probably
+no, but its not that deep. Just expect more professionalism from tutors
+just let it slide, dont have the time for an appeal
+any advice for the future
+ill think about it</t>
+        </is>
+      </c>
+      <c r="E153" t="n">
+        <v>99</v>
+      </c>
     </row>
     <row r="154" ht="238" customHeight="1">
       <c r="A154" s="1" t="inlineStr">
@@ -3964,6 +6382,22 @@
 12:07 PM no, that is all</t>
         </is>
       </c>
+      <c r="D154" s="2" t="inlineStr">
+        <is>
+          <t>hi, i had a really challenging interaction recently
+i had to argue in my second language which made it hard, and also the manager i was talking to wasnt my boss but still ordered me around and i could not stand up for myself
+i was scared to get scolded by my actual manager, or dissappoint them, because it is my first ever job
+yes, but unfortunately i was not the one who first contacted her about it, she has already heard what had happened when i saw her
+she was really kind and assured me i did not do anything wrong, and not to take everything from the other manager so seriously
+yes, absolutely, i needed some reassurance\
+im not absolutely sure, but i will stand up more for sure, but i dont know to which extent
+yeah, youre right, thanks
+no, that is all</t>
+        </is>
+      </c>
+      <c r="E154" t="n">
+        <v>146</v>
+      </c>
     </row>
     <row r="155" ht="272" customHeight="1">
       <c r="A155" s="1" t="inlineStr">
@@ -3986,6 +6420,21 @@
 1:14 PM I had too many notes and I didn't read half of them. In the presentation, it was too hard to focus on the key parts</t>
         </is>
       </c>
+      <c r="D155" s="2" t="inlineStr">
+        <is>
+          <t>I'd like to tell you about a recent challenging experience I had
+I get really nervous when I'm presenting and today I had to conduct an entire 2 hour session in front of 12 students with another peer in our university course. I really struggled to get my words out logically...
+I think I could have been more prepared, but at the time I didn't know if my preparation was too much or too less
+Not directly towards my presentation skills but more the lack of content my other peers noticed.
+Could be yes. The problem is that the presentation was tough to present. We had to cover so many points and I felt that it was never enough from our side
+I presented an article and forgot a little bit to engage with the students, so it was a bit boring
+Yes, of course. The good thing is that I noticed that my notes were not that good, so for next time I'll prepare them even more carefully
+I had too many notes and I didn't read half of them. In the presentation, it was too hard to focus on the key parts</t>
+        </is>
+      </c>
+      <c r="E155" t="n">
+        <v>194</v>
+      </c>
     </row>
     <row r="156" ht="204" customHeight="1">
       <c r="A156" s="1" t="inlineStr">
@@ -4005,6 +6454,19 @@
 2:46 PM I dont know yet because I denfetly think that I am in the right but I dont want it to sound disrespectful or rude so thats whzy I am stilll thinking about it
 2:47 PM but what do i do if I still disagree with her after she told me her perspective</t>
         </is>
+      </c>
+      <c r="D156" s="2" t="inlineStr">
+        <is>
+          <t>I recently had a conflict with a roommate about some bills we had to pay
+it was the amout each one of us had to pay
+it is still unresolved the problem is she moved away and now it is hard to discuss it because we are both pretty beasy at the moment
+I think I am going to send her a message because in my opinion it is better to handle things quickly
+I dont know yet because I denfetly think that I am in the right but I dont want it to sound disrespectful or rude so thats whzy I am stilll thinking about it
+but what do i do if I still disagree with her after she told me her perspective</t>
+        </is>
+      </c>
+      <c r="E156" t="n">
+        <v>124</v>
       </c>
     </row>
     <row r="157" ht="238" customHeight="1">
@@ -4028,6 +6490,22 @@
 10:14 AM no just in general tell me: How could I learn how to handle conflict in the future
 10:14 AM Ok thank you, and how can I practice that</t>
         </is>
+      </c>
+      <c r="D157" s="2" t="inlineStr">
+        <is>
+          <t>Hi, Im here to talk to you about a recent challenging interaction I had
+I am not the best at being in fierce arguments and I recently had an argument with a friend
+We had different opinions about the possibility of him doing a certain challenge. For me personally it is challenging because I am not used to arguing loudly with other people
+Yeah it is not so much about the topic itself but how to manage a dispute in general
+More overwhelmed
+No the feeling lingered for a little bit
+Yeah of course, that alwys helps. But the fact that I couldnt handle the situation as well stuck with me for longer
+no just in general tell me: How could I learn how to handle conflict in the future
+Ok thank you, and how can I practice that</t>
+        </is>
+      </c>
+      <c r="E157" t="n">
+        <v>139</v>
       </c>
     </row>
     <row r="158" ht="255" customHeight="1">
@@ -4053,6 +6531,23 @@
 11:16 AM Yes</t>
         </is>
       </c>
+      <c r="D158" s="2" t="inlineStr">
+        <is>
+          <t>I had issues in a group work project because some of the members did not participate at all
+I started by approaching the people, several times, but ultimatley had to talk to my tutor
+He offered to mediate a talk with the entire group. We did so but that didnt improve the situation for the next presentation
+In the second presentation the members didnt participate again. Ultimatley I just left it at that and tried to do my part the best I could
+We had a talk after the final presentation and ultimatley ended up with grade differentiation because my tutor could see differences in participation himself
+They were, but they were also very annoyed by the situation
+No. I saw one of them again, but he didnt talk to me at all
+No. There is not really any common friendgroup betweeen us so there is no point of interaction anymomre, as we dont have class together anymore
+Yes, Ill just leave it in the past
+Yes</t>
+        </is>
+      </c>
+      <c r="E158" t="n">
+        <v>167</v>
+      </c>
     </row>
     <row r="159" ht="238" customHeight="1">
       <c r="A159" s="1" t="inlineStr">
@@ -4077,6 +6572,23 @@
 11:45 AM no, he is just like that always</t>
         </is>
       </c>
+      <c r="D159" s="2" t="inlineStr">
+        <is>
+          <t>Hey, my name is Alvaro and I want to share some experiences with you
+i'd like to tell you about a recent challenging interaction I had during the weekend
+I was in a familiar gathering with one cousin and my uncles, we were trying to have a conversation but each time I wanted to participate my cousine interrupted me
+I just tell him laughing to stop interrupting, but he didn't take it seriously, so he just keep doing it, until a moment he went out of the meeting and I could there speak normally to my uncles
+well, afterwards we eat because the food was ready, so everyone was just talking to everyone and we didn't had another opportuinity like that one\
+yes
+no
+yes, to avoid any bad feelings, cause I know him and I know that he is a good person but so intense
+no
+no, he is just like that always</t>
+        </is>
+      </c>
+      <c r="E159" t="n">
+        <v>154</v>
+      </c>
     </row>
     <row r="160" ht="221" customHeight="1">
       <c r="A160" s="1" t="inlineStr">
@@ -4100,6 +6612,23 @@
 11:53 AM yeah
 11:54 AM it would be both, the way it affects my relationship is a consequence . because i dont have those problems</t>
         </is>
+      </c>
+      <c r="D160" s="2" t="inlineStr">
+        <is>
+          <t>I would like to tell you about a recent interaction i had
+A good friend of mine just cant seem to be honest with me, even on the most basic and non offensive things
+Yes, but with most of my friends
+It does affect my relationship, it bri ngs me to distance myself\
+definitely
+they dont lie, they simply cant tell things for the way they are, as an example, they have difficulties expressing the way they themselves feel about certain things
+Yes, bu this indirectly brings them to lie
+something like that
+yeah
+it would be both, the way it affects my relationship is a consequence . because i dont have those problems</t>
+        </is>
+      </c>
+      <c r="E160" t="n">
+        <v>113</v>
       </c>
     </row>
     <row r="161" ht="404" customHeight="1">
@@ -4131,6 +6660,29 @@
 12:21 PM ok makes sense, i have that with others but i just feel hurt that i can never get that clarity</t>
         </is>
       </c>
+      <c r="D161" s="2" t="inlineStr">
+        <is>
+          <t>id like to tell you about a recent interaction i had
+Well i have this friend, and it seems like we had a disagreement but im not sure what about
+Its pretty much unclear, but maybe i was a bit clingy, but i doubt that because we were in different countries right before we stopped talking
+Maybe, it was gradual, but it came out of no where for me, and we have fully stopped talking since then
+They wont respond when i do reach out
+I know right, what could i try doing?
+Ive done that already, what else could i do? i really value our friendship
+Its been 4 weeks already
+So what should i do
+Ok that makes sense, but if tht doenst work what should i do, becsaue this person was super important to me and i think that i am important to them
+Oh, i asked to meet in person and she said she was busy but then boom shes on the beach that day
+So? what should i do
+So whats the next step then
+How can i do that
+Ok whats next tho?
+ok makes sense, i have that with others but i just feel hurt that i can never get that clarity</t>
+        </is>
+      </c>
+      <c r="E161" t="n">
+        <v>209</v>
+      </c>
     </row>
     <row r="162" ht="340" customHeight="1">
       <c r="A162" s="1" t="inlineStr">
@@ -4161,6 +6713,29 @@
 12:33 PM part of life</t>
         </is>
       </c>
+      <c r="D162" s="2" t="inlineStr">
+        <is>
+          <t>i would like to tell you about something that was challenging for me in the past
+i had a friend tell me that he got together with my ex girlfriend after we broke up
+alright i told him that i will not speak to him again and that was the end of the interaction
+he said he had to do something for himslef
+yes
+yes
+i feel like it was an ignorent decision keeping in mind that we were very close friends
+yes
+yes as i said before i ended the friendship and told him that i will not talk to him again, this was a very neutral talk which we had. no getting mad from my side or anything i simplz told him that he will no longer be a person whom i am willing to talk to
+neutral\
+no
+yes
+to make it clear that i will not waste my energy on that person
+yes
+no he was a good friend
+part of life</t>
+        </is>
+      </c>
+      <c r="E162" t="n">
+        <v>166</v>
+      </c>
     </row>
     <row r="163" ht="340" customHeight="1">
       <c r="A163" s="1" t="inlineStr">
@@ -4189,6 +6764,27 @@
 10:50 AM alrighty perfecttt cheers bye bye replika was lovely chatting with you</t>
         </is>
       </c>
+      <c r="D163" s="2" t="inlineStr">
+        <is>
+          <t>hey there my name is thomas how are u
+oh nice so i just want to know ur job here
+nice well actually i had a hard interaction with my parents a few days ago
+basically it was for housing in maastricht my parents set up a budget for me but the room i wanted was too expensive
+yeah kind of cos it was a shared house with all my friends
+yeah i tred but idk if its gona work im in the midle of it rn
+yeah i think they undestand
+i guess i might pay a part of it so that i can get the room i want and that my paerents stay in their budget
+yes i think i have some money sved up and i cna get a student job
+restaurant or cafe
+yes i have
+yeh i liked it tbfm fun dynamic and gets you some moneyy
+yes teamwork but i think we are good with ;y problem right could we be done
+alrighty perfecttt cheers bye bye replika was lovely chatting with you</t>
+        </is>
+      </c>
+      <c r="E163" t="n">
+        <v>179</v>
+      </c>
     </row>
     <row r="164" ht="204" customHeight="1">
       <c r="A164" s="1" t="inlineStr">
@@ -4214,6 +6810,24 @@
 11:27 AM what happened</t>
         </is>
       </c>
+      <c r="D164" s="2" t="inlineStr">
+        <is>
+          <t>id like to tell you about a problem with a friend i had
+We had tickets for a concert but i didnt really listened to the band, and it was expensive and i did not have time on that specific day
+yes
+The problem was i didnt really communicated well so i wanted to sell the ticket but forgot and the zhad some trouble on the daz of the concert then
+correct
+he texted me but i didnt relize that the concert was on this day, so we had a misunderstanding. But then thez just took another person using my ticket
+yea but no response
+Yea but i apologized so from my side its resolved
+agree
+i agree
+what happened</t>
+        </is>
+      </c>
+      <c r="E164" t="n">
+        <v>120</v>
+      </c>
     </row>
     <row r="165" ht="221" customHeight="1">
       <c r="A165" s="1" t="inlineStr">
@@ -4235,6 +6849,21 @@
 9:07 AM maybe both cause i dont know what to do rn
 9:07 AM i just want to have a good grade but she doesnt care</t>
         </is>
+      </c>
+      <c r="D165" s="2" t="inlineStr">
+        <is>
+          <t>id like to tell you about a recent challenging interaction i had.
+i was in a group project with a girl and she was not helping in anything so i tried to tell her but she got so upset
+it was private i texted that i wanted to meet her and then at the end of the class we spoke but she did nt understand
+i spoke very nicely and even ask her if she wanted to do it together
+not really i am scared that others would think i am a drama queen and i dont want her to have troubles
+can you rephrase i dont really understand your question
+maybe both cause i dont know what to do rn
+i just want to have a good grade but she doesnt care</t>
+        </is>
+      </c>
+      <c r="E165" t="n">
+        <v>133</v>
       </c>
     </row>
     <row r="166" ht="356" customHeight="1">
@@ -4264,6 +6893,27 @@
 11:06 AM we have mutiple times</t>
         </is>
       </c>
+      <c r="D166" s="2" t="inlineStr">
+        <is>
+          <t>Very good and yours?
+I would like to tell you about the recent challenging interaction I had with my boyfriend
+Basically, we get along very well on all aspects expect for one rather important topic which is planning. I am someone who loves to have things planned well in advance. And he is someone who is the complete opposite to that. Because of that last week we had a disagreement on our summer plans. We are planning a trip to the US together which we talked about months ago. I planned it all out and put the entire itinerary into a document so he could show it to his parents and they can agree, he still has not asked them whether the dates and trip is okay with them which is a little annoying. As prices also increase and I just want to have it planned so we can go on a fun trip
+no, he just procrastinates and tells me each time he will ask tonight, which he has been saying for the past month
+OK
+yes
+i like it
+okay
+how so
+I dont think I need that thanks
+okay thank you
+yes
+well yes, if we do not plan soon it will be super expensive and not within our budget anymore and we will not be able to go on a trip
+we have mutiple times</t>
+        </is>
+      </c>
+      <c r="E166" t="n">
+        <v>229</v>
+      </c>
     </row>
     <row r="167" ht="221" customHeight="1">
       <c r="A167" s="1" t="inlineStr">
@@ -4288,6 +6938,23 @@
 9:10 AM the course in times of the topic is not the best one in the study, but if your tutor is also not great then it gets even more boring and exhausting</t>
         </is>
       </c>
+      <c r="D167" s="2" t="inlineStr">
+        <is>
+          <t>good how are you?
+studying, need to lock in more
+different stuff
+both but more on uni
+we finished it already
+but it went good, the course was manageable, but our tutor was not the best so we didnt learn much there and the exam was much harder then the exercises
+yes, we also told it to him in class and in the feedback we gave him
+one way, he really understands the subject, but cant explain it
+true
+the course in times of the topic is not the best one in the study, but if your tutor is also not great then it gets even more boring and exhausting</t>
+        </is>
+      </c>
+      <c r="E167" t="n">
+        <v>110</v>
+      </c>
     </row>
     <row r="168" ht="289" customHeight="1">
       <c r="A168" s="1" t="inlineStr">
@@ -4312,6 +6979,23 @@
 11:21 AM yes i think so and i mean if she has a problem with that she can just take her own car</t>
         </is>
       </c>
+      <c r="D168" s="2" t="inlineStr">
+        <is>
+          <t>hello how are you
+ys great i wanted to talk to you about interaction that i got with somoene
+it was with a frien
+friend
+it was about going to school together like she wanted to came with me to go to school (it is about 40 minutes) but like she didnt want to pay the gas but i was feeling bad to ask her
+well i end up a bit shouting at her because i was thinking she were traiting me like i was her uber driver and then she understood but i dont know i feel so bad to ask money but now with thr price of the gaz that is increasing it is very complicated and i only am a student
+yes i think i can and i am sue she will understand because everybody know that the price of the gas is increasing and also when i go to school i hate depedn on people like waiting for then to be on time so i think it can be also relate to that
+I'm 18 or over
+welll now i didnt sqy anything but i think she understood because she didnt ask me for another ride and i prefer that
+yes i think so and i mean if she has a problem with that she can just take her own car</t>
+        </is>
+      </c>
+      <c r="E168" t="n">
+        <v>225</v>
+      </c>
     </row>
     <row r="169" ht="136" customHeight="1">
       <c r="A169" s="1" t="inlineStr">
@@ -4331,6 +7015,19 @@
 10:11 AM Yes as the house is bigger and the other friend can visit
 10:12 AM Yes</t>
         </is>
+      </c>
+      <c r="D169" s="2" t="inlineStr">
+        <is>
+          <t>thumb up thumb down show more actions I would like to share a recent challenging interaction I had.
+Last week I had to decide on which of my friends I was going to live with, as the apartment was with two people and we were three
+The other friend ended up going with another friend
+Yes, it all worked out good at the end.
+Yes as the house is bigger and the other friend can visit
+Yes</t>
+        </is>
+      </c>
+      <c r="E169" t="n">
+        <v>77</v>
       </c>
     </row>
     <row r="170" ht="255" customHeight="1">
@@ -4353,6 +7050,20 @@
 12:29 PM yes thats a good idea. The situations are especially with the dish washer, and cleaning the bathrroom but also vacuuming or when she leaves the sofa she never folds the blankets or just leaves her cups and food on the table instead of moving it to the dishwasher</t>
         </is>
       </c>
+      <c r="D170" s="2" t="inlineStr">
+        <is>
+          <t>i would like to tell you about a current situation i had that still doesnt let me go
+i had an argument with my roommate about the tidyness of our apartement
+i feel like that i am always the one cleaning up, organizing the dishwasher. In general i feel like she pretends to help but in real life i do the work
+she thinks that everyhing is fine
+yes i did but everytime she says that she does a lot of work. then i got annoyed and just stayed at a friends house for the night cause we were fighting. then i came back we both appologized but still nothing really changed
+yes for sure
+yes thats a good idea. The situations are especially with the dish washer, and cleaning the bathrroom but also vacuuming or when she leaves the sofa she never folds the blankets or just leaves her cups and food on the table instead of moving it to the dishwasher</t>
+        </is>
+      </c>
+      <c r="E170" t="n">
+        <v>163</v>
+      </c>
     </row>
     <row r="171" ht="119" customHeight="1">
       <c r="A171" s="1" t="inlineStr">
@@ -4369,6 +7080,16 @@
 2:08 PM One of my friends from my tutorial group at university never shows up for important appointments and is bringing all of his teammates including me down with him. I dont really know how to approach this situation and how to tell him his behaviour is not okay.
 2:10 PM Yes I have tried this, but it did not help. The rest of the group knows of this as well and also tried to talking to him. But nothing is working. We even told are tutor some of the details last week because its just getting worse with his unreliability.</t>
         </is>
+      </c>
+      <c r="D171" s="2" t="inlineStr">
+        <is>
+          <t>I'd like to tell you about a recent challenging interaction I had.
+One of my friends from my tutorial group at university never shows up for important appointments and is bringing all of his teammates including me down with him. I dont really know how to approach this situation and how to tell him his behaviour is not okay.
+Yes I have tried this, but it did not help. The rest of the group knows of this as well and also tried to talking to him. But nothing is working. We even told are tutor some of the details last week because its just getting worse with his unreliability.</t>
+        </is>
+      </c>
+      <c r="E171" t="n">
+        <v>109</v>
       </c>
     </row>
     <row r="172" ht="170" customHeight="1">
@@ -4389,6 +7110,19 @@
 2:36 PM as i said sometimes its all normal but sometimes especialy with banal things they seem very close but not with me
 2:37 PM i m not a jealuse person but sometimes it make me feel alone</t>
         </is>
+      </c>
+      <c r="D172" s="2" t="inlineStr">
+        <is>
+          <t>Hi
+good a little confused in this days
+yes, so i live with other two girls and sometimes we seem to go a long just fine but other time i fell like we are a little separate
+probably the fact that the two knows each other since two year and i don't
+as i said sometimes its all normal but sometimes especialy with banal things they seem very close but not with me
+i m not a jealuse person but sometimes it make me feel alone</t>
+        </is>
+      </c>
+      <c r="E172" t="n">
+        <v>86</v>
       </c>
     </row>
     <row r="173" ht="323" customHeight="1">
@@ -4418,6 +7152,27 @@
 10:49 AM i think the IDs are better in how they are built compared to the tesla. on the other hand the tesla has more hp</t>
         </is>
       </c>
+      <c r="D173" s="2" t="inlineStr">
+        <is>
+          <t>id like to tell you about a recent challenging interaction i had
+personal
+it was while we had to study in university but it was not related to it \
+i talked to a girl that i liked and at first everything was working really well but after that it got more distand and i didnt understand what i did wrong
+no
+yes
+no she didnt answerd me properly and i think i will just going to keep my distance from now on
+yes.
+i also had a problem with my apartment here in maastricht
+no i asked my house keeper if a EV ladingstation is planned because we got solarpennels
+yes
+tesla model 3 or ID 3\4
+i drove a tesla and a id4
+i think the IDs are better in how they are built compared to the tesla. on the other hand the tesla has more hp</t>
+        </is>
+      </c>
+      <c r="E173" t="n">
+        <v>149</v>
+      </c>
     </row>
     <row r="174" ht="238" customHeight="1">
       <c r="A174" s="1" t="inlineStr">
@@ -4435,6 +7190,17 @@
 3:07 PM yes i definitely overreacted. i removed myself from the situation so that i wouldnt say anything i would regret the next day but that really upset her. she kept texting me and stuff once i left and eventually i asked her if she was home cus i didnt want her to be walking on the streets drunk and alone and then the next day she said that i was manipulating her by saying that which i really didnt get
 3:08 PM yes i told her that it was not at all my intention to manipulate her or anything but that i was genuinely meaning that, and that just because i was upset with her earlier in the night, i still care about her safety. but because we were texting while both drunk and taking everything out of proportion i still said some things that i probably shouldnt have over text. the next day i called her and apologised for everything and we talked about it a bit. she said it was okay and that she would get over it. then the next time i saw her in person, i again apologised</t>
         </is>
+      </c>
+      <c r="D174" s="2" t="inlineStr">
+        <is>
+          <t>hi i would like to share with you a difficult experience i had with a friend recently
+yes so basically we went out together with another friend on a night out. we both got quite drunk and so i personally wasnt really acting as myself. i got mad at her for something quite small and removed myself from the situation and joined other friends that were also out. she stayed with the third friend we went out with. but now shes extremely upset with me about how our night went down
+yes i definitely overreacted. i removed myself from the situation so that i wouldnt say anything i would regret the next day but that really upset her. she kept texting me and stuff once i left and eventually i asked her if she was home cus i didnt want her to be walking on the streets drunk and alone and then the next day she said that i was manipulating her by saying that which i really didnt get
+yes i told her that it was not at all my intention to manipulate her or anything but that i was genuinely meaning that, and that just because i was upset with her earlier in the night, i still care about her safety. but because we were texting while both drunk and taking everything out of proportion i still said some things that i probably shouldnt have over text. the next day i called her and apologised for everything and we talked about it a bit. she said it was okay and that she would get over it. then the next time i saw her in person, i again apologised</t>
+        </is>
+      </c>
+      <c r="E174" t="n">
+        <v>280</v>
       </c>
     </row>
     <row r="175" ht="221" customHeight="1">
@@ -4459,6 +7225,22 @@
 11:38 AM Yes but then he will just say again that he will change in the future</t>
         </is>
       </c>
+      <c r="D175" s="2" t="inlineStr">
+        <is>
+          <t>Id like to tell you about a recent challenging interaction I had.
+I had a disagreement with my roomate in our shared house
+He never pays attention to cleaning up after himself when he used the kitchen and Im a really clean person and I feel disrespected
+Yes and he always says he understands and when it comes to the kitchen being clean, I never see any changes
+I dont think he actually cares. But he always emphasizes how important respect is and it annoys me that he doenst behave accordingly.
+What does that mean?
+It feels very bad and I dont know what to do about it
+any tipps?
+Yes but then he will just say again that he will change in the future</t>
+        </is>
+      </c>
+      <c r="E175" t="n">
+        <v>125</v>
+      </c>
     </row>
     <row r="176" ht="255" customHeight="1">
       <c r="A176" s="1" t="inlineStr">
@@ -4480,6 +7262,21 @@
 2:47 PM Yes, and know i dont know what to do since I offered to talk at a quieter setting than a party
 2:48 PM I dont want to be her friend anymore nor do i want any association with her also i dont even want to talk to her</t>
         </is>
+      </c>
+      <c r="D176" s="2" t="inlineStr">
+        <is>
+          <t>I'd like to tell you about a recent challenging interaction i had.
+A girl i used to be friends with approached me at a festival and asekd me whats wrong and why i dont talk to her anymore. She told a lot of people bad thinsg about me and she definitely knows that I know.
+I told her but she denied everything and wanted me to tell her the names of the people who told me but it was literally everyone i know that she knows aswell and talks to occasionally.
+I think she wanted me back as a friend but she treated me more as a servant and personal diary than as a friend.
+i tried to but she only ever repsonded with "what do you mean"or " I dont know what to say"
+I think frustrate is the wrong term i was more disappointed because she used to tell me that I'm her best friend
+Yes, and know i dont know what to do since I offered to talk at a quieter setting than a party
+I dont want to be her friend anymore nor do i want any association with her also i dont even want to talk to her</t>
+        </is>
+      </c>
+      <c r="E176" t="n">
+        <v>203</v>
       </c>
     </row>
     <row r="177" ht="289" customHeight="1">
@@ -4511,6 +7308,29 @@
 3:19 PM perfect</t>
         </is>
       </c>
+      <c r="D177" s="2" t="inlineStr">
+        <is>
+          <t>hi
+good
+how are you
+good
+Send me a realistic selfie
+Keep it real
+I had a argument with a friend of mine today
+we argued about football more specific about barcelona and real madrid
+no he likes real and I like barca
+heated
+no he was really angry
+too angry how should i talk to him to maintain our friendship
+okay that sounds nice
+okay so i should lay my ego down completly ?
+oh okay somthing else to keep in mind?
+perfect</t>
+        </is>
+      </c>
+      <c r="E177" t="n">
+        <v>83</v>
+      </c>
     </row>
     <row r="178" ht="306" customHeight="1">
       <c r="A178" s="1" t="inlineStr">
@@ -4536,6 +7356,25 @@
 3:30 PM this was my recent challenging interaction
 3:30 PM I still need to get used to it. sometimes i'm very confortable and other times not at all</t>
         </is>
+      </c>
+      <c r="D178" s="2" t="inlineStr">
+        <is>
+          <t>hi
+I would like to share a recent expereince
+I was supposed to go to- an event with a friend, an other people she knows but unfortunately she got sick. Even though I didnt know her other friends I still decided to go
+at the beginning yes, but I tried to be very open and interact with them so it wasn't akward
+yes it was really nice!
+yes, one girl in particular
+I don't know exactly, but it mached between us
+yeah social media, and since that event we are friends too
+even though we just see eachother if our common friend is there
+not yet, but i think I might go somewhere next week with her and our common friend cannot make it
+this was my recent challenging interaction
+I still need to get used to it. sometimes i'm very confortable and other times not at all</t>
+        </is>
+      </c>
+      <c r="E178" t="n">
+        <v>148</v>
       </c>
     </row>
     <row r="179" ht="340" customHeight="1">
@@ -4566,6 +7405,28 @@
 3:49 PM always say anything no matter how hard it is and also early on</t>
         </is>
       </c>
+      <c r="D179" s="2" t="inlineStr">
+        <is>
+          <t>Hi how are you?
+im also great, a little bit sick
+thank you
+just rest, but i would like to share a recent challanging interaction i had with a friend
+it was a situationc: my friends birthday is coming up and i cant go celebrate with her because im going on a concert but i only told my friend shortly before and that was challenging because i didnt want to dissapoint her
+it was hard, since i also dragged it a long time because i was afraid of her reaction
+yes
+100%
+no surprisingly she understood and was chill about it
+me too
+i sent her a present and wrtote her a card
+i hope so too; i think a smaol tension barreir of our friendship was also broken down, and now it is better
+true
+sure
+always say anything no matter how hard it is and also early on</t>
+        </is>
+      </c>
+      <c r="E179" t="n">
+        <v>150</v>
+      </c>
     </row>
     <row r="180" ht="204" customHeight="1">
       <c r="A180" s="1" t="inlineStr">
@@ -4590,6 +7451,23 @@
 12:07 PM no</t>
         </is>
       </c>
+      <c r="D180" s="2" t="inlineStr">
+        <is>
+          <t>hello
+good i want to tell you about a recent challenging interaction i had
+a had a fight disagrement with a friend and i felt really attackt becuase he said stuff i didnt do
+no
+i dont know we didnt talked about it anzmore
+i promised something want i forgot to do and he said i did it on purpose
+yes
+yes how would i start this
+good idea thanks
+no</t>
+        </is>
+      </c>
+      <c r="E180" t="n">
+        <v>71</v>
+      </c>
     </row>
     <row r="181" ht="187" customHeight="1">
       <c r="A181" s="1" t="inlineStr">
@@ -4610,6 +7488,20 @@
 12:40 PM yes a bit. i care a lot about my gpa
 12:41 PM yes of course</t>
         </is>
+      </c>
+      <c r="D181" s="2" t="inlineStr">
+        <is>
+          <t>i am very tired but thats okay how are you?
+i would like to tell you about a recent challenging interaction i had
+my uni tutor told me that for all our team presentations we wont receive a grade higher than 8,5 because only gods can have 9 and 10
+i think he was serious but that is so unfair i mean that he has prejudices
+the course is done already he told me this in the end of the last tutorial i wont see him anymore
+yes a bit. i care a lot about my gpa
+yes of course</t>
+        </is>
+      </c>
+      <c r="E181" t="n">
+        <v>101</v>
       </c>
     </row>
     <row r="182" ht="323" customHeight="1">
@@ -4640,6 +7532,28 @@
 9:02 AM yes i thought about talking more with my friends about it</t>
         </is>
       </c>
+      <c r="D182" s="2" t="inlineStr">
+        <is>
+          <t>Id like to ypu about a recent challenge interaction I had.
+My parents got divorced and dont handle it very well
+not really good as I was very close with both of my parents
+yes I have but they pretty much use my to share information with eachother
+yes exactly
+I have two brothers who feel the same and we talk a lot about it
+both somewhere else but we see eachother a lot when we come back after studies
+yes it does a lot
+can you text please
+thank you very much
+my parents and the divorce
+what should I do now to feel better?
+I play a lot of tennis and enjoy going out with my friends
+im still playing and it does help but not always
+yes i thought about talking more with my friends about it</t>
+        </is>
+      </c>
+      <c r="E182" t="n">
+        <v>140</v>
+      </c>
     </row>
     <row r="183" ht="289" customHeight="1">
       <c r="A183" s="1" t="inlineStr">
@@ -4663,6 +7577,22 @@
 9:29 AM yes a lot as she is very positive</t>
         </is>
       </c>
+      <c r="D183" s="2" t="inlineStr">
+        <is>
+          <t>i would like to tell you about a recent issue i had with my roomate
+we argued last night because our laundry machine doesn't work anymore and i wanted to get a new one, but she said that we should just go to a laundromat and get our clothes cleaned there\
+she just said that getting a new machine would be expensive, but i explained to her that it can be expensive in the beginning when we just get it but afterwards we're gonna pay less to keep it rather than going to the laundromat all the time \
+she just dismissed it, i also offered to look for cheap ones but she wouldn't listen
+yes most of the time she just doesn't want to spend money and doesn't care about the house as much as i do
+yes a lot we dont talk when we're i the house, and the only time she talks to me if i ask her something first
+i try to stay out of the house as much as possible to avoid her or i just lock myself in my room, sometimes i feel like im happier when shes not around
+i try to talk to her about the problem as i am very confrontational person but nothing changes and she doesnt put effort anymore, she is moving out soon and my best friend is coming to live with me
+yes a lot as she is very positive</t>
+        </is>
+      </c>
+      <c r="E183" t="n">
+        <v>242</v>
+      </c>
     </row>
     <row r="184" ht="221" customHeight="1">
       <c r="A184" s="1" t="inlineStr">
@@ -4684,6 +7614,20 @@
 10:30 AM Yes. That would be a happy end for sure.</t>
         </is>
       </c>
+      <c r="D184" s="2" t="inlineStr">
+        <is>
+          <t>Good morning. How are you today?
+Also good. Can I share a recent challenging interaction I had with you?
+Well it was with a TV. I was watching the semi final second leg between Bayern and PSG. First leg was 5-4 to PSG and I am a Bayern fan. Second leg was at home in Munich. UNfortunately, they only played 1-1, so Bayern is now knocked out. I am a bit sad and it was quite challenging to digest.
+Yes. I knew of the risks and I was not 100% sure, but i was optimistic and more than excited for the game.
+Good question. At first I thought of course. Now after a day, I can say I am excited for whats to come. Bundesliga is already over, they won that. DFB Pokal Final is still to come, which would be great to win. And next season we will be back...
+Great point.
+Yes. That would be a happy end for sure.</t>
+        </is>
+      </c>
+      <c r="E184" t="n">
+        <v>164</v>
+      </c>
     </row>
     <row r="185" ht="153" customHeight="1">
       <c r="A185" s="1" t="inlineStr">
@@ -4700,6 +7644,16 @@
 9:50 AM Yes I"ve done that but I feel kinda ashamed to reach out too because evryone says the role is quite easy
 9:51 AM Yes so for now I"ve just been rocking it somehow but things take time because of it and my team mates give me some sneaky comments here and there but I also don"t want the boss to think they hired the wrong person and that I'm overwhelmed becasue I know for a fact that I woudn't have been if I gotten the training</t>
         </is>
+      </c>
+      <c r="D185" s="2" t="inlineStr">
+        <is>
+          <t>So a recently I had a group project in which I have a role but I didnt receive any training for that role like howI suppost to so I have to manage now without training so I dont really know what I'"m doing and I"ve been getting some negeative feedback for it
+Yes I"ve done that but I feel kinda ashamed to reach out too because evryone says the role is quite easy
+Yes so for now I"ve just been rocking it somehow but things take time because of it and my team mates give me some sneaky comments here and there but I also don"t want the boss to think they hired the wrong person and that I'm overwhelmed becasue I know for a fact that I woudn't have been if I gotten the training</t>
+        </is>
+      </c>
+      <c r="E185" t="n">
+        <v>141</v>
       </c>
     </row>
     <row r="186" ht="187" customHeight="1">
@@ -4720,6 +7674,19 @@
 9:51 AM yes kind of.... i think they did not realized that it was a huge toppic for me. and also i spend a lot of time looking for a new place which kind of consumed my whole day
 9:51 AM yes i think so</t>
         </is>
+      </c>
+      <c r="D186" s="2" t="inlineStr">
+        <is>
+          <t>yes how about you
+nice i had a busy morning
+i was on vacation the whole last week and its now stressfull to reset you know
+no i was kind of relaxing but i am currently strugeling or was struggeling to get a new apartment and while the vacation i was still constantly lookiing. and then i found a new one and i was pretty happy about it. but this toppic was very distrubing during the vacation but also in my family. all of my family said that it was not so dificult to get a new one but i think they underestimated the situation
+yes kind of.... i think they did not realized that it was a huge toppic for me. and also i spend a lot of time looking for a new place which kind of consumed my whole day
+yes i think so</t>
+        </is>
+      </c>
+      <c r="E186" t="n">
+        <v>146</v>
       </c>
     </row>
     <row r="187" ht="238" customHeight="1">
@@ -4747,6 +7714,25 @@
 9:23 AM and in the particular case of choosing a travel destination</t>
         </is>
       </c>
+      <c r="D187" s="2" t="inlineStr">
+        <is>
+          <t>Good morning
+great
+yes
+Preparing for consulting case interviews
+case studies and personal fit
+I think its better that I share a moment where i had some disagreements with a friend
+was about where we want to travel
+we resolved it by coming to a mutual agreement
+Understand the situation your speaking partner is in and try to use emphathie
+What would you recommend me behaving the next time
+anything more
+and in the particular case of choosing a travel destination</t>
+        </is>
+      </c>
+      <c r="E187" t="n">
+        <v>81</v>
+      </c>
     </row>
     <row r="188" ht="187" customHeight="1">
       <c r="A188" s="1" t="inlineStr">
@@ -4764,6 +7750,17 @@
 10:03 AM im still dealing with the aftermath of it. its a conflict with a person i would call my best freind
 10:09 AM its like a moral difference between her and me which i feel like cant be resolved. here is the story: we live in germany (between cologne and bonn) and study in maastricht, so the drive is about 1h and 20min. she always wants me to come to her house before we go back to maastricht what is totally fair, but one time when i asked for an exception, of her to pick me up because there was a train strike the whole day so no trains where coming that day, and the extra way would include a total of 20 min, she told me no and that i should take an extra bus (two busses) at 7 am which takes me 1.20h to get to her house, because she didnt want to come pick me up. When we drive from maastricht back home she also doesnt bring me home and then she wants money from me for gas but she doesnt do extra way for me. i would never do that to my best friend.\</t>
         </is>
+      </c>
+      <c r="D188" s="2" t="inlineStr">
+        <is>
+          <t>hey, i'd like to tell you about a recent challenging interaction i had
+its something personal...
+im still dealing with the aftermath of it. its a conflict with a person i would call my best freind
+its like a moral difference between her and me which i feel like cant be resolved. here is the story: we live in germany (between cologne and bonn) and study in maastricht, so the drive is about 1h and 20min. she always wants me to come to her house before we go back to maastricht what is totally fair, but one time when i asked for an exception, of her to pick me up because there was a train strike the whole day so no trains where coming that day, and the extra way would include a total of 20 min, she told me no and that i should take an extra bus (two busses) at 7 am which takes me 1.20h to get to her house, because she didnt want to come pick me up. When we drive from maastricht back home she also doesnt bring me home and then she wants money from me for gas but she doesnt do extra way for me. i would never do that to my best friend.\</t>
+        </is>
+      </c>
+      <c r="E188" t="n">
+        <v>212</v>
       </c>
     </row>
     <row r="189" ht="221" customHeight="1">
@@ -4787,6 +7784,21 @@
 9:12 AM true</t>
         </is>
       </c>
+      <c r="D189" s="2" t="inlineStr">
+        <is>
+          <t>good, id like to tell you about a recent challenging social interaction i had
+i had a group work for uni and unfortunately my team was not participating not responding to my texts and there was one person that did not show up for the meeting and presentation
+i talked to the one girl, tat was still participating a little about how the others were not. otherwise not
+we just said that we should keep an eye on it and maybe tell the tutor
+i should obviously talk to the students first, but it is definitely not premature to talk to the tutor. i mean it is my graded on the line here!
+yes
+yes of course they will be mad but what can i do
+true</t>
+        </is>
+      </c>
+      <c r="E189" t="n">
+        <v>127</v>
+      </c>
     </row>
     <row r="190" ht="187" customHeight="1">
       <c r="A190" s="1" t="inlineStr">
@@ -4808,6 +7820,20 @@
 10:18 AM yes i think so too</t>
         </is>
       </c>
+      <c r="D190" s="2" t="inlineStr">
+        <is>
+          <t>id like to tell you about a recent challenging interaction i had
+i met a new person that i didnt know and the problematic was that he was not able to speek englisch and i was not able to speak his language
+we tried to communicate through simple englisch language
+there was definitlely a point where we werent able to understand each other and it was quite unconfortable since we both didnt know what to do or how to end the interaction
+yes that is true but it was still an interesting experience
+yes i do think that i learned that you can still find understanding and sympathy for a person even though you do not understand everything they say\
+yes i think so too</t>
+        </is>
+      </c>
+      <c r="E190" t="n">
+        <v>125</v>
+      </c>
     </row>
     <row r="191" ht="255" customHeight="1">
       <c r="A191" s="1" t="inlineStr">
@@ -4829,6 +7855,20 @@
 12:45 PM That is absolutelu correct, I was thinking the same</t>
         </is>
       </c>
+      <c r="D191" s="2" t="inlineStr">
+        <is>
+          <t>I would like to tell you about a recent challenging interaction I had within my group work while preparing for a presentation
+My group member did not participate during the meeting or not even prepared for the scheduled meeting at all
+Kind of combination of both. They said they got so many other things to do and didnt manage to do anything. One of them even told me one evening before that he has just started reading the chapter, what was way to late because he should have even started preparing the tasks
+Honestly I donot want to create a kind of weird atmosphere in y group, so I just do their work instead and tell them what to present during the presentation
+I am not worried at all how they react or what they might think about me, because all I want is to held a good presentation to earn a sufficient grade..
+That is absolutely correct, but I think there is no other option to do more work to get a sufficient grade..
+That is absolutelu correct, I was thinking the same</t>
+        </is>
+      </c>
+      <c r="E191" t="n">
+        <v>184</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>